<commit_message>
Refresh scraped TradeIndia product data
Re-running the existing scrapers picked up more products now exposed
on TradeIndia's listing pages: clinical analyzers grew 61 -> 63, and
the four TradeIndia manufacturer listing sources grew from 3-5 products
each to 95-99. medicalexpo.com (source_03) remains blocked by an active
Cloudflare bot challenge and was left untouched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tradeindia_products.xlsx
+++ b/tradeindia_products.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Products" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Products'!$A$1:$U$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Products'!$A$1:$V$64</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U30"/>
+  <dimension ref="A1:V64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -442,6 +442,7 @@
     <col width="35" customWidth="1" min="19" max="19"/>
     <col width="35" customWidth="1" min="20" max="20"/>
     <col width="35" customWidth="1" min="21" max="21"/>
+    <col width="35" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -548,6 +549,11 @@
       <c r="U1" t="inlineStr">
         <is>
           <t>tests_performed</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>seller_phone</t>
         </is>
       </c>
     </row>
@@ -637,6 +643,7 @@
         </is>
       </c>
       <c r="U2" s="1" t="inlineStr"/>
+      <c r="V2" s="1" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -729,6 +736,7 @@
         </is>
       </c>
       <c r="U3" s="1" t="inlineStr"/>
+      <c r="V3" s="1" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -833,100 +841,97 @@
         </is>
       </c>
       <c r="U4" s="1" t="inlineStr"/>
+      <c r="V4" s="1" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Human Humastar 600 Automated Clinical Chemistry Analyzer - Dimension (L*w*h): 1000*740*1130 Mm</t>
+          <t>Fully Automated Biochemistry Analyzer</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>INORBVICT HEALTHCARE INDIA PVT. LTD.</t>
+          <t>PATHIMAGE INSTRUMENTS CO.</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>Human Humastar 600 Automated Clinical Chemistry Analyzer</t>
+          <t>Fully Automated Biochemistry Analyzer</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>https://www.tradeindia.com/products/human-humastar-600-automated-clinical-chemistry-analyzer-c10877025.html</t>
+          <t>https://www.tradeindia.com/products/fully-automated-biochemistry-analyzer-c10598070.html</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>https://cpimg.tistatic.com/10877025/b/4/Human-Humastar-600-Automated-Clinical-Chemistry-Analyzer.png</t>
+          <t>https://cpimg.tistatic.com/10598070/b/4/Fully-Automated-Biochemistry-Analyzer..jpg</t>
         </is>
       </c>
       <c r="F5" s="1" t="inlineStr"/>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>Routine clinical chemistry testing in medium to high-throughput laboratories</t>
+          <t>Hospital</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>Portable Biogas Analyzer - Accuracy: 2 %: https://www.tradeindia.com/products/portable-biogas-analyzer-c3391801.html
-Circuit Breaker Operational Analyzer - Automation Grade: Automatic: https://www.tradeindia.com/products/circuit-breaker-operational-analyzer-c11224952.html
-Sodium Analyzer Equipment: https://www.tradeindia.com/products/sodium-analyzer-equipment-c7911608.html
-Lightweight Meco 9009 Digital Solar Module Analyzer Equipment: https://www.tradeindia.com/products/solar-module-analyzer-1239923.html
-Circuit Breaker Analyzer Equipment: https://www.tradeindia.com/products/circuit-breaker-analyzer-equipment-587020.html
-Buchi Encapsulator B390, B395 - Application: Controlled Drug Delivery Systems: https://www.tradeindia.com/products/buchi-encapsulator-b390-b395-c10866048.html
-Bruker Ft-Nir Spectrometer Mpa Iii - Dimension (L*W*H): 70*50*100 Cm: https://www.tradeindia.com/products/bruker-ft-nir-spectrometer-mpa-iii-c10867804.html
-Bruker Tango Ft-Nir Spectrometer - Dimension (L*W*H): 49*42*29 Cm: https://www.tradeindia.com/products/bruker-tango-ft-nir-spectrometer-c10868572.html
-Sartorius Ambr 250 Modular - Dimension (L*W*H): 885*455* 600 Mm Millimeter (Mm): https://www.tradeindia.com/products/sartorius-ambr-250-modular-c10833593.html
-Sigma 4-16Ks Refrigerated Benchtop Centrifuge - Application: Clinical Diagnostics: https://www.tradeindia.com/products/sigma-4-16ks-refrigerated-benchtop-centrifuge-c10870007.html
-Qiastat-Dx Gastrointestinal Panel 2 - Application: Laboratory: https://www.tradeindia.com/products/qiastat-dx-gastrointestinal-panel-2-c9582175.html
-Sigma 3-30Khs Refrigerated And Heated Benchtop Centrifuge - Application: Cellular Biology: https://www.tradeindia.com/products/sigma-3-30khs-refrigerated-and-heated-benchtop-centrifuge-c10870486.html
-Tanner Scientific Cuttec S Sliding Microtome - Dimension (L*W*H): 450A A A 150A A A 200A Mm Micromete (Micron): https://www.tradeindia.com/products/tanner-scientific-cuttec-s-sliding-microtome-c10873453.html
-Hitachi Thermo Mechanical Analyzers (Tma): Tma7100 - Dimension (L*W*H): 545*295*430 Millimeter (Mm): https://www.tradeindia.com/products/hitachi-thermo-mechanical-analyzers-tma-tma7100-c10843894.html
-Sigma 4-5Krl Refrigerated Automated Centrifuge - Dimension (L*W*H): 655*570*489 Mm: https://www.tradeindia.com/products/sigma-4-5krl-refrigerated-automated-centrifuge-c10869336.html
-Biochemistry Analyzer Fully Automatic For Laboratory Use: https://www.tradeindia.com/products/biochemistry-analyzer-fully-automatic-for-laboratory-use-c10877154.html</t>
+          <t>White Bene Sphera C61 Semi Automatic Biochemistry Analyzer: https://www.tradeindia.com/products/bene-sphera-c61-semi-automatic-biochemistry-analyzer-c7839533.html
+Cst-180 Automatic Biochemistry Analyzer - Accuracy: 100 %: https://www.tradeindia.com/products/cst-180-automatic-biochemistry-analyzer-c11539500.html
+Semi Automatic Biochemistry Analyzer - CE Certified, 220V Voltage, Blue Color | 1 Year Warranty for Clinical Use: https://www.tradeindia.com/products/semi-automatic-biochemistry-analyzer-for-laboratory-and-clinical-use-7576255.html
+Semi Auto Biochemistry Analyzer - Plastic Material, 7-Inch TFT LCD Display, Grey Color | 8 Filters Including 700nm, Dual Mode Operation, Real-Time Reaction Graph, 2,00,000 Result Storage: https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-4856083.html
+Fully Automatic Biochemistry Analyzer - 150 to 300 Tests Per Hour | I.S.E. Module Options Available: https://www.tradeindia.com/products/fully-automatic-biochemistry-analyzer-1205665.html
+Ge Refurbished Ct Scan Machine - Application: Hospital: https://www.tradeindia.com/products/ge-refurbished-ct-scan-machine-c10598268.html
+Mammography X-Ray Machine - Application: Hospital: https://www.tradeindia.com/products/mammography-x-ray-machine-c10598228.html
+300 Ma X-Ray Machine - Color: White: https://www.tradeindia.com/products/300-ma-x-ray-machine-c10598224.html
+Bpl Biphasic Defibrillator - Application: Hospital: https://www.tradeindia.com/products/bpl-biphasic-defibrillator-copy-c10598248.html
+Portable Ultrasound Machine - Application: Hospital: https://www.tradeindia.com/products/portable-ultrasound-machine-c10598044.html
+0.3T Refurbished Hitachi VENTO LT MRI Machine - Open Design, White Color, Automatic Operation, Portable, 22 mT/m Amplitude, Warranty Included: https://www.tradeindia.com/products/0-3t-refurbished-hitachi-vento-lt-mri-machine-c10598168.html
+Hf Series X-Ray Machine - Application: Nursing Home: https://www.tradeindia.com/products/hf-series-x-ray-machine-c10598223.html
+100Ma X Ray Machine Console - Application: Hospital: https://www.tradeindia.com/products/100ma-x-ray-machine-console-c10598243.html
+Laparoscopic Co2 Insufflator - Application: Hospital: https://www.tradeindia.com/products/laparoscopic-co2-insufflator-c10598082.html
+Cd 25 Color Doppler - Attributes: Strong &amp; Durable: https://www.tradeindia.com/products/konica-minolta-cd-25-color-doppler-c10598111.html</t>
         </is>
       </c>
       <c r="I5" s="1" t="inlineStr">
         <is>
-          <t>INORBVICT HEALTHCARE INDIA PVT. LTD.</t>
+          <t>PATHIMAGE INSTRUMENTS CO.</t>
         </is>
       </c>
       <c r="J5" s="1" t="inlineStr"/>
       <c r="K5" s="1" t="inlineStr"/>
       <c r="L5" s="1" t="inlineStr">
         <is>
-          <t>INORBVICT HEALTHCARE INDIA PVT. LTD.</t>
+          <t>PATHIMAGE INSTRUMENTS CO.</t>
         </is>
       </c>
       <c r="M5" s="1" t="inlineStr">
         <is>
-          <t>INORBVICT HEALTHCARE INDIA PVT. LTD.</t>
+          <t>PATHIMAGE INSTRUMENTS CO.</t>
         </is>
       </c>
       <c r="N5" s="1" t="inlineStr">
         <is>
-          <t>At Inorbvict Healthcare India Pvt. Ltd. , we are passionate about delivering quality healthcare solutions to the world. As a dedicated exporter, we work closely with healthcare providers, hospitals, and institutions across the globe to supply reliable, advanced medical equipment that supports better patient care. We offer a wide range of products including Dental &amp; ENT equipment, OT &amp; ICU setups, Endoscopy systems, X-Ray and Ultrasound machines, NICU and Neurology tools, Radiology and Imaging equipment, Blood bank solutions, Dialysis machines, Dermatology and Ophthalmology equipment, Laboratory instruments, Cardiology devices, Respiratory care systems , and Operating Microscopes . What sets us apart is our commitment to quality, trusted brand associations, and a hands-on approach to every clienta s needs. Whether youa re setting up a new facility or expanding your services, wea re here to make global medical sourcing easier, faster, and more reliable. Business Type Exporter, Manufacturer Employee Count 50 Establishment 2014 Working Days Monday To Saturday GST NO 27AADCI6120M1ZH Payment Mode Others Certification ISO 9001:2015 Related Products Portable Biogas Analyzer - Accuracy: 2 % Price: 280000 INR MOQ - 1 Piece/Pieces Hnl Systems Pvt. Ltd. Mumbai, Maharashtra</t>
+          <t>n this fast pace life, people have completely neglected the care, a body needs to continue working. Toiling hard days and nights for materialistic things results in fatigued body, mind and spirit. A good health is the real secret to an eternal bliss and this understanding is the real reason behind formation of Pathimage Instruments Co. Our business enterprise is formed to make hospitals, clinics, medical research centers and laboratories have an impressive line of Medical Equipment. Business Type Supplier, Trading Company Employee Count 11 Establishment 2008 Working Days Monday To Saturday GST NO 19AAKFP4862D1Z0 Payment Mode Cheque/DD, Online Payments (NEFT/RTGS/IMPS), Cash Related Products White Bene Sphera C61 Semi Automatic Biochemistry Analyzer Price: 80000 INR MOQ - 1 Piece/Pieces Ambay Enterprises Kolkata, West Bengal</t>
         </is>
       </c>
       <c r="O5" s="1" t="inlineStr"/>
       <c r="P5" s="1" t="inlineStr"/>
       <c r="Q5" s="1" t="inlineStr">
         <is>
-          <t>https://www.tradeindia.com/inorbvict-healthcare-india-pvt-ltd-8372692/</t>
+          <t>https://www.tradeindia.com/pathimage-instruments-co-5057644/</t>
         </is>
       </c>
       <c r="R5" s="1" t="inlineStr"/>
       <c r="S5" s="1" t="inlineStr"/>
       <c r="T5" s="1" t="inlineStr">
         <is>
-          <t>Routine clinical chemistry testing in medium to high-throughput laboratories</t>
-        </is>
-      </c>
-      <c r="U5" s="1" t="inlineStr">
-        <is>
-          <t>Routine clinical chemistry testing in medium to high-throughput laboratories</t>
-        </is>
-      </c>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="U5" s="1" t="inlineStr"/>
+      <c r="V5" s="1" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -1017,6 +1022,7 @@
         </is>
       </c>
       <c r="U6" s="1" t="inlineStr"/>
+      <c r="V6" s="1" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -1111,6 +1117,7 @@
         </is>
       </c>
       <c r="U7" s="1" t="inlineStr"/>
+      <c r="V7" s="1" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -1214,6 +1221,7 @@
         </is>
       </c>
       <c r="U8" s="1" t="inlineStr"/>
+      <c r="V8" s="1" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -1309,129 +1317,41 @@
         </is>
       </c>
       <c r="U9" s="1" t="inlineStr"/>
+      <c r="V9" s="1" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Fully Automated Biochemistry Analyzer</t>
+          <t>Semi-automated Biochemistry Analyzer</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>PATHIMAGE INSTRUMENTS CO.</t>
+          <t>AISTECH GLOBAL PRIVATE LIMITED</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>Fully Automated Biochemistry Analyzer</t>
+          <t>Semi-automated Biochemistry Analyzer</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>https://www.tradeindia.com/products/fully-automated-biochemistry-analyzer-c10598070.html</t>
+          <t>https://www.tradeindia.com/products/biochemistry-analyzer-c10543245.html</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>https://cpimg.tistatic.com/10598070/b/4/Fully-Automated-Biochemistry-Analyzer..jpg</t>
+          <t>https://cpimg.tistatic.com/10543245/b/4/Semi-automated-Biochemistry-Analyzer.jpeg</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr"/>
       <c r="G10" s="1" t="inlineStr">
         <is>
-          <t>Hospital</t>
+          <t>ANLYZER</t>
         </is>
       </c>
       <c r="H10" s="1" t="inlineStr">
-        <is>
-          <t>White Bene Sphera C61 Semi Automatic Biochemistry Analyzer: https://www.tradeindia.com/products/bene-sphera-c61-semi-automatic-biochemistry-analyzer-c7839533.html
-Cst-180 Automatic Biochemistry Analyzer - Accuracy: 100 %: https://www.tradeindia.com/products/cst-180-automatic-biochemistry-analyzer-c11539500.html
-Semi Automatic Biochemistry Analyzer - CE Certified, 220V Voltage, Blue Color | 1 Year Warranty for Clinical Use: https://www.tradeindia.com/products/semi-automatic-biochemistry-analyzer-for-laboratory-and-clinical-use-7576255.html
-Semi Auto Biochemistry Analyzer - Plastic Material, 7-Inch TFT LCD Display, Grey Color | 8 Filters Including 700nm, Dual Mode Operation, Real-Time Reaction Graph, 2,00,000 Result Storage: https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-4856083.html
-Fully Automatic Biochemistry Analyzer - 150 to 300 Tests Per Hour | I.S.E. Module Options Available: https://www.tradeindia.com/products/fully-automatic-biochemistry-analyzer-1205665.html
-Ge Refurbished Ct Scan Machine - Application: Hospital: https://www.tradeindia.com/products/ge-refurbished-ct-scan-machine-c10598268.html
-Mammography X-Ray Machine - Application: Hospital: https://www.tradeindia.com/products/mammography-x-ray-machine-c10598228.html
-300 Ma X-Ray Machine - Color: White: https://www.tradeindia.com/products/300-ma-x-ray-machine-c10598224.html
-Bpl Biphasic Defibrillator - Application: Hospital: https://www.tradeindia.com/products/bpl-biphasic-defibrillator-copy-c10598248.html
-Portable Ultrasound Machine - Application: Hospital: https://www.tradeindia.com/products/portable-ultrasound-machine-c10598044.html
-0.3T Refurbished Hitachi VENTO LT MRI Machine - Open Design, White Color, Automatic Operation, Portable, 22 mT/m Amplitude, Warranty Included: https://www.tradeindia.com/products/0-3t-refurbished-hitachi-vento-lt-mri-machine-c10598168.html
-Hf Series X-Ray Machine - Application: Nursing Home: https://www.tradeindia.com/products/hf-series-x-ray-machine-c10598223.html
-100Ma X Ray Machine Console - Application: Hospital: https://www.tradeindia.com/products/100ma-x-ray-machine-console-c10598243.html
-Laparoscopic Co2 Insufflator - Application: Hospital: https://www.tradeindia.com/products/laparoscopic-co2-insufflator-c10598082.html
-Cd 25 Color Doppler - Attributes: Strong &amp; Durable: https://www.tradeindia.com/products/konica-minolta-cd-25-color-doppler-c10598111.html</t>
-        </is>
-      </c>
-      <c r="I10" s="1" t="inlineStr">
-        <is>
-          <t>PATHIMAGE INSTRUMENTS CO.</t>
-        </is>
-      </c>
-      <c r="J10" s="1" t="inlineStr"/>
-      <c r="K10" s="1" t="inlineStr"/>
-      <c r="L10" s="1" t="inlineStr">
-        <is>
-          <t>PATHIMAGE INSTRUMENTS CO.</t>
-        </is>
-      </c>
-      <c r="M10" s="1" t="inlineStr">
-        <is>
-          <t>PATHIMAGE INSTRUMENTS CO.</t>
-        </is>
-      </c>
-      <c r="N10" s="1" t="inlineStr">
-        <is>
-          <t>n this fast pace life, people have completely neglected the care, a body needs to continue working. Toiling hard days and nights for materialistic things results in fatigued body, mind and spirit. A good health is the real secret to an eternal bliss and this understanding is the real reason behind formation of Pathimage Instruments Co. Our business enterprise is formed to make hospitals, clinics, medical research centers and laboratories have an impressive line of Medical Equipment. Business Type Supplier, Trading Company Employee Count 11 Establishment 2008 Working Days Monday To Saturday GST NO 19AAKFP4862D1Z0 Payment Mode Cheque/DD, Online Payments (NEFT/RTGS/IMPS), Cash Related Products White Bene Sphera C61 Semi Automatic Biochemistry Analyzer Price: 80000 INR MOQ - 1 Piece/Pieces Ambay Enterprises Kolkata, West Bengal</t>
-        </is>
-      </c>
-      <c r="O10" s="1" t="inlineStr"/>
-      <c r="P10" s="1" t="inlineStr"/>
-      <c r="Q10" s="1" t="inlineStr">
-        <is>
-          <t>https://www.tradeindia.com/pathimage-instruments-co-5057644/</t>
-        </is>
-      </c>
-      <c r="R10" s="1" t="inlineStr"/>
-      <c r="S10" s="1" t="inlineStr"/>
-      <c r="T10" s="1" t="inlineStr">
-        <is>
-          <t>Hospital</t>
-        </is>
-      </c>
-      <c r="U10" s="1" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>Semi-automated Biochemistry Analyzer</t>
-        </is>
-      </c>
-      <c r="B11" s="1" t="inlineStr">
-        <is>
-          <t>AISTECH GLOBAL PRIVATE LIMITED</t>
-        </is>
-      </c>
-      <c r="C11" s="1" t="inlineStr">
-        <is>
-          <t>Semi-automated Biochemistry Analyzer</t>
-        </is>
-      </c>
-      <c r="D11" s="1" t="inlineStr">
-        <is>
-          <t>https://www.tradeindia.com/products/biochemistry-analyzer-c10543245.html</t>
-        </is>
-      </c>
-      <c r="E11" s="1" t="inlineStr">
-        <is>
-          <t>https://cpimg.tistatic.com/10543245/b/4/Semi-automated-Biochemistry-Analyzer.jpeg</t>
-        </is>
-      </c>
-      <c r="F11" s="1" t="inlineStr"/>
-      <c r="G11" s="1" t="inlineStr">
-        <is>
-          <t>ANLYZER</t>
-        </is>
-      </c>
-      <c r="H11" s="1" t="inlineStr">
         <is>
           <t>Semiautomatic HBA1C Abbott Afinion 2 For Laboratory Use: https://www.tradeindia.com/products/auto-biochemistry-analyzer-8968392.html
 Semi Auto Biochemistry Analyzer C61: https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-c61-8163441.html
@@ -1455,81 +1375,82 @@
 Carbon Nitrogen Analyzer: https://www.tradeindia.com/products/carbon-nitrogen-analyzer-c9908969.html</t>
         </is>
       </c>
-      <c r="I11" s="1" t="inlineStr">
+      <c r="I10" s="1" t="inlineStr">
         <is>
           <t>AISTECH GLOBAL PRIVATE LIMITED</t>
         </is>
       </c>
-      <c r="J11" s="1" t="inlineStr"/>
-      <c r="K11" s="1" t="inlineStr"/>
-      <c r="L11" s="1" t="inlineStr">
+      <c r="J10" s="1" t="inlineStr"/>
+      <c r="K10" s="1" t="inlineStr"/>
+      <c r="L10" s="1" t="inlineStr">
         <is>
           <t>AISTECH GLOBAL PRIVATE LIMITED</t>
         </is>
       </c>
-      <c r="M11" s="1" t="inlineStr">
+      <c r="M10" s="1" t="inlineStr">
         <is>
           <t>AISTECH GLOBAL PRIVATE LIMITED</t>
         </is>
       </c>
-      <c r="N11" s="1" t="inlineStr">
+      <c r="N10" s="1" t="inlineStr">
         <is>
           <t>Aistech Global Private Limited has supportive partners because of which we are able to serve customers in exceptionally well manner. As a supplier and trader, our expertise lies in catering to demand for products like Plastic Big Survey Prism, Bosch Hammer Drill Machine, Langry Rebound Hammer, Wooden Tripod Stand For Total Station, etc. We are happy to state that buyer who have placed their trust on us have received the best and their satisfaction is the key of our prompt success. We do not trust anyone blindly when it comes to quality and thus conduct in-house quality check of products before dispatch. Only after getting assured about the quality of the products, we allow them to leave from our premises. Business Type Distributor, Supplier, Trading Company Employee Count 2 Establishment 2020 Working Days Monday To Sunday GST NO 19AATCA7893D1ZZ Related Products Semiautomatic HBA1C Abbott Afinion 2 For Laboratory Use Price: 190000 INR MOQ - 1 Piece/Pieces Pathimage Instruments Co. Kolkata, West Bengal</t>
         </is>
       </c>
-      <c r="O11" s="1" t="inlineStr"/>
-      <c r="P11" s="1" t="inlineStr"/>
-      <c r="Q11" s="1" t="inlineStr">
+      <c r="O10" s="1" t="inlineStr"/>
+      <c r="P10" s="1" t="inlineStr"/>
+      <c r="Q10" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/aistech-global-private-limited-40038445/</t>
         </is>
       </c>
-      <c r="R11" s="1" t="inlineStr"/>
-      <c r="S11" s="1" t="inlineStr"/>
-      <c r="T11" s="1" t="inlineStr">
+      <c r="R10" s="1" t="inlineStr"/>
+      <c r="S10" s="1" t="inlineStr"/>
+      <c r="T10" s="1" t="inlineStr">
         <is>
           <t>ANLYZER</t>
         </is>
       </c>
-      <c r="U11" s="1" t="inlineStr"/>
+      <c r="U10" s="1" t="inlineStr"/>
+      <c r="V10" s="1" t="inlineStr"/>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>Biochemistry Analyzer</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>SUNSHINE SCIENTIFIC EQUIPMENTS</t>
         </is>
       </c>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>Biochemistry Analyzer</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/biochemistry-analyzer-c6350610.html</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>https://cpimg.tistatic.com/06350610/b/4/Biochemistry-Analyzer.jpg</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="F11" s="1" t="inlineStr">
         <is>
           <t>Precise analysis, Reliable results, Easy operation, Compact design, Cost effective Power Supply Elec</t>
         </is>
       </c>
-      <c r="G12" s="1" t="inlineStr">
+      <c r="G11" s="1" t="inlineStr">
         <is>
           <t>Clinical biochemistry testing in labs and hospitals. Provides quantitative analysis of various blood and serum components.</t>
         </is>
       </c>
-      <c r="H12" s="1" t="inlineStr">
+      <c r="H11" s="1" t="inlineStr">
         <is>
           <t>Full Automatic Chemistry Analyzer - Application: Commercial: https://www.tradeindia.com/products/full-automatic-chemistry-analyzer-c9474134.html
 Meril Autoquant 400 Fully Automatic Biochemistry Analyzer - Attributes: Easy To Operate: https://www.tradeindia.com/products/meril-autoquant-400-fully-automatic-biochemistry-analyzer-c10317325.html
@@ -1562,82 +1483,83 @@
 Microlab 300 Biochemistry Analyzer: https://www.tradeindia.com/products/microlab-300-biochemistry-analyzer-5482147.html</t>
         </is>
       </c>
-      <c r="I12" s="1" t="inlineStr">
+      <c r="I11" s="1" t="inlineStr">
         <is>
           <t>SUNSHINE SCIENTIFIC EQUIPMENTS</t>
         </is>
       </c>
-      <c r="J12" s="1" t="inlineStr"/>
-      <c r="K12" s="1" t="inlineStr"/>
-      <c r="L12" s="1" t="inlineStr">
+      <c r="J11" s="1" t="inlineStr"/>
+      <c r="K11" s="1" t="inlineStr"/>
+      <c r="L11" s="1" t="inlineStr">
         <is>
           <t>SUNSHINE SCIENTIFIC EQUIPMENTS</t>
         </is>
       </c>
-      <c r="M12" s="1" t="inlineStr">
+      <c r="M11" s="1" t="inlineStr">
         <is>
           <t>SUNSHINE SCIENTIFIC EQUIPMENTS</t>
         </is>
       </c>
-      <c r="N12" s="1" t="inlineStr">
+      <c r="N11" s="1" t="inlineStr">
         <is>
           <t>Incepted in the year 2007, Sunshine Scientific Equipments is a reputed firm. We are highly involved Exporter of Dairy Equipment, Laboratory Testing Instruments, Soil Testing Equipments, Bomb Calorimeter, Bitumen &amp; Asphalt Testing, Laboratory Testing Equipment and many more. These products are highly known in the market for their long service life and optimum performance. Our offered assortment is manufactured and designed using quality approved raw material and sophisticated technology in compliance with international quality principles and norms. Business Type Exporter, Manufacturer, Supplier Employee Count 10 Establishment 2007 Working Days Monday To Saturday GST NO 07AFHPN3371D1ZL Payment Mode Telegraphic Transfer (T/T) Certification An ISO : 9001:2015 , CE Certified Related Products Full Automatic Chemistry Analyzer - Application: Commercial MOQ - 1 Unit/Units Weldon Biotech (india) Pvt. Ltd. Delhi, Delhi</t>
         </is>
       </c>
-      <c r="O12" s="1" t="inlineStr"/>
-      <c r="P12" s="1" t="inlineStr"/>
-      <c r="Q12" s="1" t="inlineStr">
+      <c r="O11" s="1" t="inlineStr"/>
+      <c r="P11" s="1" t="inlineStr"/>
+      <c r="Q11" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/sunshine-scientific-equipments-12356009/</t>
         </is>
       </c>
-      <c r="R12" s="1" t="inlineStr"/>
-      <c r="S12" s="1" t="inlineStr"/>
-      <c r="T12" s="1" t="inlineStr">
+      <c r="R11" s="1" t="inlineStr"/>
+      <c r="S11" s="1" t="inlineStr"/>
+      <c r="T11" s="1" t="inlineStr">
         <is>
           <t>Clinical biochemistry testing in labs and hospitals. Provides quantitative analysis of various blood and serum components.</t>
         </is>
       </c>
-      <c r="U12" s="1" t="inlineStr">
+      <c r="U11" s="1" t="inlineStr">
         <is>
           <t>Clinical biochemistry testing in labs and hospitals. Provides quantitative analysis of various blood and serum components.</t>
         </is>
       </c>
+      <c r="V11" s="1" t="inlineStr"/>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>Clinical Middle Ear Analyzer at Best Price in Ambala Cantt | Contemporary Export Industry</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr"/>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr"/>
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>Contemporary Export Industry - Offering low price Clinical Middle Ear Analyzer in Science Market, Ambala Cantt with product details &amp; company information.</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/conxport-clinical-middle-ear-analyzer-r-36-m-c7243895.html</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>https://cpimg.tistatic.com/07243895/b/4/Clinical-Middle-Ear-Analyzer.jpg</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>Automatic and manual mode, data storage, user-friendly interface Type Other, Clinical Middle Ear Ana
 Clinical Middle Ear Analyzer R 36 M Manufactured By Conxport Company Details We, Contemporary Export</t>
         </is>
       </c>
-      <c r="G13" s="1" t="inlineStr">
+      <c r="G12" s="1" t="inlineStr">
         <is>
           <t>Clinical diagnosis and measurement of middle ear conditions</t>
         </is>
       </c>
-      <c r="H13" s="1" t="inlineStr">
+      <c r="H12" s="1" t="inlineStr">
         <is>
           <t>ConXport Bio-Chemistry Analyzer: https://www.tradeindia.com/products/conxport-bio-chemistry-analyzer-c7208608.html
 Bio Chemistry Analyzer - Silver, 33x32x12.5cm | Absorbance Mono and Bi-Chromatic, 100 Test Memory, LCD Display, Thermostat Control 25-37Â°C: https://www.tradeindia.com/products/bio-chemistry-analyzer-c2951949.html
@@ -1672,69 +1594,70 @@
 Thermo Scientific Sorvall St 16 Benchtop Lab Centrifuge: https://www.tradeindia.com/products/thermo-scientific-sorvall-st-16-benchtop-lab-centrifuge-c10859546.html</t>
         </is>
       </c>
-      <c r="I13" s="1" t="inlineStr">
+      <c r="I12" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="J13" s="1" t="inlineStr"/>
-      <c r="K13" s="1" t="inlineStr"/>
-      <c r="L13" s="1" t="inlineStr">
+      <c r="J12" s="1" t="inlineStr"/>
+      <c r="K12" s="1" t="inlineStr"/>
+      <c r="L12" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="M13" s="1" t="inlineStr">
+      <c r="M12" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="N13" s="1" t="inlineStr">
+      <c r="N12" s="1" t="inlineStr">
         <is>
           <t>We, Contemporary Export Industry are a company that values customers. Everyday, we work hard under the leadership of Mr. Akhil Trehan, to offer the best to clients. We design and customize a fine assortment of Single Person Grossing Workstations, Advance Rotary Microtomes, Disintegration Test Apparatus Tablets, Projectors, etc. Quality of our offered items exceeds the expectations of clients, without any interruption. The gamut is renowned for not just its unrivaled quality but also its seamless finish and durability. One can order our phenomenal collection in bulk, while just paying a small sum of money. Our prestigious enterprise is registered with Ministry of Consumer Affairs, Business Type Exporter, Manufacturer, Supplier, Trading Company Employee Count 8 Establishment 2012 Working Days Monday To Sunday GST NO 06AJMPT4011D1ZG Certification ISO 9001-2008 Related Products ConXport Bio-Chemistry Analyzer Contemporary Export Industry Ambala Cantt, Haryana</t>
         </is>
       </c>
-      <c r="O13" s="1" t="inlineStr"/>
-      <c r="P13" s="1" t="inlineStr"/>
-      <c r="Q13" s="1" t="inlineStr">
+      <c r="O12" s="1" t="inlineStr"/>
+      <c r="P12" s="1" t="inlineStr"/>
+      <c r="Q12" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/conxport-clinical-middle-ear-analyzer-r-36-m-c7243895.html</t>
         </is>
       </c>
-      <c r="R13" s="1" t="inlineStr"/>
-      <c r="S13" s="1" t="inlineStr"/>
-      <c r="T13" s="1" t="inlineStr">
+      <c r="R12" s="1" t="inlineStr"/>
+      <c r="S12" s="1" t="inlineStr"/>
+      <c r="T12" s="1" t="inlineStr">
         <is>
           <t>Clinical diagnosis and measurement of middle ear conditions</t>
         </is>
       </c>
-      <c r="U13" s="1" t="inlineStr"/>
+      <c r="U12" s="1" t="inlineStr"/>
+      <c r="V12" s="1" t="inlineStr"/>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>Uriscan Pro Urine Chemistry Analyzer - Color: Different Availabe - Color: Different Availabe at Best Price in Mathura | Biosolution Technologies</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr"/>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr"/>
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>Biosolution Technologies - Offering low price Uriscan Pro Urine Chemistry Analyzer - Color: Different Availabe - Color: Different Availabe in Chandra Puri, Mathura with product details &amp; company information.</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/uriscan-pro-urine-chemistry-analyzer-c10651715.html</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>https://cpimg.tistatic.com/10651715/b/4/Uriscan-Pro-Urine-Chemistry-Analyzer..jpg</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr"/>
-      <c r="G14" s="1" t="inlineStr"/>
-      <c r="H14" s="1" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr"/>
+      <c r="G13" s="1" t="inlineStr"/>
+      <c r="H13" s="1" t="inlineStr">
         <is>
           <t>Uriscan Super Urine Chemistry Analyzer - Color: Different Availabe: https://www.tradeindia.com/products/uriscan-super-urine-chemistry-analyzer-c10651716.html
 Urine Analyzer ( Bi-400) - Color: White: https://www.tradeindia.com/products/urine-analyzer-bi-400-c8781154.html
@@ -1758,43 +1681,139 @@
 Accurex ACR Albumin Creatinine Ratio Urine Analyzer: https://www.tradeindia.com/products/accurex-acr-albumin-creatinine-ratio-urine-analyzer-7968045.html</t>
         </is>
       </c>
+      <c r="I13" s="1" t="inlineStr">
+        <is>
+          <t>Trusted Seller</t>
+        </is>
+      </c>
+      <c r="J13" s="1" t="inlineStr"/>
+      <c r="K13" s="1" t="inlineStr"/>
+      <c r="L13" s="1" t="inlineStr">
+        <is>
+          <t>Trusted Seller</t>
+        </is>
+      </c>
+      <c r="M13" s="1" t="inlineStr">
+        <is>
+          <t>Trusted Seller</t>
+        </is>
+      </c>
+      <c r="N13" s="1" t="inlineStr">
+        <is>
+          <t>Biosolution Technologies, established in 2024, is a trusted trader and supplier based in Mathura, Uttar Pradesh, India. We specialize in providing cutting-edge medical diagnostic equipment, including Semi Automatic Biochemistry Analyzer, Hemoglobin Analyzer, Medonic Hematology Analyzer, ESR Analyzer and Hemoglobin Testing Meter. With a focus on quality, innovation, and reliability, we aim to serve the healthcare sector with advanced diagnostic solutions to improve patient outcomes.We recognize that medicadiagnostics evolve rapidly, and we are dedicated to staying ahead of the curve. By incorporating the latest technological advancements, we provide equipment that guarantees precision and reliability. Our focus on constant innovation ensures that our clients always have access to the best tools to meet their di Business Type Supplier, Trading Company Employee Count 2 Establishment 2024 Working Days Monday To Sunday GST NO 09BNFPK4044M1ZP Payment Mode Online Payments (NEFT/RTGS/IMPS), Cheque/DD Related Products Uriscan Pro Urine Chemistry Analyzer - Color: Different Availabe MOQ - 1 Unit/Units Biosolution Technologies Mathura, Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="O13" s="1" t="inlineStr"/>
+      <c r="P13" s="1" t="inlineStr"/>
+      <c r="Q13" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/uriscan-pro-urine-chemistry-analyzer-c10651715.html</t>
+        </is>
+      </c>
+      <c r="R13" s="1" t="inlineStr"/>
+      <c r="S13" s="1" t="inlineStr"/>
+      <c r="T13" s="1" t="inlineStr">
+        <is>
+          <t>Biosolution Technologies - Offering low price Uriscan Pro Urine Chemistry Analyzer - Color: Different Availabe - Color: Different Availabe in Chandra Puri, Mathura with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="U13" s="1" t="inlineStr"/>
+      <c r="V13" s="1" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Human Humastar 600 Automated Clinical Chemistry Analyzer - Dimension (L*w*h): 1000*740*1130 Mm</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>INORBVICT HEALTHCARE INDIA PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>Human Humastar 600 Automated Clinical Chemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/human-humastar-600-automated-clinical-chemistry-analyzer-c10877025.html</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/10877025/b/4/Human-Humastar-600-Automated-Clinical-Chemistry-Analyzer.png</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr"/>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>Routine clinical chemistry testing in medium to high-throughput laboratories</t>
+        </is>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>Portable Biogas Analyzer - Accuracy: 2 %: https://www.tradeindia.com/products/portable-biogas-analyzer-c3391801.html
+Circuit Breaker Operational Analyzer - Automation Grade: Automatic: https://www.tradeindia.com/products/circuit-breaker-operational-analyzer-c11224952.html
+Sodium Analyzer Equipment: https://www.tradeindia.com/products/sodium-analyzer-equipment-c7911608.html
+Lightweight Meco 9009 Digital Solar Module Analyzer Equipment: https://www.tradeindia.com/products/solar-module-analyzer-1239923.html
+Circuit Breaker Analyzer Equipment: https://www.tradeindia.com/products/circuit-breaker-analyzer-equipment-587020.html
+Buchi Encapsulator B390, B395 - Application: Controlled Drug Delivery Systems: https://www.tradeindia.com/products/buchi-encapsulator-b390-b395-c10866048.html
+Bruker Ft-Nir Spectrometer Mpa Iii - Dimension (L*W*H): 70*50*100 Cm: https://www.tradeindia.com/products/bruker-ft-nir-spectrometer-mpa-iii-c10867804.html
+Bruker Tango Ft-Nir Spectrometer - Dimension (L*W*H): 49*42*29 Cm: https://www.tradeindia.com/products/bruker-tango-ft-nir-spectrometer-c10868572.html
+Sartorius Ambr 250 Modular - Dimension (L*W*H): 885*455* 600 Mm Millimeter (Mm): https://www.tradeindia.com/products/sartorius-ambr-250-modular-c10833593.html
+Sigma 4-16Ks Refrigerated Benchtop Centrifuge - Application: Clinical Diagnostics: https://www.tradeindia.com/products/sigma-4-16ks-refrigerated-benchtop-centrifuge-c10870007.html
+Qiastat-Dx Gastrointestinal Panel 2 - Application: Laboratory: https://www.tradeindia.com/products/qiastat-dx-gastrointestinal-panel-2-c9582175.html
+Sigma 3-30Khs Refrigerated And Heated Benchtop Centrifuge - Application: Cellular Biology: https://www.tradeindia.com/products/sigma-3-30khs-refrigerated-and-heated-benchtop-centrifuge-c10870486.html
+Tanner Scientific Cuttec S Sliding Microtome - Dimension (L*W*H): 450A A A 150A A A 200A Mm Micromete (Micron): https://www.tradeindia.com/products/tanner-scientific-cuttec-s-sliding-microtome-c10873453.html
+Hitachi Thermo Mechanical Analyzers (Tma): Tma7100 - Dimension (L*W*H): 545*295*430 Millimeter (Mm): https://www.tradeindia.com/products/hitachi-thermo-mechanical-analyzers-tma-tma7100-c10843894.html
+Sigma 4-5Krl Refrigerated Automated Centrifuge - Dimension (L*W*H): 655*570*489 Mm: https://www.tradeindia.com/products/sigma-4-5krl-refrigerated-automated-centrifuge-c10869336.html
+Biochemistry Analyzer Fully Automatic For Laboratory Use: https://www.tradeindia.com/products/biochemistry-analyzer-fully-automatic-for-laboratory-use-c10877154.html</t>
+        </is>
+      </c>
       <c r="I14" s="1" t="inlineStr">
         <is>
-          <t>Trusted Seller</t>
+          <t>INORBVICT HEALTHCARE INDIA PVT. LTD.</t>
         </is>
       </c>
       <c r="J14" s="1" t="inlineStr"/>
       <c r="K14" s="1" t="inlineStr"/>
       <c r="L14" s="1" t="inlineStr">
         <is>
-          <t>Trusted Seller</t>
+          <t>INORBVICT HEALTHCARE INDIA PVT. LTD.</t>
         </is>
       </c>
       <c r="M14" s="1" t="inlineStr">
         <is>
-          <t>Trusted Seller</t>
+          <t>INORBVICT HEALTHCARE INDIA PVT. LTD.</t>
         </is>
       </c>
       <c r="N14" s="1" t="inlineStr">
         <is>
-          <t>Biosolution Technologies, established in 2024, is a trusted trader and supplier based in Mathura, Uttar Pradesh, India. We specialize in providing cutting-edge medical diagnostic equipment, including Semi Automatic Biochemistry Analyzer, Hemoglobin Analyzer, Medonic Hematology Analyzer, ESR Analyzer and Hemoglobin Testing Meter. With a focus on quality, innovation, and reliability, we aim to serve the healthcare sector with advanced diagnostic solutions to improve patient outcomes.We recognize that medicadiagnostics evolve rapidly, and we are dedicated to staying ahead of the curve. By incorporating the latest technological advancements, we provide equipment that guarantees precision and reliability. Our focus on constant innovation ensures that our clients always have access to the best tools to meet their di Business Type Supplier, Trading Company Employee Count 2 Establishment 2024 Working Days Monday To Sunday GST NO 09BNFPK4044M1ZP Payment Mode Online Payments (NEFT/RTGS/IMPS), Cheque/DD Related Products Uriscan Pro Urine Chemistry Analyzer - Color: Different Availabe MOQ - 1 Unit/Units Biosolution Technologies Mathura, Uttar Pradesh</t>
+          <t>At Inorbvict Healthcare India Pvt. Ltd. , we are passionate about delivering quality healthcare solutions to the world. As a dedicated exporter, we work closely with healthcare providers, hospitals, and institutions across the globe to supply reliable, advanced medical equipment that supports better patient care. We offer a wide range of products including Dental &amp; ENT equipment, OT &amp; ICU setups, Endoscopy systems, X-Ray and Ultrasound machines, NICU and Neurology tools, Radiology and Imaging equipment, Blood bank solutions, Dialysis machines, Dermatology and Ophthalmology equipment, Laboratory instruments, Cardiology devices, Respiratory care systems , and Operating Microscopes . What sets us apart is our commitment to quality, trusted brand associations, and a hands-on approach to every clienta s needs. Whether youa re setting up a new facility or expanding your services, wea re here to make global medical sourcing easier, faster, and more reliable. Business Type Exporter, Manufacturer Employee Count 50 Establishment 2014 Working Days Monday To Saturday GST NO 27AADCI6120M1ZH Payment Mode Others Certification ISO 9001:2015 Related Products Portable Biogas Analyzer - Accuracy: 2 % Price: 280000 INR MOQ - 1 Piece/Pieces Hnl Systems Pvt. Ltd. Mumbai, Maharashtra</t>
         </is>
       </c>
       <c r="O14" s="1" t="inlineStr"/>
       <c r="P14" s="1" t="inlineStr"/>
       <c r="Q14" s="1" t="inlineStr">
         <is>
-          <t>https://www.tradeindia.com/products/uriscan-pro-urine-chemistry-analyzer-c10651715.html</t>
+          <t>https://www.tradeindia.com/inorbvict-healthcare-india-pvt-ltd-8372692/</t>
         </is>
       </c>
       <c r="R14" s="1" t="inlineStr"/>
       <c r="S14" s="1" t="inlineStr"/>
       <c r="T14" s="1" t="inlineStr">
         <is>
-          <t>Biosolution Technologies - Offering low price Uriscan Pro Urine Chemistry Analyzer - Color: Different Availabe - Color: Different Availabe in Chandra Puri, Mathura with product details &amp; company information.</t>
-        </is>
-      </c>
-      <c r="U14" s="1" t="inlineStr"/>
+          <t>Routine clinical chemistry testing in medium to high-throughput laboratories</t>
+        </is>
+      </c>
+      <c r="U14" s="1" t="inlineStr">
+        <is>
+          <t>Routine clinical chemistry testing in medium to high-throughput laboratories</t>
+        </is>
+      </c>
+      <c r="V14" s="1" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr">
@@ -1883,6 +1902,7 @@
         </is>
       </c>
       <c r="U15" s="1" t="inlineStr"/>
+      <c r="V15" s="1" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
@@ -1991,6 +2011,7 @@
           <t>Diagnostic Equipment</t>
         </is>
       </c>
+      <c r="V16" s="1" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr">
@@ -2100,6 +2121,7 @@
         </is>
       </c>
       <c r="U17" s="1" t="inlineStr"/>
+      <c r="V17" s="1" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr">
@@ -2193,6 +2215,7 @@
         </is>
       </c>
       <c r="U18" s="1" t="inlineStr"/>
+      <c r="V18" s="1" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr">
@@ -2279,6 +2302,7 @@
         </is>
       </c>
       <c r="U19" s="1" t="inlineStr"/>
+      <c r="V19" s="1" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="inlineStr">
@@ -2367,6 +2391,7 @@
         </is>
       </c>
       <c r="U20" s="1" t="inlineStr"/>
+      <c r="V20" s="1" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr">
@@ -2465,6 +2490,7 @@
           <t>Water Analysis, Clinical and Industrial Laboratories</t>
         </is>
       </c>
+      <c r="V21" s="1" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="1" t="inlineStr">
@@ -2562,6 +2588,7 @@
         </is>
       </c>
       <c r="U22" s="1" t="inlineStr"/>
+      <c r="V22" s="1" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="1" t="inlineStr">
@@ -2668,36 +2695,132 @@
         </is>
       </c>
       <c r="U23" s="1" t="inlineStr"/>
+      <c r="V23" s="1" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="1" t="inlineStr">
         <is>
+          <t>Fully Automatic CLIA Analyzer (BI-2000)</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>BIOGENIX INC. PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>Fully Automatic CLIA Analyzer (BI-2000)</t>
+        </is>
+      </c>
+      <c r="D24" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/fully-automatic-clia-analyzer-bi-2000-c8969808.html</t>
+        </is>
+      </c>
+      <c r="E24" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/08969808/b/4/Fully-Automatic-CLIA-Analyzer-BI-2000-.jpg</t>
+        </is>
+      </c>
+      <c r="F24" s="1" t="inlineStr"/>
+      <c r="G24" s="1" t="inlineStr"/>
+      <c r="H24" s="1" t="inlineStr">
+        <is>
+          <t>Semi Auto Biosystem Bts Analyser - Color: Different Available: https://www.tradeindia.com/products/semi-auto-biosystem-bts-analyser-c11872784.html
+Bonavera Chem Uno Plus Biochemistry Semi Auto Analyzer: https://www.tradeindia.com/products/bonavera-chem-uno-plus-biochemistry-semi-auto-analyzer-c12491575.html
+Biochemistry Auto Analyzer (Cat No Bgs-278): https://www.tradeindia.com/products/biochemistry-auto-analyzer-cat-no-bgs-278-4448353.html
+Ez Scan-Auto Analyzer - 45x30x20 cm, Gray, 15 Inch Screen | Non-Invasive, Instant Diabetes Screening, Easy Use: https://www.tradeindia.com/products/ez-scan-auto-analyzer-3490051.html
+Merilyzer Cliniquant Semi Automated Biochemistry Analyzer - Application: Hospital: https://www.tradeindia.com/products/merilyzer-cliniquant-semi-automated-biochemistry-analyzer-c11787577.html
+Welchem Semi Automatic Analyzer - Equipment Materials: Metal: https://www.tradeindia.com/products/welchem-semi-automatic-analyzer-c9474156.html
+Semi-Automated Biochemistry Analyzer - Application: Anlyzer: https://www.tradeindia.com/products/biochemistry-analyzer-c10543245.html
+Semi-Auto Chemistry Analyzer - Color: White: https://www.tradeindia.com/products/semi-auto-chemistry-analyzer-c11771231.html
+Semi Automated Clinical Chemistry Analyzer - Application: Laboratory: https://www.tradeindia.com/products/semi-automated-clinical-chemistry-analyzer-c11825292.html
+Welchem Semi - Auto Analyzer - Attributes: Higher Level Of Accuracy: https://www.tradeindia.com/products/welchem-semi-auto-analyzer-c8452573.html
+Skyla Clinical Chemistry Analyzer D-66386 - Blue Color, Designed for Hospital Use | Advanced Diagnostic Capabilities: https://www.tradeindia.com/products/skyla-hb1-poc-clinical-chemistry-auto-analyzer-c7901963.html
+Semi Auto Turbidimetry Analyzer - Color: White: https://www.tradeindia.com/products/semi-auto-turbidimetry-analyzer-c6374634.html
+EDAN Calibrant Fluid - Arterial Blood Gas (ABG) Analyzer: https://www.tradeindia.com/products/edan-calibrant-fluid-arterial-blood-gas-abg-analyzer-c11827725.html
+DENGUE NS1 Antigen Rapid Test - High Sensitivity, Fast Results | Ideal for Immediate Diagnosis: https://www.tradeindia.com/products/dengue-test-kit-c5376520.html
+Prolactin Elisa Kit - Color: Multi Color: https://www.tradeindia.com/products/prolactin-elisa-kit-c5376524.html
+Cholera AG: https://www.tradeindia.com/products/cholera-ag-c5559402.html
+H. Pylori Ab: https://www.tradeindia.com/products/h-pylori-ab-c5559585.html
+CK-MB KIT: https://www.tradeindia.com/products/ck-mb-kit-c5569340.html
+LDL DIRECT CHOLESTEROL (Liquid): https://www.tradeindia.com/products/ldl-direct-kit-c5569401.html
+MULTIPARAMETER 10P: https://www.tradeindia.com/products/multiparameter-10p-c5889507.html
+FILARIASIS IgG/IgM RAPID TEST: https://www.tradeindia.com/products/filariasis-igg-igm-rapid-test-c8791650.html
+GONORRHEA Ag RAPID TEST: https://www.tradeindia.com/products/gonorrhea-ag-rapid-test-c8791706.html
+Fully Automatic CLIA Analyzer (BI-1000: https://www.tradeindia.com/products/fully-automatic-clia-analyzer-bi-1000-c8969939.html
+15C COD Analyzer: https://www.tradeindia.com/products/15c-cod-analyzer-c7489980.html</t>
+        </is>
+      </c>
+      <c r="I24" s="1" t="inlineStr">
+        <is>
+          <t>BIOGENIX INC. PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="J24" s="1" t="inlineStr"/>
+      <c r="K24" s="1" t="inlineStr"/>
+      <c r="L24" s="1" t="inlineStr">
+        <is>
+          <t>BIOGENIX INC. PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="M24" s="1" t="inlineStr">
+        <is>
+          <t>BIOGENIX INC. PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="N24" s="1" t="inlineStr">
+        <is>
+          <t>Biogenix , has backed a large number of medical facilities throughout the globe with its best quality Diagnostics Kits &amp; Laboratory Equipment. Our inception dates back to 2007, and all this time of our business activities has been highly appreciated throughout the globe as a large number of our pathologists and doctors have been highly satisfied with the usage of our products. Operating from Lucknow (Uttar Pradesh, India), we are highly praised by national as well as international medical facilities for our role as a prominent manufacturing and trading company. This renomination of our company has been possible due to our business policies and work ethics, that are to manufacture the products of the utmost quality and highly satisfy the clients with our business dealings. Business Type Exporter, Manufacturer, Supplier Employee Count 48 Establishment 2007 Working Days Monday To Sunday GST NO 09AAGCB6941G1ZJ Related Products Semi Auto Biosystem Bts Analyser - Color: Different Available MOQ - 10 Unit/Units Biomedical And Services Varanasi, Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="O24" s="1" t="inlineStr"/>
+      <c r="P24" s="1" t="inlineStr"/>
+      <c r="Q24" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/biogenix-inc-pvt-ltd-9029995/</t>
+        </is>
+      </c>
+      <c r="R24" s="1" t="inlineStr"/>
+      <c r="S24" s="1" t="inlineStr"/>
+      <c r="T24" s="1" t="inlineStr">
+        <is>
+          <t>Fully Automatic CLIA Analyzer (BI-2000)</t>
+        </is>
+      </c>
+      <c r="U24" s="1" t="inlineStr"/>
+      <c r="V24" s="1" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr">
+        <is>
           <t>Bio Chemistry Analyzer - Silver, 33x32x12.5cm | Absorbance Mono and Bi-Chromatic, 100 Test Memory, LCD Display, Thermostat Control 25-37Â°C - Silver, 33x32x12.5cm | Absorbance Mono And Bi-chromatic, 100 Test Memory, Lcd Display, Thermostat Control 25-37â°c at Best Price in Ambala Cantt | Edutek Instrumentation</t>
         </is>
       </c>
-      <c r="B24" s="1" t="inlineStr"/>
-      <c r="C24" s="1" t="inlineStr">
+      <c r="B25" s="1" t="inlineStr"/>
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>Edutek Instrumentation - Offering low price Bio Chemistry Analyzer - Silver, 33x32x12.5cm | Absorbance Mono and Bi-Chromatic, 100 Test Memory, LCD Display, Thermostat Control 25-37Â°C - Silver, 33x32x12.5cm | Absorbance Mono And Bi-chromatic, 100 Test Memory, Lcd Display, Thermostat Control 25-37â°c in Jagadhri Road, Ambala Cantt with product details &amp; company information.</t>
         </is>
       </c>
-      <c r="D24" s="1" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/bio-chemistry-analyzer-c2951949.html</t>
         </is>
       </c>
-      <c r="E24" s="1" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>https://cpimg.tistatic.com/02951949/b/5/Bio-Chemistry-Analyzer.png</t>
         </is>
       </c>
-      <c r="F24" s="1" t="inlineStr"/>
-      <c r="G24" s="1" t="inlineStr">
+      <c r="F25" s="1" t="inlineStr"/>
+      <c r="G25" s="1" t="inlineStr">
         <is>
           <t>Hospitals, Laboratories, Clinics, Research Institutes</t>
         </is>
       </c>
-      <c r="H24" s="1" t="inlineStr">
+      <c r="H25" s="1" t="inlineStr">
         <is>
           <t>Touch Screen Bio Chemistry Analyzer - Compact Design , Clear Digital Display Screen , User-Friendly Controls: https://www.tradeindia.com/products/touch-screen-bio-chemistry-analyzer-c6965405.html
 Bio Chemistry Analyzer - Absorbency, Mono-Chromatic &amp; Bi-Chromatic Methods | 100-Test Memory, Inbuilt Thermal Printer, 4x20 LCD Display: https://www.tradeindia.com/products/bio-chemistry-analyzer-c2505822.html
@@ -2731,77 +2854,78 @@
 Automated Hematology Analyzer - Advanced Diagnostic Technology | High-Throughput, User-Friendly Interface, Accurate Blood Analysis: https://www.tradeindia.com/products/automated-hematology-analyzer-c3013903.html</t>
         </is>
       </c>
-      <c r="I24" s="1" t="inlineStr">
+      <c r="I25" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="J24" s="1" t="inlineStr"/>
-      <c r="K24" s="1" t="inlineStr"/>
-      <c r="L24" s="1" t="inlineStr">
+      <c r="J25" s="1" t="inlineStr"/>
+      <c r="K25" s="1" t="inlineStr"/>
+      <c r="L25" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="M24" s="1" t="inlineStr">
+      <c r="M25" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="N24" s="1" t="inlineStr">
+      <c r="N25" s="1" t="inlineStr">
         <is>
           <t>Manufacturer and Exporter of all type engineering lab equipment, civil engineering lab equipment, science lab equipment, soil testing lab equipment, concrete Testing Lab Equipment, Vocational Training Equipment, Teaching lab equipment, Pharmacy Lab Equipment, Mechanical Lab for engineering college, fluid mechanic lab for engineering students, etc Business Type Exporter, Manufacturer, Supplier Employee Count 25 Establishment 1973 Working Days Monday To Saturday GST NO 06AEWPJ6896D1ZU Certification AN ISO 9001:2008 Related Products Touch Screen Bio Chemistry Analyzer - Compact Design , Clear Digital Display Screen , User-Friendly Controls Contemporary Export Industry Ambala Cantt, Haryana</t>
         </is>
       </c>
-      <c r="O24" s="1" t="inlineStr"/>
-      <c r="P24" s="1" t="inlineStr"/>
-      <c r="Q24" s="1" t="inlineStr">
+      <c r="O25" s="1" t="inlineStr"/>
+      <c r="P25" s="1" t="inlineStr"/>
+      <c r="Q25" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/bio-chemistry-analyzer-c2951949.html</t>
         </is>
       </c>
-      <c r="R24" s="1" t="inlineStr"/>
-      <c r="S24" s="1" t="inlineStr"/>
-      <c r="T24" s="1" t="inlineStr">
+      <c r="R25" s="1" t="inlineStr"/>
+      <c r="S25" s="1" t="inlineStr"/>
+      <c r="T25" s="1" t="inlineStr">
         <is>
           <t>Hospitals, Laboratories, Clinics, Research Institutes</t>
         </is>
       </c>
-      <c r="U24" s="1" t="inlineStr"/>
+      <c r="U25" s="1" t="inlineStr"/>
+      <c r="V25" s="1" t="inlineStr"/>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
         <is>
           <t>Fully Automatic Biochemistry Analyzer</t>
         </is>
       </c>
-      <c r="B25" s="1" t="inlineStr">
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>MARKEN HEALTHTECH LIMITED</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>Fully Automatic Biochemistry Analyzer</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
+      <c r="D26" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/fully-automatic-biochemistry-analyzer-c11810500.html</t>
         </is>
       </c>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E26" s="1" t="inlineStr">
         <is>
           <t>https://cpimg.tistatic.com/11810500/b/4/Fully-Automatic-Biochemistry-Analyzer.png</t>
         </is>
       </c>
-      <c r="F25" s="1" t="inlineStr"/>
-      <c r="G25" s="1" t="inlineStr">
+      <c r="F26" s="1" t="inlineStr"/>
+      <c r="G26" s="1" t="inlineStr">
         <is>
           <t>Hospital, Diagnostic Laboratory, Pathology Lab</t>
         </is>
       </c>
-      <c r="H25" s="1" t="inlineStr">
+      <c r="H26" s="1" t="inlineStr">
         <is>
           <t>Semi Automatic Biochemistry Analyzer - Application: Hospital: https://www.tradeindia.com/products/semi-automatic-biochemistry-analyzer-c5301831.html
 KANAD 6FX Semi Automatic Biochemistry Analyzer - ABS Plastic, 320x270x140mm, White, LED Light Source with 6 Wavelengths | Quartz Flowcell 32ul, 3-inch Graphical Display, 100 User Programs, RT to 37Â°C Testing: https://www.tradeindia.com/products/kanad-6fx-semi-automatic-biochemistry-analyzer-5631458.html
@@ -2823,81 +2947,82 @@
 Clinical Labmate: https://www.tradeindia.com/products/clinical-labmate-c3874769.html</t>
         </is>
       </c>
-      <c r="I25" s="1" t="inlineStr">
+      <c r="I26" s="1" t="inlineStr">
         <is>
           <t>MARKEN HEALTHTECH LIMITED</t>
         </is>
       </c>
-      <c r="J25" s="1" t="inlineStr"/>
-      <c r="K25" s="1" t="inlineStr"/>
-      <c r="L25" s="1" t="inlineStr">
+      <c r="J26" s="1" t="inlineStr"/>
+      <c r="K26" s="1" t="inlineStr"/>
+      <c r="L26" s="1" t="inlineStr">
         <is>
           <t>MARKEN HEALTHTECH LIMITED</t>
         </is>
       </c>
-      <c r="M25" s="1" t="inlineStr">
+      <c r="M26" s="1" t="inlineStr">
         <is>
           <t>MARKEN HEALTHTECH LIMITED</t>
         </is>
       </c>
-      <c r="N25" s="1" t="inlineStr">
+      <c r="N26" s="1" t="inlineStr">
         <is>
           <t>Marken Healthtech Private Limited was formed in 2018 with the name Mark Enterprises. Since inception, we have been passionately running our operations with a vision to provide easily accessible and dependable Cold Chain Solutions for the Healthcare Sector. We have become a renowned manufacturer and exporter of Solar Direct Drive Refrigerator, Ice Lined Refrigerator, Blood Bank Refrigerator, Laminar Air Flow, Gel Card Incubator, Laboratory Autoclave, Ultrasonic Cleaner, Pediatric Bed, etc.We perform our job duties with an unwavering commitment to quality and focus on gaining complete satisfaction of customers. This has earned us recognition and accreditation from many renowned names of the market, including the All State Governments, Central government of India, Research Institutes, Defense forces, and more. Business Type Exporter, Importer, Manufacturer, Service Provider, Distributor, Supplier, Trading Company, Wholesaler, Retailer, Dealer, Fabricator, Producer Employee Count 250 Establishment 2017 Working Days Monday To Sunday GST NO 27AARCM9404E1Z7 Related Products Fully Automatic Biochemistry Analyzer - Accuracy: Cv 1% % Price: 474999.0 INR MOQ - 1 Piece/Pieces Marken Healthtech Limited Nashik, Maharashtra</t>
         </is>
       </c>
-      <c r="O25" s="1" t="inlineStr"/>
-      <c r="P25" s="1" t="inlineStr"/>
-      <c r="Q25" s="1" t="inlineStr">
+      <c r="O26" s="1" t="inlineStr"/>
+      <c r="P26" s="1" t="inlineStr"/>
+      <c r="Q26" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/marken-healthtech-limited-32168396/</t>
         </is>
       </c>
-      <c r="R25" s="1" t="inlineStr"/>
-      <c r="S25" s="1" t="inlineStr"/>
-      <c r="T25" s="1" t="inlineStr">
+      <c r="R26" s="1" t="inlineStr"/>
+      <c r="S26" s="1" t="inlineStr"/>
+      <c r="T26" s="1" t="inlineStr">
         <is>
           <t>Hospital, Diagnostic Laboratory, Pathology Lab</t>
         </is>
       </c>
-      <c r="U25" s="1" t="inlineStr">
+      <c r="U26" s="1" t="inlineStr">
         <is>
           <t>Hospital, Diagnostic Laboratory, Pathology Lab</t>
         </is>
       </c>
+      <c r="V26" s="1" t="inlineStr"/>
     </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
         <is>
           <t>Semi Automated Clinical Chemistry Analyzer - Application: Laboratory</t>
         </is>
       </c>
-      <c r="B26" s="1" t="inlineStr">
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Lifeline Distribution</t>
         </is>
       </c>
-      <c r="C26" s="1" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>Semi Automated Clinical Chemistry Analyzer</t>
         </is>
       </c>
-      <c r="D26" s="1" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/semi-automated-clinical-chemistry-analyzer-c11825292.html</t>
         </is>
       </c>
-      <c r="E26" s="1" t="inlineStr">
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>https://cpimg.tistatic.com/11825292/b/4/Semi-Automated-Clinical-Chemistry-Analyzer..webp</t>
         </is>
       </c>
-      <c r="F26" s="1" t="inlineStr"/>
-      <c r="G26" s="1" t="inlineStr">
+      <c r="F27" s="1" t="inlineStr"/>
+      <c r="G27" s="1" t="inlineStr">
         <is>
           <t>Laboratory</t>
         </is>
       </c>
-      <c r="H26" s="1" t="inlineStr">
+      <c r="H27" s="1" t="inlineStr">
         <is>
           <t>Erba Chem 5X Clinical Chemistry Analyzer - Application: Laboratory: https://www.tradeindia.com/products/erba-chem-5x-clinical-chemistry-analyzer-c11825289.html
 Om-120 Biochemistry Analyzer - Application: Industrial: https://www.tradeindia.com/products/om-120-biochemistry-analyzer-c11636025.html
@@ -2924,73 +3049,74 @@
 20 X 17 X 11 Inch 1.16 Kilogram ABS And Mild Steel Clinical Chemistry Analyzer: https://www.tradeindia.com/products/20-x-17-x-11-inch-1-16-kilogram-abs-mild-steel-clinical-chemistry-analyzer-8319759.html</t>
         </is>
       </c>
-      <c r="I26" s="1" t="inlineStr">
+      <c r="I27" s="1" t="inlineStr">
         <is>
           <t>Lifeline Distribution</t>
         </is>
       </c>
-      <c r="J26" s="1" t="inlineStr"/>
-      <c r="K26" s="1" t="inlineStr"/>
-      <c r="L26" s="1" t="inlineStr">
+      <c r="J27" s="1" t="inlineStr"/>
+      <c r="K27" s="1" t="inlineStr"/>
+      <c r="L27" s="1" t="inlineStr">
         <is>
           <t>Lifeline Distribution</t>
         </is>
       </c>
-      <c r="M26" s="1" t="inlineStr">
+      <c r="M27" s="1" t="inlineStr">
         <is>
           <t>Lifeline Distribution</t>
         </is>
       </c>
-      <c r="N26" s="1" t="inlineStr">
+      <c r="N27" s="1" t="inlineStr">
         <is>
           <t>Lifeline Distribution operates with the objective of strengthening healthcare delivery by ensuring dependable access to essential medical and diagnostic products. Based in Srinagar, Jammu and Kashmir, we are a trusted trader, wholesaler, supplier, and service provider, addressing the evolving needs of laboratories, hospitals, and healthcare professionals. Our business approach emphasizes reliability, accuracy, and professional engagement across every transaction.Our portfolio includes Centrifuge Machine, Micron CXL Microscope, Pathology Lab Management Software, Chemiluminescence Analyzer and Surgical Hand Gloves. These products play a critical role in diagnostics, laboratory efficiency, and clinical safety. We ensure that all offerings are sourced and supplied with attention to performance standards and application sui Business Type Service Provider, Supplier, Trading Company, Wholesaler Employee Count 10 Establishment 2017 Working Days Monday To Sunday GST NO 01EMXPA3156A1ZI Related Products Erba Chem 5X Clinical Chemistry Analyzer - Application: Laboratory Price: 75000 INR MOQ - 1 Unit/Units Lifeline Distribution Srinagar, Jammu and Kashmir</t>
         </is>
       </c>
-      <c r="O26" s="1" t="inlineStr"/>
-      <c r="P26" s="1" t="inlineStr"/>
-      <c r="Q26" s="1" t="inlineStr">
+      <c r="O27" s="1" t="inlineStr"/>
+      <c r="P27" s="1" t="inlineStr"/>
+      <c r="Q27" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/lifeline-distribution-35105571/</t>
         </is>
       </c>
-      <c r="R26" s="1" t="inlineStr"/>
-      <c r="S26" s="1" t="inlineStr"/>
-      <c r="T26" s="1" t="inlineStr">
+      <c r="R27" s="1" t="inlineStr"/>
+      <c r="S27" s="1" t="inlineStr"/>
+      <c r="T27" s="1" t="inlineStr">
         <is>
           <t>Laboratory</t>
         </is>
       </c>
-      <c r="U26" s="1" t="inlineStr"/>
+      <c r="U27" s="1" t="inlineStr"/>
+      <c r="V27" s="1" t="inlineStr"/>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>Clover A1c (hba1c Analyzer) at Best Price in Bengaluru | Benaka Health Care</t>
         </is>
       </c>
-      <c r="B27" s="1" t="inlineStr"/>
-      <c r="C27" s="1" t="inlineStr">
+      <c r="B28" s="1" t="inlineStr"/>
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>Benaka Health Care - Offering low price Clover A1c (hba1c Analyzer) in Bsk 3rd Stage, Bengaluru with product details &amp; company information.</t>
         </is>
       </c>
-      <c r="D27" s="1" t="inlineStr">
+      <c r="D28" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/clover-a1c-hba1c-analyzer-c9513981.html</t>
         </is>
       </c>
-      <c r="E27" s="1" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>https://cpimg.tistatic.com/09513981/b/4/Clover-A1c-HbA1c-Analyzer-.jpg</t>
         </is>
       </c>
-      <c r="F27" s="1" t="inlineStr"/>
-      <c r="G27" s="1" t="inlineStr">
+      <c r="F28" s="1" t="inlineStr"/>
+      <c r="G28" s="1" t="inlineStr">
         <is>
           <t>Diagnostics for Glycated Hemoglobin (HbA1c)</t>
         </is>
       </c>
-      <c r="H27" s="1" t="inlineStr">
+      <c r="H28" s="1" t="inlineStr">
         <is>
           <t>Medical Machinery: https://www.tradeindia.com/products/medical-machinery-9641281.html
 ENDOMED DUO - Medical Grade Material, Variable Dimensions | Compact Size, Durable Design, Precise Control, Ergonomic, Reliable Performance: https://www.tradeindia.com/products/endomed-duo-21-5919013.html
@@ -3011,69 +3137,70 @@
 Hospital Phototherapy Machine: https://www.tradeindia.com/products/hospital-phototherapy-machine-5539798.html</t>
         </is>
       </c>
-      <c r="I27" s="1" t="inlineStr"/>
-      <c r="J27" s="1" t="inlineStr"/>
-      <c r="K27" s="1" t="inlineStr"/>
-      <c r="L27" s="1" t="inlineStr"/>
-      <c r="M27" s="1" t="inlineStr"/>
-      <c r="N27" s="1" t="inlineStr">
+      <c r="I28" s="1" t="inlineStr"/>
+      <c r="J28" s="1" t="inlineStr"/>
+      <c r="K28" s="1" t="inlineStr"/>
+      <c r="L28" s="1" t="inlineStr"/>
+      <c r="M28" s="1" t="inlineStr"/>
+      <c r="N28" s="1" t="inlineStr">
         <is>
           <t>Know Us Benaka Health Care (A Division Of Benaka Business Consultancy) is a reputed name in the sector of Syringe Pump, Digital X Ray System, Radiation Protection Products, Ultrasound System, Cardiology System, ECG Machine, Critical Care Product, Patient Monitor, etc. Committed to provide innovative, branded and cost-effective products, we have been offering the best solutions to the medical industry. We have developed a business alliance with the major names of the industry to provide clients with the matchless range. With prompt sales, customer service and service efficiency, we have become the icon of trust for the patrons. Incepted in the year of 2009, we Business Type Manufacturer, Service Provider, Supplier, Trading Company Employee Count 25 Establishment 2009 Working Days Monday To Sunday GST NO 29ADHPC5601P1ZC Payment Mode Online Payments (NEFT/RTGS/IMPS), Cheque/DD, Wallet &amp; UPI Related Products Medical Machinery Price: 5000 INR MOQ - 100 Piece/Pieces Naturoinfra Private Limited Indore, Madhya Pradesh</t>
         </is>
       </c>
-      <c r="O27" s="1" t="inlineStr"/>
-      <c r="P27" s="1" t="inlineStr"/>
-      <c r="Q27" s="1" t="inlineStr">
+      <c r="O28" s="1" t="inlineStr"/>
+      <c r="P28" s="1" t="inlineStr"/>
+      <c r="Q28" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/clover-a1c-hba1c-analyzer-c9513981.html</t>
         </is>
       </c>
-      <c r="R27" s="1" t="inlineStr"/>
-      <c r="S27" s="1" t="inlineStr"/>
-      <c r="T27" s="1" t="inlineStr">
+      <c r="R28" s="1" t="inlineStr"/>
+      <c r="S28" s="1" t="inlineStr"/>
+      <c r="T28" s="1" t="inlineStr">
         <is>
           <t>Diagnostics for Glycated Hemoglobin (HbA1c)</t>
         </is>
       </c>
-      <c r="U27" s="1" t="inlineStr">
+      <c r="U28" s="1" t="inlineStr">
         <is>
           <t>Diagnostics for Glycated Hemoglobin (HbA1c)</t>
         </is>
       </c>
+      <c r="V28" s="1" t="inlineStr"/>
     </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t>Semi Automatic Analyzer - Features: Stable Operation - Features: Stable Operation at Best Price in Coimbatore | Venus Health Care</t>
         </is>
       </c>
-      <c r="B28" s="1" t="inlineStr"/>
-      <c r="C28" s="1" t="inlineStr">
+      <c r="B29" s="1" t="inlineStr"/>
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>Venus Health Care - Offering low price Semi Automatic Analyzer - Features: Stable Operation - Features: Stable Operation in Brindavan Nagar, Coimbatore with product details &amp; company information.</t>
         </is>
       </c>
-      <c r="D28" s="1" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/semi-automatic-analyzer-c11541591.html</t>
         </is>
       </c>
-      <c r="E28" s="1" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>https://cpimg.tistatic.com/11541591/b/4/Semi-Automatic-Analyzer..jpg</t>
         </is>
       </c>
-      <c r="F28" s="1" t="inlineStr">
+      <c r="F29" s="1" t="inlineStr">
         <is>
           <t>Stable operation Payment Terms Cash in Advance (CID) Supply Ability 15 Per Month Delivery Time 2-10</t>
         </is>
       </c>
-      <c r="G28" s="1" t="inlineStr">
+      <c r="G29" s="1" t="inlineStr">
         <is>
           <t>Laboratory</t>
         </is>
       </c>
-      <c r="H28" s="1" t="inlineStr">
+      <c r="H29" s="1" t="inlineStr">
         <is>
           <t>Semi Auto Analyzer - ABS Plastic, 10x12x15 cm, 220V AC | Automatic Calibration, LCD Display, Microprocessor Based, Portable: https://www.tradeindia.com/products/semi-auto-analyzer-c3738939.html
 Semi Auto Analyzer 2 Year Warranty Application: Industrial: https://www.tradeindia.com/products/semi-auto-analyser-2-year-warranty-c8093789.html
@@ -3099,73 +3226,74 @@
 Mission U120 Urine Analyzer - Automation Grade: Semi - Automatic: https://www.tradeindia.com/products/mission-u120-urine-analyzer-c11541593.html</t>
         </is>
       </c>
-      <c r="I28" s="1" t="inlineStr">
+      <c r="I29" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="J28" s="1" t="inlineStr"/>
-      <c r="K28" s="1" t="inlineStr"/>
-      <c r="L28" s="1" t="inlineStr">
+      <c r="J29" s="1" t="inlineStr"/>
+      <c r="K29" s="1" t="inlineStr"/>
+      <c r="L29" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="M28" s="1" t="inlineStr">
+      <c r="M29" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="N28" s="1" t="inlineStr">
+      <c r="N29" s="1" t="inlineStr">
         <is>
           <t>Venus Health Care is a trusted and professionally managed organization engaged in supplying and trading a wide range of high-quality medical and diagnostic equipment. With a strong commitment to reliability, innovation, and customer satisfaction, we have established ourselves as a preferred partner for healthcare professionals, laboratories, hospitals, and clinics across the region. Our product portfolio includes advanced and precision-engineered instruments such as Immunoassay Analyzers, Blood Pressure Monitors, Digital Hemoglobin (Hb) Meters, On Call Plus Blood Glucose Test Strips, Blood Glucose Monitors, and many other diagnostic and medical devices.At Venus Health Care, we believe that access to accurate and efficient healthcare technology is vital for improving patient outcomes and enhancing clinical performance. Business Type Supplier, Trading Company Employee Count 2 Establishment 2017 Working Days Monday To Sunday GST NO 33ASFPR8169J2Z5 Related Products Semi Auto Analyzer - ABS Plastic, 10x12x15 cm, 220V AC | Automatic Calibration, LCD Display, Microprocessor Based, Portable Analyze Biotech Private Limited Chennai, Tamil Nadu</t>
         </is>
       </c>
-      <c r="O28" s="1" t="inlineStr"/>
-      <c r="P28" s="1" t="inlineStr"/>
-      <c r="Q28" s="1" t="inlineStr">
+      <c r="O29" s="1" t="inlineStr"/>
+      <c r="P29" s="1" t="inlineStr"/>
+      <c r="Q29" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/semi-automatic-analyzer-c11541591.html</t>
         </is>
       </c>
-      <c r="R28" s="1" t="inlineStr"/>
-      <c r="S28" s="1" t="inlineStr"/>
-      <c r="T28" s="1" t="inlineStr">
+      <c r="R29" s="1" t="inlineStr"/>
+      <c r="S29" s="1" t="inlineStr"/>
+      <c r="T29" s="1" t="inlineStr">
         <is>
           <t>Laboratory</t>
         </is>
       </c>
-      <c r="U28" s="1" t="inlineStr"/>
+      <c r="U29" s="1" t="inlineStr"/>
+      <c r="V29" s="1" t="inlineStr"/>
     </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr">
         <is>
           <t>Clinical Chemistry Analyzer</t>
         </is>
       </c>
-      <c r="B29" s="1" t="inlineStr"/>
-      <c r="C29" s="1" t="inlineStr">
+      <c r="B30" s="1" t="inlineStr"/>
+      <c r="C30" s="1" t="inlineStr">
         <is>
           <t>Buy low price Clinical Chemistry Analyzer in Kidwai Nagar, Kanpur. Clinical Chemistry Analyzer offered by Jks Enterprises is available with multiple payment options and easy delivery.</t>
         </is>
       </c>
-      <c r="D29" s="1" t="inlineStr">
+      <c r="D30" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/clinical-chemistry-analyzer-c11977827.html</t>
         </is>
       </c>
-      <c r="E29" s="1" t="inlineStr">
+      <c r="E30" s="1" t="inlineStr">
         <is>
           <t>https://cpimg.tistatic.com/11977827/b/4/Clinical-Chemistry-Analyzer..png</t>
         </is>
       </c>
-      <c r="F29" s="1" t="inlineStr"/>
-      <c r="G29" s="1" t="inlineStr">
+      <c r="F30" s="1" t="inlineStr"/>
+      <c r="G30" s="1" t="inlineStr">
         <is>
           <t>Biochemical Analysis in Medical Laboratories</t>
         </is>
       </c>
-      <c r="H29" s="1" t="inlineStr">
+      <c r="H30" s="1" t="inlineStr">
         <is>
           <t>Smart Biochemistry Analyzer: https://www.tradeindia.com/products/smart-biochemistry-analyzer-c11977823.html
 Horiba Yumizen Ca60 Clinical Chemistry Analyzer - Color: Blue And White: https://www.tradeindia.com/products/horiba-yumizen-ca60-clinical-chemistry-analyzer-c11160991.html
@@ -3187,140 +3315,3156 @@
 Chemistry Analyzer (BS-380): https://www.tradeindia.com/products/chemistry-analyzer-bs-380-4552405.html</t>
         </is>
       </c>
-      <c r="I29" s="1" t="inlineStr">
+      <c r="I30" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="J29" s="1" t="inlineStr"/>
-      <c r="K29" s="1" t="inlineStr"/>
-      <c r="L29" s="1" t="inlineStr">
+      <c r="J30" s="1" t="inlineStr"/>
+      <c r="K30" s="1" t="inlineStr"/>
+      <c r="L30" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="M29" s="1" t="inlineStr">
+      <c r="M30" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="N29" s="1" t="inlineStr">
+      <c r="N30" s="1" t="inlineStr">
         <is>
           <t>JKS Enterprises is a trusted supplier and trader of advanced diagnostic and medical testing solutions, committed to supporting accurate, efficient, and reliable healthcare delivery. With a strong focus on quality and performance, we provide a carefully selected range of products that meet the evolving needs of hospitals, diagnostic laboratories, clinics, and healthcare professionals. Our product portfolio includes the Z5 Hematology Analyzer, designed for precise and dependable blood analysis, and the Aphera Fully Automated Biochemistry Analyzer, known for its high throughput, automation, and consistent results. We also supply the Xpress Gluco Blood Glucose Monitoring System and Xpress Glucometer, which offer quick, user-friendly, and accurate glucose testing for both clinical and personal use. At JKS Enterprises, we believe that dependable diagnostics are the foundation of effective medical car Business Type Supplier, Trading Company Employee Count 12 Establishment 2018 Working Days Monday To Sunday GST NO 09BXHPP5458C1Z7 Payment Mode Online Payments (NEFT/RTGS/IMPS), Cheque/DD, Wallet &amp; UPI, Cash Related Products Smart Biochemistry Analyzer MOQ - 10 Unit/Units Jks Enterprises Kanpur, Uttar Pradesh</t>
         </is>
       </c>
-      <c r="O29" s="1" t="inlineStr"/>
-      <c r="P29" s="1" t="inlineStr"/>
-      <c r="Q29" s="1" t="inlineStr">
+      <c r="O30" s="1" t="inlineStr"/>
+      <c r="P30" s="1" t="inlineStr"/>
+      <c r="Q30" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/clinical-chemistry-analyzer-c11977827.html</t>
         </is>
       </c>
-      <c r="R29" s="1" t="inlineStr"/>
-      <c r="S29" s="1" t="inlineStr"/>
-      <c r="T29" s="1" t="inlineStr">
+      <c r="R30" s="1" t="inlineStr"/>
+      <c r="S30" s="1" t="inlineStr"/>
+      <c r="T30" s="1" t="inlineStr">
         <is>
           <t>Biochemical Analysis in Medical Laboratories</t>
         </is>
       </c>
-      <c r="U29" s="1" t="inlineStr">
+      <c r="U30" s="1" t="inlineStr">
         <is>
           <t>Biochemical Analysis in Medical Laboratories</t>
         </is>
       </c>
+      <c r="V30" s="1" t="inlineStr"/>
     </row>
-    <row r="30">
-      <c r="A30" s="1" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
         <is>
           <t>Bs 430 Mindray Clinical Chemistry Analyzer - Attributes: Easy To Operate</t>
         </is>
       </c>
-      <c r="B30" s="1" t="inlineStr">
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>ROYAL DIAGNOSTIC &amp; SURGICAL</t>
         </is>
       </c>
-      <c r="C30" s="1" t="inlineStr">
+      <c r="C31" s="1" t="inlineStr">
         <is>
           <t>BS 430 Mindray Clinical Chemistry Analyzer</t>
         </is>
       </c>
-      <c r="D30" s="1" t="inlineStr">
+      <c r="D31" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/bs-430-mindray-clinical-chemistry-analyzer-c8458715.html</t>
         </is>
       </c>
-      <c r="E30" s="1" t="inlineStr">
+      <c r="E31" s="1" t="inlineStr">
         <is>
           <t>https://cpimg.tistatic.com/08458715/b/4/BS-430-Mindray-Clinical-Chemistry-Analyzer.jpg</t>
         </is>
       </c>
-      <c r="F30" s="1" t="inlineStr"/>
-      <c r="G30" s="1" t="inlineStr">
+      <c r="F31" s="1" t="inlineStr"/>
+      <c r="G31" s="1" t="inlineStr">
         <is>
           <t>Hospital</t>
         </is>
       </c>
-      <c r="H30" s="1" t="inlineStr">
+      <c r="H31" s="1" t="inlineStr">
         <is>
           <t>Clinical Chemistry Analyzer - Color: White: https://www.tradeindia.com/products/clinical-chemistry-analyzer-c11771172.html
 Electrolyte Analyzer Erma El-120 ( Agd ) - Color: White: https://www.tradeindia.com/products/electrolyte-analyzer-erma-el-120-agd-c8438396.html
 Hematology Analyzer Application: Laboratory/Hospital/Pharmaceutical Industry: https://www.tradeindia.com/products/hematology-analyzer-c8355968.html
 Labman Bod Analyzer - Accuracy: A 1.0 %: https://www.tradeindia.com/products/labman-bod-analyzer-c11508527.html
 Semi Automatic Clinical Analyzer Application: Diagnostic Lab: https://www.tradeindia.com/products/semi-automatic-clinical-analyzer-4227341.html
-Bpl Smartoxy Fingertip Pulse Oximeter - Material: Plastic: https://www.tradeindia.com/products/bpl-smartoxy-fingertip-pulse-oximeter-c7998308.html
-Fully Auto Hematology Analyzer - 5 Part - Attributes: Higher Level Of Accuracy: https://www.tradeindia.com/products/fully-auto-hematology-analyzer-5-part-c8639165.html
-Accurex Semi Automatic 5 Parameters Automated Electrolyte Analyzer - Color: White: https://www.tradeindia.com/products/accurex-semi-automatic-5-parameters-automated-electrolyte-analyzer-c8440576.html
-Sd Biosensor Fully Automatic Standard F200 Immunoassay Analyzer - Attributes: Higher Level Of Accuracy: https://www.tradeindia.com/products/sd-biosensor-fully-automatic-standard-f200-immunoassay-analyzer-c8531788.html
-Paper Bayer Keto Diastix Reagent 50 Strips For Urinalysis - Grade: Industrial: https://www.tradeindia.com/products/paper-bayer-keto-diastix-reagent-50-strips-for-urinalysis-c7998228.html
-500 Ml Acetone Solvent - Grade: Commercial: https://www.tradeindia.com/products/500-ml-acetone-solvent-c7998255.html
-Creatinine 200 Reagent - Grade: Commercial: https://www.tradeindia.com/products/creatinine-200-reagent-c7998265.html
-Cotton Swab Stick - 100 Pcs Sterilized Medical Grade , Disposable with Cuff for Easy Sampling: https://www.tradeindia.com/products/100-pcs-easy-pick-sampler-axiom-swab-stick-c7998305.html
-Semi Automatic Esr Automated Analyzer Model Esr 20Plus - Attributes: Higher Level Of Accuracy: https://www.tradeindia.com/products/semi-automatic-esr-automated-analyzer-model-esr-20plus-c8445392.html
-5-Part Haematology Analyzer Zybio Z5 Hematology Analyser - Attributes: Easy To Operate: https://www.tradeindia.com/products/5-part-haematology-analyzer-zybio-z5-hematology-analyser-c8501902.html
+Black Remi Flabo X Phlebotomy Chair - Usage: Hospital: https://www.tradeindia.com/products/black-remi-flabo-x-phlebotomy-chair-c8445403.html
+Rbc Semi Automatic Agd 300 Hematology Analyzers - Attributes: Higher Level Of Accuracy: https://www.tradeindia.com/products/rbc-semi-automatic-agd-300-hematology-analyzers-c8452768.html
+Mindray Bs 240 E Analyzer - Attributes: Higher Level Of Accuracy: https://www.tradeindia.com/products/mindray-bs-240-e-analyzer-c8459363.html
+Bt 4500 Semi Automatic Biochemistry Analyzer - Attributes: Easy To Operate: https://www.tradeindia.com/products/bt-4500-fully-automatic-biochemistry-analyzer-c8624757.html
+Cell Counter Eurocount 5L - Attributes: Higher Level Of Accuracy: https://www.tradeindia.com/products/cell-counter-eurocount-5l-c8471224.html
+J Mitra Iquant Immunoassay Analyzer - Attributes: Easy To Operate: https://www.tradeindia.com/products/j-mitra-iquant-immunoassay-analyzer-c8515468.html
+Mispa I3 Protein Analyzer - Color: Red: https://www.tradeindia.com/products/mispa-i3-protein-analyzer-c7998231.html
+Leishman Stain Solution - Commercial Grade, 99% Purity | Ideal for Blood Smears and Pathogen Analysis, High-Quality Industrial Lab Chemical: https://www.tradeindia.com/products/leishman-stain-solution-c7998263.html
+J. Mitra Elisa Reader - Attributes: Higher Level Of Accuracy: https://www.tradeindia.com/products/j-mitra-elisa-reader-c8524395.html
+Diasys Hematology Analyzer - Attributes: Safe To Use: https://www.tradeindia.com/products/diasys-hematology-analyzer-c8082665.html
 RD 50+ Smart Touch Semi - Auto Biochemistry Analyzer: https://www.tradeindia.com/products/rd-50-smart-touch-semi-auto-biochemistry-analyzer-c4568987.html</t>
         </is>
       </c>
-      <c r="I30" s="1" t="inlineStr">
+      <c r="I31" s="1" t="inlineStr">
         <is>
           <t>ROYAL DIAGNOSTIC &amp; SURGICAL</t>
         </is>
       </c>
-      <c r="J30" s="1" t="inlineStr"/>
-      <c r="K30" s="1" t="inlineStr"/>
-      <c r="L30" s="1" t="inlineStr">
+      <c r="J31" s="1" t="inlineStr"/>
+      <c r="K31" s="1" t="inlineStr"/>
+      <c r="L31" s="1" t="inlineStr">
         <is>
           <t>ROYAL DIAGNOSTIC &amp; SURGICAL</t>
         </is>
       </c>
-      <c r="M30" s="1" t="inlineStr">
+      <c r="M31" s="1" t="inlineStr">
         <is>
           <t>ROYAL DIAGNOSTIC &amp; SURGICAL</t>
         </is>
       </c>
-      <c r="N30" s="1" t="inlineStr">
+      <c r="N31" s="1" t="inlineStr">
         <is>
           <t>With the exponential growth of diseases, the need for various medical and research-related products like Agar Plate, ESR Pipette, Vacutainer Blood Collection Tubes, Yumizen H500 Ct Hematology Analyzer, Cotton Crepe Bandage, Binocular Microscope, etc., have grown rapidly. Our company, Royal Diagnostic &amp; Surgical, is known as one of the leading traders, suppliers, and retailers of such products. We provide our customers with top-quality products and that has helped us set a strong foothold for ourselves in the market. Our good market reputation and professional work ethic have helped us gain the trust of our clients. We give our hundred percent to each project and make sure that we uphold the trust that our customers have put in us. Moreover, our more than 10 years of experience in this industry gives us an edge over our competitors. Our expert team of professional analy Business Type Exporter, Manufacturer, Distributor, Supplier, Trading Company, Wholesaler, Retailer, Dealer Employee Count 10 Establishment 2009 Working Days Monday To Sunday GST NO 07BCKPP5842C1ZJ Payment Mode Online Payments (NEFT/RTGS/IMPS), Cheque/DD Related Products Clinical Chemistry Analyzer - Color: White Price: 580000 INR MOQ - 1 Piece/Pieces Drx Laboratories India Inc New Delhi, Delhi</t>
         </is>
       </c>
-      <c r="O30" s="1" t="inlineStr"/>
-      <c r="P30" s="1" t="inlineStr"/>
-      <c r="Q30" s="1" t="inlineStr">
+      <c r="O31" s="1" t="inlineStr"/>
+      <c r="P31" s="1" t="inlineStr"/>
+      <c r="Q31" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/royal-diagnostic-surgical-29441814/</t>
         </is>
       </c>
-      <c r="R30" s="1" t="inlineStr"/>
-      <c r="S30" s="1" t="inlineStr"/>
-      <c r="T30" s="1" t="inlineStr">
+      <c r="R31" s="1" t="inlineStr"/>
+      <c r="S31" s="1" t="inlineStr"/>
+      <c r="T31" s="1" t="inlineStr">
         <is>
           <t>Hospital</t>
         </is>
       </c>
-      <c r="U30" s="1" t="inlineStr"/>
+      <c r="U31" s="1" t="inlineStr"/>
+      <c r="V31" s="1" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>Labcare Export Auto Biochemistry Analyzer at Best Price in Ambala Cantt | Labcare Instruments &amp; International Services</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr"/>
+      <c r="C32" s="1" t="inlineStr">
+        <is>
+          <t>Labcare Instruments &amp; International Services - Offering low price Labcare Export Auto Biochemistry Analyzer in Pragati Vihar, Ambala Cantt with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="D32" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/labcare-export-auto-biochemistry-analyzer-c6741418.html</t>
+        </is>
+      </c>
+      <c r="E32" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/06741418/b/4/Labcare-Export-Auto-Biochemistry-Analyzer.png</t>
+        </is>
+      </c>
+      <c r="F32" s="1" t="inlineStr">
+        <is>
+          <t>Labcare Instruments And International Services Ambala labcare India. Labcare instruments And Interna</t>
+        </is>
+      </c>
+      <c r="G32" s="1" t="inlineStr">
+        <is>
+          <t>Hospital, Clinic, Laboratory</t>
+        </is>
+      </c>
+      <c r="H32" s="1" t="inlineStr">
+        <is>
+          <t>Digital Thermometers - Color: Blue: https://www.tradeindia.com/products/digital-thermometers-c5467261.html
+Digital Thermometer: https://www.tradeindia.com/products/digital-thermometer-c9590069.html
+Digital Tele Thermometer - Stainless Steel, Clinical Use | 220 Voltage, Cream Color: https://www.tradeindia.com/products/digital-tele-thermometer-c4305901.html
+Digital Thermometer - Automation Grade: No: https://www.tradeindia.com/products/digital-thermometer-c11621035.html
+Digital Thermometer - Color: White: https://www.tradeindia.com/products/digital-thermometer-c11821762.html
+Temperature Meters - External Size: Handheld Perch: https://www.tradeindia.com/products/temperature-meters-c4399878.html
+Black Digital Temperature Meter: https://www.tradeindia.com/products/digital-temperature-meter-c5377869.html
+Digital Temperature Meter - 3Â½ Digit LED Display, 0-100ÂºC Temperature Range | Exceptional Accuracy Â± 0.01 pH, Long Service Life: https://www.tradeindia.com/products/digital-temperature-meter-1791028.html
+Kjeldhal flask with joint: https://www.tradeindia.com/products/kjeldhal-flask-with-joint-c5968097.html
+Labcare Export Fridge Storage Container: https://www.tradeindia.com/products/labcare-export-fridge-storage-container-c6455952.html
+Labcare Export Milk Chiller: https://www.tradeindia.com/products/labcare-export-milk-chiller-c6743910.html
+Labcare Export Kitchen Rack Stand: https://www.tradeindia.com/products/labcare-export-kitchen-rack-stand-c6453711.html
+Labcare Export Decorador Papa Confeito: https://www.tradeindia.com/products/labcare-export-decorador-papa-confeito-c6453757.html
+Labcare Export Wet Grinder: https://www.tradeindia.com/products/labcare-export-wet-grinder-c6743707.html
+boss head (any angal ) labcare: https://www.tradeindia.com/products/boss-head-any-angal-labcare-c5916578.html
+Laboratory jack Labcare: https://www.tradeindia.com/products/laboratory-jack-labcare-c5917920.html
+LABCARE EDUCATIONAL EQUIPMENT IN DEHRADUN: https://www.tradeindia.com/products/labcare-educational-equipment-in-dehradun-c6222567.html
+Labcare Secondary Science Lab Kit In Ambala: https://www.tradeindia.com/products/labcare-secondary-science-lab-kit-in-ambala-c6239987.html
+Labcare Export Microprocessor pH Cond. mV-Temp. Meter - ABS Body, 230x180x70 mm, pH 0-14, Conductivity 0-200 ms/cm, Temp 0-100Â°C | Multi-Parameter Measurement, Large Backlit LCD, Auto Temperature Compensation, 1000 Data Storage: https://www.tradeindia.com/products/labcare-export-microprocessor-ph-cond-mv-temp-meter-c6741282.html
+Labcare Export Digital pH Meter (Portable): https://www.tradeindia.com/products/labcare-export-digital-ph-meter-portable-c6742292.html
+Labcare Export Microprocessor pH-MV-Temp.Meter LB-961 - ABS Plastic Body, 230x200x90 mm, pH 0.00-14.00, mV Â±1999.9, Temp 0-100Â°C | 3-Point Auto Calibration, Auto Buffer Recognition, Digital LCD, Glass Combination Electrode: https://www.tradeindia.com/products/labcare-export-microprocessor-ph-mv-temp-meter-c6741128.html
+Labcare Export Digital Leak Test Apparatus: https://www.tradeindia.com/products/labcare-export-digital-leak-test-apparatus-c6741933.html
+Labcare Export Auto Karl Fischer Titrimeter: https://www.tradeindia.com/products/labcare-export-auto-karl-fischer-titrimeter-c6740503.html
+Labcare Export Digital Dissolved Meter (Portable) - ABS Plastic, 185x40x35 mm, 0.0-20.0 mg/L Range, Replaceable Electrode, Digital LCD Display, Battery Powered: https://www.tradeindia.com/products/labcare-export-digital-dissolved-meter-portable-c6742378.html
+Labcare Export Digital pH Meter: https://www.tradeindia.com/products/labcare-export-digital-ph-meter-c6741087.html
+Labcare Export Digital Dissolved Oxygen Meter: https://www.tradeindia.com/products/labcare-export-digital-dissolved-oxygen-meter-c6741226.html</t>
+        </is>
+      </c>
+      <c r="I32" s="1" t="inlineStr"/>
+      <c r="J32" s="1" t="inlineStr"/>
+      <c r="K32" s="1" t="inlineStr"/>
+      <c r="L32" s="1" t="inlineStr"/>
+      <c r="M32" s="1" t="inlineStr"/>
+      <c r="N32" s="1" t="inlineStr">
+        <is>
+          <t>LABCARE INSTRUMENTS &amp; INTERNATIONAL SERVICES , Established in 1986 at Ambala Cantt in Haryana, is a leading service provider of Scientific Instruments in India. LABCARE INSTRUMENTS &amp; INTERNATIONAL SERVICES is one of Trade India's verified and trusted names for listed services. With extensive experience in the field of Scientific Instruments, LABCARE INSTRUMENTS &amp; INTERNATIONAL SERVICES has made a reputed name for itself in the market with satisfactory Double Beam UV VIS Spectrophotometer, 2 Jar Digital Programmable Disintegration Apparatus, For Industrial, ABS Bedside locker, etc. Focusing on a customer-centric approach, LABCARE INSTRUMENTS &amp; INTERNATIONAL SERVICES has a pan-India presence and caters to a huge consumer base throughout the country. Get Scientific Instruments from LABCARE INSTRUMENTS &amp; INTERNATIONAL SERVICES at Trade India quality-assured services. Business Type Exporter, Importer, Manufacturer, Service Provider, Distributor, Supplier, Trading Company Employee Count 45 Establishment 1986 Working Days Monday To Sunday GST NO 06DCLPA2906P1ZF Certification ISO 9001 : 2O15 CERTIFIED CO. CE CERTIFIED Related Products Digital Thermometers - Color: Blue Price: 500.0 INR MOQ - 10 Piece/Pieces Micro Teknik Ambala Cantt, Haryana</t>
+        </is>
+      </c>
+      <c r="O32" s="1" t="inlineStr"/>
+      <c r="P32" s="1" t="inlineStr"/>
+      <c r="Q32" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/labcare-export-auto-biochemistry-analyzer-c6741418.html</t>
+        </is>
+      </c>
+      <c r="R32" s="1" t="inlineStr"/>
+      <c r="S32" s="1" t="inlineStr"/>
+      <c r="T32" s="1" t="inlineStr">
+        <is>
+          <t>Hospital, Clinic, Laboratory</t>
+        </is>
+      </c>
+      <c r="U32" s="1" t="inlineStr"/>
+      <c r="V32" s="1" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr">
+        <is>
+          <t>Hematology Analyzer</t>
+        </is>
+      </c>
+      <c r="B33" s="1" t="inlineStr">
+        <is>
+          <t>SURGICAL WHOLESALE MART PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="C33" s="1" t="inlineStr">
+        <is>
+          <t>Hematology Analyzer</t>
+        </is>
+      </c>
+      <c r="D33" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/hematology-analyzer-c8355968.html</t>
+        </is>
+      </c>
+      <c r="E33" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/08355968/b/6/Hematology-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F33" s="1" t="inlineStr"/>
+      <c r="G33" s="1" t="inlineStr"/>
+      <c r="H33" s="1" t="inlineStr">
+        <is>
+          <t>Celquant Edge 3 Part Hematology Analyzer - Color: As Per Availability: https://www.tradeindia.com/products/celquant-edge-3-part-hematology-analyzer-c9144592.html
+3 Part Hematology Analyzer Eurocount Plus Cell Counter - Color: White: https://www.tradeindia.com/products/3-part-hematology-analyzer-eurocount-plus-cell-counter-c7998229.html
+Hospital Automatic Hematology Analyzer: https://www.tradeindia.com/products/hospital-automatic-hematology-analyzer-c2734751.html
+2 Chambers 220 Volts Electrical Hematology Analyzers For Run Tests On Blood Samples Application: Clinical: https://www.tradeindia.com/products/2-chambers-220-volt-clinical-hematology-analyzers-8376330.html
+Reliable Nature Easily Operate Veterinary Hematology Analyzer For Pets (Mek-6550J/K) Application: Food: https://www.tradeindia.com/products/to-conduct-a-complete-blood-count-gentle-veterinary-care-hematology-analyzer-7487639.html
+Carecell-23 Hematology Analyzer: https://www.tradeindia.com/products/carecell-23-hematology-analyzer-209254.html
+Fully Automatic Hematology Analyzer: https://www.tradeindia.com/products/fully-automatic-hematology-analyzer-c3704793.html
+Easy To Operate 3 Part Hematology Analyzer: https://www.tradeindia.com/products/3-part-hematology-analyzer-c5656091.html
+Fully Automatic Hematology Analyzer - 43x32x50 cm, Electro-impedance, 22 Parameters | Easy Operation, 24/7 Standby, Built-in Thermal Printer: https://www.tradeindia.com/products/fully-automatic-hematology-analyzer-c948652.html
+Black Om-51-5 Part Hematology Analyzer: https://www.tradeindia.com/products/om-51-5-part-hematology-analyzer-c7737370.html
+Five Part Hematology Analyzer: https://www.tradeindia.com/products/five-part-hematology-analyzer-3216232.html
+Telescopic Delivery Obstetric Bed - Dimension (L*W*H): 100 L X 80 W X 75 H Cm: https://www.tradeindia.com/products/telescopic-delivery-obstetric-bed-c8591283.html
+Icu Bed Five Functional Electric (Eco Model) - General Use: Commercial Furniture: https://www.tradeindia.com/products/icu-bed-five-functional-electric-eco-model-c8584461.html
+Eco-Friendly Electric Icu Beds: https://www.tradeindia.com/products/electric-icu-beds-c8355917.html
+Delivery Table Three Fold - Furniture Type: Hospital Bed: https://www.tradeindia.com/products/delivery-table-three-fold-c8590920.html
+I.C.U BED FIVE FUNCTIONAL ELECTRIC: https://www.tradeindia.com/products/i-c-u-bed-five-functional-electric-c8583068.html
+SIMPLE TABLE DELIVERY - Two Section Foam Padded Upholstered Top 187L x 51W x 81H , Gas Spring Adjustability, Three Drawers, Epoxy Coated Finish: https://www.tradeindia.com/products/simple-table-delivery-c8591254.html
+Plain Bed Deluxe Dimension(L*W*H): 220L * 100W * 60-80H Cm: https://www.tradeindia.com/products/plain-bed-deluxe-c8617955.html
+Manual Delivery Table - Stainless Steel Bowl, 180 L x 60 W x 82 H cms, Adjustable Backrest and Knee Crutches, Rubber Shoes Mounted Design: https://www.tradeindia.com/products/manual-delivery-table-3-section-c8591168.html
+O.T TABLE HYDRAULIC - Heavy Duty Steel Base with Nylon Wheels, Five Sectional Top with Perianal Drainage Tray and Kidney Bridge, Smooth Gear Mechanism: https://www.tradeindia.com/products/o-t-table-haydraulic-c8625571.html
+Electro-Mechanical Operation Table - MS Tubular Framework, X-Ray Permeable 8 mm Thick Top | Motorised Height Adjustment, Lateral Tilt, Trendelenburg &amp; Reverse Trendelenburg, Detachable Head Rest and Leg Rest, SS Side Rails: https://www.tradeindia.com/products/electro-mechanical-operation-table-c8625800.html
+ConXport Fully Automatic Hematology Analyzer: https://www.tradeindia.com/products/conxport-fully-automatic-hematology-analyzer-c7208553.html
+BI-H60S 5 Part Hematology Analyzer: https://www.tradeindia.com/products/bi-h60s-5-part-hematology-analyzer-c9145394.html</t>
+        </is>
+      </c>
+      <c r="I33" s="1" t="inlineStr">
+        <is>
+          <t>SURGICAL WHOLESALE MART PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="J33" s="1" t="inlineStr"/>
+      <c r="K33" s="1" t="inlineStr"/>
+      <c r="L33" s="1" t="inlineStr">
+        <is>
+          <t>SURGICAL WHOLESALE MART PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="M33" s="1" t="inlineStr">
+        <is>
+          <t>SURGICAL WHOLESALE MART PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="N33" s="1" t="inlineStr">
+        <is>
+          <t>Surgical Wholesale Mart Private Limited is one of the most renowned companies in India which was established in 2022 under the guidance of its Jalandhar based parent company holding more than 60 years of experience in import, export and trading of medical equipment. The head office of our company is situated in New Delhi whereas the regional offices are located in Bihar and Punjab. Our products like Hospital Beds, Hospital ICU Equipment, Autoclave Pressure Cooker, Mobile OT Light, BPL Anesthesia Workstation, etc. are also supplied across the country through our distributors to government &amp; private hospitals, nursing homes, medical colleges, etc. The hospital equipm Business Type Manufacturer, Supplier Employee Count 101 Establishment 2022 Working Days Monday To Sunday GST NO 07ABJCS0271Q1ZT Related Products Celquant Edge 3 Part Hematology Analyzer - Color: As Per Availability Price: 210000 INR MOQ - 5 Unit/Units Drx Laboratories India Inc New Delhi, Delhi</t>
+        </is>
+      </c>
+      <c r="O33" s="1" t="inlineStr"/>
+      <c r="P33" s="1" t="inlineStr"/>
+      <c r="Q33" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/surgical-wholesale-mart-private-limited-39977655/</t>
+        </is>
+      </c>
+      <c r="R33" s="1" t="inlineStr"/>
+      <c r="S33" s="1" t="inlineStr"/>
+      <c r="T33" s="1" t="inlineStr">
+        <is>
+          <t>Hematology Analyzer</t>
+        </is>
+      </c>
+      <c r="U33" s="1" t="inlineStr"/>
+      <c r="V33" s="1" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>Acon Mission U500 Urine Analyzer at Best Price in Chennai | Saaskin Corporation Private Limited.</t>
+        </is>
+      </c>
+      <c r="B34" s="1" t="inlineStr"/>
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>Saaskin Corporation Private Limited. - Offering low price Acon Mission U500 Urine Analyzer in Kilpauk, Chennai with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/acon-mission-u500-urine-analyzer-c9992154.html</t>
+        </is>
+      </c>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/09992154/b/4/Acon-Mission-U500-Urine-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F34" s="1" t="inlineStr"/>
+      <c r="G34" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Laboratory, Hospital, Diagnostic Center</t>
+        </is>
+      </c>
+      <c r="H34" s="1" t="inlineStr">
+        <is>
+          <t>Mission U120 Urine Analyzer - Manual Operation, White Color | 120 Tests Per Hour, 2000 Results Memory, Accurate Real-Time Results: https://www.tradeindia.com/products/urine-analyzer-9189312.html
+Urine Analyzer - Compact Design with Large LCD Display | Automatic Calibration, Cold Light Source, Memory for 1000 Samples: https://www.tradeindia.com/products/urine-analyzer-595445.html
+Lab U Reader Plus - Semi-Automated Benchtop Urine Analyzer | 500 Samples Per Hour, Enhanced User Interface, Automated Data Reporting: https://www.tradeindia.com/products/urine-analyzer-1010126.html
+Semi Auto Analyzer - ABS Plastic, 10x12x15 cm, 220V AC | Automatic Calibration, LCD Display, Microprocessor Based, Portable: https://www.tradeindia.com/products/semi-auto-analyzer-c3738939.html
+UROGB 120 Urine Analyzer with RS 232 Interface: https://www.tradeindia.com/products/genuine-urine-analyzer-ranges-5431201.html
+Compact Urine Analyzer Application: Industrial: https://www.tradeindia.com/products/compact-urine-analyzer-c5213945.html
+Urine Analyzers - Compact Size, Low Weight, 5 LCD Display | 11 Test Items, Auto Save Data, Cold Light Source, User-DIY Maintenance, Thermal Printer: https://www.tradeindia.com/products/urine-analyzers-c1882364.html
+Digital Urine Analyzer - Application: Hospital: https://www.tradeindia.com/products/digital-urine-analyzer-9831442.html
+URIT-50 Urine Analyzer - ABS Plastic, 13x10x5 inches, 5 kg | LCD Display, Fast Analysis, 1000 Tests Memory, Efficient Workflow, Thermal Printer: https://www.tradeindia.com/products/urit-50-urine-analyzer-5350023.html
+Medtronic Resolute Integrity DES Drug-Eluting Stent 2.75mm Diameter, Cobalt-Chromium Alloy, Continuous Sinusoidal Design, Zotarolimus-Coated: https://www.tradeindia.com/products/medtronic-resolute-integrity-des-drug-eluting-stent-sd-2-75-c10353391.html
+Abbott HI-TORQUE BALANCE MIDDLEWEIGHT UNIVERSAL Guide Wire: https://www.tradeindia.com/products/abbott-hi-torque-balance-middleweight-universal-guide-wire-c10124515.html
+Abbott HI-TORQUE IRONMAN Guide Wires (300 cm): https://www.tradeindia.com/products/abbott-hi-torque-ironman-guide-wires-300-cm-c10126035.html
+Terumo Ryujin Plus PTCA Dilatation Catheter - Polyamide Balloon 3.00mm Diameter, 135cm Length, Transparent Color Coding, Semi-Compliant: https://www.tradeindia.com/products/terumo-ryujin-plus-ptca-dilatation-catheter-bd-3-00-c10124383.html
+Abbott HI-TORQUE CROSS-IT 100XT Guidewire (300 cm) - Nitinol Core with Hydrophilic Coating, Blue Hydrophilic Tip, Radiopaque Distal Tip | Flexible, Steerable, Kink-Resistant, High Precision Navigation: https://www.tradeindia.com/products/abbott-hi-torque-cross-it-100xt-guidewire-300-cm-c10125278.html
+Abbott HI-TORQUE IRONMAN Guide Wires - Stainless Steel, 190 cm, Metallic | Hydrophilic Tip, Enhanced Radiopacity, Kink Resistant: https://www.tradeindia.com/products/abbott-hi-torque-ironman-guide-wires-190-cm-c10125970.html
+Terumo Accuforce Ptca Dilatation Catheter (Bd 2.50) - Accuracy: High Precision Balloon: https://www.tradeindia.com/products/terumo-accuforce-ptca-dilatation-catheter-bd-2-50-c10124103.html
+Terumo Tazuna PTCA Dilatation Catheter (RX) (BD 2.25) - Polyamide Balloon 2.25mm x 12mm, Transparent/Blue Shaft, Dual Platinum Markers, Rapid Exchange System: https://www.tradeindia.com/products/terumo-tazuna-ptca-dilatation-catheter-rx-bd-2-25-c10124387.html
+Terumo Radifocus Introducer II Standard Kit B: https://www.tradeindia.com/products/terumo-radifocus-introducer-ii-standard-kit-b-c10127217.html
+Terumo Accuforce PTCA Dilatation Catheter (BD 3.25): https://www.tradeindia.com/products/terumo-accuforce-ptca-dilatation-catheter-bd-3-25-c10124150.html
+Combilyzer 13 Urine Analyzer: https://www.tradeindia.com/products/combilyzer-13-urine-analyzer-6561901.html
+Mini Urine Analyzer For Medical Use: https://www.tradeindia.com/products/mini-urine-analyzer-for-medical-use-139649.html</t>
+        </is>
+      </c>
+      <c r="I34" s="1" t="inlineStr"/>
+      <c r="J34" s="1" t="inlineStr"/>
+      <c r="K34" s="1" t="inlineStr"/>
+      <c r="L34" s="1" t="inlineStr"/>
+      <c r="M34" s="1" t="inlineStr"/>
+      <c r="N34" s="1" t="inlineStr">
+        <is>
+          <t>SAASKIN Corporation Private Limited is a Healthcare and Life Sciences Company that provides Manufacturing , Distribution and Consulting to different markets across globe. Business Type Exporter, Manufacturer, Distributor, Supplier, Trading Company, Wholesaler, Dealer Employee Count 10 Establishment 2011 Working Days Monday To Saturday GST NO 33AAZCS6003M1ZU Payment Mode Telegraphic Transfer (T/T) Certification IS0 9001 : 2015 Related Products Mission U120 Urine Analyzer - Manual Operation, White Color | 120 Tests Per Hour, 2000 Results Memory, Accurate Real-Time Results Price: 30000 INR MOQ - 2 Unit/Units Saaskin Corporation Private Limited. Chennai, Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="O34" s="1" t="inlineStr"/>
+      <c r="P34" s="1" t="inlineStr"/>
+      <c r="Q34" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/acon-mission-u500-urine-analyzer-c9992154.html</t>
+        </is>
+      </c>
+      <c r="R34" s="1" t="inlineStr"/>
+      <c r="S34" s="1" t="inlineStr"/>
+      <c r="T34" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Laboratory, Hospital, Diagnostic Center</t>
+        </is>
+      </c>
+      <c r="U34" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Laboratory, Hospital, Diagnostic Center</t>
+        </is>
+      </c>
+      <c r="V34" s="1" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr">
+        <is>
+          <t>Zybio- EXC 200 Fully auto Biochemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="B35" s="1" t="inlineStr">
+        <is>
+          <t>ANVI DIAGNOSTICS</t>
+        </is>
+      </c>
+      <c r="C35" s="1" t="inlineStr">
+        <is>
+          <t>General Feature:Throughput : 240 T/H for single reagent, 160 T/H for dual reagentsMethodology : End point, Fixed-time (two point),KineticPrinciple: Absorbance photometry,TurbidimetryProgramming: Open/Close system(optional)Optical System:Light Source: Halogen-Tungsten lampWavelenght: (340-800) nm, in total 12 wavelenghtsAbsorpition range: 0-4.0 AbsResoltion: 0.0001 AbsSample System:Sample Capacity: 40 positionsSample Volume: 2 L - 50 L, step by 0.25 LSample Probe: Liquid level detection, auto-dept adjustment, and collision protectionSample Type: Serum, Plasma, urine, and CSFReagent System:Reagent Capacity: 40 positionsReagent Volume: 10 L- 400 L, step by 0.5 LReaction System:Cuvette: 63 cuvettes with 5mm optical path diameterReaction Volume: 90 L- 450 LReaction Tempreature: 37 + 0.1 CCuvette Washing:6- step washing stationControl:Control Type: Real-time, within-day, between-day control and etcControl Rule: WestgardCalibration:Calibration mode: One-point, two-point, multi- point, Logistic-Log4/5P, Exponential-5P, Polynomial-5P and SplineOperation System:Operation System: Windows 10, support USHost interface: RS232, TCP/POthers:Power supply: 100-240 V- , 50/60 HzCooling way: Constant air coolingWater consumption: &lt; 5 L/HDimension (mm): 710 (W) x 705(D) x 635 (H)Weight: 65 Kg</t>
+        </is>
+      </c>
+      <c r="D35" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/zybio-exc-200-fully-auto-biochemistry-analyzer-c12532199.html</t>
+        </is>
+      </c>
+      <c r="E35" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/12532199/b/4/Zybio-EXC-200-Fully-auto-Biochemistry-Analyzer..jpg</t>
+        </is>
+      </c>
+      <c r="F35" s="1" t="inlineStr">
+        <is>
+          <t>General Feature</t>
+        </is>
+      </c>
+      <c r="G35" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Laboratory, Diagnostic Centers</t>
+        </is>
+      </c>
+      <c r="H35" s="1" t="inlineStr">
+        <is>
+          <t>Mindray Albumin Reagent Kits For Fully Auto Biochemistry Analyzer Bs 240 System Pack - Application: Hospital: https://www.tradeindia.com/products/mindray-albumin-reagent-kits-for-fully-auto-biochemistry-analyzer-bs-240-system-pack-c11788063.html
+Mindray Calcium Reagent Kits for Fully Auto Biochemistry Analyzer: https://www.tradeindia.com/products/mindray-calcium-reagent-kits-for-fully-auto-biochemistry-analyzer-c13222497.html
+Semiautomatic HBA1C Abbott Afinion 2 For Laboratory Use: https://www.tradeindia.com/products/auto-biochemistry-analyzer-8968392.html
+Fully Auto Biochemistry Analyzer (BI-200) - 200 Tests/Hour, Double Reagents for Serum &amp; Urine Analysis | Liver &amp; Kidney Function Testing, Cardiac Markers: https://www.tradeindia.com/products/fully-auto-biochemistry-analyzer-bi-200-c8779733.html
+Meril Autoquant 100I Fully Auto Biochemistry Analyzer - Color: White: https://www.tradeindia.com/products/meril-autoquant-100i-fully-auto-biochemistry-analyzer-c10317331.html
+Fully Auto Biochemistry Analyzer: https://www.tradeindia.com/products/fully-auto-biochemistry-analyzer-c3261548.html
+Fully Auto Biochemistry Analyzer: https://www.tradeindia.com/products/fully-auto-biochemistry-analyzer-10120199.html
+Fully Auto Biochemistry Analyzer: https://www.tradeindia.com/products/fully-auto-biochemistry-analyzer-c1223951.html
+Fully Auto Biochemistry Analyzer: https://www.tradeindia.com/products/fully-auto-biochemistry-analyzer-c3310427.html
+Oscar Fully Auto Biochemistry Analyzer OS-200 - Constant Speed 200 Tests Per Hour, Automatic 8-Step Washing System, User-Friendly Windows Software: https://www.tradeindia.com/products/oscar-fully-auto-biochemistry-analyzer-os-200-c8527308.html
+Easy To Operate Fully Auto Biochemistry Analyzer: https://www.tradeindia.com/products/fully-auto-biochemistry-analyzer-c5656075.html
+Zybio-Z50 Hematology Analyzer - Accuracy: 100 %: https://www.tradeindia.com/products/zybio-z50-hematology-analyzer-c10586736.html
+Zybio- Z3 Hematology Analyzer - Accuracy: Meets Iec/En61010 And Quality Control Standards: https://www.tradeindia.com/products/zybio-z3-hematology-analyzer-c12532194.html
+Pa - 100 Electrolyte Analyzer - Accuracy: 1% (For Na+: https://www.tradeindia.com/products/pa-100-electrolyte-analyzer-c12532197.html
+Exr-110 Fluorescence Immunochromatography Analyzer - Accuracy: 100 %: https://www.tradeindia.com/products/exr-110-fluorescence-immunochromatography-analyzer-c10586743.html
+Eelectrolyte Analyzer ST-200 aqua: https://www.tradeindia.com/products/eelectrolyte-analyzer-st-200-aqua-c13098643.html
+Mml-Ha-300 Hematology Analyzer - Accuracy: High Precision: https://www.tradeindia.com/products/mml-ha-300-hematology-analyzer-c12532191.html
+Bc-20S Auto Hematology Analyzer - Accuracy: 100 %: https://www.tradeindia.com/products/bc-20s-auto-hematology-analyzer-c10586738.html
+Exz-6000 Hematology Analyzer - Accuracy: 100 %: https://www.tradeindia.com/products/exz-6000-hematology-analyzer-c10586737.html
+Zybio- Exs 2600 -Mass Spectrometry System - Accuracy: 98% For Microbial Identification: https://www.tradeindia.com/products/zybio-exs-2600-mass-spectrometry-system-c12532200.html
+Easy To Operate Semi Automatic Biochemistry Analyzer: https://www.tradeindia.com/products/easy-to-operate-semi-automatic-biochemistry-analyzer-6620791.html</t>
+        </is>
+      </c>
+      <c r="I35" s="1" t="inlineStr">
+        <is>
+          <t>ANVI DIAGNOSTICS</t>
+        </is>
+      </c>
+      <c r="J35" s="1" t="inlineStr"/>
+      <c r="K35" s="1" t="inlineStr"/>
+      <c r="L35" s="1" t="inlineStr">
+        <is>
+          <t>ANVI DIAGNOSTICS</t>
+        </is>
+      </c>
+      <c r="M35" s="1" t="inlineStr">
+        <is>
+          <t>ANVI DIAGNOSTICS</t>
+        </is>
+      </c>
+      <c r="N35" s="1" t="inlineStr">
+        <is>
+          <t>Founded in 2023 and based in Mumbai, Maharashtra, Anvi Diagnostics is a trusted manufacturer and supplier of advanced diagnostic equipment. We specialize in offering a wide range of diagnostic analyzers, including EXZ Hematology Analyzer, Zybio Hematology Analyzer, Automatic Clinical Chemistry Analyzer, Semi Automatic Blood Coagulation Analyzer and Fluorescence Immunochromatography Analyzer. With a commitment to providing high-quality, innovative solutions, we aim to support healthcare providers with accurate and efficient diagnostic tools that improve patient outcomes. Business Type Manufacturer, Supplier, Trading Company Employee Count 8 Establishment 2023 Working Days Monday To Saturday GST NO 27AELPT8817R1Z9 Payment Mode Cheque/DD, Online Payments (NEFT/RTGS/IMPS), Wallet &amp; UPI Related Products Zybio- Exc 200 Fully Auto Biochemistry Analyzer - Accuracy: 1% (Analytical Variation Price: 500000 INR MOQ - 1 Unit/Units Anvi Diagnostics Mumbai, Maharashtra</t>
+        </is>
+      </c>
+      <c r="O35" s="1" t="inlineStr"/>
+      <c r="P35" s="1" t="inlineStr"/>
+      <c r="Q35" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/anvi-diagnostics-61709470/</t>
+        </is>
+      </c>
+      <c r="R35" s="1" t="inlineStr"/>
+      <c r="S35" s="1" t="inlineStr"/>
+      <c r="T35" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Laboratory, Diagnostic Centers</t>
+        </is>
+      </c>
+      <c r="U35" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Laboratory, Diagnostic Centers</t>
+        </is>
+      </c>
+      <c r="V35" s="1" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr">
+        <is>
+          <t>Labman Bod Analyzer</t>
+        </is>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>P&amp;C Enterprises</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="inlineStr">
+        <is>
+          <t>Labman Bod Analyzer</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/labman-bod-analyzer-c11508527.html</t>
+        </is>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/11508527/b/4/Labman-Bod-Analyzer..webp</t>
+        </is>
+      </c>
+      <c r="F36" s="1" t="inlineStr">
+        <is>
+          <t>Durable Accuracy A+-1.0 % Usage Laboratory Control Mode Automatic Payment Terms Cash in Advance (CID
+Durable Easy to install Efficient Accuracy A+-1.0 % 100 % Usage Laboratory Laboratory Use Measuring</t>
+        </is>
+      </c>
+      <c r="G36" s="1" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+      <c r="H36" s="1" t="inlineStr">
+        <is>
+          <t>BOD Analyzer - Compact Design with Digital Control Panel | Customizable User Interface, Barcode Identification, Reduced Human Error: https://www.tradeindia.com/products/bod-analyzer-c5023669.html
+Bod Analyzer - Application: Blood Bio Chemistry: https://www.tradeindia.com/products/bod-analyzer-c12942422.html
+BOD Monitoring System: https://www.tradeindia.com/products/bod-monitoring-system-c4070277.html
+BOD Analyzer - 10.4" Touch Screen , Real-Time Visualization &amp; Auto-Cleaning Functionality: https://www.tradeindia.com/products/bod-analyzer-2079224.html
+BOD Analyzer - Advanced Online Connectivity, Exceptional Durability &amp; Low Maintenance: https://www.tradeindia.com/products/bod-analyzer-4631395.html
+BOD Analyzer - Premium Quality Material, Advanced Technology Integration | Highly Admired for Excellent Performance, Versatile Applications: https://www.tradeindia.com/products/bod-analyzer-1456961.html
+Online Conductivity Controller - Accuracy: +/- 1 %: https://www.tradeindia.com/products/online-conductivity-controller-c11508489.html
+Digital Ultrasonic Cleaner - Material: Stainless Steel: https://www.tradeindia.com/products/digital-ultrasonic-cleaner-c11508484.html
+Alcohol Breath Analyzer Tester - Dimension (L*W*H): 180Mm X 70Mm X 30 Millimeter (Mm): https://www.tradeindia.com/products/alcohol-breath-analyzer-tester-c11508535.html
+Lark La 228 37401 91 Detector Lamp - Color: Transparent: https://www.tradeindia.com/products/lark-la-228-37401-91-detector-lamp-c11508598.html
+Lark Alumina Crucible - Color: White: https://www.tradeindia.com/products/lark-alumina-crucible-c11508606.html
+Kerro Mc 7806 Grain Moisture Meter - Color: Black: https://www.tradeindia.com/products/kerro-mc-7806-grain-moisture-meter-c11508622.html
+Kerro Jewellery Weighing Balance - Load: 300 Gram (G): https://www.tradeindia.com/products/kerro-jewellery-weighing-balance-c11508631.html
+Disposable Quartz Cuvettes - Color: Transparent: https://www.tradeindia.com/products/disposable-quartz-cuvettes-c11508661.html
+5L Digital Ultrasonic Cleaner - Frequency: 40 Kilohertz ( Khz ): https://www.tradeindia.com/products/5l-digital-ultrasonic-cleaner-c11508684.html
+Lmif30T Ice Flaker - Material: Stainless Steel: https://www.tradeindia.com/products/lmif30t-ice-flaker-c11508692.html
+Reckon Getein-1100 Poct Analyzer: https://www.tradeindia.com/products/reckon-getein-1100-poct-analyzer-c10564201.html
+Online TOC Meter: https://www.tradeindia.com/products/online-toc-meter-c10169365.html</t>
+        </is>
+      </c>
+      <c r="I36" s="1" t="inlineStr">
+        <is>
+          <t>P&amp;C Enterprises</t>
+        </is>
+      </c>
+      <c r="J36" s="1" t="inlineStr"/>
+      <c r="K36" s="1" t="inlineStr"/>
+      <c r="L36" s="1" t="inlineStr">
+        <is>
+          <t>P&amp;C Enterprises</t>
+        </is>
+      </c>
+      <c r="M36" s="1" t="inlineStr">
+        <is>
+          <t>P&amp;C Enterprises</t>
+        </is>
+      </c>
+      <c r="N36" s="1" t="inlineStr">
+        <is>
+          <t>P&amp;C Enterprises is committed to delivering advanced laboratory instruments designed for precision, reliability, and performance. As a trader, supplier, and exporter, the company specializes in providing top-tier equipment such as Labman Biochemistry Analyzer, Labman Gradient Thermal Cycler, Online Conductivity Controller, Digital Ultrasonic Cleaner, Photoelectric Colorimeter, Hsetin Digital Tachometer, Digital Food Thermometer, Lark Deuterium Lamp, and Pocket Sized pH Meter. Every product reflects a dedication to technological excellence, built to meet the evolving needs of modern laboratories and scientific industries worldwide.Engineered with cutting-edge digital calibration systems, these instruments guarantee consistent and dependable results across diverse applications. Their compact and durable design ensures Business Type Exporter, Supplier, Trading Company, Wholesaler, Retailer Employee Count 10 Establishment 2020 Working Days Monday To Sunday GST NO 07FTSPK5264G1Z5 Payment Mode Cash, Online Payments (NEFT/RTGS/IMPS), Wallet &amp; UPI, Cheque/DD Related Products BOD Analyzer - Compact Design with Digital Control Panel | Customizable User Interface, Barcode Identification, Reduced Human Error MOQ - 1 Box/Boxes Shreetech Life Science Pvt. Ltd. New Delhi, Delhi</t>
+        </is>
+      </c>
+      <c r="O36" s="1" t="inlineStr"/>
+      <c r="P36" s="1" t="inlineStr"/>
+      <c r="Q36" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/pc-enterprises-149880218/</t>
+        </is>
+      </c>
+      <c r="R36" s="1" t="inlineStr"/>
+      <c r="S36" s="1" t="inlineStr"/>
+      <c r="T36" s="1" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+      <c r="U36" s="1" t="inlineStr"/>
+      <c r="V36" s="1" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr">
+        <is>
+          <t>Vector V Chem Next Programmable Biochemistry Analyzer - Color: As Per Demand - Color: As Per Demand at Best Price in Varanasi | Biomedical And Services</t>
+        </is>
+      </c>
+      <c r="B37" s="1" t="inlineStr"/>
+      <c r="C37" s="1" t="inlineStr">
+        <is>
+          <t>Biomedical And Services - Offering low price Vector V Chem Next Programmable Biochemistry Analyzer - Color: As Per Demand - Color: As Per Demand in Baullia Lahartara, Varanasi with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="D37" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/vector-v-chem-next-programmable-biochemistry-analyzer-c11872770.html</t>
+        </is>
+      </c>
+      <c r="E37" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/11872770/b/4/Vector-V-Chem-Next-Programmable-Biochemistry-Analyzer..webp</t>
+        </is>
+      </c>
+      <c r="F37" s="1" t="inlineStr">
+        <is>
+          <t>High Quality Power Supply Electric Usage Laboratories Size Various Sizes Available Color As Per Dema</t>
+        </is>
+      </c>
+      <c r="G37" s="1" t="inlineStr">
+        <is>
+          <t>Laboratories</t>
+        </is>
+      </c>
+      <c r="H37" s="1" t="inlineStr">
+        <is>
+          <t>Vector V Chem Next Biochemistry Analyzer - Color: As Per Demand: https://www.tradeindia.com/products/vector-v-chem-next-biochemistry-analyzer-c11872765.html
+Bx-3010 Automated Bio Chemistry Analyzer - Accuracy: Cv 1% For Repeatability %: https://www.tradeindia.com/products/bx-3010-automated-chemistry-analyzer-c12491620.html
+Biochemistry Analyzer - Premium Quality Raw Material, Advanced Technology | Rigorous Quality Testing, Flawless Performance: https://www.tradeindia.com/products/biochemistry-analyzer-3309405.html
+Innolab 200 Semi Automatic Biochemistry Analyzer - Application: Laboratories: https://www.tradeindia.com/products/innolab-200-semi-automatic-biochemistry-analyzer-c10651688.html
+Fully Auto Biochemistry Analyzer (BI-200) - 200 Tests/Hour, Double Reagents for Serum &amp; Urine Analysis | Liver &amp; Kidney Function Testing, Cardiac Markers: https://www.tradeindia.com/products/fully-auto-biochemistry-analyzer-bi-200-c8779733.html
+Smart Biochemistry Analyzer: https://www.tradeindia.com/products/smart-biochemistry-analyzer-c11977823.html
+Electric Fully Automatic A15 Biosystems Analyzer - Color: As Per Demand: https://www.tradeindia.com/products/electric-fully-automatic-a15-biosystems-analyzer-c11872774.html
+Bonavera Chem 200 Fully Automated Biochemistry Analyzer: https://www.tradeindia.com/products/bonavera-chem-200-fully-automated-biochemistry-analyzer-c12491574.html
+Erbachem 5X Biochemistry Analyzer - Color: White: https://www.tradeindia.com/products/erbachem-5x-biochemistry-analyzer-c10206917.html
+Horiba Pentra 400 Fully Automatic Biochemistry Analyzer - Color: Customized: https://www.tradeindia.com/products/horiba-pentra-400-fully-automatic-biochemistry-analyzer-c11160977.html
+Pictus-700 Fully Automatic Biochemistry Analyzer - Feature: High Quality: https://www.tradeindia.com/products/pictus-700-fully-automatic-biochemistry-analyzer-c10778212.html
+Clinical Use Metrolab 1600 Dr Biochemistry Analyzer: https://www.tradeindia.com/products/clinical-use-metrolab-1600-dr-biochemistry-analyzer-8510126.html
+Coagulation Analyzing Machine - Automation Grade: Semi Automatic: https://www.tradeindia.com/products/coagulation-analyzing-machine-c11872787.html
+Immunoshop Life Dx H3Pro Automated Hematology Analyzer - Automation Grade: Semi Automatic: https://www.tradeindia.com/products/immunoshop-life-dx-h3pro-automated-hematology-analyzer-c11872757.html
+Horiba Yumizen H500 Hematology Analyzer - Color: As Per Demand: https://www.tradeindia.com/products/horiba-yumizen-h500-hematology-analyzer-c11872775.html
+02_Automatic Lw E60 Electrolyte Analyzer - Color: Different Available: https://www.tradeindia.com/products/02-automatic-lw-e60-electrolyte-analyzer-c11872778.html
+01_Automatic Lw E60 Electrolyte Analyzer - Color: Different Available: https://www.tradeindia.com/products/01-automatic-lw-e60-electrolyte-analyzer-c11872777.html
+Immunoshop Maglumi 800 Analyzer - Color: Different Available: https://www.tradeindia.com/products/immunoshop-maglumi-800-analyzer-c11872780.html
+Sysmex Xn 350 Hematology Analyzer - Feature: Easy To Operate: https://www.tradeindia.com/products/sysmex-xn-350-hematology-analyzer-c11872759.html
+Automatic Ba 200 Biochemistry Analyzer - Feature: Easy To Operate: https://www.tradeindia.com/products/automatic-ba-200-biochemistry-analyzer-c11872760.html
+Fully Automatic Sysmex Xn 550 Cell Counter - Feature: Easy To Operate: https://www.tradeindia.com/products/fully-automatic-sysmex-xn-550-cell-counter-c11872754.html
+Biochemistry Analyzer Mispa Viva Agappe: https://www.tradeindia.com/products/biochemistry-analyzer-mispa-viva-agappe-10167226.html
+Biochemistry Analyzer: https://www.tradeindia.com/products/biochemistry-analyzer-4482395.html</t>
+        </is>
+      </c>
+      <c r="I37" s="1" t="inlineStr">
+        <is>
+          <t>Trusted Seller</t>
+        </is>
+      </c>
+      <c r="J37" s="1" t="inlineStr"/>
+      <c r="K37" s="1" t="inlineStr"/>
+      <c r="L37" s="1" t="inlineStr">
+        <is>
+          <t>Trusted Seller</t>
+        </is>
+      </c>
+      <c r="M37" s="1" t="inlineStr">
+        <is>
+          <t>Trusted Seller</t>
+        </is>
+      </c>
+      <c r="N37" s="1" t="inlineStr">
+        <is>
+          <t>Biomedical and Services is a dependable Trader, Supplier, and Service Provider catering to the growing needs of diagnostic laboratories, hospitals, and healthcare institutions. We supply Automated Hematology Analyzer, Hematology Analyzer, Biochemistry Analyzer, Automated Hematology Analyzer, Auto Hematology Analyzer, etc. We specialize in providing reliable and technologically advanced diagnostic equipment that supports accurate and timely medical testing. With a clear focus on quality and service excellence, our organization has built a strong presence in the medical equipment supply sector by consistently meeting the expectations of healthcare professionals.Technical Expertise and SupportBeyond supplying equipment, Biomedical and Services is known for its professional technical support. Our experienced service team provides installation, calibration, preventive maintenance Business Type Service Provider, Supplier, Trading Company Employee Count 6 Establishment 2020 Working Days Monday To Sunday GST NO 09AAVFB5802E1ZC Related Products Vector V Chem Next Biochemistry Analyzer - Color: As Per Demand MOQ - 10 Unit/Units Biomedical And Services Varanasi, Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="O37" s="1" t="inlineStr"/>
+      <c r="P37" s="1" t="inlineStr"/>
+      <c r="Q37" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/vector-v-chem-next-programmable-biochemistry-analyzer-c11872770.html</t>
+        </is>
+      </c>
+      <c r="R37" s="1" t="inlineStr"/>
+      <c r="S37" s="1" t="inlineStr"/>
+      <c r="T37" s="1" t="inlineStr">
+        <is>
+          <t>Laboratories</t>
+        </is>
+      </c>
+      <c r="U37" s="1" t="inlineStr"/>
+      <c r="V37" s="1" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>Fully Automated Biochemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>MEDICA SOLUTIONS</t>
+        </is>
+      </c>
+      <c r="C38" s="1" t="inlineStr">
+        <is>
+          <t>Fully Automated Biochemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="D38" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/fully-automated-biochemistry-analyzer-c10317328.html</t>
+        </is>
+      </c>
+      <c r="E38" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/10317328/b/4/Fully-Automated-Biochemistry-Analyzer..jpg</t>
+        </is>
+      </c>
+      <c r="F38" s="1" t="inlineStr"/>
+      <c r="G38" s="1" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="H38" s="1" t="inlineStr">
+        <is>
+          <t>Full Automatic Chemistry Analyzer - Application: Commercial: https://www.tradeindia.com/products/full-automatic-chemistry-analyzer-c9474134.html
+Meril Autoquant 400 Fully Automatic Biochemistry Analyzer - Attributes: Easy To Operate: https://www.tradeindia.com/products/meril-autoquant-400-fully-automatic-biochemistry-analyzer-c10317325.html
+SpectraChem Bioassay-240Plus - 220V, Reusable Plastic Cuvette | Fully Automatic Biochemistry Analyzer, 240 Tests/Hour, Up to 90 Sample Positions, Sleek White Design: https://www.tradeindia.com/products/fully-automatic-biochemistry-analyzer-8522041.html
+Semi Automatic Biochemistry Analyzers - Semi Automatic Analyzer, White, Digital Display | Easy To Use, 1 Year Warranty: https://www.tradeindia.com/products/semi-automatic-biochemistry-analyzers-9855456.html
+Automatic Biochemistry Analyzer: https://www.tradeindia.com/products/automatic-biochemistry-analyzer-c1303684.html
+Biochemistry Analyzer: https://www.tradeindia.com/products/biochemistry-analyzer-c556611.html
+Fully Automatic Biochemistry Analyzer: https://www.tradeindia.com/products/fully-automatic-biochemistry-analyzer-4983039.html
+Semi Automatic Biochemistry Analyzer - ABS Plastic, 20x30x15 cm | LCD Display, Data Storage, Programmable Tests, 60 Tests/Hour: https://www.tradeindia.com/products/semi-automatic-biochemistry-analyzer-c4092450.html
+Fully Automatic Biochemistry Analyser: https://www.tradeindia.com/products/fully-automatic-biochemistry-analyser-c1285859.html
+Csense 100Fully Automatic Biochemistry Analyzer - White, Durable | Hospital Use, Automatic, Very Good Quality: https://www.tradeindia.com/products/csense-100fully-automatic-biochemistry-analyzer-9910186.html
+Meril Cliniquant Semi Auto Biochemistry Analyzer - Attributes: Easy To Operate: https://www.tradeindia.com/products/meril-cliniquant-semi-auto-biochemistry-analyzer-c10317333.html
+Ever Life Ex-Ds Electrolyte Analyser - Color Code: Grey: https://www.tradeindia.com/products/ever-life-ex-ds-electrolyte-analyser-c10317337.html
+Blood Gas And Chemistry Analyzer - Color: White: https://www.tradeindia.com/products/blood-gas-and-chemistry-analyzer-c10317339.html
+Total Protein Test Kit - Attributes: Safe To Use: https://www.tradeindia.com/products/total-protein-test-kit-c10317341.html
+Crp Test Kit - Attributes: Safe To Use: https://www.tradeindia.com/products/crp-test-kit-c10317345.html
+Abbott Urine Analyzer - Color: White: https://www.tradeindia.com/products/abbott-urine-analyzer-c10317350.html
+Meril Cliniquant Micro Semi Auto Biochemistry Analyzer - Color: White: https://www.tradeindia.com/products/meril-cliniquant-micro-semi-auto-biochemistry-analyzer-c10317332.html
+Immunoassay Analyzer - Color: White: https://www.tradeindia.com/products/i-croma-iii-fluorescence-immunoassay-analyzer-c10317335.html
+Alkaline Phosphatase Kit - Attributes: Safe To Use: https://www.tradeindia.com/products/alkaline-phosphatase-kit-c10317346.html
+Auto Biochemistry Analyzer: https://www.tradeindia.com/products/auto-biochemistry-analyzer-c5375373.html
+SemiAutomatic Biochemistry Analyzer ERBA CHEM7: https://www.tradeindia.com/products/semiautomatic-biochemistry-analyzer-erba-chem7-c8169376.html</t>
+        </is>
+      </c>
+      <c r="I38" s="1" t="inlineStr">
+        <is>
+          <t>MEDICA SOLUTIONS</t>
+        </is>
+      </c>
+      <c r="J38" s="1" t="inlineStr"/>
+      <c r="K38" s="1" t="inlineStr"/>
+      <c r="L38" s="1" t="inlineStr">
+        <is>
+          <t>MEDICA SOLUTIONS</t>
+        </is>
+      </c>
+      <c r="M38" s="1" t="inlineStr">
+        <is>
+          <t>MEDICA SOLUTIONS</t>
+        </is>
+      </c>
+      <c r="N38" s="1" t="inlineStr">
+        <is>
+          <t>Medica Solutions is a trusted company that deals with medical equipment and diagnostic solutions, providing advanced healthcare technologies. We are a trader and supplier of critical medical diagnostic instruments including Covid Test Kits, Biochemistry Analyzers, Immunoassay Analyzers, Hematology Analyzers, and more. We are committed to helping healthcare professionals with high-quality, precision-engineered diagnostic equipment that allows for accurate and efficient medical testing. Our comprehensive portfolio of products, which is designed by certified manufacturing companies for the specific requirements of a constantly evolving medical laboratory, hospitals, and other health care institution needs. Thus bringing the finest cutting-edge technologies of diagnostics at the doorstep of the healthcare service provider. Business Type Exporter, Importer, Manufacturer, Distributor, Supplier, Trading Company, Wholesaler, Dealer Employee Count 10 Establishment 2018 Working Days Monday To Sunday GST NO 07ABJFM6010C1ZP Payment Mode Cheque/DD, Online Payments (NEFT/RTGS/IMPS), Cash Related Products Full Automatic Chemistry Analyzer - Application: Commercial MOQ - 1 Unit/Units Weldon Biotech (india) Pvt. Ltd. Delhi, Delhi</t>
+        </is>
+      </c>
+      <c r="O38" s="1" t="inlineStr"/>
+      <c r="P38" s="1" t="inlineStr"/>
+      <c r="Q38" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/medica-solutions-26010478/</t>
+        </is>
+      </c>
+      <c r="R38" s="1" t="inlineStr"/>
+      <c r="S38" s="1" t="inlineStr"/>
+      <c r="T38" s="1" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="U38" s="1" t="inlineStr"/>
+      <c r="V38" s="1" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr">
+        <is>
+          <t>Unikon Gh Hba1c Analyzer at Best Price in Varanasi | M/s Elite Biomedicals</t>
+        </is>
+      </c>
+      <c r="B39" s="1" t="inlineStr"/>
+      <c r="C39" s="1" t="inlineStr">
+        <is>
+          <t>M/s Elite Biomedicals - Offering low price Unikon Gh Hba1c Analyzer in Mahesh Pur Industrial Estate, Varanasi with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="D39" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/unikon-gh-hba1c-analyzer-c12491593.html</t>
+        </is>
+      </c>
+      <c r="E39" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/12491593/b/4/Unikon-GH-HBA1C-Analyzer..png</t>
+        </is>
+      </c>
+      <c r="F39" s="1" t="inlineStr">
+        <is>
+          <t>High Precision, Fast Results, User-friendly Interface, Internal Printer Display Type LCD Touch Scree
+High Precision, Fast Results, User-friendly Interface, Internal Printer Open system, memory storage</t>
+        </is>
+      </c>
+      <c r="G39" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Laboratory, HbA1c Testing</t>
+        </is>
+      </c>
+      <c r="H39" s="1" t="inlineStr">
+        <is>
+          <t>Vector V Chem Next Biochemistry Analyzer - Color: As Per Demand: https://www.tradeindia.com/products/vector-v-chem-next-biochemistry-analyzer-c11872765.html
+Bx-3010 Automated Bio Chemistry Analyzer - Accuracy: Cv 1% For Repeatability %: https://www.tradeindia.com/products/bx-3010-automated-chemistry-analyzer-c12491620.html
+Uriscan Optima Urine Chemistry Analyzer - Color: Different Availabe: https://www.tradeindia.com/products/uriscan-optima-urine-chemistry-analyzer-c10651714.html
+Urine Analyzer ( Bi-400) - Color: White: https://www.tradeindia.com/products/urine-analyzer-bi-400-c8781154.html
+Automated Floor Stand Chemistry Analyzer: https://www.tradeindia.com/products/automated-floor-stand-chemistry-analyzer-c11977825.html
+Vector V Chem Next Programmable Biochemistry Analyzer - Color: As Per Demand: https://www.tradeindia.com/products/vector-v-chem-next-programmable-biochemistry-analyzer-c11872770.html
+Unikon 480 Fully Automatic Clinical Bio Chemistry Analyzer - Accuracy: Cv 1% (Repeatability) %: https://www.tradeindia.com/products/unikon-480-fully-automatic-clinical-chemistry-analyzer-c12491622.html
+Erba Chem 5X Clinical Chemistry Analyzer - Application: Commercial: https://www.tradeindia.com/products/erba-chem-5x-clinical-chemistry-analyzer-c10206968.html
+Plastic Fully Automatic Bio Chemistry Analyzer: https://www.tradeindia.com/products/fully-automatic-bio-chemistry-analyzer-c8200085.html
+Horiba Yumizen Ca60 Clinical Chemistry Analyzer - Color: Blue And White: https://www.tradeindia.com/products/horiba-yumizen-ca60-clinical-chemistry-analyzer-c11160991.html
+Urine Analyzer - ABS Plastic, 10x12x15 inches, USB Connectivity | Accurate Readings, Automated Testing, Digital Display, Fast Results, Multiple Parameters: https://www.tradeindia.com/products/urine-analyzer-c4469663.html
+Plastic Chemistry Analyzer - 430 x 360 x 170 mm, White Plastic Design, 6.8 kg Weight, Semi-Automatic Operation, LED Display, 220 Volt Voltage, Detects Over 30 Compounds: https://www.tradeindia.com/products/plastic-chemistry-analyzer-with-6-8-kg-weight-for-hospitals-and-clinics-8168732.html
+Bonavera Chem 200 Fully Automated Biochemistry Analyzer: https://www.tradeindia.com/products/bonavera-chem-200-fully-automated-biochemistry-analyzer-c12491574.html
+Nulyte Aqua Electrolyte Analyzer: https://www.tradeindia.com/products/nulyte-aqua-electrolyte-analyzer-c12491676.html
+Elite Count 72 3 Part Diff Automated Hematology Analyzer: https://www.tradeindia.com/products/elite-count-72-3-part-diff-automated-hematology-analyzer-c12491750.html
+Bonavera Chem Uno Plus Biochemistry Semi Auto Analyzer: https://www.tradeindia.com/products/bonavera-chem-uno-plus-biochemistry-semi-auto-analyzer-c12491575.html
+CA-600 Fully Automated Coagulation Analyzer: https://www.tradeindia.com/products/ca-600-fully-automated-coagulation-analyzer-c12491648.html
+Unikon Lyte 3 Unique Electrolyte Analyzer: https://www.tradeindia.com/products/unikon-lyte-3-unique-electrolyte-analyzer-c12491678.html
+IFlash 1800 Immunoassay Analyzer: https://www.tradeindia.com/products/iflash-1800-immunoassay-analyzer-c12491847.html
+Ichroma Iii Advanced Compact Immuno Analyzer - Application: Quantitative Immunoassays For Clinical Diagnostics: https://www.tradeindia.com/products/ichroma-ii-advanced-compact-immuno-analyzer-c12491844.html
+AFIAS-6 Desktop Fluorescence Immuno Analyzer - 370x165x280 mm, 6-Cartridge Capacity, 7-Inch Touchscreen | Multi-Parameter Testing, LIS/HIS Connectivity, Automated QC/Calibration: https://www.tradeindia.com/products/afias-6-wersatile-desktop-fluorescence-immuno-analyzer-c12491842.html
+Semi Auto Chemistry Analyzer: https://www.tradeindia.com/products/semi-auto-chemistry-analyzer-c7303681.html
+Semi Automatic Nitrogen Analyzer: https://www.tradeindia.com/products/semi-automatic-nitrogen-analyzer-c1567488.html</t>
+        </is>
+      </c>
+      <c r="I39" s="1" t="inlineStr">
+        <is>
+          <t>Trusted Seller</t>
+        </is>
+      </c>
+      <c r="J39" s="1" t="inlineStr"/>
+      <c r="K39" s="1" t="inlineStr"/>
+      <c r="L39" s="1" t="inlineStr">
+        <is>
+          <t>Trusted Seller</t>
+        </is>
+      </c>
+      <c r="M39" s="1" t="inlineStr">
+        <is>
+          <t>Trusted Seller</t>
+        </is>
+      </c>
+      <c r="N39" s="1" t="inlineStr">
+        <is>
+          <t>Elite Biomedicals is a dependable Supplier and Trader of advanced diagnostic and laboratory equipment, committed to supporting the evolving needs of the healthcare sector. With a strong presence in the market, the company offers a wide portfolio of high-performance products including Biochemistry Analyzers, Blood Gas and Chemistry Analyzers, Coagulation Analyzers, Electrolyte Analyzers, and Hematology Analyzers. Each product is sourced from trusted manufacturers and designed to deliver accurate, consistent, and timely results essential for effective clinical decision-making. Business Type Supplier, Trading Company Employee Count 8 Establishment 2016 Working Days Monday To Saturday GST NO 09BAMPS3687N1ZK Payment Mode Cheque/DD, Cash, Online Payments (NEFT/RTGS/IMPS) Related Products Vector V Chem Next Biochemistry Analyzer - Color: As Per Demand MOQ - 10 Unit/Units Biomedical And Services Varanasi, Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="O39" s="1" t="inlineStr"/>
+      <c r="P39" s="1" t="inlineStr"/>
+      <c r="Q39" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/unikon-gh-hba1c-analyzer-c12491593.html</t>
+        </is>
+      </c>
+      <c r="R39" s="1" t="inlineStr"/>
+      <c r="S39" s="1" t="inlineStr"/>
+      <c r="T39" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Laboratory, HbA1c Testing</t>
+        </is>
+      </c>
+      <c r="U39" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Laboratory, HbA1c Testing</t>
+        </is>
+      </c>
+      <c r="V39" s="1" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
+        <is>
+          <t>CST-180 Automatic Biochemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="B40" s="1" t="inlineStr">
+        <is>
+          <t>Majumder Enterprises</t>
+        </is>
+      </c>
+      <c r="C40" s="1" t="inlineStr">
+        <is>
+          <t>CST-180 Automatic Biochemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="D40" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/cst-180-automatic-biochemistry-analyzer-c11539500.html</t>
+        </is>
+      </c>
+      <c r="E40" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/11539500/b/4/CST-180-Automatic-Biochemistry-Analyzer..jpeg</t>
+        </is>
+      </c>
+      <c r="F40" s="1" t="inlineStr">
+        <is>
+          <t>High quality Accuracy 100 % Usage Clinical diagnostics Voltage 220 Volt (v) Material Metal, plastic</t>
+        </is>
+      </c>
+      <c r="G40" s="1" t="inlineStr">
+        <is>
+          <t>Clinical diagnostics</t>
+        </is>
+      </c>
+      <c r="H40" s="1" t="inlineStr">
+        <is>
+          <t>White Bene Sphera C61 Semi Automatic Biochemistry Analyzer: https://www.tradeindia.com/products/bene-sphera-c61-semi-automatic-biochemistry-analyzer-c7839533.html
+Semi Automatic Biochemistry Analyzer - CE Certified, 220V Voltage, Blue Color | 1 Year Warranty for Clinical Use: https://www.tradeindia.com/products/semi-automatic-biochemistry-analyzer-for-laboratory-and-clinical-use-7576255.html
+Semi Auto Biochemistry Analyzer - Plastic Material, 7-Inch TFT LCD Display, Grey Color | 8 Filters Including 700nm, Dual Mode Operation, Real-Time Reaction Graph, 2,00,000 Result Storage: https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-4856083.html
+Fully Automatic Biochemistry Analyzer - 150 to 300 Tests Per Hour | I.S.E. Module Options Available: https://www.tradeindia.com/products/fully-automatic-biochemistry-analyzer-1205665.html
+Cst- 240 Plus Automatic Biochemistry Analyzer - Accuracy: 100 %: https://www.tradeindia.com/products/cst-240-plus-automatic-biochemistry-analyzer-c11539499.html
+Mispa Nano Plus Fully Automated Biochemistry Analyzer - Accuracy: 100 %: https://www.tradeindia.com/products/mispa-nano-plus-fully-automated-biochemistry-analyzer-c11539501.html
+Volton Base Plus Electrolyte Analyzer - Automation Grade: Automatic: https://www.tradeindia.com/products/volton-base-plus-electrolyte-analyzer-c11539513.html
+Dirui Bf-6900 Automatic Hematology Analyzer - Accuracy: 100 %: https://www.tradeindia.com/products/dirui-bf-6900-automatic-hematology-analyzer-c11539526.html
+Maglumi 800 Immunoassay Analyzer - Accuracy: 100 %: https://www.tradeindia.com/products/maglumi-800-immunoassay-analyzer-c11539546.html</t>
+        </is>
+      </c>
+      <c r="I40" s="1" t="inlineStr">
+        <is>
+          <t>Majumder Enterprises</t>
+        </is>
+      </c>
+      <c r="J40" s="1" t="inlineStr"/>
+      <c r="K40" s="1" t="inlineStr"/>
+      <c r="L40" s="1" t="inlineStr">
+        <is>
+          <t>Majumder Enterprises</t>
+        </is>
+      </c>
+      <c r="M40" s="1" t="inlineStr">
+        <is>
+          <t>Majumder Enterprises</t>
+        </is>
+      </c>
+      <c r="N40" s="1" t="inlineStr">
+        <is>
+          <t>Majumder Enterprises is a trusted and reputed Supplier and Trader of advanced medical and laboratory diagnostic equipment, committed to excellence, innovation, and customer satisfaction. We offer Automatic Biochemistry Analyzer, Mispa Nano Plus Fully Automated Biochemistry Analyzer, Automatic Biochemistry Analyzer, Volton Base Plus Electrolyte Analyzer, Automatic Hematology Analyzer, and more. Based on years of experience in the healthcare industry, we have established ourselves as a dependable partner for hospitals, diagnostic centers, research institutions, and laboratories across India.We specialize in providing cutting-edge analytical instruments that deliver accurate, efficient, and reliable diagnostic results. Our mission is to bridge the gap between advanced medical technology and accessibility, ensuring that ev Business Type Supplier, Trading Company Employee Count 11 Establishment 2004 Working Days Monday To Sunday GST NO 19AMEPM7449K1ZF Payment Mode Online Payments (NEFT/RTGS/IMPS), Cheque/DD, Wallet &amp; UPI Related Products White Bene Sphera C61 Semi Automatic Biochemistry Analyzer Price: 80000 INR MOQ - 1 Piece/Pieces Ambay Enterprises Kolkata, West Bengal</t>
+        </is>
+      </c>
+      <c r="O40" s="1" t="inlineStr"/>
+      <c r="P40" s="1" t="inlineStr"/>
+      <c r="Q40" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/majumder-enterprises-27873101/</t>
+        </is>
+      </c>
+      <c r="R40" s="1" t="inlineStr"/>
+      <c r="S40" s="1" t="inlineStr"/>
+      <c r="T40" s="1" t="inlineStr">
+        <is>
+          <t>Clinical diagnostics</t>
+        </is>
+      </c>
+      <c r="U40" s="1" t="inlineStr">
+        <is>
+          <t>Clinical diagnostics</t>
+        </is>
+      </c>
+      <c r="V40" s="1" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
+        <is>
+          <t>BCA80 Bio Chemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="B41" s="1" t="inlineStr">
+        <is>
+          <t>TESTCARE INSTRUMENTS</t>
+        </is>
+      </c>
+      <c r="C41" s="1" t="inlineStr">
+        <is>
+          <t>BCA80 Bio Chemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="D41" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/bca80-bio-chemistry-analyzer-c12307715.html</t>
+        </is>
+      </c>
+      <c r="E41" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/12307715/b/4/BCA80-Bio-Chemistry-Analyzer..jpg</t>
+        </is>
+      </c>
+      <c r="F41" s="1" t="inlineStr">
+        <is>
+          <t>Automated Operation, Barcode Reader, Data Storage, User-Friendly Interface Speed Range 80 Tests/Hour</t>
+        </is>
+      </c>
+      <c r="G41" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Laboratory, Hospital, Research</t>
+        </is>
+      </c>
+      <c r="H41" s="1" t="inlineStr">
+        <is>
+          <t>Erba Em Destiny 180 - Fully Automated Biochemistry Analyzer - Automation Grade: Automatic: https://www.tradeindia.com/products/erba-em-destiny-180-fully-automated-biochemistry-analyzer-c11787573.html
+Erba Biochemistry Analyzer Application: Industrial: https://www.tradeindia.com/products/erba-biochemistry-analyzer-c8544174.html
+Erba Biochemistry Analyzer: https://www.tradeindia.com/products/erba-biochemistry-analyzer-10254106.html
+Erba Biochemistry Analyzer - Plastic, Digital Display, Grey | Compact Design, Automatic/Semi-Automatic/Manual Operation, Low Power Consumption: https://www.tradeindia.com/products/erba-biochemistry-analyzer-c7874879.html
+Erba Biochemistry Analyzer: https://www.tradeindia.com/products/erba-biochemistry-analyzer-c12360320.html
+Top Quality Erba Biochemistry Analyzer: https://www.tradeindia.com/products/top-quality-erba-biochemistry-analyzer-5037931.html
+Chem 7 Erba Biochemistry Analyzer - Reliable Optical System, Easy to Use Interface, Heavy Duty, Industrial Laboratory Use: https://www.tradeindia.com/products/chem-7-erba-biochemistry-analyzer-10167227.html
+Kab2L Analytical Balance Keypad - Application: Lab: https://www.tradeindia.com/products/kab2l-analytical-balance-keypad-c12711599.html
+LMSPV325 Visible Spectrophotometer: https://www.tradeindia.com/products/lmspv325-visible-spectrophotometer-c12307686.html
+Lmph12 Ph Meter - Application: Laboratory: https://www.tradeindia.com/products/lmph9-economic-ph-meter-c12307702.html
+Lmif200T Ice Flaker - Touch Screen - Application: Hotels: https://www.tradeindia.com/products/lmif200t-touchscreen-ice-flaker-c12307673.html
+Adp100Cfr High Speed Automatic Polarimeter - Application: Laboratory: https://www.tradeindia.com/products/adp100cfr-high-speed-automatic-polarimeter-c12307665.html
+ESS300M Electromagnetic Sieve Shaker: https://www.tradeindia.com/products/ess300m-electromagnetic-sieve-shaker-c12662310.html
+AAS4M Atomic Absorption Spectrophotometer: https://www.tradeindia.com/products/aas4m-atomic-absorption-spectrophotometer-c12662307.html
+KAB10L Semi Micro Balance: https://www.tradeindia.com/products/kab10l-semi-micro-balance-c12711012.html
+Lmms300 Hotplate Magnetic Stirrer - Accuracy: 1%: https://www.tradeindia.com/products/lmms300-hotplate-magnetic-stirrer-c12307711.html
+Dbi11T Touch Screen Dry Bath Incubator - Accuracy: +/-0.3 C: https://www.tradeindia.com/products/dbi11t-touch-screen-dry-bath-incubator-c12307694.html</t>
+        </is>
+      </c>
+      <c r="I41" s="1" t="inlineStr">
+        <is>
+          <t>TESTCARE INSTRUMENTS</t>
+        </is>
+      </c>
+      <c r="J41" s="1" t="inlineStr"/>
+      <c r="K41" s="1" t="inlineStr"/>
+      <c r="L41" s="1" t="inlineStr">
+        <is>
+          <t>TESTCARE INSTRUMENTS</t>
+        </is>
+      </c>
+      <c r="M41" s="1" t="inlineStr">
+        <is>
+          <t>TESTCARE INSTRUMENTS</t>
+        </is>
+      </c>
+      <c r="N41" s="1" t="inlineStr">
+        <is>
+          <t>Testcare Instruments is a trusted supplier and trader of high-quality laboratory equipment, committed to supporting scientific excellence across diverse industries. With a strong focus on reliability, precision, and innovation, we provide a comprehensive range of instruments designed to meet the evolving needs of research laboratories, educational institutions, healthcare facilities, and industrial testing environments. Our portfolio includes advanced analytical instruments, measuring devices, testing equipment, and essential lab accessories sourced from reputable manufacturers, ensuring consistent performance and durability.At Testcare Instruments, we understand the critical role that accurate and dependable equipment plays in achieving meaningful results. Therefore, we prioritize quality assurance, timely delivery, and competitive pricing to ensure complete customer satisfaction. Business Type Supplier, Trading Company Employee Count 6 Establishment 2022 Working Days Monday To Saturday GST NO 29AOGPV0958N1Z1 Payment Mode Wallet &amp; UPI, Online Payments (NEFT/RTGS/IMPS), Cheque/DD, Cash Related Products Erba Em Destiny 180 - Fully Automated Biochemistry Analyzer - Automation Grade: Automatic Price: 550000 INR MOQ - 1 Unit/Units Global Biomedicals Inc Jaipur, Rajasthan</t>
+        </is>
+      </c>
+      <c r="O41" s="1" t="inlineStr"/>
+      <c r="P41" s="1" t="inlineStr"/>
+      <c r="Q41" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/testcare-instruments-90878291/</t>
+        </is>
+      </c>
+      <c r="R41" s="1" t="inlineStr"/>
+      <c r="S41" s="1" t="inlineStr"/>
+      <c r="T41" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Laboratory, Hospital, Research</t>
+        </is>
+      </c>
+      <c r="U41" s="1" t="inlineStr"/>
+      <c r="V41" s="1" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
+        <is>
+          <t>Reckon Getein-1100 Poct Analyzer</t>
+        </is>
+      </c>
+      <c r="B42" s="1" t="inlineStr">
+        <is>
+          <t>Darshi Biomedical</t>
+        </is>
+      </c>
+      <c r="C42" s="1" t="inlineStr">
+        <is>
+          <t>Reckon Getein-1100 Poct Analyzer</t>
+        </is>
+      </c>
+      <c r="D42" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/reckon-getein-1100-poct-analyzer-c10564197.html</t>
+        </is>
+      </c>
+      <c r="E42" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/10564197/b/4/Reckon-Getein-1100-Poct-Analyzer..jpg</t>
+        </is>
+      </c>
+      <c r="F42" s="1" t="inlineStr">
+        <is>
+          <t>High quality Display Type 7 inch Weight 1.9 Kilograms (kg) Power Supply Digital Dimension (L*W*H) 26</t>
+        </is>
+      </c>
+      <c r="G42" s="1" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+      <c r="H42" s="1" t="inlineStr">
+        <is>
+          <t>Portable Dissolved Gas Analyzer: https://www.tradeindia.com/products/portable-dissolved-gas-analyzer-c10344999.html
+Portable Combustion Analyzer: https://www.tradeindia.com/products/portable-combustion-analyzer-c1100168.html
+Portable Oxygen And Carbon Dioxide Analyzer - Application: Detecting O2 &amp; Co2: https://www.tradeindia.com/products/portable-oxygen-and-carbon-dioxide-analyzer-c9624051.html
+Krykard Portable Analyzer ALM 31: https://www.tradeindia.com/products/krykard-portable-analyser-alm-31-2679305.html
+Xrf Portable Analyzer: https://www.tradeindia.com/products/xrf-portable-analyzer-c9396325.html
+Hand Held Portable Xrf Analyzer - Color: White: https://www.tradeindia.com/products/xrf-portable-spectrometer-c8806870.html
+Hitachi Handheld Xrf Spectrometer Analyzers - Dimension (L*W*H): 10*93*272 Millimeter (Mm): https://www.tradeindia.com/products/hitachi-handheld-xrf-spectrometer-analyzers-c10845500.html
+Portable Xrf Analyzer - 220x300x220 mm, 130 eV Resolution, 4.3-Inch Touchscreen, Handheld, Battery Operated, USB Bluetooth Wi-Fi Connectivity: https://www.tradeindia.com/products/portable-xrf-analyzer-c2789274.html
+Kt220 Handheld Ct-Pt Analyzer - Color: Different Available: https://www.tradeindia.com/products/kt220-handheld-ct-pt-analyzer-c11930714.html
+2Nd Hand Analyzer - Features: High Quality: https://www.tradeindia.com/products/2nd-hand-analyzer-c11825413.html
+Portable Power Quality Analyzer - Compact Design , High-Precision Measurements, User-Friendly Interface, Real-Time Data Logging, Multi-Channel Monitoring: https://www.tradeindia.com/products/metravi-ce-0102pa-portable-power-quality-analyzer-c7040682.html
+Thermo Fisher Niton Xl5 Plus Handheld Xrf Analyzer - Features: Good Quality: https://www.tradeindia.com/products/thermo-fisher-niton-xl5-plus-handheld-xrf-analyzer-c10396889.html
+Semi Auto Analyser - Application: For Biochemistry Parameters: https://www.tradeindia.com/products/semi-auto-analyser-c10564175.html
+Fully Automated Biochemistry Analyzer - Application: Laboratory: https://www.tradeindia.com/products/fully-automated-biochemistry-analyzer-c10564184.html
+Cbs- 300 Diagnostic Electrolyte Analyzer - Automation Grade: Semi Automatic: https://www.tradeindia.com/products/cbs-300-diagnostic-electrolyte-analyzer-c10564189.html
+Cbs- 400 B And E Diagnostic Electrolyte Analyzer - Automation Grade: Automatic: https://www.tradeindia.com/products/cbs-400-b-and-e-diagnostic-electrolyte-analyzer-c10564188.html
+Semi Auto Biochemistry Analyzer - Application: Laboratory And Hospitals: https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-c10564185.html
+Reckon Getein-1100 Poct Analyzer - PVC Material, 261 x 241 x 115 mm, White &amp; Blue Color, 1.9 kg Weight, 220-240 Volt Voltage, 7-inch Display | Easy to Install, Compact Design: https://www.tradeindia.com/products/reckon-getein-1100-poct-analyzer-c10564201.html
+Reckon Crp Turbi Latex - Attributes: Safe To Use: https://www.tradeindia.com/products/reckon-crp-turbi-latex-c10564161.html
+Abbott Uro Meter 120 Urine Analyzer - Feature: Reliable &amp; Efficient: https://www.tradeindia.com/products/abbott-uro-meter-120-urine-analyzer-c10564193.html
+Crp Turbi Sure - Material: Plastic: https://www.tradeindia.com/products/crp-turbi-sure-c10564166.html
+Portable Trace H2s Hydrogen Sulfide Analyzer: https://www.tradeindia.com/products/portable-trace-h2s-hydrogen-sulfide-analyzer-c7574351.html
+Explorer 5000: https://www.tradeindia.com/products/explorer-5000-c5874493.html</t>
+        </is>
+      </c>
+      <c r="I42" s="1" t="inlineStr">
+        <is>
+          <t>Darshi Biomedical</t>
+        </is>
+      </c>
+      <c r="J42" s="1" t="inlineStr"/>
+      <c r="K42" s="1" t="inlineStr"/>
+      <c r="L42" s="1" t="inlineStr">
+        <is>
+          <t>Darshi Biomedical</t>
+        </is>
+      </c>
+      <c r="M42" s="1" t="inlineStr">
+        <is>
+          <t>Darshi Biomedical</t>
+        </is>
+      </c>
+      <c r="N42" s="1" t="inlineStr">
+        <is>
+          <t>Darshi Biomedical envisions a future where healthcare is defined by accuracy, accessibility, and unwavering trust. As a manufacturer, supplier, and trader of advanced diagnostic tools, the mission is cleara to empower healthcare professionals with precision instruments that transform patient care. Every product, from the CRP test kit and coral sgpt alat to the fully automatic biochemistry analyzer and diagnostic electrolyte analyzer, is designed to bridge the gap between innovation and real-world application. It is not just about tools; it is about creating pathways to faster diagnosis, informed decisions, and healthier lives. In a world where every second counts, we deliver rapid turnaround time, reliable results, and intuitive technology that simplifies the complexities of modern diagnostics. Whether it is the digital glucometer providing point-of-care convenience or the coral creat Business Type Manufacturer, Supplier, Trading Company Employee Count 5 Establishment 2014 Working Days Monday To Saturday GST NO 24AMMPP7307D1Z3 Payment Mode Cash in Advance (CID) Related Products Portable Dissolved Gas Analyzer Price: 4500000 INR MOQ - 1 Piece/Pieces Chromatography And Instrument Co Pvt Ltd Vadodara, Gujarat</t>
+        </is>
+      </c>
+      <c r="O42" s="1" t="inlineStr"/>
+      <c r="P42" s="1" t="inlineStr"/>
+      <c r="Q42" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/darshi-biomedical-5228411/</t>
+        </is>
+      </c>
+      <c r="R42" s="1" t="inlineStr"/>
+      <c r="S42" s="1" t="inlineStr"/>
+      <c r="T42" s="1" t="inlineStr">
+        <is>
+          <t>Laboratory</t>
+        </is>
+      </c>
+      <c r="U42" s="1" t="inlineStr"/>
+      <c r="V42" s="1" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr">
+        <is>
+          <t>Bio-chemistry Analyzer - Abs Plastic, Stainless Steel, 860x600x420 Mm, Fully Automatic, 300 Tests/hour, 7-inch Tft Touchscreen, Â¤2% Cv Accuracy at Best Price in Ambala Cantt | Kfw Scientific Industries</t>
+        </is>
+      </c>
+      <c r="B43" s="1" t="inlineStr"/>
+      <c r="C43" s="1" t="inlineStr">
+        <is>
+          <t>Kfw Scientific Industries - Offering low price Bio-chemistry Analyzer - Abs Plastic, Stainless Steel, 860x600x420 Mm, Fully Automatic, 300 Tests/hour, 7-inch Tft Touchscreen, Â¤2% Cv Accuracy in Science Market, Ambala Cantt with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="D43" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/bio-chemistry-analyzer-c2393205.html</t>
+        </is>
+      </c>
+      <c r="E43" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/02393205/b/4/Bio-Chemistry-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F43" s="1" t="inlineStr"/>
+      <c r="G43" s="1" t="inlineStr"/>
+      <c r="H43" s="1" t="inlineStr">
+        <is>
+          <t>Touch Screen Bio Chemistry Analyzer - Compact Design , Clear Digital Display Screen , User-Friendly Controls: https://www.tradeindia.com/products/touch-screen-bio-chemistry-analyzer-c6965405.html
+Bio Chemistry Analyzer - Absorbency, Mono-Chromatic &amp; Bi-Chromatic Methods | 100-Test Memory, Inbuilt Thermal Printer, 4x20 LCD Display: https://www.tradeindia.com/products/bio-chemistry-analyzer-c2505822.html
+Metal Bio-Chemistry Analyzer: https://www.tradeindia.com/products/bio-chemistry-analyzer-c1736368.html
+Bio Chemistry Analyzer - Application: Industrial: https://www.tradeindia.com/products/bio-chemistry-analyzer-c3205326.html
+Bio Chemistry Analyzer - Silver, 33x32x12.5cm | Absorbance Mono and Bi-Chromatic, 100 Test Memory, LCD Display, Thermostat Control 25-37Â°C: https://www.tradeindia.com/products/bio-chemistry-analyzer-c2951949.html
+Bio Chemistry Analyser Machine Weight: 1-10 Kilograms (Kg): https://www.tradeindia.com/products/bio-chemistry-analyser-c4408987.html
+Labcare Export Auto Biochemistry Analyzer: https://www.tradeindia.com/products/labcare-export-auto-biochemistry-analyzer-c6741418.html
+Touch Screen Bio Chemistry Analyzer: https://www.tradeindia.com/products/touch-screen-bio-chemistry-analyzer-c2392934.html
+Erba Semi Bio Chemistry Analyzer: https://www.tradeindia.com/products/erba-semi-bio-chemistry-analyzer-c5466456.html
+BIO-CHEMISTRY ANALYZER: https://www.tradeindia.com/products/bio-chemistry-analyzer-c2924176.html
+Bio Chemistry Analyzer: https://www.tradeindia.com/products/bio-chemistry-analyzer-10427689.html
+Bio Chemistry Analyzer - Photometry Optical System, 340-630nm Wavelength, 220V 50Hz, LCD Display, Thermostat 25-37Â°C, Multi-Method Analysis, Data Storage: https://www.tradeindia.com/products/bio-chemistry-analyzer-c2665759.html
+FTIR Spectrometer System: https://www.tradeindia.com/products/ftir-spectrometer-system-c2404900.html
+Hot Plate Rectangular: https://www.tradeindia.com/products/hot-plate-rectangular-c2402648.html
+Atomic Absporption Spectrophotometer: https://www.tradeindia.com/products/atomic-absporption-spectrophotometer-c2404919.html
+Atomic Absporption Spectrophotometer: https://www.tradeindia.com/products/atomic-absporption-spectrophotometer-c2404915.html
+Auto Karl Fischer Titrimeter: https://www.tradeindia.com/products/auto-karl-fischer-titrimeter-c2402996.html
+Clinical Digital Thermometer - ABS Plastic, 100x15x5 mm, White | Digital Display, Measurement Range 32-42Â°C, Â±0.1Â°C Accuracy, Battery Powered: https://www.tradeindia.com/products/clinical-digital-thermometer-c1199269.html
+Boy's law apparatus: https://www.tradeindia.com/products/boy-s-law-apparatus-c1204008.html
+Camera Lucida (Mirror Type) - Metal, Glass, 150x100x80 mm, Black Matte | 50x50 mm Mirror, 500g Weight, Hinge for Quick Eyepiece Change: https://www.tradeindia.com/products/camera-lucida-mirror-type-c2404611.html
+Digital Flame Photometers: https://www.tradeindia.com/products/digital-flame-photometers-c2404273.html
+Compound Bar Pendulum (Iron): https://www.tradeindia.com/products/compound-bar-pendulum-iron-c3255898.html
+Fully Auto Chemistry Analyzer BCH240: https://www.tradeindia.com/products/fully-auto-chemistry-analyzer-bch240-4929612.html
+High Performance Premium Chemistry Analyzer: https://www.tradeindia.com/products/high-performance-premium-chemistry-analyzer-4804529.html</t>
+        </is>
+      </c>
+      <c r="I43" s="1" t="inlineStr">
+        <is>
+          <t>Trusted Seller</t>
+        </is>
+      </c>
+      <c r="J43" s="1" t="inlineStr"/>
+      <c r="K43" s="1" t="inlineStr"/>
+      <c r="L43" s="1" t="inlineStr">
+        <is>
+          <t>Trusted Seller</t>
+        </is>
+      </c>
+      <c r="M43" s="1" t="inlineStr">
+        <is>
+          <t>Trusted Seller</t>
+        </is>
+      </c>
+      <c r="N43" s="1" t="inlineStr">
+        <is>
+          <t>We have a well-developed infrastructure, which is managed by a team of professionals. All our personnel are highly experienced and skilled in their specific work domain. They assist us in choosing the raw materials, carrying the production process, and delivering the products to our clients with the assurance of high quality.KFW Scientific Industries is a name to be reckoned with the best manufacturers, exporters, and suppliers of scientific instruments, pharma instruments, laboratory glassware, chemistry/ physics/ biological instruments, biological laboratory instruments and models, and agriculture instruments. In addition, we also deal in electrical &amp; Business Type Exporter, Manufacturer, Distributor, Supplier, Trading Company Employee Count 12 Establishment 1978 Working Days Monday To Sunday GST NO 06BLIPK7612L1ZU Related Products Touch Screen Bio Chemistry Analyzer - Compact Design , Clear Digital Display Screen , User-Friendly Controls Contemporary Export Industry Ambala Cantt, Haryana</t>
+        </is>
+      </c>
+      <c r="O43" s="1" t="inlineStr"/>
+      <c r="P43" s="1" t="inlineStr"/>
+      <c r="Q43" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/bio-chemistry-analyzer-c2393205.html</t>
+        </is>
+      </c>
+      <c r="R43" s="1" t="inlineStr"/>
+      <c r="S43" s="1" t="inlineStr"/>
+      <c r="T43" s="1" t="inlineStr">
+        <is>
+          <t>Kfw Scientific Industries - Offering low price Bio-chemistry Analyzer - Abs Plastic, Stainless Steel, 860x600x420 Mm, Fully Automatic, 300 Tests/hour, 7-inch Tft Touchscreen, Â¤2% Cv Accuracy in Science Market, Ambala Cantt with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="U43" s="1" t="inlineStr"/>
+      <c r="V43" s="1" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
+        <is>
+          <t>ERBACHEM 5X Biochemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="B44" s="1" t="inlineStr">
+        <is>
+          <t>BIOTEX LIFE SCIENCE</t>
+        </is>
+      </c>
+      <c r="C44" s="1" t="inlineStr">
+        <is>
+          <t>ERBACHEM 5X Biochemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="D44" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/erbachem-5x-biochemistry-analyzer-c10206917.html</t>
+        </is>
+      </c>
+      <c r="E44" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/10206917/b/4/ERBACHEM-5X-Biochemistry-Analyzer..jpg</t>
+        </is>
+      </c>
+      <c r="F44" s="1" t="inlineStr"/>
+      <c r="G44" s="1" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="H44" s="1" t="inlineStr">
+        <is>
+          <t>Erba Em Destiny 180 - Fully Automated Biochemistry Analyzer - Automation Grade: Automatic: https://www.tradeindia.com/products/erba-em-destiny-180-fully-automated-biochemistry-analyzer-c11787573.html
+Erba Biochemistry Analyzer Application: Industrial: https://www.tradeindia.com/products/erba-biochemistry-analyzer-c8544174.html
+Erba Biochemistry Analyzer - Plastic, Digital Display, Grey | Compact Design, Automatic/Semi-Automatic/Manual Operation, Low Power Consumption: https://www.tradeindia.com/products/erba-biochemistry-analyzer-c7874879.html
+Erba Biochemistry Analyzer: https://www.tradeindia.com/products/erba-biochemistry-analyzer-10254106.html
+Erba Biochemistry Analyzer: https://www.tradeindia.com/products/erba-biochemistry-analyzer-c12360320.html
+Top Quality Erba Biochemistry Analyzer: https://www.tradeindia.com/products/top-quality-erba-biochemistry-analyzer-5037931.html
+Chem 7 Erba Biochemistry Analyzer - Reliable Optical System, Easy to Use Interface, Heavy Duty, Industrial Laboratory Use: https://www.tradeindia.com/products/chem-7-erba-biochemistry-analyzer-10167227.html
+5X20Ml Sgpt Kit - Material: Plastic: https://www.tradeindia.com/products/5x20ml-sgpt-kit-c10206786.html
+Glucospark Blood Glucose Strips - Material: Plastic: https://www.tradeindia.com/products/glucospark-blood-glucose-strips-c10206821.html
+3 Ply Disposable Face Mask - Age Group: Suitable For All Ages: https://www.tradeindia.com/products/3-ply-disposable-face-mask-c10206829.html
+Htc-1 Digital Thermo Hygrometer - Color: White: https://www.tradeindia.com/products/htc-1-digital-thermo-hygrometer-c10206841.html
+Lab Microscope Binocular - Color: White: https://www.tradeindia.com/products/lab-microscope-binocular-c10206930.html
+5 Ltr Surgical Spirit - Color: Blue: https://www.tradeindia.com/products/5-ltr-surgical-spirit-c10206932.html
+Blood Collection Tube - Color: Transparent: https://www.tradeindia.com/products/blood-collection-tube-c10206939.html
+Glass Test Tube - Color: Transparent: https://www.tradeindia.com/products/glass-test-tube-c10206936.html
+Medico Centrifuge Machine - Color: Black: https://www.tradeindia.com/products/medico-centrifuge-machine-c10206945.html
+Digital Auto Calorimeter - Application: Commercial: https://www.tradeindia.com/products/digital-auto-calorimeter-c10206972.html
+Erba Chem 5x Semi Biochemistry Analyzer: https://www.tradeindia.com/products/erba-chem-5x-semi-biochemistry-analyzer-7167037.html
+Ergonomic Bioreactor: https://www.tradeindia.com/products/ergonomic-bioreactor-c10914315.html</t>
+        </is>
+      </c>
+      <c r="I44" s="1" t="inlineStr">
+        <is>
+          <t>BIOTEX LIFE SCIENCE</t>
+        </is>
+      </c>
+      <c r="J44" s="1" t="inlineStr"/>
+      <c r="K44" s="1" t="inlineStr"/>
+      <c r="L44" s="1" t="inlineStr">
+        <is>
+          <t>BIOTEX LIFE SCIENCE</t>
+        </is>
+      </c>
+      <c r="M44" s="1" t="inlineStr">
+        <is>
+          <t>BIOTEX LIFE SCIENCE</t>
+        </is>
+      </c>
+      <c r="N44" s="1" t="inlineStr">
+        <is>
+          <t>Biotex Life Science is one of the leading traders and suppliers of health and laboratory products. Our vast product range includes Test Kits, Test Strips, Cell Counters, Face Masks, and Micro Pipette Tips, etc. We cater to both healthcare professionals and research institutions. We focus on improving health outcomes by providing reliable diagnostics and protective equipment. At our company, we prioritize quality and customer satisfaction to ensure that our products meet stringent industry standards. Our mission is to support the scientific community and healthcare sector by providing innovative solutions that promote health and safety for all. We are also open to new collaborations that can help us to serve medical sector with exclusive array. Product Packaging Quality Business Type Manufacturer, Distributor, Supplier, Trading Company Employee Count 3 Establishment 2020 Working Days Monday To Sunday GST NO 09AIIPG7825K1ZU Payment Mode Online Payments (NEFT/RTGS/IMPS), Cheque/DD, Cash Related Products Erba Em Destiny 180 - Fully Automated Biochemistry Analyzer - Automation Grade: Automatic Price: 550000 INR MOQ - 1 Unit/Units Global Biomedicals Inc Jaipur, Rajasthan</t>
+        </is>
+      </c>
+      <c r="O44" s="1" t="inlineStr"/>
+      <c r="P44" s="1" t="inlineStr"/>
+      <c r="Q44" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/biotex-life-science-5237582/</t>
+        </is>
+      </c>
+      <c r="R44" s="1" t="inlineStr"/>
+      <c r="S44" s="1" t="inlineStr"/>
+      <c r="T44" s="1" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="U44" s="1" t="inlineStr"/>
+      <c r="V44" s="1" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Chemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="B45" s="1" t="inlineStr"/>
+      <c r="C45" s="1" t="inlineStr">
+        <is>
+          <t>Buy low price Clinical Chemistry Analyzer in Badambadi, Cuttack. Clinical Chemistry Analyzer offered by River View Bio Chemical is available with multiple payment options and easy delivery.</t>
+        </is>
+      </c>
+      <c r="D45" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/clinical-chemistry-analyzer-c13295107.html</t>
+        </is>
+      </c>
+      <c r="E45" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/13295107/b/4/Clinical-Chemistry-Analyzer..webp</t>
+        </is>
+      </c>
+      <c r="F45" s="1" t="inlineStr">
+        <is>
+          <t>User-friendly software, onboard printer, real-time result display, multiple test modes Temperature R</t>
+        </is>
+      </c>
+      <c r="G45" s="1" t="inlineStr">
+        <is>
+          <t>Biochemistry and pathology laboratory chemical analysis</t>
+        </is>
+      </c>
+      <c r="H45" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Chemistry Analyzer - 20x17x11 Inch, White and Blue, ABS Plastic and Mild Steel, 12 Watt Power, 1.16 kg Weight, Fast Blood Sample Analysis: https://www.tradeindia.com/products/20-x-17-x-11-inch-1-16-kilogram-abs-plastic-and-mild-steel-clinical-chemistry-analyzers-8319759.html
+Om-120 Biochemistry Analyzer - Application: Industrial: https://www.tradeindia.com/products/om-120-biochemistry-analyzer-c11636025.html
+Grey Semi-Automated Clinical Chemistry Analyzer: https://www.tradeindia.com/products/semi-automated-clinical-chemistry-analyzer-4018708.html
+Mispa Clinia Plus Fully Automated Clinical Chemistry Analyzer: https://www.tradeindia.com/products/mispa-clinia-plus-fully-automated-clinical-chemistry-analyzer-c13222463.html
+Full Automatic Chemistry Analyzer - Application: Commercial: https://www.tradeindia.com/products/full-automatic-chemistry-analyzer-c9474134.html
+Clinical Chemistry Analyzer - Application: Laboratory Use: https://www.tradeindia.com/products/clinical-chemistry-analyzer-c5395097.html
+Semi Auto Biochemistry Analyzer - Color: White: https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-c10598125.html
+Semi-Automated Biochemistry Analyzer - Application: Anlyzer: https://www.tradeindia.com/products/biochemistry-analyzer-c10543245.html
+Biochemistry Analyzer - Color: White Black: https://www.tradeindia.com/products/biochemistry-analyzer-c6350610.html
+Bio-Chemistry Analyzer - Advanced Diagnostic Performance | High Precision, User-Friendly Interface, Real-Time Data Analysis, Compact Design: https://www.tradeindia.com/products/bio-chemistry-analyzer-c6965407.html
+Bio Chemistry Analyzer - Absorbency, Mono-Chromatic &amp; Bi-Chromatic Methods | 100-Test Memory, Inbuilt Thermal Printer, 4x20 LCD Display: https://www.tradeindia.com/products/bio-chemistry-analyzer-c2505822.html
+Sensa Core ST 200 Aqua Electrolyte Analyzer: https://www.tradeindia.com/products/sensa-core-st-200-aqua-electrolyte-analyzer-c13295092.html
+Meril Celquant Edge Diluent: https://www.tradeindia.com/products/meril-celquant-edge-diluent-c13295121.html
+Urine Chemistry Analyzer: https://www.tradeindia.com/products/urine-chemistry-analyzer-c13295131.html
+CQ5 Ultima Merilyzer Celquant With Auto Loader: https://www.tradeindia.com/products/cq5-ultima-merilyzer-celquant-with-auto-loader-c13295175.html
+Cbc Hematology Analyzer: https://www.tradeindia.com/products/cbc-hematology-analyzer-c13295086.html
+500ml Edge Lyse Meril Celquant: https://www.tradeindia.com/products/500ml-meril-celquant-edge-lyse-c13295129.html
+Meril Clotquant 2 Hematology Analyzer: https://www.tradeindia.com/products/meril-clotquant-2-hematology-analyzer-c13295085.html
+Horiba Hematology Analyzer: https://www.tradeindia.com/products/horiba-hematology-analyzer-c13295091.html
+Robonik Biochemistry Analyzer: https://www.tradeindia.com/products/robonik-biochemistry-analyzer-c13295108.html
+Microlab 300 Biochemistry Analyzer: https://www.tradeindia.com/products/microlab-300-biochemistry-analyzer-5482147.html
+KANAD 8MPC PLUS Clinical Chemistry Analyzer: https://www.tradeindia.com/products/kanad-8mpc-plus-clinical-chemistry-analyzer-6521743.html</t>
+        </is>
+      </c>
+      <c r="I45" s="1" t="inlineStr"/>
+      <c r="J45" s="1" t="inlineStr"/>
+      <c r="K45" s="1" t="inlineStr"/>
+      <c r="L45" s="1" t="inlineStr"/>
+      <c r="M45" s="1" t="inlineStr"/>
+      <c r="N45" s="1" t="inlineStr">
+        <is>
+          <t>Welcome to River View Bio Chemical, where precision diagnostics meet dependable supply. As a trusted supplier and trader in the field of laboratory and healthcare solutions, we are committed to empowering diagnostic centers, hospitals, and pathology labs with reliable, high-quality products that support accurate patient care.Our comprehensive product range includes Hematology Analyzers, Edge Lyse, Analyzer Quality Control Kit, Rinse Cleanzer and many more, each carefully sourced to meet the diverse needs of modern diagnostic laboratories. From accurate blood cell analysis to optimal cell lysis, quality control, and analyzer maintenance, our range covers the essential requirements of a well-equipped, efficient laboratory setup.At River View Bio Chemical, we understand that in healthcare, precision is not just important it is essential. That is why we prioritize sourcing q Business Type Supplier, Trading Company Employee Count 6 Establishment 2020 Working Days Monday To Sunday GST NO 21FTKPS4474J1Z6 Payment Mode Online Payments (NEFT/RTGS/IMPS), Cheque/DD, Cash Related Products Clinical Chemistry Analyzer MOQ - 1 Unit/Units River View Bio Chemical Cuttack, Odisha</t>
+        </is>
+      </c>
+      <c r="O45" s="1" t="inlineStr"/>
+      <c r="P45" s="1" t="inlineStr"/>
+      <c r="Q45" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/clinical-chemistry-analyzer-c13295107.html</t>
+        </is>
+      </c>
+      <c r="R45" s="1" t="inlineStr"/>
+      <c r="S45" s="1" t="inlineStr"/>
+      <c r="T45" s="1" t="inlineStr">
+        <is>
+          <t>Biochemistry and pathology laboratory chemical analysis</t>
+        </is>
+      </c>
+      <c r="U45" s="1" t="inlineStr">
+        <is>
+          <t>Biochemistry and pathology laboratory chemical analysis</t>
+        </is>
+      </c>
+      <c r="V45" s="1" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>Truchem 48 Biochemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="B46" s="1" t="inlineStr">
+        <is>
+          <t>TRUVIC HEALTHCARE</t>
+        </is>
+      </c>
+      <c r="C46" s="1" t="inlineStr">
+        <is>
+          <t>Truchem 48 Biochemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="D46" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/truchem-48-biochemistry-analyzer-c11160976.html</t>
+        </is>
+      </c>
+      <c r="E46" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/11160976/b/4/Truchem-48-Biochemistry-Analyzer..jpg</t>
+        </is>
+      </c>
+      <c r="F46" s="1" t="inlineStr">
+        <is>
+          <t>High quality Usage Clinical Size Different available Voltage 65V Volt (v) Warranty Yes Payment Terms
+High quality High-quality Usage Clinical Industrial For Laboratory Size Different available Standard</t>
+        </is>
+      </c>
+      <c r="G46" s="1" t="inlineStr">
+        <is>
+          <t>Clinical</t>
+        </is>
+      </c>
+      <c r="H46" s="1" t="inlineStr">
+        <is>
+          <t>Smart Biochemistry Analyzer: https://www.tradeindia.com/products/smart-biochemistry-analyzer-c11977823.html
+Horiba Pentra 400 Fully Automatic Biochemistry Analyzer - Color: Customized: https://www.tradeindia.com/products/horiba-pentra-400-fully-automatic-biochemistry-analyzer-c11160977.html
+Innolab 200 Semi Automatic Biochemistry Analyzer - Application: Laboratories: https://www.tradeindia.com/products/innolab-200-semi-automatic-biochemistry-analyzer-c10651688.html
+Fully Auto Biochemistry Analyzer (BI-200) - 200 Tests/Hour, Double Reagents for Serum &amp; Urine Analysis | Liver &amp; Kidney Function Testing, Cardiac Markers: https://www.tradeindia.com/products/fully-auto-biochemistry-analyzer-bi-200-c8779733.html
+Semiautomated Biochemistry Analyzer: https://www.tradeindia.com/products/semiautomated-biochemistry-analyzer-c11977824.html
+Vector V Chem Next Biochemistry Analyzer - Color: As Per Demand: https://www.tradeindia.com/products/vector-v-chem-next-biochemistry-analyzer-c11872765.html
+Bx-3010 Automated Bio Chemistry Analyzer - Accuracy: Cv 1% For Repeatability %: https://www.tradeindia.com/products/bx-3010-automated-chemistry-analyzer-c12491620.html
+Erbachem 5X Biochemistry Analyzer - Color: White: https://www.tradeindia.com/products/erbachem-5x-biochemistry-analyzer-c10206917.html
+Pictus-700 Fully Automatic Biochemistry Analyzer - Feature: High Quality: https://www.tradeindia.com/products/pictus-700-fully-automatic-biochemistry-analyzer-c10778212.html
+Horiba Yumizen Ca60 Clinical Chemistry Analyzer - Color: Blue And White: https://www.tradeindia.com/products/horiba-yumizen-ca60-clinical-chemistry-analyzer-c11160991.html
+Clinical Use Metrolab 1600 Dr Biochemistry Analyzer: https://www.tradeindia.com/products/clinical-use-metrolab-1600-dr-biochemistry-analyzer-8510126.html
+Biochemistry Analyzer: https://www.tradeindia.com/products/biochemistry-analyzer-c4469651.html
+Horiba Yumizen G200 Hemostasis Analyzer - Feature: High Quality: https://www.tradeindia.com/products/horiba-yumizen-g200-hemostasis-analyzer-c11160967.html
+Magnus Mlx B Plus - Color: Black And Silver: https://www.tradeindia.com/products/magnus-mlx-b-plus-c11160984.html
+Horiba Yumizen Ca40 Analyser - Color: Multicolour: https://www.tradeindia.com/products/horiba-yumizen-ca40-analyser-c11160993.html
+Horiba Diluent Hematology Reagents - Color: Customized: https://www.tradeindia.com/products/horiba-diluent-hematology-reagents-c11161001.html
+100 Ma Mobile X Ray Machine - Color: Customized: https://www.tradeindia.com/products/100-ma-mobile-x-ray-machine-c11161010.html
+Horiba Abx Micro Es60 Hematology Analyzer - Color: Transparent: https://www.tradeindia.com/products/horiba-abx-micro-es60-hematology-analyzer-c11160966.html
+Finecar Fully-Automatic Fia Analyzer - Color: Multiple: https://www.tradeindia.com/products/finecar-fully-automatic-fia-analyzer-c11160969.html
+Sonorad V8 Ultrasound Machine - Color: Customized: https://www.tradeindia.com/products/sonorad-v8-ultrasound-machine-c11161044.html
+Nulyte Digital Display Electrolyte Analyzer - Color: Multicolour: https://www.tradeindia.com/products/nulyte-digital-display-electrolyte-analyzer-c11161048.html
+Biochemistry Analyzer: https://www.tradeindia.com/products/biochemistry-analyzer-c6350610.html
+High Performance Automatic Biochemistry Analyzer For Laboratory: https://www.tradeindia.com/products/high-performance-automatic-biochemistry-analyzer-for-laboratory-8579675.html</t>
+        </is>
+      </c>
+      <c r="I46" s="1" t="inlineStr">
+        <is>
+          <t>TRUVIC HEALTHCARE</t>
+        </is>
+      </c>
+      <c r="J46" s="1" t="inlineStr"/>
+      <c r="K46" s="1" t="inlineStr"/>
+      <c r="L46" s="1" t="inlineStr">
+        <is>
+          <t>TRUVIC HEALTHCARE</t>
+        </is>
+      </c>
+      <c r="M46" s="1" t="inlineStr">
+        <is>
+          <t>TRUVIC HEALTHCARE</t>
+        </is>
+      </c>
+      <c r="N46" s="1" t="inlineStr">
+        <is>
+          <t>Established in 2016 and based in Kanpur, Uttar Pradesh, Truvic Healthcare has emerged as a dynamic force in the healthcare and diagnostics equipment industry. As a trusted manufacturer, trader, and supplier, we are committed to delivering advanced medical and laboratory solutions that empower healthcare professionals to achieve greater diagnostic accuracy and operational efficiency.We offer a premium portfolio of products that includes Finecar FIA Meter X2 Hematology Analyzer, Finecar Fully-Automatic FIA Analyzer, Magnus CH20i Microscope, Horiba Pentra C200 Clinical Chemistry Analyzer, Horiba Diluent Hematology Reagents, Carestream Vita Flex CR System, etc. With a focus on quality, precision, and customer satisfaction, we serve diagnostic centers, hospitals, l Business Type Manufacturer, Supplier, Trading Company Employee Count 10 Establishment 2016 Working Days Monday To Sunday GST NO 09AMXPD9527E2ZJ Payment Mode Online Payments (NEFT/RTGS/IMPS), Cheque/DD, Wallet &amp; UPI, Cash Related Products Smart Biochemistry Analyzer MOQ - 10 Unit/Units Jks Enterprises Kanpur, Uttar Pradesh</t>
+        </is>
+      </c>
+      <c r="O46" s="1" t="inlineStr"/>
+      <c r="P46" s="1" t="inlineStr"/>
+      <c r="Q46" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/truvic-healthcare-40589588/</t>
+        </is>
+      </c>
+      <c r="R46" s="1" t="inlineStr"/>
+      <c r="S46" s="1" t="inlineStr"/>
+      <c r="T46" s="1" t="inlineStr">
+        <is>
+          <t>Clinical</t>
+        </is>
+      </c>
+      <c r="U46" s="1" t="inlineStr"/>
+      <c r="V46" s="1" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr">
+        <is>
+          <t>C-71 Clinical Chemistry Analyzer Application: Industrial</t>
+        </is>
+      </c>
+      <c r="B47" s="1" t="inlineStr">
+        <is>
+          <t>PSJ Biochem Diagnostic Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="C47" s="1" t="inlineStr">
+        <is>
+          <t>C-71 Clinical Chemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="D47" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/c-71-clinical-chemistry-analyzer-c8544197.html</t>
+        </is>
+      </c>
+      <c r="E47" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/08544197/b/4/C-71-Clinical-Chemistry-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F47" s="1" t="inlineStr"/>
+      <c r="G47" s="1" t="inlineStr"/>
+      <c r="H47" s="1" t="inlineStr">
+        <is>
+          <t>Full Automatic Chemistry Analyzer - Application: Commercial: https://www.tradeindia.com/products/full-automatic-chemistry-analyzer-c9474134.html
+Biochemistry Analyzer - Color: White Black: https://www.tradeindia.com/products/biochemistry-analyzer-c6350610.html
+Maglumi Chemiluminescence Immunoassay Analyzer - Color: White: https://www.tradeindia.com/products/maglumi-chemiluminescence-immunoassay-analyzer-c10317334.html
+Stainless Steel Semi Automated Clinical Chemistry Analyzer For Hospital Use: https://www.tradeindia.com/products/semi-automated-clinical-chemistry-analyzer-for-hospital-use-8531403.html
+Aspen Star 20 Clinical Chemistry Analyzer: https://www.tradeindia.com/products/aspen-star-20-clinical-chemistry-analyzer-c9495036.html
+Semi Automatic Clinical Chemistry Analyzer: https://www.tradeindia.com/products/semi-automatic-clinical-chemistry-analyzer-c515950.html
+Semi Automated Clinical Chemistry Analyzer: https://www.tradeindia.com/products/semi-automated-clinical-chemistry-analyzer-9910184.html
+Erba Biochemistry Analyzer Application: Industrial: https://www.tradeindia.com/products/erba-biochemistry-analyzer-c8544174.html
+Bc 5800 Hemotology Analyzer Application: Industrial: https://www.tradeindia.com/products/bc-5800-hemotology-analyzer-c8544173.html
+Hematology Analayzer - Application: Medical Purpose: https://www.tradeindia.com/products/hematology-analayzer-c8633293.html
+I800 Hormone Analyzer Application: Industrial: https://www.tradeindia.com/products/i800-hormone-analyzer-c8544236.html
+I800 Immunoassay Analyzer - Application: Industrial: https://www.tradeindia.com/products/i800-immunoassay-analyzer-c8544237.html
+10 W Siemens Bayer Lamp - Application: Industrial: https://www.tradeindia.com/products/10-w-siemens-bayer-lamp-c8544220.html
+Micros60 Abx Waste Sensor Application: Industrial: https://www.tradeindia.com/products/micros60-abx-waste-sensor-c8544130.html
+Bc-2800 Mindray 2.5Ml Syringe Application: Industrial: https://www.tradeindia.com/products/bc-2800-mindray-2-5ml-syringe-c8544162.html
+7.5 Ml Mindray Hematology Analyzer Syringe Application: Industrial: https://www.tradeindia.com/products/7-5-ml-mindray-hematology-analyzer-syringe-c8544140.html
+Nihon Kohden Peristaltic Pump Tube Application: Industrial: https://www.tradeindia.com/products/nihon-kohden-peristaltic-pump-tube-c8544161.html
+POCT Analyzer (BI-180: https://www.tradeindia.com/products/poct-analyzer-bi-180-c8781013.html
+Semi-Auto Biochemistry Analyzer: https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-3988337.html</t>
+        </is>
+      </c>
+      <c r="I47" s="1" t="inlineStr">
+        <is>
+          <t>PSJ Biochem Diagnostic Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="J47" s="1" t="inlineStr"/>
+      <c r="K47" s="1" t="inlineStr"/>
+      <c r="L47" s="1" t="inlineStr">
+        <is>
+          <t>PSJ Biochem Diagnostic Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="M47" s="1" t="inlineStr">
+        <is>
+          <t>PSJ Biochem Diagnostic Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="N47" s="1" t="inlineStr">
+        <is>
+          <t>PSJ Biochem Diagnostic Pvt. Ltd. is a company that is well-recognized for offering a wide range of Mindray Chemistry Analyzer Big Pumps, Rotation Motor Position Sensors, Hormone Analyzers, Erba Biochemistry Analyzers, and other products. We are established as one of the leading manufacturers, suppliers, and traders of the aforementioned products. All our products are of high quality and comply with predefined industry standards. Each product is made using the finest quality raw materials at our advanced manufacturing unit under the guidance of our team of professionals. Our professionals are highly intelligent, experienced, and competent to design and develop such a range that holds the power to be instantly liked by a wide range of customers. We Business Type Manufacturer, Distributor, Supplier, Trading Company Employee Count 20 Establishment 2006 Working Days Monday To Sunday GST NO 07AAECP0016C1Z5 Payment Mode Cash Advance (CA) Related Products Full Automatic Chemistry Analyzer - Application: Commercial MOQ - 1 Unit/Units Weldon Biotech (india) Pvt. Ltd. Delhi, Delhi</t>
+        </is>
+      </c>
+      <c r="O47" s="1" t="inlineStr"/>
+      <c r="P47" s="1" t="inlineStr"/>
+      <c r="Q47" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/psj-biochem-diagnostic-pvt-ltd-2376460/</t>
+        </is>
+      </c>
+      <c r="R47" s="1" t="inlineStr"/>
+      <c r="S47" s="1" t="inlineStr"/>
+      <c r="T47" s="1" t="inlineStr">
+        <is>
+          <t>C-71 Clinical Chemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="U47" s="1" t="inlineStr"/>
+      <c r="V47" s="1" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Biochemistry Analyzer at Best Price in New Delhi, Delhi | Martand Medical Services</t>
+        </is>
+      </c>
+      <c r="B48" s="1" t="inlineStr"/>
+      <c r="C48" s="1" t="inlineStr">
+        <is>
+          <t>Buy low price Clinical Biochemistry Analyzer in Vijay Enclave, New Delhi. Clinical Biochemistry Analyzer offered by Martand Medical Services is available with multiple payment options and easy delivery.</t>
+        </is>
+      </c>
+      <c r="D48" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/clinical-biochemistry-analyzer-c3774440.html</t>
+        </is>
+      </c>
+      <c r="E48" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/03774440/b/4/Clinical-Biochemistry-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F48" s="1" t="inlineStr">
+        <is>
+          <t>Semi-automated, Easy-to-use, Cost-effective, Reliable, High-performance, Compact Company Details Mar</t>
+        </is>
+      </c>
+      <c r="G48" s="1" t="inlineStr">
+        <is>
+          <t>Clinical biochemistry analysis in labs</t>
+        </is>
+      </c>
+      <c r="H48" s="1" t="inlineStr">
+        <is>
+          <t>Autoquant 400 Supremus Biochemistry Analyzer - Color: Different Available: https://www.tradeindia.com/products/autoquant-400-supremus-biochemistry-analyzer-c9144587.html
+Agd 2260 Fully Automatic Clinical Chemistry Analyzer - Attributes: Higher Level Of Accuracy: https://www.tradeindia.com/products/agd-2260-fully-automatic-clinical-chemistry-analyzer-c8452668.html
+Biochemistry Analyzer Application: Laboratory/Hospital/Pharmaceutical Industry: https://www.tradeindia.com/products/biochemistry-analyzer-c8355970.html
+Labman Biochemistry Analyzer - Features: Durable: https://www.tradeindia.com/products/labman-biochemistry-analyzer-c11508492.html
+SEMI BIOCHEMISTRY ANALYZER: https://www.tradeindia.com/products/semi-biochemistry-analyzer-c7947308.html
+Biochemistry Analyzer: https://www.tradeindia.com/products/biochemistry-analyzer-c3303495.html
+Semi Auto Biochemistry Analyzer(Coagulation &amp; Incubator): https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-coagulation-incubator-c3704795.html
+Semi Auto Biochemistry Analyzer - 7.0 Inch True Color Touch Screen, 300 Programmable Tests &amp; 200,000 Result Storage, Auto Sleep &amp; Lamp Protection, Dual Wavelength Absorbance &amp; Coagulation Measurement: https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-1790459.html
+Accukine Biochemistry Analyzer - Color: Black: https://www.tradeindia.com/products/accukine-biochemistry-analyzer-9205582.html
+Os-3000M Semi-Automatic Biochemistry Analyze Touch Screen - Power Source: Electric: https://www.tradeindia.com/products/os-3000m-semi-automatic-biochemistry-analyze-touch-screen-c7737366.html
+Biochemistry Analyzer Dimension(L*W*H): 50X 6 X 6 Inch (In): https://www.tradeindia.com/products/biochemistry-analyzer-4251323.html
+Analyzer Auto Biochemistry Analyzer-Emerald: https://www.tradeindia.com/products/auto-biochemistry-analyzer-emerald-c6779909.html
+Glass Capillary Tube for Newborn Jaundice: https://www.tradeindia.com/products/glass-capillary-tube-for-newborn-jaundice-c3704822.html
+Multipara Monitor - Compact, Lightweight, 320 x 160 x 270mm | Multi-Patient Monitoring, Portable Design, Rechargeable Battery, Comprehensive Alarms: https://www.tradeindia.com/products/multipara-monitor-c3704802.html
+Radiant Heat Warmer - Metal &amp; Plastic, Variable Dimensions | Digital Control, LED Display, Accurate Results, Long Battery Life, Heat Preservation, Metabolism Control: https://www.tradeindia.com/products/radiant-heat-warmer-c3704819.html
+Mobile OT Lights: https://www.tradeindia.com/products/mobile-ot-lights-c3763322.html
+Pneumotrac Vitalograph: https://www.tradeindia.com/products/pneumotrac-vitalograph-c3771869.html
+Capillary Bilirubinometer: https://www.tradeindia.com/products/capillary-bilirubinometer-c3776783.html
+Neo-Tee Infant T-Piece Resuscitator: https://www.tradeindia.com/products/neo-tee-infant-t-piece-resuscitator-c3783283.html
+Common NICU equipment: https://www.tradeindia.com/products/common-nicu-equipment-c3783274.html
+Blood Bag Centrifuge - ABS &amp; SS, 330x420x275 mm, Max Speed 12000 RPM, 24 Capillary Rotor, Timer 0-15 min | Digital Display, Compact Design, Durable Build: https://www.tradeindia.com/products/blood-bag-centrifuges-c3778689.html
+Transcutaneous Meter - 65x135x35 mm, Reflectance Photometry, Two LEDs, Photocell Detector | Non-Invasive, Jaundice Screening, Fast, Accurate LCD Display: https://www.tradeindia.com/products/testing-spirometer-c3778681.html
+Meril Auto Quant 100 AMARA -Fully Automated Biochemistry Analyzer: https://www.tradeindia.com/products/meril-auto-quant-100-amara-fully-automated-biochemistry-analyzer-c10862941.html
+Stable Performance Biochemistry Analyzer: https://www.tradeindia.com/products/stable-performance-biochemistry-analyzer-85757.html</t>
+        </is>
+      </c>
+      <c r="I48" s="1" t="inlineStr"/>
+      <c r="J48" s="1" t="inlineStr"/>
+      <c r="K48" s="1" t="inlineStr"/>
+      <c r="L48" s="1" t="inlineStr"/>
+      <c r="M48" s="1" t="inlineStr"/>
+      <c r="N48" s="1" t="inlineStr">
+        <is>
+          <t>Martand Medical Services is a renowned supplier of haematology analyser and other biochemistry analyser and laboratory testing equipment. Established in 2015, we have been providing advanced laboratory testing equipment and analyser including Business Type Exporter, Importer, Distributor, Supplier, Trading Company Employee Count 20 Establishment 2015 Working Days Monday To Sunday Related Products Autoquant 400 Supremus Biochemistry Analyzer - Color: Different Available Price: 1060000 INR MOQ - 5 Unit/Units Drx Laboratories India Inc New Delhi, Delhi</t>
+        </is>
+      </c>
+      <c r="O48" s="1" t="inlineStr"/>
+      <c r="P48" s="1" t="inlineStr"/>
+      <c r="Q48" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/clinical-biochemistry-analyzer-c3774440.html</t>
+        </is>
+      </c>
+      <c r="R48" s="1" t="inlineStr"/>
+      <c r="S48" s="1" t="inlineStr"/>
+      <c r="T48" s="1" t="inlineStr">
+        <is>
+          <t>Clinical biochemistry analysis in labs</t>
+        </is>
+      </c>
+      <c r="U48" s="1" t="inlineStr">
+        <is>
+          <t>Clinical biochemistry analysis in labs</t>
+        </is>
+      </c>
+      <c r="V48" s="1" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Chemistry Analyzer - Quartz Colorimetric Tank, 330x310x175mm, Halogen Lamp, 340-630nm | Large Memory, Multifunctional Software, Convenient Maintenance</t>
+        </is>
+      </c>
+      <c r="B49" s="1" t="inlineStr"/>
+      <c r="C49" s="1" t="inlineStr">
+        <is>
+          <t>U. R. Diagnostics Pvt. Ltd. - Offering low price Clinical Chemistry Analyzer - Quartz Colorimetric Tank, 330x310x175mm, Halogen Lamp, 340-630nm | Large Memory, Multifunctional Software, Convenient Maintenance - Quartz Colorimetric Tank, 330x310x175mm, Halogen Lamp, 340-630nm | Large Memory, Multifunctional Software, Convenient Maintenance in NH-5 Nissan Hut (NIT), Faridabad with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="D49" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/clinical-chemistry-analyzer-c720406.html</t>
+        </is>
+      </c>
+      <c r="E49" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/00720406/b/4/Clinical-Chemistry-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F49" s="1" t="inlineStr">
+        <is>
+          <t>Accurate results, Easy operation, Large memory, Cost effective, Reliable analysis, Convenient mainte
+Bluefic Industrial &amp; Scientific Technologies Ambala, Haryana Send Inquiry Touch Screen Bio Chemistry</t>
+        </is>
+      </c>
+      <c r="G49" s="1" t="inlineStr"/>
+      <c r="H49" s="1" t="inlineStr">
+        <is>
+          <t>Mediray- Semi Auto Biochemistry Analyzer - Material: Plastic: https://www.tradeindia.com/products/mediray-semi-auto-biochemistry-analyzer-c10608461.html
+Auto Chemistry Analyzer: https://www.tradeindia.com/products/auto-chemistry-analyzer-c720401.html
+Bio Chemistry Analyzer Fully Automatic: https://www.tradeindia.com/products/bio-chemistry-analyzer-fully-automatic-c5375379.html
+U-Ra Semi Automated Clinical Chemistry Analyzer Application: Hospital: https://www.tradeindia.com/products/u-ra-semi-automated-clinical-chemistry-analyzer-6561623.html
+Semi Auto Chemistry Analyzer - Compact Design, High Throughput Capability, Enhanced Accuracy Features: https://www.tradeindia.com/products/semi-auto-chemistry-analyzer-c7303681.html
+Touch Screen Bio Chemistry Analyzer - Compact Design , Clear Digital Display Screen , User-Friendly Controls: https://www.tradeindia.com/products/touch-screen-bio-chemistry-analyzer-c6965405.html
+Bio Chemistry Analyzer - Absorbency, Mono-Chromatic &amp; Bi-Chromatic Methods | 100-Test Memory, Inbuilt Thermal Printer, 4x20 LCD Display: https://www.tradeindia.com/products/bio-chemistry-analyzer-c2505822.html
+Metal Bio-Chemistry Analyzer: https://www.tradeindia.com/products/bio-chemistry-analyzer-c1736368.html
+Bio Chemistry Analyzer - Application: Industrial: https://www.tradeindia.com/products/bio-chemistry-analyzer-c3205326.html
+Bio Chemistry Analyzer - Silver, 33x32x12.5cm | Absorbance Mono and Bi-Chromatic, 100 Test Memory, LCD Display, Thermostat Control 25-37Â°C: https://www.tradeindia.com/products/bio-chemistry-analyzer-c2951949.html
+Bio Chemistry Analyser Machine Weight: 1-10 Kilograms (Kg): https://www.tradeindia.com/products/bio-chemistry-analyser-c4408987.html
+Labcare Export Auto Biochemistry Analyzer: https://www.tradeindia.com/products/labcare-export-auto-biochemistry-analyzer-c6741418.html
+Automated Urine Analyzer - Battery/AC Powered, 60 Seconds Test Time, 500 Sample Memory, 210g Portable Design | Accurate Results, Fast Testing, Easy Operation: https://www.tradeindia.com/products/automated-urine-analyzer-c720408.html
+Hematology Analyzers Comparison: https://www.tradeindia.com/products/hematology-analyzers-comparison-c720396.html
+I Chroma Hormone Analyzer: https://www.tradeindia.com/products/i-chroma-hormone-analyzer-c3082588.html
+Portable Hemoglobin Analyzer: https://www.tradeindia.com/products/portable-hemoglobin-analyzer-c3082592.html
+ISE Electrolyte Analyzer: https://www.tradeindia.com/products/ise-electrolyte-analyzer-c720392.html
+Microplate Reader Fluorescence: https://www.tradeindia.com/products/microplate-reader-fluorescence-c720398.html
+Glucose Meter - 88x64x22mm, LCD Display | Fast Testing, 20~600mg/dL Range, 200 Memory Capacity, Lightweight 59g: https://www.tradeindia.com/products/glucose-meter-c3082587.html
+Elisa Microplate Washer: https://www.tradeindia.com/products/elisa-microplate-washer-c3082594.html
+Clinical Chemistry Analyzer: https://www.tradeindia.com/products/clinical-chemistry-analyzer-c720399.html
+Neo 4000 Chemistry Analyzer: https://www.tradeindia.com/products/neo-4000-chemistry-analyzer-6469074.html</t>
+        </is>
+      </c>
+      <c r="I49" s="1" t="inlineStr"/>
+      <c r="J49" s="1" t="inlineStr"/>
+      <c r="K49" s="1" t="inlineStr"/>
+      <c r="L49" s="1" t="inlineStr"/>
+      <c r="M49" s="1" t="inlineStr"/>
+      <c r="N49" s="1" t="inlineStr">
+        <is>
+          <t>Company Preface To cater to the requirements of pharmaceutical and diagnostic industries, we, U.R. Diagnostics Pvt Ltd., were founded in 2007. Since our foundation, we have remained committed in meeting and exceeding our clients expectations with our entire assortment of quality assured products. Acquisition of immense knowledge and rich experience has assisted in achieving a prominent position of one of the noted importers, traders and suppliers in this competitive industry. Banking on valuable contribution of reliable vendors, we are able to showcase a quality range of products such as Clinical Chemistry (Two Reagents ), Clinical Chemistry ( Single Reagents), Serology ( Including Blood Group Business Type Exporter, Supplier, Trading Company Employee Count 50 Establishment 2001 Related Products Mediray- Semi Auto Biochemistry Analyzer - Material: Plastic Price: 52000 INR MOQ - 1 Piece/Pieces Mediray Healthcare Faridabad, Haryana</t>
+        </is>
+      </c>
+      <c r="O49" s="1" t="inlineStr"/>
+      <c r="P49" s="1" t="inlineStr"/>
+      <c r="Q49" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/clinical-chemistry-analyzer-c720406.html</t>
+        </is>
+      </c>
+      <c r="R49" s="1" t="inlineStr"/>
+      <c r="S49" s="1" t="inlineStr"/>
+      <c r="T49" s="1" t="inlineStr">
+        <is>
+          <t>U. R. Diagnostics Pvt. Ltd. - Offering low price Clinical Chemistry Analyzer - Quartz Colorimetric Tank, 330x310x175mm, Halogen Lamp, 340-630nm | Large Memory, Multifunctional Software, Convenient Maintenance - Quartz Colorimetric Tank, 330x310x175mm, Halogen Lamp, 340-630nm | Large Memory, Multifunctional Software, Convenient Maintenance in NH-5 Nissan Hut (NIT), Faridabad with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="U49" s="1" t="inlineStr"/>
+      <c r="V49" s="1" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr">
+        <is>
+          <t>Erba Chem 5x Clinical Chemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>Udit Agencies</t>
+        </is>
+      </c>
+      <c r="C50" s="1" t="inlineStr">
+        <is>
+          <t>Erba Chem 5x Clinical Chemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="D50" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/erba-chem-5x-clinical-chemistry-analyzer-c13260384.html</t>
+        </is>
+      </c>
+      <c r="E50" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/13260384/b/4/Erba-Chem-5x-Clinical-Chemistry-Analyzer..webp</t>
+        </is>
+      </c>
+      <c r="F50" s="1" t="inlineStr"/>
+      <c r="G50" s="1" t="inlineStr">
+        <is>
+          <t>Clinical chemistry assays</t>
+        </is>
+      </c>
+      <c r="H50" s="1" t="inlineStr">
+        <is>
+          <t>Erba Biochemistry Analyzer: https://www.tradeindia.com/products/erba-biochemistry-analyzer-c12360320.html
+Erba Em Destiny 180 - Fully Automated Biochemistry Analyzer - Automation Grade: Automatic: https://www.tradeindia.com/products/erba-em-destiny-180-fully-automated-biochemistry-analyzer-c11787573.html
+Erba Biochemistry Analyzer Application: Industrial: https://www.tradeindia.com/products/erba-biochemistry-analyzer-c8544174.html
+Erba Biochemistry Analyzer: https://www.tradeindia.com/products/erba-biochemistry-analyzer-10254106.html
+Erba Biochemistry Analyzer - Plastic, Digital Display, Grey | Compact Design, Automatic/Semi-Automatic/Manual Operation, Low Power Consumption: https://www.tradeindia.com/products/erba-biochemistry-analyzer-c7874879.html
+Top Quality Erba Biochemistry Analyzer: https://www.tradeindia.com/products/top-quality-erba-biochemistry-analyzer-5037931.html
+Chem 7 Erba Biochemistry Analyzer - Reliable Optical System, Easy to Use Interface, Heavy Duty, Industrial Laboratory Use: https://www.tradeindia.com/products/chem-7-erba-biochemistry-analyzer-10167227.html
+Automated Coagulation Analyzer: https://www.tradeindia.com/products/automated-coagulation-analyzer-c13260391.html
+Semi Automated Bio Chemistry Anlayzer: https://www.tradeindia.com/products/semi-automated-bio-chemistry-anlayzer-c13260379.html
+Automatic Biochemistry Analyzer: https://www.tradeindia.com/products/automatic-biochemistry-analyzer-c13260385.html
+Roche Diagnostics AVL 9180 Series Electrolyte Analyzers: https://www.tradeindia.com/products/roche-diagnostics-avl-9180-series-electrolyte-analyzers-c13260395.html
+Erba Ec 90 Electrolyte Analyzer: https://www.tradeindia.com/products/erba-ec-90-electrolyte-analyzer-c13260396.html
+Semi Automated ESR Analyzer: https://www.tradeindia.com/products/semi-automated-esr-analyzer-c13260398.html
+Turbodyne SC Tulip Diagnostics Analyzer: https://www.tradeindia.com/products/turbodyne-sc-tulip-diagnostics-analyzer-c13260406.html
+Turbodyne SC Tulip Diagnostics Analyzer: https://www.tradeindia.com/products/turbodyne-sc-tulip-diagnostics-analyzer-c13260408.html
+Digital Hemoglobin Meter: https://www.tradeindia.com/products/digital-hemoglobin-meter-c13260415.html
+Fully Automated Biochemistry Analyzer: https://www.tradeindia.com/products/fully-automated-biochemistry-analyzer-c13260381.html
+SemiAutomatic Biochemistry Analyzer ERBA CHEM7: https://www.tradeindia.com/products/semiautomatic-biochemistry-analyzer-erba-chem7-c8169376.html</t>
+        </is>
+      </c>
+      <c r="I50" s="1" t="inlineStr">
+        <is>
+          <t>Udit Agencies</t>
+        </is>
+      </c>
+      <c r="J50" s="1" t="inlineStr"/>
+      <c r="K50" s="1" t="inlineStr"/>
+      <c r="L50" s="1" t="inlineStr">
+        <is>
+          <t>Udit Agencies</t>
+        </is>
+      </c>
+      <c r="M50" s="1" t="inlineStr">
+        <is>
+          <t>Udit Agencies</t>
+        </is>
+      </c>
+      <c r="N50" s="1" t="inlineStr">
+        <is>
+          <t>Udit Agencies is committed to supporting laboratories, diagnostic centres, healthcare institutions, and medical professionals with dependable diagnostic solutions and professional equipment support. As a trader, supplier, retailer, wholesaler, service provider, we focus on bringing together quality, accuracy, technology, and responsive assistance to address the practical requirements of modern diagnostic environments. The product range includes Sysmex Cell Counter, Automated Coagulation Analyzer, Electrolyte Analyzer, Hemoglobin Meter, and Immunoassay Analyzer, selected to support reliable laboratory testing and efficient diagnostic workflows. Alongside equipment, Medical Equipment Repair Services strengthen the overall offering by helping customers maintain dependable performance and continuity in their operations. Business Type Service Provider, Supplier, Trading Company, Wholesaler, Retailer Employee Count 6 Establishment 1999 Working Days Monday To Sunday GST NO 23ABOPM6436H1ZH Payment Mode Others, Online Payments (NEFT/RTGS/IMPS), Cheque/DD, Cash Related Products Erba Biochemistry Analyzer Price: 90000 INR MOQ - 1 Piece/Pieces Arnavi Enterprises Bhopal, Madhya Pradesh</t>
+        </is>
+      </c>
+      <c r="O50" s="1" t="inlineStr"/>
+      <c r="P50" s="1" t="inlineStr"/>
+      <c r="Q50" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/udit-agencies-2241277/</t>
+        </is>
+      </c>
+      <c r="R50" s="1" t="inlineStr"/>
+      <c r="S50" s="1" t="inlineStr"/>
+      <c r="T50" s="1" t="inlineStr">
+        <is>
+          <t>Clinical chemistry assays</t>
+        </is>
+      </c>
+      <c r="U50" s="1" t="inlineStr">
+        <is>
+          <t>Clinical chemistry assays</t>
+        </is>
+      </c>
+      <c r="V50" s="1" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Chemistry Analyzer - Permanent Hard Glass Cuvettes, Throughput 600 Tests/hr | Automated Process, Sapphire Lamp, Barcoded Samples, 50 On-board Tests</t>
+        </is>
+      </c>
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>Didac International</t>
+        </is>
+      </c>
+      <c r="C51" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Chemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="D51" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/clinical-chemistry-analyzer-c3597846.html</t>
+        </is>
+      </c>
+      <c r="E51" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/03597846/b/4/Clinical-Chemistry-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F51" s="1" t="inlineStr">
+        <is>
+          <t>High throughput, Fast results, High accuracy, Automated process, Barcoded samples, Wide test choices</t>
+        </is>
+      </c>
+      <c r="G51" s="1" t="inlineStr"/>
+      <c r="H51" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Chemistry Analyzer - Color: White: https://www.tradeindia.com/products/clinical-chemistry-analyzer-c11771172.html
+Euro Lab 200 Clinical Chemistry Analyzer - Attributes: Higher Level Of Accuracy: https://www.tradeindia.com/products/euro-lab-200-clinical-chemistry-analyzer-c8614148.html
+Biochemistry Analyzer Application: Laboratory/Hospital/Pharmaceutical Industry: https://www.tradeindia.com/products/biochemistry-analyzer-c8355970.html
+Labman Biochemistry Analyzer - Features: Durable: https://www.tradeindia.com/products/labman-biochemistry-analyzer-c11508492.html
+Clinical Chemistry Analyzers - 120 Tests/Hour Throughput | Random Access, STAT Capability, Open System with 40 Programmable Methods: https://www.tradeindia.com/products/clinical-chemistry-analyzers-4173450.html
+Semi Auto Biochemistry Analyzer - 7.0 Inch True Color Touch Screen, 300 Programmable Tests &amp; 200,000 Result Storage, Auto Sleep &amp; Lamp Protection, Dual Wavelength Absorbance &amp; Coagulation Measurement: https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-1790459.html
+Clinical Chemistry Analyzer - Unique Triple Cuvette System | 56 Direct Access Keys, Low Reagent Consumption, Online Display of Reaction Curve, Quality Control Monitoring: https://www.tradeindia.com/products/clinical-chemistry-analyzer-3897482.html
+Clinical chemistry analyzers: https://www.tradeindia.com/products/clinical-chemistry-analyzers-c3774451.html
+Biochemistry Analyser - High Efficiency, Rectangular Shape, Semi-Automatic Operation | Portable, Easy to Operate, Manual Control, White Plastic Design: https://www.tradeindia.com/products/biochemistry-analyser-9086318.html
+Portable Compact Medical Device - Polycarbonate Sheet, 75.0 x 50.0 x 28.0 cm, Chromatic Grey | 40 Watt Power, 13 kg Weight, Suitable for Pathology Lab: https://www.tradeindia.com/products/portable-compact-mobile-lab-7067570.html
+Fully Automated Clinical Chemistry Analyzer - High-Precision Manufacturing Using Quality Raw Materials | International Standards Compliance, User-Friendly Interface, Efficient Performance: https://www.tradeindia.com/products/fully-automated-clinical-chemistry-analyzer-4169034.html
+Clinical Chemistry Analyzer - 675x450x300 mm Dimensions, 180 Tests/Hour Throughput | Automated Random Access, Adjustable Sample Volume, Extensive QC Programme: https://www.tradeindia.com/products/clinical-chemistry-analyzer-c3597751.html
+Bino Metallurgical Microscope MT7000EH - 30W Koehler Illumination, Ergonomic Controls, Binocular Head, Brightfield Observation: https://www.tradeindia.com/products/bino-metallurgical-microscope-mt7000eh-c3553808.html
+Tail Flick Analgesia Meters - Methacrylate, 350x350x130 mm, Halogen Lamp | Precise Measurement, Automated Testing, Sensitive Analysis: https://www.tradeindia.com/products/tail-flick-analgesia-meters-c3647051.html
+Complete Instrument With Cell - Portable Conductivity Meter, Auto Calibration, LCD Display, 0.1 1 10 Cell Constant, 0-80Â°C Temperature Range: https://www.tradeindia.com/products/complete-instrument-with-cell-c3653430.html
+Electronic Pipettes - 0.1-5000 ÂµL, 1/8/12-Channel, DC-Motor | Optiload Tip Sealing, 9 Speeds, Ergonomic Design: https://www.tradeindia.com/products/electronic-pipettes-c3714384.html
+Heating Block System - Silver Modular Base Plates, Up to 500ml Flask Capacity, Flexible Multiple Blocks: https://www.tradeindia.com/products/heating-block-system-c3582838.html
+Microbiological Safety Cabinet Class II - Stainless Steel, Variable Dimensions, Centrifugal Fans | Microprocessor Control, HEPA Filtration, Removable Work Surface: https://www.tradeindia.com/products/microbiological-safety-cabinet-class-ii-c3602342.html
+PuriCare Procedure Stations - 304 Stainless Steel, Powder-Coated Steel, Tempered Glass | Air Recirculation 70%, Filter Monitoring, Security Lock: https://www.tradeindia.com/products/puricare-procedure-stations-c3604199.html
+Neurobiology Teaching System - Blue, PowerLab 4/26, LabChart Software, Amplifiers, Headstages | Neurobiology Teaching, Data Acquisition, Nerve Chamber: https://www.tradeindia.com/products/neurobiology-teaching-system-c3633048.html
+Digital Melting Point Apparatus: https://www.tradeindia.com/products/digital-melting-point-apparatus-c3583237.html
+Dry Block Heater 4: https://www.tradeindia.com/products/dry-block-heater-4-c3614965.html
+RD-50 Clinical Chemistry Analyzer: https://www.tradeindia.com/products/rd-50-clinical-chemistry-analyzer-4607540.html
+Clinical Auto Chemistry Analyzer: https://www.tradeindia.com/products/clinical-auto-chemistry-analyzer-4865643.html
+EM 360 Automated Clinical Chemistry Analyzer: https://www.tradeindia.com/products/em-360-automated-clinical-chemistry-analyzer-5070236.html
+Fully Automated Clinical Chemistry Analyzer - Hard Glass Cuvettes, 200 Tests/Hr | Automated Pipetting, Onboard Cooling, Reagent Saving, Quality Control: https://www.tradeindia.com/products/fully-automated-clinical-chemistry-analyzer-c3597762.html
+Semi Automated Clinical Chemistry Analyzer - Touch Screen Interface, Wide Temperature Range 20-40Â°C, Unique Triple Cuvette System, Built-In Quality Control, Advanced Real-Time Graphs, Non-Linear Calibration Up to 10 Standards: https://www.tradeindia.com/products/semi-automated-clinical-chemistry-analyzer-c3597952.html
+Open System Clinical Chemistry Analyzer: https://www.tradeindia.com/products/open-system-clinical-chemistry-analyzer-c3597788.html
+Clinical Chemistry Analyzer - Application: Laboratory Use: https://www.tradeindia.com/products/clinical-chemistry-analyzer-c5395097.html
+Semi Auto Chemistry Analyzer: https://www.tradeindia.com/products/semi-auto-chemistry-analyzer-c4258308.html
+Neo 4000 Chemistry Analyzer: https://www.tradeindia.com/products/neo-4000-chemistry-analyzer-6469074.html</t>
+        </is>
+      </c>
+      <c r="I51" s="1" t="inlineStr">
+        <is>
+          <t>Didac International</t>
+        </is>
+      </c>
+      <c r="J51" s="1" t="inlineStr"/>
+      <c r="K51" s="1" t="inlineStr"/>
+      <c r="L51" s="1" t="inlineStr">
+        <is>
+          <t>Didac International</t>
+        </is>
+      </c>
+      <c r="M51" s="1" t="inlineStr">
+        <is>
+          <t>Didac International</t>
+        </is>
+      </c>
+      <c r="N51" s="1" t="inlineStr">
+        <is>
+          <t>An Introduction For updating the technological set up of several research centers and medical labs and giving the experts of them ease in completing their works, here, we, Didac International, are offering reliable equipment. The 1980 born enterprise is working sincerely as a manufacturer and supplier of Autoclaves, Microscopes, Laboratory Instruments, General Lab Equipment and Clean Air Systems. The microscopes we offer are praised for their compact design, high clarity of the lens and simple usage. 84068_HOME1.jpg 84068_HOME2.jpg Serving Quality of Expectation Quality products is the first thing every customer expects in return of his/her hard earned money. To stand upto the expectation of clients, Business Type Manufacturer, Supplier Employee Count 20 Establishment 2010 Working Days Monday To Sunday GST NO 07DCLPM4529J1Z6 Payment Mode Cash Advance (CA), Others Related Products Clinical Chemistry Analyzer - Color: White Price: 580000 INR MOQ - 1 Piece/Pieces Drx Laboratories India Inc New Delhi, Delhi</t>
+        </is>
+      </c>
+      <c r="O51" s="1" t="inlineStr"/>
+      <c r="P51" s="1" t="inlineStr"/>
+      <c r="Q51" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/didac-international-11078877/</t>
+        </is>
+      </c>
+      <c r="R51" s="1" t="inlineStr"/>
+      <c r="S51" s="1" t="inlineStr"/>
+      <c r="T51" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Chemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="U51" s="1" t="inlineStr"/>
+      <c r="V51" s="1" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Chemistry Analyzers</t>
+        </is>
+      </c>
+      <c r="B52" s="1" t="inlineStr"/>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>Buy low price Clinical Chemistry Analyzers in Sanathnagar, Hyderabad. Clinical Chemistry Analyzers offered by Elico Limited is available with multiple payment options and easy delivery.</t>
+        </is>
+      </c>
+      <c r="D52" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/clinical-chemistry-analyzers-c698758.html</t>
+        </is>
+      </c>
+      <c r="E52" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/00698758/b/5/Clinical-Chemistry-Analyzers.jpg</t>
+        </is>
+      </c>
+      <c r="F52" s="1" t="inlineStr">
+        <is>
+          <t>User friendly, Storage facility, Advanced calculations, Online printing Company Details ELICO LIMITE</t>
+        </is>
+      </c>
+      <c r="G52" s="1" t="inlineStr"/>
+      <c r="H52" s="1" t="inlineStr">
+        <is>
+          <t>Emp 168 Semi Automatic Chemistry Analyzer Dimension(L*W*H): 420(L) X 310(W) X 152(H) Centimeter (Cm): https://www.tradeindia.com/products/semi-automatic-chemistry-analyzer-c6629826.html
+Clinical Chemistry Analyzer - Semi-Automated System with Touch Screen &amp; Large LCD Display | 7 Filters (340-630nm), Dynamic Temperature Control, 112 Test Profiles Memory: https://www.tradeindia.com/products/clinical-chemistry-analyzer-5813679.html
+Semi Automatic Chemistry Analyzer - High-Quality Manufacturing, Ideal for Laboratories | Advanced Functionality, Suitable for Various Applications, Great Performance in Hyderabad: https://www.tradeindia.com/products/semi-automatic-biochemistry-analyzer-5571420.html
+Clinical Chemistry Analyzer - Plastic Material, 220V Voltage, White Color, 50/60 Hz Frequency | Semi-Automatic Medical Use: https://www.tradeindia.com/products/clinical-chemistry-analyzer-8581804.html
+Semi-Automatic Clinical Chemistry Analyzer - BAS-100, Powerful Data Processing, Built-in Printer, Suction Pump System, Kinetic Testing at 25-30-37Â°C, Measures All Blood Elements: https://www.tradeindia.com/products/semi-automatic-clinical-chemistry-analyzer-747976.html
+Clinical Chemistry Analyzer - Semi-Automatic Flow Cell Model | User-Friendly Microcontroller, 40 Pre-Programmed Assays, Built-in Thermal Printer: https://www.tradeindia.com/products/clinical-chemistry-analyzers-6103155.html
+High Quality BS200 Chemistry Analyzer - Aluminum, 50x70mm, 12V, 2kg | Precise Analysis, Reliable Results, Easy to Use: https://www.tradeindia.com/products/high-quality-bs200-chemistry-analyzer-4694085.html
+Redefine Fully Automatic Chemistry Analyzer: https://www.tradeindia.com/products/redefine-fully-automatic-chemistry-analyzer-6632153.html
+Water Quality Analyser: https://www.tradeindia.com/products/water-quality-analyser-c698764.html
+Colorimeters: https://www.tradeindia.com/products/colorimeters-c698755.html
+NIR Spectrophotometer: https://www.tradeindia.com/products/nir-spectrophotometer-c698766.html
+Single Beam Atomic Absorption Spectrophotometer: https://www.tradeindia.com/products/single-beam-atomic-absorption-spectrophotometer-c698769.html
+Ph Meter: https://www.tradeindia.com/products/ph-meter-c698763.html
+Fluoroscence Spectrophotometer &amp; Analyzer: https://www.tradeindia.com/products/fluoroscence-spectrophotometer-analyzer-c698770.html
+Visible Spectrophotometers: https://www.tradeindia.com/products/visible-spectrophotometers-c698752.html
+Diode Array Spectrophotometers: https://www.tradeindia.com/products/diode-array-spectrophotometers-c698765.html
+PH Analyser: https://www.tradeindia.com/products/ph-analyser-c698762.html</t>
+        </is>
+      </c>
+      <c r="I52" s="1" t="inlineStr"/>
+      <c r="J52" s="1" t="inlineStr"/>
+      <c r="K52" s="1" t="inlineStr"/>
+      <c r="L52" s="1" t="inlineStr"/>
+      <c r="M52" s="1" t="inlineStr"/>
+      <c r="N52" s="1" t="inlineStr">
+        <is>
+          <t>ELICO LIMITED , Established in 1959 at Hyderabad in Telangana, is a leading Exporter,Manufacturer,Supplier of Measuring Tools &amp; Equipment in India. ELICO LIMITED is one of Trade India's verified and trusted sellers of listed products. With extensive experience in supplying and trading Clinical Chemistry Analyzers, ELICO LIMITED has made a reputed name for itself in the market with high-quality True Double Beam Atomic Absorption Spectrophotometer, Variable Bandwidth UV VIS Spectrophotometers, Bio Spectrophotometers, etc. Focusing on a customer-centric approach, ELICO LIMITED has a pan-India presence and caters to a huge consumer base throughout the country. Buy Measuring Tools &amp; Equipment in bulk from ELICO LIMITED at Trade India quality-assured products. Business Type Exporter, Manufacturer, Supplier Establishment 1959 Working Days Monday To Sunday GST NO 36AAACE5140L1ZP Certification ISO:9001 Related Products Emp 168 Semi Automatic Chemistry Analyzer Dimension(L*W*H): 420(L) X 310(W) X 152(H) Centimeter (Cm) Vishnu Bio Sciences Hyderabad, Telangana</t>
+        </is>
+      </c>
+      <c r="O52" s="1" t="inlineStr"/>
+      <c r="P52" s="1" t="inlineStr"/>
+      <c r="Q52" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/clinical-chemistry-analyzers-c698758.html</t>
+        </is>
+      </c>
+      <c r="R52" s="1" t="inlineStr"/>
+      <c r="S52" s="1" t="inlineStr"/>
+      <c r="T52" s="1" t="inlineStr">
+        <is>
+          <t>Buy low price Clinical Chemistry Analyzers in Sanathnagar, Hyderabad. Clinical Chemistry Analyzers offered by Elico Limited is available with multiple payment options and easy delivery.</t>
+        </is>
+      </c>
+      <c r="U52" s="1" t="inlineStr"/>
+      <c r="V52" s="1" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>C Sense Biochemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>Pulse Medical Services</t>
+        </is>
+      </c>
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>C Sense Biochemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="D53" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/c-sense-biocemistry-analyzer-c8016368.html</t>
+        </is>
+      </c>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/08016368/b/4/C-Sense-Biochemistry-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F53" s="1" t="inlineStr"/>
+      <c r="G53" s="1" t="inlineStr"/>
+      <c r="H53" s="1" t="inlineStr">
+        <is>
+          <t>Stainless Steel Ura Semi Auto Chemistry Analyzer: https://www.tradeindia.com/products/ura-semi-auto-chemistry-analyzer-c8016419.html
+Reliable Biochemistry Analyzer: https://www.tradeindia.com/products/reliable-biochemistry-analyzer-5311260.html
+Semi Automatic Chemistry Analyzer - High-Quality Manufacturing, Ideal for Laboratories | Advanced Functionality, Suitable for Various Applications, Great Performance in Hyderabad: https://www.tradeindia.com/products/semi-automatic-biochemistry-analyzer-5571420.html
+BioChemistry Analyzers: https://www.tradeindia.com/products/biochemistry-analyzers-3386381.html
+Biochemistry Analyzer: https://www.tradeindia.com/products/biochemistry-analyzer-10375688.html
+YK 8000C ECG Machine - Plastic, Portable, White | Multi-Parameter Monitoring, Real-Time S-T Segment Analysis, Pacemaker Detection: https://www.tradeindia.com/products/yk-8000c-ecg-machine-c8016383.html
+Innova Portable Baby Warmer - Material: Stainless Steel And Plastic: https://www.tradeindia.com/products/innova-baby-warmer-c8016377.html
+C Arm Machine 1K X 1K Cam - Attributes: Strong &amp; Durable: https://www.tradeindia.com/products/c-arm-machine-1k-x-1k-cam-c10611367.html
+White Eva 500 Surgical Ot Light: https://www.tradeindia.com/products/eva-500-light-c8016403.html
+Hematology Analyzer - Material: Plastic: https://www.tradeindia.com/products/hematology-analyzer-c8016309.html
+Asteros Lite Ventilator - FRP Fibre Body, 220V, 60Hz | Stainless Steel Writing Tray, Low Flow Anaesthesia Capability, Three Storage Drawers: https://www.tradeindia.com/products/asteros-lite-ventilator-c8016401.html
+Cms 8000 Ecg Machine - Color: White: https://www.tradeindia.com/products/cms-8000-ecg-machine-c8016380.html
+Stainless Steel Specific Protein Analyzer: https://www.tradeindia.com/products/specfic-protein-analyzer-c8016405.html</t>
+        </is>
+      </c>
+      <c r="I53" s="1" t="inlineStr">
+        <is>
+          <t>Pulse Medical Services</t>
+        </is>
+      </c>
+      <c r="J53" s="1" t="inlineStr"/>
+      <c r="K53" s="1" t="inlineStr"/>
+      <c r="L53" s="1" t="inlineStr">
+        <is>
+          <t>Pulse Medical Services</t>
+        </is>
+      </c>
+      <c r="M53" s="1" t="inlineStr">
+        <is>
+          <t>Pulse Medical Services</t>
+        </is>
+      </c>
+      <c r="N53" s="1" t="inlineStr">
+        <is>
+          <t>Pulse Medical Services is a rising name in the Indian industry of medical equipment and tools. We are a supplier and trader of ESR Analyzer, C Sense Biochemistry Analyzer, Turbine Driven Ventilator, Hematology Analyzer and many more. These equipment are used in hospitals and medical institutions for diagnosing diseases and monitoring patients. Our products are known for providing accurate results, affordability and sturdy design. We rely on our reputed vendors to supply the best products from the market. Our vendors are chosen after being checked on various parameters such as past performance, delivery capabilities, quality of the goods and other factors. Business Type Supplier, Trading Company Employee Count 6 Establishment 2020 Working Days Monday To Saturday GST NO 36EYSPP1028M1ZR Payment Mode Online Payments (NEFT/RTGS/IMPS) Related Products Stainless Steel Ura Semi Auto Chemistry Analyzer Price: 100300 INR MOQ - 1 Unit/Units Pulse Medical Services Secunderabad, Telangana</t>
+        </is>
+      </c>
+      <c r="O53" s="1" t="inlineStr"/>
+      <c r="P53" s="1" t="inlineStr"/>
+      <c r="Q53" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/pulse-medical-services-9769229/</t>
+        </is>
+      </c>
+      <c r="R53" s="1" t="inlineStr"/>
+      <c r="S53" s="1" t="inlineStr"/>
+      <c r="T53" s="1" t="inlineStr">
+        <is>
+          <t>C Sense Biochemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="U53" s="1" t="inlineStr"/>
+      <c r="V53" s="1" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr">
+        <is>
+          <t>Cpc Turbochem Prime Fully Automated Clinical Chemistry Analyzer - Dimension (L*w*h): 756 X 834 X 643 Millimeter (Mm)</t>
+        </is>
+      </c>
+      <c r="B54" s="1" t="inlineStr"/>
+      <c r="C54" s="1" t="inlineStr">
+        <is>
+          <t>Ank Cares Pvt Ltd - Offering low price Cpc Turbochem Prime Fully Automated Clinical Chemistry Analyzer - Dimension (l*w*h): 756 X 834 X 643 Millimeter (mm) in Ashram Road, Ahmedabad with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="D54" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/cpc-turbochem-prime-fully-automated-clinical-chemistry-analyzer-c8761098.html</t>
+        </is>
+      </c>
+      <c r="E54" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/08761098/b/4/CPC-Turbochem-Prime-Fully-Automated-Clinical-Chemistry-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F54" s="1" t="inlineStr">
+        <is>
+          <t>CPC Turbochem Prime Fully Automated Clinical Chemistry Analyzer FEATURES - Constant Throughput of 18</t>
+        </is>
+      </c>
+      <c r="G54" s="1" t="inlineStr">
+        <is>
+          <t>Hospital / Pathlab / Clinic</t>
+        </is>
+      </c>
+      <c r="H54" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Chemistry Analyzer - Application: Laboratory Use: https://www.tradeindia.com/products/clinical-chemistry-analyzer-c5395097.html
+Mispa Viva Semi Automated Bio Chemistry Clinical Chemistry Analyzer: https://www.tradeindia.com/products/mispa-viva-semi-automated-bio-chemistry-clinical-chemistry-analyzer-8487557.html
+Clinical Chemistry Analyzers Application: Laboratories And Hospitals: https://www.tradeindia.com/products/clinical-chemistry-analyzers-3989621.html
+Nihon Kohden Chm 4100K Biochemistry Analyzer - Application: Laboratory: https://www.tradeindia.com/products/nihon-kohden-chm-4100k-biochemistry-analyzer-c10564183.html
+Erba Chem 5X Clinical Chemistry Analyzer Color Code: White: https://www.tradeindia.com/products/erba-chem-5x-clinical-chemistry-analyzer-c8379215.html
+RD-50 Clinical Chemistry Analyzer: https://www.tradeindia.com/products/rd-50-clinical-chemistry-analyzer-4607540.html
+Fully-Automated Clinical Chemistry Analyzer: https://www.tradeindia.com/products/fully-automated-clinical-chemistry-analyzer-4725825.html
+Uric Acid Coral Kit - Suitable For: Hospital: https://www.tradeindia.com/products/uric-acid-coral-kit-c8379274.html
+Immuno Science Covid 19 Antigen Rapid Test Kit Icmr Approved - Unisex, Hospital/Pathlab Usage | Fast &amp; Reliable Results: https://www.tradeindia.com/products/immuno-science-covid-19-antigen-rapid-test-kit-icmr-approved-c8379242.html
+Non Vacuum Blood Collection Tube - PET &amp; Other Material, New Condition | Ideal for Hospital Use: https://www.tradeindia.com/products/non-vacuum-blood-collection-tube-c8379313.html
+HIV Rapid Test Kit Trustline - Plastic Material | Unisex Design for Hospital Usage, Reliable and Efficient Testing Solution: https://www.tradeindia.com/products/hiv-rapid-test-kit-trustline-c8379079.html
+Urine Test Strip - New, Clinical Grade | For Hospital and Pathlab Use, Reliable Equipment Type for Accurate Results: https://www.tradeindia.com/products/urine-test-strip-c8379285.html
+Sinocare Glucose Test Strips and Uric Strips - 50 Test Strips, FAD-GDH Material | Compatible with Safe AQ Smart, Voice, Air Glucometers, No Manual Coding, Multi-Material Resistance: https://www.tradeindia.com/products/sinocare-glucose-test-strips-and-uric-strips-c8639589.html
+Finecare - FIA Meter Plus Analyser 112: https://www.tradeindia.com/products/finecare-fia-meter-plus-analyser-112-c8520179.html
+Bioassay Homocysteine Elisa Kit Human - Gender: Unisex: https://www.tradeindia.com/products/bioassay-homocysteine-elisa-kit-human-c9276379.html
+Corona Virus Pcr Test Kit - Gender: Unisex: https://www.tradeindia.com/products/corona-virus-pcr-test-kit-c6109531.html
+Sinocare Safe-Accu (Bood Glucose Monitoring System) - Use: Pathlab / Hospital / Clinic: https://www.tradeindia.com/products/sinocare-safe-accu-bood-glucose-monitoring-system-c8639911.html</t>
+        </is>
+      </c>
+      <c r="I54" s="1" t="inlineStr"/>
+      <c r="J54" s="1" t="inlineStr"/>
+      <c r="K54" s="1" t="inlineStr"/>
+      <c r="L54" s="1" t="inlineStr"/>
+      <c r="M54" s="1" t="inlineStr"/>
+      <c r="N54" s="1" t="inlineStr">
+        <is>
+          <t>Ank Cares Pvt Ltd , Established in 2015 at Ahmedabad in Gujarat, is a leading Exporter,Manufacturer,Supplier,Trading Company of Personal Safety Equipment in India. Ank Cares Pvt Ltd is one of Trade India's verified and trusted sellers of listed products. With extensive experience in supplying and trading CPC Turbochem Prime Fully Automated Clinical Chemistry Analyzer, Ank Cares Pvt Ltd has made a reputed name for itself in the market with high-quality 100 Bp DNA Ladder 500ul, Abon Multi Drug Test Kit 6 Panel, Abon-Alere Multi Line Drug Screen Test (Urine) 10 Para, etc. Focusing on a customer-centric approach, Ank Cares Pvt Ltd has a pan-India presence and caters to a huge consumer base throughout the country. Buy Personal Safety Equipment in bulk from Ank Cares Pvt Ltd at Trade India quality-assured products. Business Type Exporter, Manufacturer, Supplier, Trading Company Employee Count 25 Establishment 2015 Working Days Monday To Sunday GST NO 24AAQCA0109F1Z4 Payment Mode Cash Advance (CA) Related Products Clinical Chemistry Analyzer - Application: Laboratory Use Price: 105000.00 INR MOQ - 1 Piece/Pieces Microlab Instruments Private Limited Ahmedabad, Gujarat</t>
+        </is>
+      </c>
+      <c r="O54" s="1" t="inlineStr"/>
+      <c r="P54" s="1" t="inlineStr"/>
+      <c r="Q54" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/cpc-turbochem-prime-fully-automated-clinical-chemistry-analyzer-c8761098.html</t>
+        </is>
+      </c>
+      <c r="R54" s="1" t="inlineStr"/>
+      <c r="S54" s="1" t="inlineStr"/>
+      <c r="T54" s="1" t="inlineStr">
+        <is>
+          <t>Hospital / Pathlab / Clinic</t>
+        </is>
+      </c>
+      <c r="U54" s="1" t="inlineStr"/>
+      <c r="V54" s="1" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr">
+        <is>
+          <t>Star 20 Clinical Chemistry Analyzer Application: Hospital</t>
+        </is>
+      </c>
+      <c r="B55" s="1" t="inlineStr"/>
+      <c r="C55" s="1" t="inlineStr">
+        <is>
+          <t>Health Tech Healthcare - Offering low price Star 20 Clinical Chemistry Analyzer Application: Hospital Application: Hospital in Rani Bagh, Delhi with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="D55" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/star-20-clinical-chemistry-analyzer-c9495038.html</t>
+        </is>
+      </c>
+      <c r="E55" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/09495038/b/4/Star-20-Clinical-Chemistry-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F55" s="1" t="inlineStr"/>
+      <c r="G55" s="1" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="H55" s="1" t="inlineStr">
+        <is>
+          <t>Full Automatic Chemistry Analyzer - Application: Commercial: https://www.tradeindia.com/products/full-automatic-chemistry-analyzer-c9474134.html
+Biochemistry Analyzer - Color: White Black: https://www.tradeindia.com/products/biochemistry-analyzer-c6350610.html
+Maglumi Chemiluminescence Immunoassay Analyzer - Color: White: https://www.tradeindia.com/products/maglumi-chemiluminescence-immunoassay-analyzer-c10317334.html
+Stainless Steel Semi Automated Clinical Chemistry Analyzer For Hospital Use: https://www.tradeindia.com/products/semi-automated-clinical-chemistry-analyzer-for-hospital-use-8531403.html
+Aspen Star 20 Clinical Chemistry Analyzer: https://www.tradeindia.com/products/aspen-star-20-clinical-chemistry-analyzer-c9495036.html
+Semi Automatic Clinical Chemistry Analyzer: https://www.tradeindia.com/products/semi-automatic-clinical-chemistry-analyzer-c515950.html
+Semi Automated Clinical Chemistry Analyzer: https://www.tradeindia.com/products/semi-automated-clinical-chemistry-analyzer-9910184.html
+Immunoassay Analyzer Color Code: White: https://www.tradeindia.com/products/maccura-i-1000-c8490867.html
+Plastic Biochemistry Analyser: https://www.tradeindia.com/products/biochemistry-analyser-c8575716.html
+Plastic Clinical Chemistry Analyser: https://www.tradeindia.com/products/clinical-chemistry-analyser-c8575718.html
+Plastic Cell Counter: https://www.tradeindia.com/products/cell-counter-c8575717.html
+Fully Automated Chemistry Analyzer Chem Ultra Application: Laboratory: https://www.tradeindia.com/products/fully-automated-chemistry-analyzer-chem-ultra-c9495037.html
+Immunoassay Analyser Application: Industrial: https://www.tradeindia.com/products/immunoassay-analyser-c8575719.html
+Coagulation Analyzer Color Code: White: https://www.tradeindia.com/products/mispa-clog-c8490710.html
+Erba Chem 5x Clinical Chemistry Analyzer: https://www.tradeindia.com/products/erba-chem-5x-clinical-chemistry-analyzer-c8379215.html</t>
+        </is>
+      </c>
+      <c r="I55" s="1" t="inlineStr"/>
+      <c r="J55" s="1" t="inlineStr"/>
+      <c r="K55" s="1" t="inlineStr"/>
+      <c r="L55" s="1" t="inlineStr"/>
+      <c r="M55" s="1" t="inlineStr"/>
+      <c r="N55" s="1" t="inlineStr">
+        <is>
+          <t>HEALTH TECH HEALTHCARE , Established in 2016 at Delhi in Delhi, is a leading Supplier,Trading Company,Wholesaler of Medical Equipment in India. HEALTH TECH HEALTHCARE is one of Trade India's verified and trusted sellers of listed products. With extensive experience in supplying and trading Star 20 Clinical Chemistry Analyzer, HEALTH TECH HEALTHCARE has made a reputed name for itself in the market with high-quality 60 ABX Micros Analyzer, AD 3200 Plus Hematology Analyzers, Aspen Star 20 Clinical Chemistry Analyzer, etc. Focusing on a customer-centric approach, HEALTH TECH HEALTHCARE has a pan-India presence and caters to a huge consumer base throughout the country. Buy Medical Equipment in bulk from HEALTH TECH HEALTHCARE at Trade India quality-assured products. Business Type Supplier, Trading Company, Wholesaler Employee Count 10 Establishment 2016 Working Days Monday To Saturday GST NO 07BKMPA3262M1Z0 Payment Mode Online Payments (NEFT/RTGS/IMPS) Related Products Full Automatic Chemistry Analyzer - Application: Commercial MOQ - 1 Unit/Units Weldon Biotech (india) Pvt. Ltd. Delhi, Delhi</t>
+        </is>
+      </c>
+      <c r="O55" s="1" t="inlineStr"/>
+      <c r="P55" s="1" t="inlineStr"/>
+      <c r="Q55" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/star-20-clinical-chemistry-analyzer-c9495038.html</t>
+        </is>
+      </c>
+      <c r="R55" s="1" t="inlineStr"/>
+      <c r="S55" s="1" t="inlineStr"/>
+      <c r="T55" s="1" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="U55" s="1" t="inlineStr"/>
+      <c r="V55" s="1" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr">
+        <is>
+          <t>SQAIQ Clinical Sperm Quality Analyzer</t>
+        </is>
+      </c>
+      <c r="B56" s="1" t="inlineStr">
+        <is>
+          <t>KRISHCO MEDICAL PRODUCTS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="C56" s="1" t="inlineStr">
+        <is>
+          <t>SQAIQ Clinical Sperm Quality Analyzer</t>
+        </is>
+      </c>
+      <c r="D56" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/sqaiq-clinical-sperm-quality-analyzer-c7364690.html</t>
+        </is>
+      </c>
+      <c r="E56" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/07364690/b/4/SQAIQ-Clinical-Sperm-Quality-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F56" s="1" t="inlineStr">
+        <is>
+          <t>Fast analysis, Accurate results, Easy to use, Portable device, Cost effective, Reliable testing Supp</t>
+        </is>
+      </c>
+      <c r="G56" s="1" t="inlineStr"/>
+      <c r="H56" s="1" t="inlineStr">
+        <is>
+          <t>Dyeing Effluent Decolouring Agent: https://www.tradeindia.com/products/dyeing-effluent-decolouring-agent-c3609779.html
+Ayurvedic/Herbal Other Products General Medicines: https://www.tradeindia.com/products/ayurvedic-herbal-other-products-c1882416.html
+Other Products - Homeopathic Supplies | Glass, Plastic, Paper Material, Potency Range 3x-200x, Compliance with Pharmacopeia Standards, Professional Use: https://www.tradeindia.com/products/other-products-6087962.html
+Other Products: https://www.tradeindia.com/products/other-products-c1213927.html
+GCC Powder used in Other Products: https://www.tradeindia.com/products/gcc-powder-used-in-other-products-c373670.html
+PURE GHEE &amp; OTHER PRODUCTS: https://www.tradeindia.com/products/pure-ghee-other-products-c26797.html
+Other Products - Remy Human Hair, Various Lengths, Grey Color | Straight Style, Single Drawn, Curly Option, Intact Cuticle, Available Sizes: https://www.tradeindia.com/products/other-products-c257850.html
+GEAR PARTS,AIR FILTER,OTHER PRODUCT: https://www.tradeindia.com/products/gear-parts-air-filter-other-product-c200932.html
+Ex Wrench &amp; Other Products: https://www.tradeindia.com/products/ex-wrench-other-products-c47355.html
+'O' Rings &amp; other products: https://www.tradeindia.com/products/o-rings-other-products-c31484.html
+Other Products: https://www.tradeindia.com/products/other-products-c318230.html
+Hand Embroidry Jewellery Boxes and Other Products: https://www.tradeindia.com/products/hand-embroidry-jewellery-boxes-and-other-products-c36709.html
+Krishco Sytofix Spray - Medical Grade Plastic, 50ml &amp; 100ml Sizes , White Color for Wound Care and Skin Protection: https://www.tradeindia.com/products/sytofix-spray-c8905285.html
+Sunrise Class 2 Below Knee Stockings - Elasticity: High: https://www.tradeindia.com/products/sunrise-class-2-below-knee-stockings-c8878854.html
+Ellavi Uterine Balloon Tamponade - Grade: Medical: https://www.tradeindia.com/products/ellavi-uterine-balloon-tamponade-c8879412.html
+Ring Pessary: https://www.tradeindia.com/products/ring-pessary-c7364759.html
+Makler Counting Chamber - High-Grade Stainless Steel, Sterilized Design for Accurate Cell Counting and Particle Enumeration: https://www.tradeindia.com/products/makler-counting-chamber-c8843724.html
+Sunrise Class 1 Below Knee Stockings - Elasticity: High: https://www.tradeindia.com/products/sunrise-class-1-below-knee-stockings-c8879181.html
+Sunrise Class 1 Above Knee Stockings - Elasticity: High: https://www.tradeindia.com/products/sunrise-class-1-above-knee-stockings-c8878852.html
+Sytofix Spray - Plastic, 50 ml &amp; 100 ml Bottles | Medical-Grade, Sterilized, Polished Surface Finish, High-Quality Properties: https://www.tradeindia.com/products/sytofix-spray-c8879048.html
+Rosidal K 100% Cotton Bandage: https://www.tradeindia.com/products/rosidal-k-100-cotton-bandage-c7364771.html
+Endometrial Biopsy Curette Grade: Medical Grade: https://www.tradeindia.com/products/plastic-endometrial-biopsy-probet-c8905284.html
+Sperm Processing Kits - Premium Quality Raw Materials, Advanced Technology Driven | Strictly Quality Analyzed, Customer-Centric Design: https://www.tradeindia.com/products/sperm-processing-kits-4229351.html
+Semen Collection: https://www.tradeindia.com/products/semen-collection-c7364628.html
+Sf 14Lf Haemodialysis Dialyzer - Color: White: https://www.tradeindia.com/products/sf-14p-haemodialysis-dialyzer-c7184324.html
+Transparent Dialysis Dialyzer: https://www.tradeindia.com/products/dialysis-dialyzer-c7184319.html
+White Laparoscopic Morcellator: https://www.tradeindia.com/products/laparoscopic-morcellator-c4664095.html
+Medical Ventilator Tube - PVC, Variable Diameter and Length | Oxygen Delivery, Airflow Control, Patient Comfort, Sterile Packaging: https://www.tradeindia.com/products/medical-ventilator-tube-c6649623.html
+Manual Single Use Dialysis Kit: https://www.tradeindia.com/products/single-use-dialysis-kit-c7184321.html
+Disposable Flexible Catheter Mount - Medical Grade Plastic, 10cm x 2cm, Green | Flexible Design, Secure Mounting, Sterile, Disposable: https://www.tradeindia.com/products/disposable-flexible-catheter-mount-c6649626.html
+Oxygen Mask Tubes - PVC 2 Meter, 6mm ID Transparent | Durable, Lightweight, Sterile, Easy to Use: https://www.tradeindia.com/products/oxygen-mask-tubes-c6649625.html
+Monitor NIBP Single Tube Hose Pipe: https://www.tradeindia.com/products/monitor-nibp-single-tube-hose-pipe-c6922902.html
+8 mm Screw Thread Caps And Septa: https://www.tradeindia.com/products/8-mm-screw-thread-caps-septa-c6297012.html</t>
+        </is>
+      </c>
+      <c r="I56" s="1" t="inlineStr">
+        <is>
+          <t>KRISHCO MEDICAL PRODUCTS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="J56" s="1" t="inlineStr"/>
+      <c r="K56" s="1" t="inlineStr"/>
+      <c r="L56" s="1" t="inlineStr">
+        <is>
+          <t>KRISHCO MEDICAL PRODUCTS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="M56" s="1" t="inlineStr">
+        <is>
+          <t>KRISHCO MEDICAL PRODUCTS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="N56" s="1" t="inlineStr">
+        <is>
+          <t>We, Krishco Medical Products Pvt. Ltd., have earned a name for ourselves as an eminent Supplier and Distributor of Pharmaceutical and Medical Products. It is solely due to healthy association with reputed vendors and strong marketing network, we are able to procure high-grade products such as Disposable Gynecology Products, Bed Protectors, Diagnostic Products, Intrauterine Contraceptive Device, Latex Gloves, IUI Disposables,Cancer Screening Products, MTP Kit Products, EVA Gloves, Abdominal Belt, Vacuum Assisted Delivery Systems, IUI Media, supplying them within the stipulated period. All the aforementioned products are in compliance with international quality Business Type Supplier, Trading Company Employee Count 45 Establishment 1997 Working Days Monday To Saturday GST NO 29AAECK4138L1Z6 Payment Mode Days after Acceptance (DA) Related Products Dyeing Effluent Decolouring Agent MOQ - 1000 Kilograms/Kilograms Yixing Bluwat Chemicals Co., Ltd. Yixing, Jiangsu Sheng</t>
+        </is>
+      </c>
+      <c r="O56" s="1" t="inlineStr"/>
+      <c r="P56" s="1" t="inlineStr"/>
+      <c r="Q56" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/krishco-medical-products-pvt-ltd-3014067/</t>
+        </is>
+      </c>
+      <c r="R56" s="1" t="inlineStr"/>
+      <c r="S56" s="1" t="inlineStr"/>
+      <c r="T56" s="1" t="inlineStr">
+        <is>
+          <t>SQAIQ Clinical Sperm Quality Analyzer</t>
+        </is>
+      </c>
+      <c r="U56" s="1" t="inlineStr"/>
+      <c r="V56" s="1" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr">
+        <is>
+          <t>Semi Auto Chemistry Analyzer - Absorbance Range: -0.214~3.000, Lcd Display 240x128 | Accurate Results, User Friendly, Versatile Testing, Peltier Temperature Control at Best Price in Ujjain | Bhargava Bio - Medics</t>
+        </is>
+      </c>
+      <c r="B57" s="1" t="inlineStr"/>
+      <c r="C57" s="1" t="inlineStr">
+        <is>
+          <t>Bhargava Bio - Medics - Offering low price Semi Auto Chemistry Analyzer - Absorbance Range: -0.214~3.000, Lcd Display 240x128 | Accurate Results, User Friendly, Versatile Testing, Peltier Temperature Control in Freeganj, Ujjain with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="D57" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/semi-auto-chemistry-analyzer-c2840515.html</t>
+        </is>
+      </c>
+      <c r="E57" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/02840515/b/4/Semi-auto-Chemistry-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F57" s="1" t="inlineStr">
+        <is>
+          <t>Accurate results, Easy operation, Precise measurements, Reliable performance, Cost effective, Effici</t>
+        </is>
+      </c>
+      <c r="G57" s="1" t="inlineStr"/>
+      <c r="H57" s="1" t="inlineStr">
+        <is>
+          <t>Chemistry Analyzer - Automated, Discrete, Random Access | 330 Tests/Hour, Refrigerated Reagent Compartment, Bi-Directional LIS Interface, 40 Reagent &amp; Sample Positions, 80 Semi-Permanent Cuvettes, Automatic Cleaning &amp; Collision Protection: https://www.tradeindia.com/products/chemistry-analyzer-3578197.html
+Electrolyte Analyzer: https://www.tradeindia.com/products/electrolyte-analyzer-c2840512.html
+Agappe Chemistry Analyzer: https://www.tradeindia.com/products/agappe-chemistry-analyzer-c12360319.html
+Erba Chem 5x Semi Automatic Clinical Chemistry Analyzer: https://www.tradeindia.com/products/erba-chem-5x-semi-automatic-clinical-chemistry-analyzer-8495342.html
+New Generation Clinical Chemistry Analyzer: https://www.tradeindia.com/products/new-generation-clinical-chemistry-analyzer-3619463.html
+Semi Auto Chemistry Analyzer - ABS Plastic, 40x30x20 cm, 10 kg | LCD Screen, Accurate Results, Compact Design, Fast Analysis, User-Friendly Interface: https://www.tradeindia.com/products/semi-auto-chemistry-analyzer-c4258308.html
+Probe Cleaner: https://www.tradeindia.com/products/probe-cleaner-c2840510.html
+Lyzer Reagents: https://www.tradeindia.com/products/lyzer-reagents-c2840509.html
+Quality Check Reagent: https://www.tradeindia.com/products/quality-check-reagent-c3474107.html
+Pathology Equipment: https://www.tradeindia.com/products/pathology-equipment-c2840514.html
+Multi therapy Healthcare System: https://www.tradeindia.com/products/multi-therapy-healthcare-system-c4258286.html
+Cleaner Reagent: https://www.tradeindia.com/products/cleaner-reagent-c2840507.html
+Diluent Reagent: https://www.tradeindia.com/products/diluent-reagent-c2840508.html
+Electrolyte Reagent: https://www.tradeindia.com/products/electrolyte-reagent-c3474108.html
+Ref Electrode Filler: https://www.tradeindia.com/products/ref-electrode-filler-c3474109.html
+Clinical Chemistry Analyzer: https://www.tradeindia.com/products/clinical-chemistry-analyzer-1672714.html
+Fully Auto Chemistry Analyzers: https://www.tradeindia.com/products/fully-auto-chemistry-analyzers-2072815.html
+Semi Auto Chemistry Analyzer - Portable Design, Unmatched Precision &amp; Expert Inspected Performance: https://www.tradeindia.com/products/semi-auto-chemistry-analyzers-2072820.html
+Efficient Semi Auto Chemistry Analyzers: https://www.tradeindia.com/products/efficient-semi-auto-chemistry-analyzers-2072825.html
+Semi Auto Chemistry Analyzer - ABS Plastic, 25x30x40 cm | Accurate Results, Easy Operation, Compact Design, 100 Tests/Hour: https://www.tradeindia.com/products/semi-auto-chemistry-analyzer-3060562.html
+Semi Auto Chemistry Analyzer - 20 Position Incubator, Multiple Temperature Settings (25°C, 30°C, 37°C) | Accurate Results with Differential, Bichromatic, and Immunoturbidimetric Testing: https://www.tradeindia.com/products/semi-auto-chemistry-analyzer-3109012.html
+Fully Automatic Chemistry Analyzer (Bs 480) Application: Clinic: https://www.tradeindia.com/products/fully-automatic-chemistry-analyzer-bs-480-6530621.html
+Semi Auto Chemistry Analyzer (Ba 88A) Application: Clinic: https://www.tradeindia.com/products/semi-auto-chemistry-analyzer-ba-88a-6530623.html
+High Performance Auto Chemistry Analyzer: https://www.tradeindia.com/products/high-performance-auto-chemistry-analyzer-4804548.html
+Neo 4000 Chemistry Analyzer: https://www.tradeindia.com/products/neo-4000-chemistry-analyzer-6469074.html</t>
+        </is>
+      </c>
+      <c r="I57" s="1" t="inlineStr"/>
+      <c r="J57" s="1" t="inlineStr"/>
+      <c r="K57" s="1" t="inlineStr"/>
+      <c r="L57" s="1" t="inlineStr"/>
+      <c r="M57" s="1" t="inlineStr"/>
+      <c r="N57" s="1" t="inlineStr">
+        <is>
+          <t>About Us Based in Madhya Pradesh (India), Bhargava Bio-Medics is a reputed Manufacturer, Supplier, Exporter and Service Provider of medical instruments. Our company was set up in the year 2009 with a mission to be the preferred choice to acquire Electrolyte Analyzer, Laboratory Reagents and similar products in the marketplace. Products we offer to our reputed clients are Biochemistry Analyzer, Cleaner Reagent, Diluent Reagents, Electrolyte Analyzer, Hematology Analyzer, Laboratory Reagents, Lyzer Reagents, Pathology Instruments, Probe Cleaner, etc. We manufacture all these products adhering to the global quality parameters to serve the clients with unmatched quality in all goods. In addition to this, our infrastructure supports us efficiently to fabricate medical equipment with dimensional accuracy. Also, all our products are covered by warranty period which marks our market authenticity. We attain complete client satisfaction by surpassing our performance to keep things balanced. In our endeavor to stand apart from the regular manufacturers in the market, we also provide after sales service to focus on different requirements of our customers. Our technical team provides consultation and give information regarding the product usages. Our customer service comes under our top most priorities to achieve our organizational goals. Business Type Exporter, Manufacturer, Service Provider, Supplier Employee Count 15 Establishment 2009 Working Days Monday To Saturday GST NO 23ATQPB3374D1ZY Payment Mode Cash in Advance (CID) Related Products Chemistry Analyzer - Automated, Discrete, Random Access | 330 Tests/Hour, Refrigerated Reagent Compartment, Bi-Directional LIS Interface, 40 Reagent &amp; Sample Positions, 80 Semi-Permanent Cuvettes, Automatic Cleaning &amp; Collision Protection Bhargava Bio - Medics Ujjain, Madhya Pradesh</t>
+        </is>
+      </c>
+      <c r="O57" s="1" t="inlineStr"/>
+      <c r="P57" s="1" t="inlineStr"/>
+      <c r="Q57" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/semi-auto-chemistry-analyzer-c2840515.html</t>
+        </is>
+      </c>
+      <c r="R57" s="1" t="inlineStr"/>
+      <c r="S57" s="1" t="inlineStr"/>
+      <c r="T57" s="1" t="inlineStr">
+        <is>
+          <t>Bhargava Bio - Medics - Offering low price Semi Auto Chemistry Analyzer - Absorbance Range: -0.214~3.000, Lcd Display 240x128 | Accurate Results, User Friendly, Versatile Testing, Peltier Temperature Control in Freeganj, Ujjain with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="U57" s="1" t="inlineStr"/>
+      <c r="V57" s="1" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Chemistry Analyzer Power Source: Electric</t>
+        </is>
+      </c>
+      <c r="B58" s="1" t="inlineStr">
+        <is>
+          <t>TULJAI LABPOINT PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="C58" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Chemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="D58" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/clinical-chemistry-analyzer-c5784193.html</t>
+        </is>
+      </c>
+      <c r="E58" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/05784193/b/4/Clinical-Chemistry-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F58" s="1" t="inlineStr"/>
+      <c r="G58" s="1" t="inlineStr"/>
+      <c r="H58" s="1" t="inlineStr">
+        <is>
+          <t>Roche Cobas E 411 Analyzer - Electrochemiluminescence (ECL) Immunoassay System, 250 kg Weight | Automated, Random-Access Multichannel Analyzer: https://www.tradeindia.com/products/roche-cobas-e-411-analyzer-c10860580.html
+Rms Analytica 705 Biochemistry Analyser - Color: White: https://www.tradeindia.com/products/rms-analytica-705-biochemistry-analyser-c10260276.html
+Discrete Analyzer: https://www.tradeindia.com/products/discrete-analyzer-c9882604.html
+Plastic Bio-Chemistry Analyser: https://www.tradeindia.com/products/bio-chemistry-analyser-c8650538.html
+Zybio- Exc 200 Fully Auto Biochemistry Analyzer - Accuracy: 1% (Analytical Variation: https://www.tradeindia.com/products/zybio-exc-200-fully-auto-biochemistry-analyzer-c12532199.html
+Mini Vis Chemistry Analyser: https://www.tradeindia.com/products/mini-vis-chemistry-analyser-c6374633.html
+Evolution Semi Automated Clinical Chemistry Analyzer: https://www.tradeindia.com/products/evolution-semi-automated-clinical-chemistry-analyzer-1790220.html
+Agd2160 Clinical Chemistry Analyzer: https://www.tradeindia.com/products/agd2160-clinical-chemistry-analyzer-4239873.html
+Clinical Chemistry Analyzer - Application: Household: https://www.tradeindia.com/products/chemistry-analyser-9525616.html
+Semi Automatic Plastic Clinical Chemistry Analyzer For Hospital Use Color Code: White: https://www.tradeindia.com/products/semi-automatic-plastic-clinical-chemistry-analyzer-for-hospital-use-8444468.html
+Agd 2020 405 Nm Clinical Chemistry Analyzer - Plastic, Portable White, Semi Automatic, Touchscreen Display, Temperature Control, Battery Powered: https://www.tradeindia.com/products/agd-2020-405-nm-clinical-chemistry-analyzer-10294983.html
+Clinical Chemistry Analyzer: https://www.tradeindia.com/products/clinical-chemistry-analyzer-c6487344.html
+CRP Turbilatex Kit: https://www.tradeindia.com/products/crp-turbilatex-kit-c6824069.html
+Automated Extraction Intact Platelets - Quality Tested Material, Portable Design | 1-Year Warranty, Electric Power Source, New Condition: https://www.tradeindia.com/products/automated-prp-ultra-platelet-rich-plasma-c5784194.html
+Video Laryngoscopy: https://www.tradeindia.com/products/video-laryngoscopy-c6036481.html
+LDH Test Kit: https://www.tradeindia.com/products/ldh-test-kit-c6824365.html
+Immunoassay Analyzer: https://www.tradeindia.com/products/immunoassay-analyzer-c6487345.html
+Minicap Flex Piercing Power Source: Electric: https://www.tradeindia.com/products/minicap-flex-piercing-c5784196.html
+Chemiluminescence Immunoassay System Power Source: Electric: https://www.tradeindia.com/products/chemiluminescence-immunoassay-system-c5784202.html
+CRP Test Kit - 50ml Volume, IVD Compliant | Rapid Results, Accurate Test, Easy Usage, Reliable Analysis: https://www.tradeindia.com/products/crp-test-kit-c6824071.html
+Clinical Chemistry Analyzer - Unique Triple Cuvette System | 56 Direct Access Keys, Low Reagent Consumption, Online Display of Reaction Curve, Quality Control Monitoring: https://www.tradeindia.com/products/clinical-chemistry-analyzer-3897482.html
+Fully Automated Clinical Chemistry Analyzer Nanolab 240: https://www.tradeindia.com/products/fully-automated-clinical-chemistry-analyzer-nanolab-240-4018725.html
+Fully Automated Clinical Chemistry Analyzer - High-Precision Manufacturing Using Quality Raw Materials | International Standards Compliance, User-Friendly Interface, Efficient Performance: https://www.tradeindia.com/products/fully-automated-clinical-chemistry-analyzer-4169034.html
+Semi Automated Clinical Chemistry Analyzer - Embedded LCD System, Dual Power Supply | Rapid Test Access, Minimal Maintenance, Extended Lamp Life: https://www.tradeindia.com/products/semi-automated-clinical-chemistry-analyzer-4940915.html
+Optimum Quality Clinical Chemistry Analyzer: https://www.tradeindia.com/products/optimum-quality-clinical-chemistry-analyzer-5209825.html
+Clinical Chemistry Analyzer - 870W x 670D x 625H mm, 120 kg Weight with 5 Speed Stirring and 12 Wavelengths up to 800nm: https://www.tradeindia.com/products/clinical-chemistry-analyzer-5425529.html
+U-Ra Semi Automated Clinical Chemistry Analyzer Application: Hospital: https://www.tradeindia.com/products/u-ra-semi-automated-clinical-chemistry-analyzer-6561623.html
+Agappe Mispa Viva Clinical Chemistry Analyzer: https://www.tradeindia.com/products/agappe-mispa-viva-clinical-chemistry-analyzer-5714859.html
+Erba Chem 5x Semi Automatic Clinical Chemistry Analyzer: https://www.tradeindia.com/products/erba-chem-5x-semi-automatic-clinical-chemistry-analyzer-8495342.html</t>
+        </is>
+      </c>
+      <c r="I58" s="1" t="inlineStr">
+        <is>
+          <t>TULJAI LABPOINT PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="J58" s="1" t="inlineStr"/>
+      <c r="K58" s="1" t="inlineStr"/>
+      <c r="L58" s="1" t="inlineStr">
+        <is>
+          <t>TULJAI LABPOINT PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="M58" s="1" t="inlineStr">
+        <is>
+          <t>TULJAI LABPOINT PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="N58" s="1" t="inlineStr">
+        <is>
+          <t>Tuljai Labpoint Pvt Ltd is established to give services to all class of End Users specially Corporate Industry. Team Tuljai is specialized in Specialty product range. Thalassemia, Sickle Cell, Fertility, Diabetes, Kidney, Liver and Cardiac Markers Business Type Supplier, Trading Company Employee Count 8 Establishment 2017 Working Days Monday To Sunday GST NO 27AAGCT3094A1ZH Payment Mode Cheque Certification NABL and NABH Consultancy Related Products Clinical Chemistry Analyzer Power Source: Electric Price: 1000 INR MOQ - 1 Unit/Units Tuljai Labpoint Private Limited Nagpur, Maharashtra</t>
+        </is>
+      </c>
+      <c r="O58" s="1" t="inlineStr"/>
+      <c r="P58" s="1" t="inlineStr"/>
+      <c r="Q58" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/tuljai-labpoint-private-limited-27267008/</t>
+        </is>
+      </c>
+      <c r="R58" s="1" t="inlineStr"/>
+      <c r="S58" s="1" t="inlineStr"/>
+      <c r="T58" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Chemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="U58" s="1" t="inlineStr"/>
+      <c r="V58" s="1" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Chemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="B59" s="1" t="inlineStr"/>
+      <c r="C59" s="1" t="inlineStr">
+        <is>
+          <t>Buy low price Clinical Chemistry Analyzer in Kukatpally, Hyderabad. Clinical Chemistry Analyzer offered by Invitro Biotech Ltd is available with multiple payment options and easy delivery.</t>
+        </is>
+      </c>
+      <c r="D59" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/clinical-chemistry-analyzer-c2000683.html</t>
+        </is>
+      </c>
+      <c r="E59" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/02000683/b/4/Clinical-Chemistry-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F59" s="1" t="inlineStr">
+        <is>
+          <t>Precise accuracy, Robust design, Easy operation, Reliable results, Cost effective, Fast analysis, Lo</t>
+        </is>
+      </c>
+      <c r="G59" s="1" t="inlineStr"/>
+      <c r="H59" s="1" t="inlineStr">
+        <is>
+          <t>Emp 168 Semi Automatic Chemistry Analyzer Dimension(L*W*H): 420(L) X 310(W) X 152(H) Centimeter (Cm): https://www.tradeindia.com/products/semi-automatic-chemistry-analyzer-c6629826.html
+Clinical Chemistry Analyzer - Semi-Automated System with Touch Screen &amp; Large LCD Display | 7 Filters (340-630nm), Dynamic Temperature Control, 112 Test Profiles Memory: https://www.tradeindia.com/products/clinical-chemistry-analyzer-5813679.html
+Semi Automatic Chemistry Analyzer - High-Quality Manufacturing, Ideal for Laboratories | Advanced Functionality, Suitable for Various Applications, Great Performance in Hyderabad: https://www.tradeindia.com/products/semi-automatic-biochemistry-analyzer-5571420.html
+Clinical Chemistry Analyzer - Plastic Material, 220V Voltage, White Color, 50/60 Hz Frequency | Semi-Automatic Medical Use: https://www.tradeindia.com/products/clinical-chemistry-analyzer-8581804.html
+Semi-Automatic Clinical Chemistry Analyzer - BAS-100, Powerful Data Processing, Built-in Printer, Suction Pump System, Kinetic Testing at 25-30-37Â°C, Measures All Blood Elements: https://www.tradeindia.com/products/semi-automatic-clinical-chemistry-analyzer-747976.html
+Clinical Chemistry Analyzer - Semi-Automatic Flow Cell Model | User-Friendly Microcontroller, 40 Pre-Programmed Assays, Built-in Thermal Printer: https://www.tradeindia.com/products/clinical-chemistry-analyzers-6103155.html
+High Quality BS200 Chemistry Analyzer - Aluminum, 50x70mm, 12V, 2kg | Precise Analysis, Reliable Results, Easy to Use: https://www.tradeindia.com/products/high-quality-bs200-chemistry-analyzer-4694085.html
+Redefine Fully Automatic Chemistry Analyzer: https://www.tradeindia.com/products/redefine-fully-automatic-chemistry-analyzer-6632153.html
+Needle Syringe Destroyer - Steel, 10x5x3 cm | Compact Design, Durable Build, Easy Operation, Infection Control, Safe Disposal: https://www.tradeindia.com/products/needle-syringe-destroyer-c2056139.html
+Mini Photometer: https://www.tradeindia.com/products/mini-photometer-c2000675.html
+Hemoglobin Meter: https://www.tradeindia.com/products/hemoglobin-meter-c2000676.html
+Digital Colorimeter: https://www.tradeindia.com/products/digital-colorimeter-c2000674.html
+Doctor Centrifuges: https://www.tradeindia.com/products/doctor-centrifuges-c2000678.html
+Pipette Stand: https://www.tradeindia.com/products/pipette-stand-c2016175.html
+Sodium EP Color: https://www.tradeindia.com/products/sodium-ep-color-c2000671.html
+Disposable Sample Containers: https://www.tradeindia.com/products/disposable-sample-containers-c2019995.html
+Regular Centrifuge: https://www.tradeindia.com/products/regular-centrifuge-c2000677.html
+OM-240 Auto Bio Chemistry Analyze: https://www.tradeindia.com/products/om-240-auto-bio-chemistry-analyze-c7737368.html
+Abbott UROMETER 120 URINE CHEMISTRY ANALYZER: https://www.tradeindia.com/products/abbott-urometer-120-urine-chemistry-analyzer-c9991917.html</t>
+        </is>
+      </c>
+      <c r="I59" s="1" t="inlineStr"/>
+      <c r="J59" s="1" t="inlineStr"/>
+      <c r="K59" s="1" t="inlineStr"/>
+      <c r="L59" s="1" t="inlineStr"/>
+      <c r="M59" s="1" t="inlineStr"/>
+      <c r="N59" s="1" t="inlineStr">
+        <is>
+          <t>Laboratory Equipment &amp; Reagents - accuracy, precision and reliabilityEstablished in the year 2002, Invitro Biotech Ltd. is a renowned manufacturer, supplier and exporter of a wide array of laboratory products with application in clinical, biotech, research and college laboratories. Laboratories can avail from us microprocessor based Digital Colorimeter, Chemistry Analyzer, Hemoglobin Meter, Single and Multi Channel Micropipettes, various models of regular Lab Centrifuge, Lab Accessories Clinical Chemistry Reagents, and many more. Manufactured as per best industrial practices and norms, our products are known for best quality &amp; standards. Our quality management systems are ISO 9001: 2008 certified and SOPs are laid out for Business Type Exporter, Manufacturer, Supplier Employee Count 20 Establishment 2002 Working Days Monday To Sunday GST NO 36AAACI8264R1ZU Related Products Emp 168 Semi Automatic Chemistry Analyzer Dimension(L*W*H): 420(L) X 310(W) X 152(H) Centimeter (Cm) Vishnu Bio Sciences Hyderabad, Telangana</t>
+        </is>
+      </c>
+      <c r="O59" s="1" t="inlineStr"/>
+      <c r="P59" s="1" t="inlineStr"/>
+      <c r="Q59" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/clinical-chemistry-analyzer-c2000683.html</t>
+        </is>
+      </c>
+      <c r="R59" s="1" t="inlineStr"/>
+      <c r="S59" s="1" t="inlineStr"/>
+      <c r="T59" s="1" t="inlineStr">
+        <is>
+          <t>Buy low price Clinical Chemistry Analyzer in Kukatpally, Hyderabad. Clinical Chemistry Analyzer offered by Invitro Biotech Ltd is available with multiple payment options and easy delivery.</t>
+        </is>
+      </c>
+      <c r="U59" s="1" t="inlineStr"/>
+      <c r="V59" s="1" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="inlineStr">
+        <is>
+          <t>Semi Automatic Clinical Analyzer at Best Price in Delhi | Clindiag India (a Division Of Monash International)</t>
+        </is>
+      </c>
+      <c r="B60" s="1" t="inlineStr"/>
+      <c r="C60" s="1" t="inlineStr">
+        <is>
+          <t>Clindiag India (a Division Of Monash International) - Offering low price Semi Automatic Clinical Analyzer in Mayur Vihar - III, Delhi with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="D60" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/semi-automatic-clinical-analyzer-c478186.html</t>
+        </is>
+      </c>
+      <c r="E60" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/00478186/b/5/Semi-Automatic-Clinical-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F60" s="1" t="inlineStr">
+        <is>
+          <t>Accurate results, Easy operation, Large memory, Cost effective, Precise readings, Quick analysis, Re</t>
+        </is>
+      </c>
+      <c r="G60" s="1" t="inlineStr"/>
+      <c r="H60" s="1" t="inlineStr">
+        <is>
+          <t>Fully Automated Biochemistry Analyzer - Color: White: https://www.tradeindia.com/products/fully-automated-biochemistry-analyzer-c10317328.html
+Clinical Analyzer - Metallic Flow Cell 18Âµl , High Performance Open System with 2000+ Patient Result Memory and Instant Testing Capability: https://www.tradeindia.com/products/clinical-analyzer-325061.html
+H31 Benesphera Hematology Analyzer Application: Industrial: https://www.tradeindia.com/products/h31-benesphera-hematology-analyzer-c8544167.html
+Clinical Chemistry Analyzer - Color: White: https://www.tradeindia.com/products/clinical-chemistry-analyzer-c11771172.html
+Electrolyte Analyzer Erma El-120 ( Agd ) - Color: White: https://www.tradeindia.com/products/electrolyte-analyzer-erma-el-120-agd-c8438396.html
+Hematology Analyzer Application: Laboratory/Hospital/Pharmaceutical Industry: https://www.tradeindia.com/products/hematology-analyzer-c8355968.html
+Labman Bod Analyzer - Accuracy: A 1.0 %: https://www.tradeindia.com/products/labman-bod-analyzer-c11508527.html
+World Class Clinical Analyzer for Quality Laboratories: https://www.tradeindia.com/products/world-class-clinical-analyzer-for-quality-laboratories-325050.html
+Abx Micros 60 Hematology Analyzer Application: Industrial: https://www.tradeindia.com/products/abx-micros-60-hematology-analyzer-c8544165.html
+Semi Automatic Clinical Analyzer Application: Diagnostic Lab: https://www.tradeindia.com/products/semi-automatic-clinical-analyzer-4227341.html
+Biochemistry Analyzer Medical Equipment: https://www.tradeindia.com/products/biochemistry-analyzer-medical-equipment-c3261537.html
+Microplate Reader: https://www.tradeindia.com/products/microplate-reader-c478184.html
+Elisa Microplate Reader: https://www.tradeindia.com/products/elisa-microplate-reader-c515985.html
+Microplate Washers: https://www.tradeindia.com/products/microplate-washers-c556623.html
+Molecular Devices: https://www.tradeindia.com/products/molecular-devices-c515948.html
+Biochemistry Analysers: https://www.tradeindia.com/products/biochemistry-analysers-c3261539.html
+Maccurat Platelet Function Analyzer: https://www.tradeindia.com/products/maccurat-platelet-function-analyzer-c4152983.html
+Medical Biochemistry Analyzer: https://www.tradeindia.com/products/medical-biochemistry-analyzer-c3261535.html
+FA-160: https://www.tradeindia.com/products/fa-160-c3261540.html
+High Accuracy Handheld Portable Asthma Device Sensitive Ultrasonic Pulmonary Function Test Machine: https://www.tradeindia.com/products/high-accuracy-handheld-portable-asthma-device-sensitive-ultrasonic-pulmonary-function-test-machine-7341495.html
+Kanad Semi Auto Clinical Analyser 6FX: https://www.tradeindia.com/products/kanad-semi-auto-clinical-analyser-6fx-c8379206.html</t>
+        </is>
+      </c>
+      <c r="I60" s="1" t="inlineStr"/>
+      <c r="J60" s="1" t="inlineStr"/>
+      <c r="K60" s="1" t="inlineStr"/>
+      <c r="L60" s="1" t="inlineStr"/>
+      <c r="M60" s="1" t="inlineStr"/>
+      <c r="N60" s="1" t="inlineStr">
+        <is>
+          <t>Clindiag is a newly founded company by a group of experienced international specialists, located in Belgium, the heart of Europe. Having the many years of experience of our engineers, Clindiag provides a full range of customer orientated, innovative products to the clinical laboratory world market.By producing high quality products combined with an excellent service to our customers, Clindiag is planning to become an important player in the clinical laboratory market over the next few years... 25792_ 25792_HOME2.jpg Clindiag India a divis Business Type Exporter, Service Provider, Distributor, Supplier, Trading Company Establishment 1998 Working Days Monday To Saturday Related Products Fully Automated Biochemistry Analyzer - Color: White Price: 300000 INR MOQ - 1 Unit/Units Medica Solutions Delhi, Delhi</t>
+        </is>
+      </c>
+      <c r="O60" s="1" t="inlineStr"/>
+      <c r="P60" s="1" t="inlineStr"/>
+      <c r="Q60" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/semi-automatic-clinical-analyzer-c478186.html</t>
+        </is>
+      </c>
+      <c r="R60" s="1" t="inlineStr"/>
+      <c r="S60" s="1" t="inlineStr"/>
+      <c r="T60" s="1" t="inlineStr">
+        <is>
+          <t>Clindiag India (a Division Of Monash International) - Offering low price Semi Automatic Clinical Analyzer in Mayur Vihar - III, Delhi with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="U60" s="1" t="inlineStr"/>
+      <c r="V60" s="1" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Middle Ear Analyzer at Best Price in Bengaluru | Pika Medical (p) Ltd.</t>
+        </is>
+      </c>
+      <c r="B61" s="1" t="inlineStr"/>
+      <c r="C61" s="1" t="inlineStr">
+        <is>
+          <t>Pika Medical (p) Ltd. - Offering low price Clinical Middle Ear Analyzer in M.G. Road, Bengaluru with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="D61" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/clinical-middle-ear-analyzer-c4413153.html</t>
+        </is>
+      </c>
+      <c r="E61" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/04413153/b/8/Clinical-Middle-Ear-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F61" s="1" t="inlineStr">
+        <is>
+          <t>Accurate analysis, Middle ear tests, Easy to use, LED display, Compact design, Rapid cleaning Paymen</t>
+        </is>
+      </c>
+      <c r="G61" s="1" t="inlineStr">
+        <is>
+          <t>Hospital, clinic middle ear testing</t>
+        </is>
+      </c>
+      <c r="H61" s="1" t="inlineStr">
+        <is>
+          <t>Medical Diagnostic Equipments: https://www.tradeindia.com/products/medical-diagnostic-equipments-6042345.html
+Medical Diagnostic Equipments: https://www.tradeindia.com/products/medical-diagnostic-equipments-c315156.html
+Suspension &amp; Diagnostic Item - Metal, Lightweight, Metallic | Portable, Silent Operation, Ideal for Surgical and Diagnostic Procedures: https://www.tradeindia.com/products/suspension-diagnostic-item-c5726378.html
+Diagnostic Ecg Machine - Color: White: https://www.tradeindia.com/products/diagnostic-ecg-c4583149.html
+Medical Diagnostic Equipment: https://www.tradeindia.com/products/medical-diagnostic-equipment-c13255125.html
+Medical Instruments For Medical Applications Use: https://www.tradeindia.com/products/medical-instruments-for-medical-applications-use-8525382.html
+Metal Medical Diagnostic Equipment: https://www.tradeindia.com/products/medical-diagnostic-equipment-5933891.html
+Percussion Hammer - Rubber and Metal, 12 Inches Length, Black Color, 3 Inches Head Diameter, 0.5 lbs Weight, Ideal for Neurological Examination: https://www.tradeindia.com/products/percussion-hammer-c726188.html
+Microlisa HIV: https://www.tradeindia.com/products/microlisa-hiv-c125703.html
+Metal Medical Diagnostic Equipments: https://www.tradeindia.com/products/medical-diagnostic-equipments-5933887.html
+Medical Diagnostic Equipment: https://www.tradeindia.com/products/medical-diagnostic-equipment-c1703253.html
+VIP Compex Machine - Aluminum, 150x50x40cm, 10 Inch Screen | Easy Installation, Low Maintenance, High Efficiency, Body Shaping, Fat Reduction: https://www.tradeindia.com/products/vip-compex-machine-5933888.html
+Clarinet Ear Analyzer: https://www.tradeindia.com/products/clarinet-ear-analyzer-c4475899.html
+Diagnostic Audiometer: https://www.tradeindia.com/products/diagnostic-audiometer-c4413147.html
+Clarinet Tympanometer: https://www.tradeindia.com/products/clarinet-tympanometer-c4475897.html
+Amplitude Integrated Electroencephalography Machine(AEEG): https://www.tradeindia.com/products/amplitude-integrated-electroencephalography-machine-aeeg-c4475892.html
+Inventis Trumpet: https://www.tradeindia.com/products/inventis-trumpet-c4475939.html
+Phototherapy Unit: https://www.tradeindia.com/products/phototherapy-unit-c4475931.html
+Ambulatory EEG: https://www.tradeindia.com/products/ambulatory-eeg-c4413145.html
+PT Unit: https://www.tradeindia.com/products/pt-unit-c4475929.html
+Fetal Monitor - 7" TFT LCD, Dual Waterproof DOP Probes, 450 Hours Trend Data Save, Built-in Thermal Printer | Twin Baby Monitoring, 150 Patients Data Storage, CE &amp; FDA Certified: https://www.tradeindia.com/products/fetal-monitor-c4413136.html
+Karl Storz: https://www.tradeindia.com/products/karl-storz-c4475923.html
+Tissue Stabilizer: https://www.tradeindia.com/products/tissue-stabilizer-8317852.html
+Tissue Stabilizer: https://www.tradeindia.com/products/tissue-stabilizer-8317845.html</t>
+        </is>
+      </c>
+      <c r="I61" s="1" t="inlineStr"/>
+      <c r="J61" s="1" t="inlineStr"/>
+      <c r="K61" s="1" t="inlineStr"/>
+      <c r="L61" s="1" t="inlineStr"/>
+      <c r="M61" s="1" t="inlineStr"/>
+      <c r="N61" s="1" t="inlineStr">
+        <is>
+          <t>Founded in the year of 1994, we, Pika Medical (P) Limited, have established ourselves as a renowned Supplier and Trader of an unmatched array of medical equipment which includes Karl Storz Endoscopic Equipment, Endoscopic Medical Equipment, Inventis Audiometers, Inventi Tympanometers, Emed Electrocautery Unit, Middle Ear Analyzers and more. These are procured from a trusted base of experienced vendors who manufacture these products using licensed components. Our entire range of hospital equipment has an enormous market demand owing to their steady performance, long operational life, portable design, accurate information, low power consumption etc. We have an in-house fully Business Type Distributor, Supplier, Trading Company Employee Count 19 Establishment 1994 Working Days Monday To Sunday GST NO 29AAACP8185A1ZD Related Products Medical Diagnostic Equipments Geneva Industries Ltd. Bengaluru, Karnataka</t>
+        </is>
+      </c>
+      <c r="O61" s="1" t="inlineStr"/>
+      <c r="P61" s="1" t="inlineStr"/>
+      <c r="Q61" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/clinical-middle-ear-analyzer-c4413153.html</t>
+        </is>
+      </c>
+      <c r="R61" s="1" t="inlineStr"/>
+      <c r="S61" s="1" t="inlineStr"/>
+      <c r="T61" s="1" t="inlineStr">
+        <is>
+          <t>Hospital, clinic middle ear testing</t>
+        </is>
+      </c>
+      <c r="U61" s="1" t="inlineStr">
+        <is>
+          <t>Hospital, clinic middle ear testing</t>
+        </is>
+      </c>
+      <c r="V61" s="1" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="inlineStr">
+        <is>
+          <t>Clinical Biochemistry Analyzer at Best Price in New Delhi, Delhi | Radiant Biomed Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="B62" s="1" t="inlineStr"/>
+      <c r="C62" s="1" t="inlineStr">
+        <is>
+          <t>Buy low price Clinical Biochemistry Analyzer in Naraina - I, New Delhi. Clinical Biochemistry Analyzer offered by Radiant Biomed Pvt. Ltd. is available with multiple payment options and easy delivery.</t>
+        </is>
+      </c>
+      <c r="D62" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/clinical-biochemistry-analyzer-c3310429.html</t>
+        </is>
+      </c>
+      <c r="E62" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/03310429/b/4/Clinical-Biochemistry-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F62" s="1" t="inlineStr">
+        <is>
+          <t>Easy install, Precise finishing, Long life, High quality, Accurate results, Quick results, Durable p</t>
+        </is>
+      </c>
+      <c r="G62" s="1" t="inlineStr"/>
+      <c r="H62" s="1" t="inlineStr">
+        <is>
+          <t>Autoquant 400 Supremus Biochemistry Analyzer - Color: Different Available: https://www.tradeindia.com/products/autoquant-400-supremus-biochemistry-analyzer-c9144587.html
+Bs 430 Mindray Clinical Chemistry Analyzer - Attributes: Easy To Operate: https://www.tradeindia.com/products/bs-430-mindray-clinical-chemistry-analyzer-c8458715.html
+Biochemistry Analyzer Application: Laboratory/Hospital/Pharmaceutical Industry: https://www.tradeindia.com/products/biochemistry-analyzer-c8355970.html
+Labman Biochemistry Analyzer - Features: Durable: https://www.tradeindia.com/products/labman-biochemistry-analyzer-c11508492.html
+SEMI BIOCHEMISTRY ANALYZER: https://www.tradeindia.com/products/semi-biochemistry-analyzer-c7947308.html
+Biochemistry Analyzer: https://www.tradeindia.com/products/biochemistry-analyzer-c3303495.html
+Semi Auto Biochemistry Analyzer(Coagulation &amp; Incubator): https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-coagulation-incubator-c3704795.html
+Semi Auto Biochemistry Analyzer - 7.0 Inch True Color Touch Screen, 300 Programmable Tests &amp; 200,000 Result Storage, Auto Sleep &amp; Lamp Protection, Dual Wavelength Absorbance &amp; Coagulation Measurement: https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-1790459.html
+Accukine Biochemistry Analyzer - Color: Black: https://www.tradeindia.com/products/accukine-biochemistry-analyzer-9205582.html
+Os-3000M Semi-Automatic Biochemistry Analyze Touch Screen - Power Source: Electric: https://www.tradeindia.com/products/os-3000m-semi-automatic-biochemistry-analyze-touch-screen-c7737366.html
+Biochemistry Analyzer Dimension(L*W*H): 50X 6 X 6 Inch (In): https://www.tradeindia.com/products/biochemistry-analyzer-4251323.html
+Analyzer Auto Biochemistry Analyzer-Emerald: https://www.tradeindia.com/products/auto-biochemistry-analyzer-emerald-c6779909.html
+Fully Auto Biochemistry Analyzer: https://www.tradeindia.com/products/fully-auto-biochemistry-analyzer-c3310427.html
+Semi Auto Biochemistry Analyzer: https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-c3310426.html
+Laboratory Blood Cell Counter: https://www.tradeindia.com/products/laboratory-blood-cell-counter-c2734753.html
+Hematology Analyzer: https://www.tradeindia.com/products/hematology-analyzer-c2734745.html
+Hematology Blood Analyzers: https://www.tradeindia.com/products/hematology-blood-analyzers-c2734747.html
+Digital Blood Cell Counter: https://www.tradeindia.com/products/digital-blood-cell-counter-c2734755.html
+Fully Automatic Hematology Analyzer: https://www.tradeindia.com/products/fully-automatic-hematology-analyzer-c2734746.html
+Cell Tech Junior: https://www.tradeindia.com/products/cell-tech-junior-c2734752.html
+Semi Automatic Biochemistry Analyzer: https://www.tradeindia.com/products/semi-automatic-biochemistry-analyzer-c3310428.html
+Biochemistry Analyzer: https://www.tradeindia.com/products/biochemistry-analyzer-4482395.html
+Biochemistry Analyzer: https://www.tradeindia.com/products/biochemistry-analyzer-c4729653.html</t>
+        </is>
+      </c>
+      <c r="I62" s="1" t="inlineStr"/>
+      <c r="J62" s="1" t="inlineStr"/>
+      <c r="K62" s="1" t="inlineStr"/>
+      <c r="L62" s="1" t="inlineStr"/>
+      <c r="M62" s="1" t="inlineStr"/>
+      <c r="N62" s="1" t="inlineStr">
+        <is>
+          <t>We prefer inquiries from north India only, like Delhi NCR, Rajasthan, UP, Punjab etc. Established in 2011, we, RADIANT BIOMED PVT. LTD, are a renowned importer, supplier and wholesaler/distributor of Laboratory Equipment such as, Hematology Analyzer, (Blood Cell Counter) and Biochemistry Analyzer. We are offering these products to several hospitals, laboratories and health clinics.All our laboratory equipments are of reputed brands and appreciated for their advanced technology. They are reliable and affordable. They provide accurate results to the doctors and help them to diagnose the patient's disease Business Type Importer, Distributor, Supplier Employee Count 8 Establishment 2011 Working Days Monday To Sunday GST NO 07AAGCR7834J1ZY Related Products Autoquant 400 Supremus Biochemistry Analyzer - Color: Different Available Price: 1060000 INR MOQ - 5 Unit/Units Drx Laboratories India Inc New Delhi, Delhi</t>
+        </is>
+      </c>
+      <c r="O62" s="1" t="inlineStr"/>
+      <c r="P62" s="1" t="inlineStr"/>
+      <c r="Q62" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/clinical-biochemistry-analyzer-c3310429.html</t>
+        </is>
+      </c>
+      <c r="R62" s="1" t="inlineStr"/>
+      <c r="S62" s="1" t="inlineStr"/>
+      <c r="T62" s="1" t="inlineStr">
+        <is>
+          <t>Buy low price Clinical Biochemistry Analyzer in Naraina - I, New Delhi. Clinical Biochemistry Analyzer offered by Radiant Biomed Pvt. Ltd. is available with multiple payment options and easy delivery.</t>
+        </is>
+      </c>
+      <c r="U62" s="1" t="inlineStr"/>
+      <c r="V62" s="1" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="inlineStr">
+        <is>
+          <t>Prietest Touch Prietest Touch Biochemistry Analyzer - ABS Plastic, 380 x 320 x 150mm | LCD Display, AC 100-240V Power Supply, High Accuracy, Long Service Life - Abs Plastic, 380 X 320 X 150mm | Lcd Display, Ac 100-240v Power Supply, High Accuracy, Long Service Life at Best Price in Mumbai | Prana's 4 Ever Diagnostics</t>
+        </is>
+      </c>
+      <c r="B63" s="1" t="inlineStr"/>
+      <c r="C63" s="1" t="inlineStr">
+        <is>
+          <t>Prana's 4 Ever Diagnostics - Offering low price Prietest Touch Prietest Touch Biochemistry Analyzer - ABS Plastic, 380 x 320 x 150mm | LCD Display, AC 100-240V Power Supply, High Accuracy, Long Service Life - Abs Plastic, 380 X 320 X 150mm | Lcd Display, Ac 100-240v Power Supply, High Accuracy, Long Service Life in BORIVALI (E), Mumbai with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="D63" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/biochemistry-analyzer-c4729653.html</t>
+        </is>
+      </c>
+      <c r="E63" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/04729653/b/4/Biochemistry-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F63" s="1" t="inlineStr">
+        <is>
+          <t>Accurate Results, Optimum Performance, High Functionality, Long Service Life Company Details We are</t>
+        </is>
+      </c>
+      <c r="G63" s="1" t="inlineStr"/>
+      <c r="H63" s="1" t="inlineStr">
+        <is>
+          <t>Agappe Mispa Viva: https://www.tradeindia.com/products/agappe-mispa-viva-c9050352.html
+Plastic Bio-Chemistry Analyser: https://www.tradeindia.com/products/bio-chemistry-analyser-c8650538.html
+Zybio- Exc 200 Fully Auto Biochemistry Analyzer - Accuracy: 1% (Analytical Variation: https://www.tradeindia.com/products/zybio-exc-200-fully-auto-biochemistry-analyzer-c12532199.html
+Bio Chemistry Analyzer - Automation Grade: Semi Automatic: https://www.tradeindia.com/products/bio-chemistry-analyzer-c9762330.html
+Semi Auto Biochemistry Analyzer Color Code: Orange And White: https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-c8499679.html
+Fully Automated Biochemistry: https://www.tradeindia.com/products/fully-automated-biochemistry-c3629369.html
+Laboratory Measuring Device - Metal, Plastic, 15x10x20 cm, LCD Digital Display | Precise Viscosity Measurement, Long Lifespan, Easy Operation: https://www.tradeindia.com/products/laboratory-measuring-devices-5991687.html
+Semi Automatic Biochemistry Analyzer - Digital Display, Plastic Material, 240 Volt Power | Easy to Install, Energy Efficient, Ideal for Laboratory Use: https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-9294933.html
+XL 640 Automated Biochemistry Analyzer: https://www.tradeindia.com/products/xl-640-automated-biochemistry-analyzer-5070240.html
+Fully Automated Biochemistry Analyzer - 180 Tests/Hour, 7-Step Onboard Laundry System, Digital Liquid Level Detection, Low Residual Volume Reagent Bottles: https://www.tradeindia.com/products/fully-automated-biochemistry-analyzer-4768031.html
+Semi Automatic Biochemistry Analyzer - Superior Grade Build | Widely Appreciated for Quality and Performance: https://www.tradeindia.com/products/semi-automatic-biochemistry-analyzer-2336810.html
+Automatic Prietest Smart Biochemistry Analyzer: https://www.tradeindia.com/products/automatic-prietest-smart-biochemistry-analyzer-c4729651.html
+Electrolyte Clinical Reagents: https://www.tradeindia.com/products/electrolyte-clinical-reagents-c4729656.html
+Semi Automatic Elisa Plate Reader: https://www.tradeindia.com/products/semi-automatic-elisa-plate-reader-c4729668.html
+Enzymes Reagents: https://www.tradeindia.com/products/enzymes-reagents-c4729658.html
+Plate Incubator Shaker: https://www.tradeindia.com/products/plate-incubator-shaker-c4729663.html
+Prietest Smart Biochemistry Analyzer - Optimal Quality Materials, Advanced Testing Protocols | Versatile Technical Specifications, Lab Certified Performance: https://www.tradeindia.com/products/automatic-biochemistry-analyzer-c4729652.html
+Automatic Coagulation Analyzer - ABS Plastic, 280 x 300 x 150 mm , 5 kg Weight, Color LCD Display, 6 Channels: https://www.tradeindia.com/products/coagulation-analyzer-c4729650.html
+Automatic Microplate Washer - ABS Plastic, 350 x 350 x 250 mm | 1-96 Wells Capacity, 50-1000 µL Dispensing Volume, Versatile Software with 100 Washing Programs: https://www.tradeindia.com/products/automatic-microplate-washer-c4729672.html
+Enhanced Reagents: https://www.tradeindia.com/products/enhanced-reagents-c4729657.html
+Semi Automated Biochemistry Analyzer - Superior Quality Raw Material, Enhanced Accuracy and Reliability: https://www.tradeindia.com/products/semi-automated-biochemistry-analyzer-3936962.html
+Automatic Laboratory Biochemistry Analyzer: https://www.tradeindia.com/products/automatic-laboratory-biochemistry-analyzer-6176976.html
+Fully Automated Biochemistry Analyzer - Electric, ÃÂ± 0.02 O.D Accuracy | Durable, Lightweight Design for Hospital Use: https://www.tradeindia.com/products/fully-automated-biochemistry-analyzer-6884859.html
+Biochemistry Analyzer - Plastic, 40 x 17 x 36.6 cm Dimension | Digital Display, Electric Driven, 220 Volt, 8.5 Kg Weight, Designed for Hospital Use: https://www.tradeindia.com/products/portable-analytica-biochemistry-analyzer-7167044.html
+Biochemistry Analyzer - Plastic, 3 Meter Length, White Color | Touch Screen Display, Multiple Analyte Detection, User-Friendly Design: https://www.tradeindia.com/products/long-durable-strong-high-performance-semi-auto-biochemistry-analyzer-7863216.html
+Biochemistry Analyzer - 340-800Nm Wavelength, 5-10Min Reaction Time, 2-70Ul Sample Volume, 20-350Ul Reagent Volume | Accurate Results, Fast Analysis, Low Maintenance, Reliable System, User Friendly: https://www.tradeindia.com/products/biochemistry-analyzer-c4048252.html
+Biochemistry Analyzer - ABS Plastic, 350 x 300 x 150 mm | LCD Display, 10 kg Weight, 100-240V Power Supply: https://www.tradeindia.com/products/biochemistry-analyzer-c4048251.html
+Microlab 300 Biochemistry Analyzer: https://www.tradeindia.com/products/microlab-300-biochemistry-analyzer-5482147.html
+Biochemistry Analyzer: https://www.tradeindia.com/products/biochemistry-analyzer-c6350610.html</t>
+        </is>
+      </c>
+      <c r="I63" s="1" t="inlineStr"/>
+      <c r="J63" s="1" t="inlineStr"/>
+      <c r="K63" s="1" t="inlineStr"/>
+      <c r="L63" s="1" t="inlineStr"/>
+      <c r="M63" s="1" t="inlineStr"/>
+      <c r="N63" s="1" t="inlineStr">
+        <is>
+          <t>We are the right place for the customer who in looking for and authentic firm for buying the top-class and items like Activated Clotting Time Machine, Elisa Readwell Touch, Prietest Easylab Biochemistry Analyzer, Wash Well Strip etc. Our company named Prana's 4 Ever Diagnostics is a one-stop destinations and a leading supplier, wholesaler and trader of wide array of products. Since our foundation in 2014, we have become one of the favourite choice of the customers and have made a vast client base form various ends of the country. We feel beaming to see that our attempts are being successful, as we are getting positive reviews from our customer in majority. We promise that in future too, we will stay loyal in our business deals and satisfy the needs of the customers. Give us a chance to serve, we Business Type Distributor, Supplier, Trading Company Employee Count 5 Establishment 2014 Working Days Monday To Sunday GST NO 27ALTPS3435P1Z3 Related Products Agappe Mispa Viva Infinity Diagnochem Mumbai, Maharashtra</t>
+        </is>
+      </c>
+      <c r="O63" s="1" t="inlineStr"/>
+      <c r="P63" s="1" t="inlineStr"/>
+      <c r="Q63" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/biochemistry-analyzer-c4729653.html</t>
+        </is>
+      </c>
+      <c r="R63" s="1" t="inlineStr"/>
+      <c r="S63" s="1" t="inlineStr"/>
+      <c r="T63" s="1" t="inlineStr">
+        <is>
+          <t>Prana's 4 Ever Diagnostics - Offering low price Prietest Touch Prietest Touch Biochemistry Analyzer - ABS Plastic, 380 x 320 x 150mm | LCD Display, AC 100-240V Power Supply, High Accuracy, Long Service Life - Abs Plastic, 380 X 320 X 150mm | Lcd Display, Ac 100-240v Power Supply, High Accuracy, Long Service Life in BORIVALI (E), Mumbai with product details &amp; company information.</t>
+        </is>
+      </c>
+      <c r="U63" s="1" t="inlineStr"/>
+      <c r="V63" s="1" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="inlineStr">
+        <is>
+          <t>Chemistry Analyzers at Best Price in Gurugram, Haryana | Accuster Technologies Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="B64" s="1" t="inlineStr"/>
+      <c r="C64" s="1" t="inlineStr">
+        <is>
+          <t>Buy low price Chemistry Analyzers in 47-Sector, Gurugram offered by Accuster Technologies Pvt. Ltd.. Chemistry Analyzers is available with multiple payment options and easy delivery.</t>
+        </is>
+      </c>
+      <c r="D64" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/chemistry-analyzers-c3905784.html</t>
+        </is>
+      </c>
+      <c r="E64" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/03905784/b/4/Chemistry-Analyzers.jpg</t>
+        </is>
+      </c>
+      <c r="F64" s="1" t="inlineStr">
+        <is>
+          <t>Precise readings, Easy operation, Reliable results, Compact design, Cost effective Company Details A
+Bluefic Industrial &amp; Scientific Technologies Ambala, Haryana Send Inquiry Touch Screen Bio Chemistry</t>
+        </is>
+      </c>
+      <c r="G64" s="1" t="inlineStr">
+        <is>
+          <t>Laboratory analysis, quality control, field testing</t>
+        </is>
+      </c>
+      <c r="H64" s="1" t="inlineStr">
+        <is>
+          <t>Semi Auto Chemistry Analyzer - Compact Design, High Throughput Capability, Enhanced Accuracy Features: https://www.tradeindia.com/products/semi-auto-chemistry-analyzer-c7303681.html
+Touch Screen Bio Chemistry Analyzer - Compact Design , Clear Digital Display Screen , User-Friendly Controls: https://www.tradeindia.com/products/touch-screen-bio-chemistry-analyzer-c6965405.html
+Bio Chemistry Analyzer - Absorbency, Mono-Chromatic &amp; Bi-Chromatic Methods | 100-Test Memory, Inbuilt Thermal Printer, 4x20 LCD Display: https://www.tradeindia.com/products/bio-chemistry-analyzer-c2505822.html
+Metal Bio-Chemistry Analyzer: https://www.tradeindia.com/products/bio-chemistry-analyzer-c1736368.html
+Mediray- Semi Auto Biochemistry Analyzer - Material: Plastic: https://www.tradeindia.com/products/mediray-semi-auto-biochemistry-analyzer-c10608461.html
+Bio Chemistry Analyzer - Application: Industrial: https://www.tradeindia.com/products/bio-chemistry-analyzer-c3205326.html
+Bio Chemistry Analyzer - Silver, 33x32x12.5cm | Absorbance Mono and Bi-Chromatic, 100 Test Memory, LCD Display, Thermostat Control 25-37Â°C: https://www.tradeindia.com/products/bio-chemistry-analyzer-c2951949.html
+Bio Chemistry Analyser Machine Weight: 1-10 Kilograms (Kg): https://www.tradeindia.com/products/bio-chemistry-analyser-c4408987.html
+Labcare Export Auto Biochemistry Analyzer: https://www.tradeindia.com/products/labcare-export-auto-biochemistry-analyzer-c6741418.html
+Touch Screen Bio Chemistry Analyzer: https://www.tradeindia.com/products/touch-screen-bio-chemistry-analyzer-c2392934.html
+Auto Chemistry Analyzer: https://www.tradeindia.com/products/auto-chemistry-analyzer-c720401.html
+la bike: https://www.tradeindia.com/products/la-bike-c3905757.html
+Micropipettes: https://www.tradeindia.com/products/micropipettes-c849170.html
+Laboratary Package - Model M004, 220 Volt AC, 100-1000 ÂµL | Temperature Uniformity, Low Temp, Forced Air Circulation, Smart Tip Cone, Ergonomic Design: https://www.tradeindia.com/products/laboratary-package-c1112804.html
+Disposable Mask - Non-Woven Fabric, 17.5x9.5cm, Green | Three-Layer, BFE â¥95%, Elastic Earloop, Adjustable Nose Clip: https://www.tradeindia.com/products/disposable-mask-c3906100.html
+Mobile Lab: https://www.tradeindia.com/products/mobile-lab-c1112784.html
+Accurate-8: https://www.tradeindia.com/products/accurate-8-c810434.html
+Cell Counter (Double Chamber): https://www.tradeindia.com/products/cell-counter-double-chamber-c3905934.html
+Laboratory Centrifuge: https://www.tradeindia.com/products/laboratory-centrifuge-c849168.html
+Benedict's Reagent: https://www.tradeindia.com/products/benedict-s-reagent-c3906059.html
+KANAD 6P Clinical Chemistry Analyzer: https://www.tradeindia.com/products/kanad-6p-clinical-chemistry-analyzer-c6374629.html
+TDS Conductivity Meter with High Accuracy: https://www.tradeindia.com/products/tds-conductivity-meter-with-high-accuracy-7182450.html</t>
+        </is>
+      </c>
+      <c r="I64" s="1" t="inlineStr"/>
+      <c r="J64" s="1" t="inlineStr"/>
+      <c r="K64" s="1" t="inlineStr"/>
+      <c r="L64" s="1" t="inlineStr"/>
+      <c r="M64" s="1" t="inlineStr"/>
+      <c r="N64" s="1" t="inlineStr">
+        <is>
+          <t>ACCUSTER TECHNOLOGIES PVT. LTD. , Established in 2009 at Gurugram in Haryana, is a leading service provider of Laboratory Glassware &amp; Equipment in India. ACCUSTER TECHNOLOGIES PVT. LTD. is one of Trade India's verified and trusted names for listed services. With extensive experience in the field of Laboratory Glassware &amp; Equipment, ACCUSTER TECHNOLOGIES PVT. LTD. has made a reputed name for itself in the market with satisfactory Accurate All, Accurate-8, Autoclave, etc. Focusing on a customer-centric approach, ACCUSTER TECHNOLOGIES PVT. LTD. has a pan-India presence and caters to a huge consumer base throughout the country. Get Laboratory Glassware &amp; Equipment from ACCUSTER TECHNOLOGIES PVT. LTD. at Trade India quality-assured services. Business Type Exporter, Manufacturer, Service Provider, Supplier, Trading Company Employee Count 100 Establishment 2009 Working Days Monday To Sunday GST NO 06AABCU0629H1ZK Related Products Chemistry Analyzers Accuster Technologies Pvt. Ltd. Gurugram, Haryana</t>
+        </is>
+      </c>
+      <c r="O64" s="1" t="inlineStr"/>
+      <c r="P64" s="1" t="inlineStr"/>
+      <c r="Q64" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/chemistry-analyzers-c3905784.html</t>
+        </is>
+      </c>
+      <c r="R64" s="1" t="inlineStr"/>
+      <c r="S64" s="1" t="inlineStr"/>
+      <c r="T64" s="1" t="inlineStr">
+        <is>
+          <t>Laboratory analysis, quality control, field testing</t>
+        </is>
+      </c>
+      <c r="U64" s="1" t="inlineStr">
+        <is>
+          <t>Laboratory analysis, quality control, field testing</t>
+        </is>
+      </c>
+      <c r="V64" s="1" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U30"/>
+  <autoFilter ref="A1:V64"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Extract seller company details from TradeIndia's embedded page data
TradeIndia renders company name, address, and profile text into a
__NEXT_DATA__ JSON blob on each product page instead of visible
labeled text, so the existing extractors found nothing. Parse that
blob as a fallback (only filling fields the existing extraction left
blank) to recover company_name, address, and profile description for
every TradeIndia record, plus manufacturer_name where TradeIndia
labels the seller a manufacturer.

Phone and email remain blank by design: TradeIndia gates phone behind
its "VIEW NUMBER" form and does not publish email on product pages.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tradeindia_products.xlsx
+++ b/tradeindia_products.xlsx
@@ -635,7 +635,11 @@
           <t>https://www.tradeindia.com/kanad-vidyut-5054728/</t>
         </is>
       </c>
-      <c r="R2" s="1" t="inlineStr"/>
+      <c r="R2" s="1" t="inlineStr">
+        <is>
+          <t>B No.6/10, Erandwane, Deenanath Mangeshkar Hospital Road, Pune, Maharashtra, 411004, India</t>
+        </is>
+      </c>
       <c r="S2" s="1" t="inlineStr"/>
       <c r="T2" s="1" t="inlineStr">
         <is>
@@ -728,7 +732,11 @@
           <t>https://www.tradeindia.com/global-biomedicals-inc-8065088/</t>
         </is>
       </c>
-      <c r="R3" s="1" t="inlineStr"/>
+      <c r="R3" s="1" t="inlineStr">
+        <is>
+          <t>D-758, South Part, Jagdamba Nagar-D, Girdharipura Jaipur, Rajasthan, 302021, India</t>
+        </is>
+      </c>
       <c r="S3" s="1" t="inlineStr"/>
       <c r="T3" s="1" t="inlineStr">
         <is>
@@ -833,7 +841,11 @@
           <t>https://www.tradeindia.com/products/bio-chemistry-analyzer-c2505822.html</t>
         </is>
       </c>
-      <c r="R4" s="1" t="inlineStr"/>
+      <c r="R4" s="1" t="inlineStr">
+        <is>
+          <t>Plot No. 73, Vikaspuri, Industrial Area, Ambala Cantt, Haryana, 133001, India</t>
+        </is>
+      </c>
       <c r="S4" s="1" t="inlineStr"/>
       <c r="T4" s="1" t="inlineStr">
         <is>
@@ -846,88 +858,112 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Fully Automated Biochemistry Analyzer</t>
+          <t>Bio-Chemistry Analyzer</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>PATHIMAGE INSTRUMENTS CO.</t>
+          <t>AJANTA EXPORT INDUSTRIES</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>Fully Automated Biochemistry Analyzer</t>
+          <t>Bio-Chemistry Analyzer</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>https://www.tradeindia.com/products/fully-automated-biochemistry-analyzer-c10598070.html</t>
+          <t>https://www.tradeindia.com/products/bio-chemistry-analyzer-c1736368.html</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr">
         <is>
-          <t>https://cpimg.tistatic.com/10598070/b/4/Fully-Automated-Biochemistry-Analyzer..jpg</t>
-        </is>
-      </c>
-      <c r="F5" s="1" t="inlineStr"/>
+          <t>https://cpimg.tistatic.com/01736368/b/4/Bio-Chemistry-Analyzer.jpg</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>Automatic Sample Mixing, Inbuilt Printer, Data Storage Power Supply AC 220V A+- 10%, 50Hz Accuracy C</t>
+        </is>
+      </c>
       <c r="G5" s="1" t="inlineStr">
         <is>
-          <t>Hospital</t>
+          <t>For Hospital and Laboratory Use</t>
         </is>
       </c>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>White Bene Sphera C61 Semi Automatic Biochemistry Analyzer: https://www.tradeindia.com/products/bene-sphera-c61-semi-automatic-biochemistry-analyzer-c7839533.html
-Cst-180 Automatic Biochemistry Analyzer - Accuracy: 100 %: https://www.tradeindia.com/products/cst-180-automatic-biochemistry-analyzer-c11539500.html
-Semi Automatic Biochemistry Analyzer - CE Certified, 220V Voltage, Blue Color | 1 Year Warranty for Clinical Use: https://www.tradeindia.com/products/semi-automatic-biochemistry-analyzer-for-laboratory-and-clinical-use-7576255.html
-Semi Auto Biochemistry Analyzer - Plastic Material, 7-Inch TFT LCD Display, Grey Color | 8 Filters Including 700nm, Dual Mode Operation, Real-Time Reaction Graph, 2,00,000 Result Storage: https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-4856083.html
-Fully Automatic Biochemistry Analyzer - 150 to 300 Tests Per Hour | I.S.E. Module Options Available: https://www.tradeindia.com/products/fully-automatic-biochemistry-analyzer-1205665.html
-Ge Refurbished Ct Scan Machine - Application: Hospital: https://www.tradeindia.com/products/ge-refurbished-ct-scan-machine-c10598268.html
-Mammography X-Ray Machine - Application: Hospital: https://www.tradeindia.com/products/mammography-x-ray-machine-c10598228.html
-300 Ma X-Ray Machine - Color: White: https://www.tradeindia.com/products/300-ma-x-ray-machine-c10598224.html
-Bpl Biphasic Defibrillator - Application: Hospital: https://www.tradeindia.com/products/bpl-biphasic-defibrillator-copy-c10598248.html
-Portable Ultrasound Machine - Application: Hospital: https://www.tradeindia.com/products/portable-ultrasound-machine-c10598044.html
-0.3T Refurbished Hitachi VENTO LT MRI Machine - Open Design, White Color, Automatic Operation, Portable, 22 mT/m Amplitude, Warranty Included: https://www.tradeindia.com/products/0-3t-refurbished-hitachi-vento-lt-mri-machine-c10598168.html
-Hf Series X-Ray Machine - Application: Nursing Home: https://www.tradeindia.com/products/hf-series-x-ray-machine-c10598223.html
-100Ma X Ray Machine Console - Application: Hospital: https://www.tradeindia.com/products/100ma-x-ray-machine-console-c10598243.html
-Laparoscopic Co2 Insufflator - Application: Hospital: https://www.tradeindia.com/products/laparoscopic-co2-insufflator-c10598082.html
-Cd 25 Color Doppler - Attributes: Strong &amp; Durable: https://www.tradeindia.com/products/konica-minolta-cd-25-color-doppler-c10598111.html</t>
+          <t>Medical Microscope - Standard Steel, White Finish | Coarse &amp; Fine Motion Sensitivity 0.002 mm, Mechanical Stage, Abbe Condenser, Dual Eye Pieces: https://www.tradeindia.com/products/medical-microscope-c927191.html
+Newton'S Color Disc: https://www.tradeindia.com/products/newton-s-color-disc-516262.html
+B.O.D. Incubator - Anodized Aluminium &amp; Polished Stainless Steel | Double Wall Design, Removable Perforated Shelves: https://www.tradeindia.com/products/b-o-d-incubator-637751.html
+FLAT BOTTOM FLASK 6000 ML: https://www.tradeindia.com/products/flat-bottom-flask-6000-ml-367631.html
+Optical Bench - High Grade Raw Materials, Durable and Quality Assurance: https://www.tradeindia.com/products/optical-bench-666517.html
+Vacuum Pump - High Grade Materials, Durable &amp; Quality Performance: https://www.tradeindia.com/products/vacuum-pump-666481.html
+Amber Color, Reagent Bottles (Laboratory Glassware Equipment): https://www.tradeindia.com/products/amber-color-reagent-bottles-laboratory-glassware-equipment-c5472389.html
+Laboratory Glassware Equipment: https://www.tradeindia.com/products/laboratory-glassware-equipment-9589715.html
+Laboratory Glassware Equipment: https://www.tradeindia.com/products/laboratory-glassware-equipment-c416087.html
+Laboratory Glassware &amp; Equipment: https://www.tradeindia.com/products/laboratory-glassware-equipment-c605015.html
+Model Earth Quake - Wood Material, 75x100 cms Size | Height 127-254 mm, Weight 1-2 kg, Displays Seismic Waves and Earthquake Effects: https://www.tradeindia.com/products/model-earth-quake-c848319.html
+Stainless Steel Shinnipon Operating Microscope Op-2: https://www.tradeindia.com/products/shinnipon-operating-microscope-op-2-c3670972.html
+Abs Plastic Matronix Digital Auto Lensmeter Slk 5400: https://www.tradeindia.com/products/matronix-digital-auto-lensmeter-slk-5400-c3678055.html
+Stainless Steel Lensometer: https://www.tradeindia.com/products/lensometer-c1440090.html
+Abs Plastic Halogen Headlight: https://www.tradeindia.com/products/halogen-headlight-c1439601.html
+Stainless Steel Slit Lamp: https://www.tradeindia.com/products/slit-lamp-c1440191.html
+Abs Plastic Matronix Lens Edgers: https://www.tradeindia.com/products/matronix-lens-edgers-c3678009.html
+Stainless Steel Matronix Adjustable Trial Frame Imported: https://www.tradeindia.com/products/matronix-adjustable-trial-frame-imported-c3677912.html
+Stainless Steel Matronix Chair Unit Optical Model: https://www.tradeindia.com/products/matronix-chair-unit-optical-model-c3677938.html
+Stainless Steel Welch Alyn Pocketscopetm-Ophthalmoscope: https://www.tradeindia.com/products/welch-alyn-pocketscopetm-ophthalmoscope-c3329139.html
+Touch Screen Bio Chemistry Analyzer - Precision Engineered with Premium Raw Material | Advanced Design, Exceptional Durability, Rigorous Quality Testing: https://www.tradeindia.com/products/touch-screen-bio-chemistry-analyzer-1794313.html
+Bio-Chemistry Analyzer - Premium Quality Materials, Customizable Sizes and Dimensions: https://www.tradeindia.com/products/bio-chemistry-analyzer-1794321.html
+Bio Chemistry Analyser - 85-264V, 10-35Â°C, 20-90% Humidity | Quantitative Clinical Bio-Chemical Analysis, Lamber-Beer Law: https://www.tradeindia.com/products/bio-chemistry-analyser-c4209661.html
+ConXport Bio-Chemistry Analyzer: https://www.tradeindia.com/products/conxport-bio-chemistry-analyzer-c7208608.html
+Aagappe Semi Biio Chemistry Analyzer: https://www.tradeindia.com/products/aagappe-semi-biio-chemistry-analyzer-c5466455.html
+ConXport Touch Screen Bio Chemistry Analyzer - Plastic Stainless Steel, 430x355x340 mm, 7" HD Touch Screen | 100-240V, Photometric Detection, Automatic Sample Loading, Onboard Reagent Cooling, Integrated Incubator, USB LAN RS232 Connectivity: https://www.tradeindia.com/products/conxport-touch-screen-bio-chemistry-analyzer-c7208529.html
+BIO-CHEMISTRY ANALYZER: https://www.tradeindia.com/products/bio-chemistry-analyzer-c2924176.html
+Touch Bio Chemistry Analyzer: https://www.tradeindia.com/products/touch-bio-chemistry-analyzer-c4222428.html
+Erba Semi Bio Chemistry Analyzer: https://www.tradeindia.com/products/erba-semi-bio-chemistry-analyzer-c5466456.html
+Hot Air Oven: https://www.tradeindia.com/products/hot-air-oven-c3853103.html
+Laboratory Conical Flask: https://www.tradeindia.com/products/laboratory-conical-flask-c7045442.html</t>
         </is>
       </c>
       <c r="I5" s="1" t="inlineStr">
         <is>
-          <t>PATHIMAGE INSTRUMENTS CO.</t>
+          <t>AJANTA EXPORT INDUSTRIES</t>
         </is>
       </c>
       <c r="J5" s="1" t="inlineStr"/>
       <c r="K5" s="1" t="inlineStr"/>
       <c r="L5" s="1" t="inlineStr">
         <is>
-          <t>PATHIMAGE INSTRUMENTS CO.</t>
+          <t>AJANTA EXPORT INDUSTRIES</t>
         </is>
       </c>
       <c r="M5" s="1" t="inlineStr">
         <is>
-          <t>PATHIMAGE INSTRUMENTS CO.</t>
+          <t>AJANTA EXPORT INDUSTRIES</t>
         </is>
       </c>
       <c r="N5" s="1" t="inlineStr">
         <is>
-          <t>n this fast pace life, people have completely neglected the care, a body needs to continue working. Toiling hard days and nights for materialistic things results in fatigued body, mind and spirit. A good health is the real secret to an eternal bliss and this understanding is the real reason behind formation of Pathimage Instruments Co. Our business enterprise is formed to make hospitals, clinics, medical research centers and laboratories have an impressive line of Medical Equipment. Business Type Supplier, Trading Company Employee Count 11 Establishment 2008 Working Days Monday To Saturday GST NO 19AAKFP4862D1Z0 Payment Mode Cheque/DD, Online Payments (NEFT/RTGS/IMPS), Cash Related Products White Bene Sphera C61 Semi Automatic Biochemistry Analyzer Price: 80000 INR MOQ - 1 Piece/Pieces Ambay Enterprises Kolkata, West Bengal</t>
+          <t>Established in the year 1957 at Ambala, Haryana (India), we, “Ajanta Export Industries”, are one of the leading manufacturers, exporters &amp; wholesalers of equipment and instruments used in physics, biology and chemistry labs. Besides, we are also meeting the demands of quality laboratory glassware. The complete product range offered by us include biological models, biological charts, dental/ENT equipments, laboratory glassware, laboratory plasticwares, scientific microscopes, physics equipments, physics apparatus, pharmacy instruments, surgical equipments, hospital furnitures, mechanics equipment, soil testing and survey items, generator equipments, muffle furnaces and many more. A Proprietorshi Business Type Exporter, Manufacturer, Distributor, Supplier, Trading Company Employee Count 10 Establishment 1964 Working Days Monday To Sunday GST NO 06DCHPK3570D1ZS Related Products Medical Microscope - Standard Steel, White Finish | Coarse &amp; Fine Motion Sensitivity 0.002 mm, Mechanical Stage, Abbe Condenser, Dual Eye Pieces Price: 2700.0 INR MOQ - 1 Piece/Pieces Standard Steel Ambala Cantt, Haryana</t>
         </is>
       </c>
       <c r="O5" s="1" t="inlineStr"/>
       <c r="P5" s="1" t="inlineStr"/>
       <c r="Q5" s="1" t="inlineStr">
         <is>
-          <t>https://www.tradeindia.com/pathimage-instruments-co-5057644/</t>
-        </is>
-      </c>
-      <c r="R5" s="1" t="inlineStr"/>
+          <t>https://www.tradeindia.com/ajanta-export-industries-4895159/</t>
+        </is>
+      </c>
+      <c r="R5" s="1" t="inlineStr">
+        <is>
+          <t>Building No.-4353, Science Market, Near Geeta Gopal Temple, Ambala Cantt, Haryana, 133001, India</t>
+        </is>
+      </c>
       <c r="S5" s="1" t="inlineStr"/>
       <c r="T5" s="1" t="inlineStr">
         <is>
-          <t>Hospital</t>
+          <t>For Hospital and Laboratory Use</t>
         </is>
       </c>
       <c r="U5" s="1" t="inlineStr"/>
@@ -1014,7 +1050,11 @@
           <t>https://www.tradeindia.com/products/labmate-semi-automated-clinical-chemistry-analyzer-c11934353.html</t>
         </is>
       </c>
-      <c r="R6" s="1" t="inlineStr"/>
+      <c r="R6" s="1" t="inlineStr">
+        <is>
+          <t>A2,A3, Sipcot Industrial Area, Irungattukottai, Chennai, Tamil Nadu, 602117, India</t>
+        </is>
+      </c>
       <c r="S6" s="1" t="inlineStr"/>
       <c r="T6" s="1" t="inlineStr">
         <is>
@@ -1109,7 +1149,11 @@
           <t>https://www.tradeindia.com/raj-biosis-private-limited-5282348/</t>
         </is>
       </c>
-      <c r="R7" s="1" t="inlineStr"/>
+      <c r="R7" s="1" t="inlineStr">
+        <is>
+          <t>F4, First Floor, Plot No. 16, D Block, Satya Colony, Tagore Nagar, On 200 Ft Bypass - Ajmer Delhi, Jaipur, Rajasthan, 302021, India</t>
+        </is>
+      </c>
       <c r="S7" s="1" t="inlineStr"/>
       <c r="T7" s="1" t="inlineStr">
         <is>
@@ -1213,7 +1257,11 @@
           <t>https://www.tradeindia.com/weldon-biotech-india-pvt-ltd-3246874/</t>
         </is>
       </c>
-      <c r="R8" s="1" t="inlineStr"/>
+      <c r="R8" s="1" t="inlineStr">
+        <is>
+          <t>B No - 32-E, 1st Floor, Patparganj, Opp. Una Enclave, Mayur Vihar, Phase-1, Delhi, Delhi, 110091, India</t>
+        </is>
+      </c>
       <c r="S8" s="1" t="inlineStr"/>
       <c r="T8" s="1" t="inlineStr">
         <is>
@@ -1309,7 +1357,11 @@
           <t>https://www.tradeindia.com/microlab-instruments-private-limited-1917606/</t>
         </is>
       </c>
-      <c r="R9" s="1" t="inlineStr"/>
+      <c r="R9" s="1" t="inlineStr">
+        <is>
+          <t>327, Survey No 213, Dantali Industrial Estate, Gota- Vadsar Road, Dantali Ahmedabad, Gujarat, 382721, India</t>
+        </is>
+      </c>
       <c r="S9" s="1" t="inlineStr"/>
       <c r="T9" s="1" t="inlineStr">
         <is>
@@ -1322,36 +1374,130 @@
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
-          <t>Semi-automated Biochemistry Analyzer</t>
+          <t>Fully Automated Biochemistry Analyzer</t>
         </is>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>AISTECH GLOBAL PRIVATE LIMITED</t>
+          <t>PATHIMAGE INSTRUMENTS CO.</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>Semi-automated Biochemistry Analyzer</t>
+          <t>Fully Automated Biochemistry Analyzer</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>https://www.tradeindia.com/products/biochemistry-analyzer-c10543245.html</t>
+          <t>https://www.tradeindia.com/products/fully-automated-biochemistry-analyzer-c10598070.html</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>https://cpimg.tistatic.com/10543245/b/4/Semi-automated-Biochemistry-Analyzer.jpeg</t>
+          <t>https://cpimg.tistatic.com/10598070/b/4/Fully-Automated-Biochemistry-Analyzer..jpg</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr"/>
       <c r="G10" s="1" t="inlineStr">
         <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>White Bene Sphera C61 Semi Automatic Biochemistry Analyzer: https://www.tradeindia.com/products/bene-sphera-c61-semi-automatic-biochemistry-analyzer-c7839533.html
+Cst-180 Automatic Biochemistry Analyzer - Accuracy: 100 %: https://www.tradeindia.com/products/cst-180-automatic-biochemistry-analyzer-c11539500.html
+Semi Automatic Biochemistry Analyzer - CE Certified, 220V Voltage, Blue Color | 1 Year Warranty for Clinical Use: https://www.tradeindia.com/products/semi-automatic-biochemistry-analyzer-for-laboratory-and-clinical-use-7576255.html
+Semi Auto Biochemistry Analyzer - Plastic Material, 7-Inch TFT LCD Display, Grey Color | 8 Filters Including 700nm, Dual Mode Operation, Real-Time Reaction Graph, 2,00,000 Result Storage: https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-4856083.html
+Fully Automatic Biochemistry Analyzer - 150 to 300 Tests Per Hour | I.S.E. Module Options Available: https://www.tradeindia.com/products/fully-automatic-biochemistry-analyzer-1205665.html
+Ge Refurbished Ct Scan Machine - Application: Hospital: https://www.tradeindia.com/products/ge-refurbished-ct-scan-machine-c10598268.html
+Mammography X-Ray Machine - Application: Hospital: https://www.tradeindia.com/products/mammography-x-ray-machine-c10598228.html
+300 Ma X-Ray Machine - Color: White: https://www.tradeindia.com/products/300-ma-x-ray-machine-c10598224.html
+Bpl Biphasic Defibrillator - Application: Hospital: https://www.tradeindia.com/products/bpl-biphasic-defibrillator-copy-c10598248.html
+Portable Ultrasound Machine - Application: Hospital: https://www.tradeindia.com/products/portable-ultrasound-machine-c10598044.html
+0.3T Refurbished Hitachi VENTO LT MRI Machine - Open Design, White Color, Automatic Operation, Portable, 22 mT/m Amplitude, Warranty Included: https://www.tradeindia.com/products/0-3t-refurbished-hitachi-vento-lt-mri-machine-c10598168.html
+Hf Series X-Ray Machine - Application: Nursing Home: https://www.tradeindia.com/products/hf-series-x-ray-machine-c10598223.html
+100Ma X Ray Machine Console - Application: Hospital: https://www.tradeindia.com/products/100ma-x-ray-machine-console-c10598243.html
+Laparoscopic Co2 Insufflator - Application: Hospital: https://www.tradeindia.com/products/laparoscopic-co2-insufflator-c10598082.html
+Cd 25 Color Doppler - Attributes: Strong &amp; Durable: https://www.tradeindia.com/products/konica-minolta-cd-25-color-doppler-c10598111.html</t>
+        </is>
+      </c>
+      <c r="I10" s="1" t="inlineStr">
+        <is>
+          <t>PATHIMAGE INSTRUMENTS CO.</t>
+        </is>
+      </c>
+      <c r="J10" s="1" t="inlineStr"/>
+      <c r="K10" s="1" t="inlineStr"/>
+      <c r="L10" s="1" t="inlineStr">
+        <is>
+          <t>PATHIMAGE INSTRUMENTS CO.</t>
+        </is>
+      </c>
+      <c r="M10" s="1" t="inlineStr">
+        <is>
+          <t>PATHIMAGE INSTRUMENTS CO.</t>
+        </is>
+      </c>
+      <c r="N10" s="1" t="inlineStr">
+        <is>
+          <t>n this fast pace life, people have completely neglected the care, a body needs to continue working. Toiling hard days and nights for materialistic things results in fatigued body, mind and spirit. A good health is the real secret to an eternal bliss and this understanding is the real reason behind formation of Pathimage Instruments Co. Our business enterprise is formed to make hospitals, clinics, medical research centers and laboratories have an impressive line of Medical Equipment. Business Type Supplier, Trading Company Employee Count 11 Establishment 2008 Working Days Monday To Saturday GST NO 19AAKFP4862D1Z0 Payment Mode Cheque/DD, Online Payments (NEFT/RTGS/IMPS), Cash Related Products White Bene Sphera C61 Semi Automatic Biochemistry Analyzer Price: 80000 INR MOQ - 1 Piece/Pieces Ambay Enterprises Kolkata, West Bengal</t>
+        </is>
+      </c>
+      <c r="O10" s="1" t="inlineStr"/>
+      <c r="P10" s="1" t="inlineStr"/>
+      <c r="Q10" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/pathimage-instruments-co-5057644/</t>
+        </is>
+      </c>
+      <c r="R10" s="1" t="inlineStr">
+        <is>
+          <t>No. - 105/12, Dum Dum Road, Shil Bagan, Kolkata, West Bengal, 700074, India</t>
+        </is>
+      </c>
+      <c r="S10" s="1" t="inlineStr"/>
+      <c r="T10" s="1" t="inlineStr">
+        <is>
+          <t>Hospital</t>
+        </is>
+      </c>
+      <c r="U10" s="1" t="inlineStr"/>
+      <c r="V10" s="1" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Semi-automated Biochemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>AISTECH GLOBAL PRIVATE LIMITED</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>Semi-automated Biochemistry Analyzer</t>
+        </is>
+      </c>
+      <c r="D11" s="1" t="inlineStr">
+        <is>
+          <t>https://www.tradeindia.com/products/biochemistry-analyzer-c10543245.html</t>
+        </is>
+      </c>
+      <c r="E11" s="1" t="inlineStr">
+        <is>
+          <t>https://cpimg.tistatic.com/10543245/b/4/Semi-automated-Biochemistry-Analyzer.jpeg</t>
+        </is>
+      </c>
+      <c r="F11" s="1" t="inlineStr"/>
+      <c r="G11" s="1" t="inlineStr">
+        <is>
           <t>ANLYZER</t>
         </is>
       </c>
-      <c r="H10" s="1" t="inlineStr">
+      <c r="H11" s="1" t="inlineStr">
         <is>
           <t>Semiautomatic HBA1C Abbott Afinion 2 For Laboratory Use: https://www.tradeindia.com/products/auto-biochemistry-analyzer-8968392.html
 Semi Auto Biochemistry Analyzer C61: https://www.tradeindia.com/products/semi-auto-biochemistry-analyzer-c61-8163441.html
@@ -1375,82 +1521,86 @@
 Carbon Nitrogen Analyzer: https://www.tradeindia.com/products/carbon-nitrogen-analyzer-c9908969.html</t>
         </is>
       </c>
-      <c r="I10" s="1" t="inlineStr">
+      <c r="I11" s="1" t="inlineStr">
         <is>
           <t>AISTECH GLOBAL PRIVATE LIMITED</t>
         </is>
       </c>
-      <c r="J10" s="1" t="inlineStr"/>
-      <c r="K10" s="1" t="inlineStr"/>
-      <c r="L10" s="1" t="inlineStr">
+      <c r="J11" s="1" t="inlineStr"/>
+      <c r="K11" s="1" t="inlineStr"/>
+      <c r="L11" s="1" t="inlineStr">
         <is>
           <t>AISTECH GLOBAL PRIVATE LIMITED</t>
         </is>
       </c>
-      <c r="M10" s="1" t="inlineStr">
+      <c r="M11" s="1" t="inlineStr">
         <is>
           <t>AISTECH GLOBAL PRIVATE LIMITED</t>
         </is>
       </c>
-      <c r="N10" s="1" t="inlineStr">
+      <c r="N11" s="1" t="inlineStr">
         <is>
           <t>Aistech Global Private Limited has supportive partners because of which we are able to serve customers in exceptionally well manner. As a supplier and trader, our expertise lies in catering to demand for products like Plastic Big Survey Prism, Bosch Hammer Drill Machine, Langry Rebound Hammer, Wooden Tripod Stand For Total Station, etc. We are happy to state that buyer who have placed their trust on us have received the best and their satisfaction is the key of our prompt success. We do not trust anyone blindly when it comes to quality and thus conduct in-house quality check of products before dispatch. Only after getting assured about the quality of the products, we allow them to leave from our premises. Business Type Distributor, Supplier, Trading Company Employee Count 2 Establishment 2020 Working Days Monday To Sunday GST NO 19AATCA7893D1ZZ Related Products Semiautomatic HBA1C Abbott Afinion 2 For Laboratory Use Price: 190000 INR MOQ - 1 Piece/Pieces Pathimage Instruments Co. Kolkata, West Bengal</t>
         </is>
       </c>
-      <c r="O10" s="1" t="inlineStr"/>
-      <c r="P10" s="1" t="inlineStr"/>
-      <c r="Q10" s="1" t="inlineStr">
+      <c r="O11" s="1" t="inlineStr"/>
+      <c r="P11" s="1" t="inlineStr"/>
+      <c r="Q11" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/aistech-global-private-limited-40038445/</t>
         </is>
       </c>
-      <c r="R10" s="1" t="inlineStr"/>
-      <c r="S10" s="1" t="inlineStr"/>
-      <c r="T10" s="1" t="inlineStr">
+      <c r="R11" s="1" t="inlineStr">
+        <is>
+          <t>313/7, Nabapally, Sector- 4, Salt Lake, Kolkata, West Bengal, 700105, India</t>
+        </is>
+      </c>
+      <c r="S11" s="1" t="inlineStr"/>
+      <c r="T11" s="1" t="inlineStr">
         <is>
           <t>ANLYZER</t>
         </is>
       </c>
-      <c r="U10" s="1" t="inlineStr"/>
-      <c r="V10" s="1" t="inlineStr"/>
+      <c r="U11" s="1" t="inlineStr"/>
+      <c r="V11" s="1" t="inlineStr"/>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>Biochemistry Analyzer</t>
         </is>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>SUNSHINE SCIENTIFIC EQUIPMENTS</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>Biochemistry Analyzer</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/biochemistry-analyzer-c6350610.html</t>
         </is>
       </c>
-      <c r="E11" s="1" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>https://cpimg.tistatic.com/06350610/b/4/Biochemistry-Analyzer.jpg</t>
         </is>
       </c>
-      <c r="F11" s="1" t="inlineStr">
+      <c r="F12" s="1" t="inlineStr">
         <is>
           <t>Precise analysis, Reliable results, Easy operation, Compact design, Cost effective Power Supply Elec</t>
         </is>
       </c>
-      <c r="G11" s="1" t="inlineStr">
+      <c r="G12" s="1" t="inlineStr">
         <is>
           <t>Clinical biochemistry testing in labs and hospitals. Provides quantitative analysis of various blood and serum components.</t>
         </is>
       </c>
-      <c r="H11" s="1" t="inlineStr">
+      <c r="H12" s="1" t="inlineStr">
         <is>
           <t>Full Automatic Chemistry Analyzer - Application: Commercial: https://www.tradeindia.com/products/full-automatic-chemistry-analyzer-c9474134.html
 Meril Autoquant 400 Fully Automatic Biochemistry Analyzer - Attributes: Easy To Operate: https://www.tradeindia.com/products/meril-autoquant-400-fully-automatic-biochemistry-analyzer-c10317325.html
@@ -1483,83 +1633,87 @@
 Microlab 300 Biochemistry Analyzer: https://www.tradeindia.com/products/microlab-300-biochemistry-analyzer-5482147.html</t>
         </is>
       </c>
-      <c r="I11" s="1" t="inlineStr">
+      <c r="I12" s="1" t="inlineStr">
         <is>
           <t>SUNSHINE SCIENTIFIC EQUIPMENTS</t>
         </is>
       </c>
-      <c r="J11" s="1" t="inlineStr"/>
-      <c r="K11" s="1" t="inlineStr"/>
-      <c r="L11" s="1" t="inlineStr">
+      <c r="J12" s="1" t="inlineStr"/>
+      <c r="K12" s="1" t="inlineStr"/>
+      <c r="L12" s="1" t="inlineStr">
         <is>
           <t>SUNSHINE SCIENTIFIC EQUIPMENTS</t>
         </is>
       </c>
-      <c r="M11" s="1" t="inlineStr">
+      <c r="M12" s="1" t="inlineStr">
         <is>
           <t>SUNSHINE SCIENTIFIC EQUIPMENTS</t>
         </is>
       </c>
-      <c r="N11" s="1" t="inlineStr">
+      <c r="N12" s="1" t="inlineStr">
         <is>
           <t>Incepted in the year 2007, Sunshine Scientific Equipments is a reputed firm. We are highly involved Exporter of Dairy Equipment, Laboratory Testing Instruments, Soil Testing Equipments, Bomb Calorimeter, Bitumen &amp; Asphalt Testing, Laboratory Testing Equipment and many more. These products are highly known in the market for their long service life and optimum performance. Our offered assortment is manufactured and designed using quality approved raw material and sophisticated technology in compliance with international quality principles and norms. Business Type Exporter, Manufacturer, Supplier Employee Count 10 Establishment 2007 Working Days Monday To Saturday GST NO 07AFHPN3371D1ZL Payment Mode Telegraphic Transfer (T/T) Certification An ISO : 9001:2015 , CE Certified Related Products Full Automatic Chemistry Analyzer - Application: Commercial MOQ - 1 Unit/Units Weldon Biotech (india) Pvt. Ltd. Delhi, Delhi</t>
         </is>
       </c>
-      <c r="O11" s="1" t="inlineStr"/>
-      <c r="P11" s="1" t="inlineStr"/>
-      <c r="Q11" s="1" t="inlineStr">
+      <c r="O12" s="1" t="inlineStr"/>
+      <c r="P12" s="1" t="inlineStr"/>
+      <c r="Q12" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/sunshine-scientific-equipments-12356009/</t>
         </is>
       </c>
-      <c r="R11" s="1" t="inlineStr"/>
-      <c r="S11" s="1" t="inlineStr"/>
-      <c r="T11" s="1" t="inlineStr">
+      <c r="R12" s="1" t="inlineStr">
+        <is>
+          <t>Office No. 303, Third Floor, D-288-89/10 Wadhwa Complex, Vikas Marg, Laxmi Nagar, Delhi, Delhi, 110092, India</t>
+        </is>
+      </c>
+      <c r="S12" s="1" t="inlineStr"/>
+      <c r="T12" s="1" t="inlineStr">
         <is>
           <t>Clinical biochemistry testing in labs and hospitals. Provides quantitative analysis of various blood and serum components.</t>
         </is>
       </c>
-      <c r="U11" s="1" t="inlineStr">
+      <c r="U12" s="1" t="inlineStr">
         <is>
           <t>Clinical biochemistry testing in labs and hospitals. Provides quantitative analysis of various blood and serum components.</t>
         </is>
       </c>
-      <c r="V11" s="1" t="inlineStr"/>
+      <c r="V12" s="1" t="inlineStr"/>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>Clinical Middle Ear Analyzer at Best Price in Ambala Cantt | Contemporary Export Industry</t>
         </is>
       </c>
-      <c r="B12" s="1" t="inlineStr"/>
-      <c r="C12" s="1" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr"/>
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>Contemporary Export Industry - Offering low price Clinical Middle Ear Analyzer in Science Market, Ambala Cantt with product details &amp; company information.</t>
         </is>
       </c>
-      <c r="D12" s="1" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/conxport-clinical-middle-ear-analyzer-r-36-m-c7243895.html</t>
         </is>
       </c>
-      <c r="E12" s="1" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>https://cpimg.tistatic.com/07243895/b/4/Clinical-Middle-Ear-Analyzer.jpg</t>
         </is>
       </c>
-      <c r="F12" s="1" t="inlineStr">
+      <c r="F13" s="1" t="inlineStr">
         <is>
           <t>Automatic and manual mode, data storage, user-friendly interface Type Other, Clinical Middle Ear Ana
 Clinical Middle Ear Analyzer R 36 M Manufactured By Conxport Company Details We, Contemporary Export</t>
         </is>
       </c>
-      <c r="G12" s="1" t="inlineStr">
+      <c r="G13" s="1" t="inlineStr">
         <is>
           <t>Clinical diagnosis and measurement of middle ear conditions</t>
         </is>
       </c>
-      <c r="H12" s="1" t="inlineStr">
+      <c r="H13" s="1" t="inlineStr">
         <is>
           <t>ConXport Bio-Chemistry Analyzer: https://www.tradeindia.com/products/conxport-bio-chemistry-analyzer-c7208608.html
 Bio Chemistry Analyzer - Silver, 33x32x12.5cm | Absorbance Mono and Bi-Chromatic, 100 Test Memory, LCD Display, Thermostat Control 25-37Â°C: https://www.tradeindia.com/products/bio-chemistry-analyzer-c2951949.html
@@ -1594,70 +1748,74 @@
 Thermo Scientific Sorvall St 16 Benchtop Lab Centrifuge: https://www.tradeindia.com/products/thermo-scientific-sorvall-st-16-benchtop-lab-centrifuge-c10859546.html</t>
         </is>
       </c>
-      <c r="I12" s="1" t="inlineStr">
+      <c r="I13" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="J12" s="1" t="inlineStr"/>
-      <c r="K12" s="1" t="inlineStr"/>
-      <c r="L12" s="1" t="inlineStr">
+      <c r="J13" s="1" t="inlineStr"/>
+      <c r="K13" s="1" t="inlineStr"/>
+      <c r="L13" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="M12" s="1" t="inlineStr">
+      <c r="M13" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="N12" s="1" t="inlineStr">
+      <c r="N13" s="1" t="inlineStr">
         <is>
           <t>We, Contemporary Export Industry are a company that values customers. Everyday, we work hard under the leadership of Mr. Akhil Trehan, to offer the best to clients. We design and customize a fine assortment of Single Person Grossing Workstations, Advance Rotary Microtomes, Disintegration Test Apparatus Tablets, Projectors, etc. Quality of our offered items exceeds the expectations of clients, without any interruption. The gamut is renowned for not just its unrivaled quality but also its seamless finish and durability. One can order our phenomenal collection in bulk, while just paying a small sum of money. Our prestigious enterprise is registered with Ministry of Consumer Affairs, Business Type Exporter, Manufacturer, Supplier, Trading Company Employee Count 8 Establishment 2012 Working Days Monday To Sunday GST NO 06AJMPT4011D1ZG Certification ISO 9001-2008 Related Products ConXport Bio-Chemistry Analyzer Contemporary Export Industry Ambala Cantt, Haryana</t>
         </is>
       </c>
-      <c r="O12" s="1" t="inlineStr"/>
-      <c r="P12" s="1" t="inlineStr"/>
-      <c r="Q12" s="1" t="inlineStr">
+      <c r="O13" s="1" t="inlineStr"/>
+      <c r="P13" s="1" t="inlineStr"/>
+      <c r="Q13" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/conxport-clinical-middle-ear-analyzer-r-36-m-c7243895.html</t>
         </is>
       </c>
-      <c r="R12" s="1" t="inlineStr"/>
-      <c r="S12" s="1" t="inlineStr"/>
-      <c r="T12" s="1" t="inlineStr">
+      <c r="R13" s="1" t="inlineStr">
+        <is>
+          <t>B No. 4353, Main Road, Near Geeta Gopal Temple, Ambala Cantt, Haryana, 133001, India</t>
+        </is>
+      </c>
+      <c r="S13" s="1" t="inlineStr"/>
+      <c r="T13" s="1" t="inlineStr">
         <is>
           <t>Clinical diagnosis and measurement of middle ear conditions</t>
         </is>
       </c>
-      <c r="U12" s="1" t="inlineStr"/>
-      <c r="V12" s="1" t="inlineStr"/>
+      <c r="U13" s="1" t="inlineStr"/>
+      <c r="V13" s="1" t="inlineStr"/>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
         <is>
           <t>Uriscan Pro Urine Chemistry Analyzer - Color: Different Availabe - Color: Different Availabe at Best Price in Mathura | Biosolution Technologies</t>
         </is>
       </c>
-      <c r="B13" s="1" t="inlineStr"/>
-      <c r="C13" s="1" t="inlineStr">
+      <c r="B14" s="1" t="inlineStr"/>
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>Biosolution Technologies - Offering low price Uriscan Pro Urine Chemistry Analyzer - Color: Different Availabe - Color: Different Availabe in Chandra Puri, Mathura with product details &amp; company information.</t>
         </is>
       </c>
-      <c r="D13" s="1" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/uriscan-pro-urine-chemistry-analyzer-c10651715.html</t>
         </is>
       </c>
-      <c r="E13" s="1" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>https://cpimg.tistatic.com/10651715/b/4/Uriscan-Pro-Urine-Chemistry-Analyzer..jpg</t>
         </is>
       </c>
-      <c r="F13" s="1" t="inlineStr"/>
-      <c r="G13" s="1" t="inlineStr"/>
-      <c r="H13" s="1" t="inlineStr">
+      <c r="F14" s="1" t="inlineStr"/>
+      <c r="G14" s="1" t="inlineStr"/>
+      <c r="H14" s="1" t="inlineStr">
         <is>
           <t>Uriscan Super Urine Chemistry Analyzer - Color: Different Availabe: https://www.tradeindia.com/products/uriscan-super-urine-chemistry-analyzer-c10651716.html
 Urine Analyzer ( Bi-400) - Color: White: https://www.tradeindia.com/products/urine-analyzer-bi-400-c8781154.html
@@ -1681,78 +1839,82 @@
 Accurex ACR Albumin Creatinine Ratio Urine Analyzer: https://www.tradeindia.com/products/accurex-acr-albumin-creatinine-ratio-urine-analyzer-7968045.html</t>
         </is>
       </c>
-      <c r="I13" s="1" t="inlineStr">
+      <c r="I14" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="J13" s="1" t="inlineStr"/>
-      <c r="K13" s="1" t="inlineStr"/>
-      <c r="L13" s="1" t="inlineStr">
+      <c r="J14" s="1" t="inlineStr"/>
+      <c r="K14" s="1" t="inlineStr"/>
+      <c r="L14" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="M13" s="1" t="inlineStr">
+      <c r="M14" s="1" t="inlineStr">
         <is>
           <t>Trusted Seller</t>
         </is>
       </c>
-      <c r="N13" s="1" t="inlineStr">
+      <c r="N14" s="1" t="inlineStr">
         <is>
           <t>Biosolution Technologies, established in 2024, is a trusted trader and supplier based in Mathura, Uttar Pradesh, India. We specialize in providing cutting-edge medical diagnostic equipment, including Semi Automatic Biochemistry Analyzer, Hemoglobin Analyzer, Medonic Hematology Analyzer, ESR Analyzer and Hemoglobin Testing Meter. With a focus on quality, innovation, and reliability, we aim to serve the healthcare sector with advanced diagnostic solutions to improve patient outcomes.We recognize that medicadiagnostics evolve rapidly, and we are dedicated to staying ahead of the curve. By incorporating the latest technological advancements, we provide equipment that guarantees precision and reliability. Our focus on constant innovation ensures that our clients always have access to the best tools to meet their di Business Type Supplier, Trading Company Employee Count 2 Establishment 2024 Working Days Monday To Sunday GST NO 09BNFPK4044M1ZP Payment Mode Online Payments (NEFT/RTGS/IMPS), Cheque/DD Related Products Uriscan Pro Urine Chemistry Analyzer - Color: Different Availabe MOQ - 1 Unit/Units Biosolution Technologies Mathura, Uttar Pradesh</t>
         </is>
       </c>
-      <c r="O13" s="1" t="inlineStr"/>
-      <c r="P13" s="1" t="inlineStr"/>
-      <c r="Q13" s="1" t="inlineStr">
+      <c r="O14" s="1" t="inlineStr"/>
+      <c r="P14" s="1" t="inlineStr"/>
+      <c r="Q14" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/uriscan-pro-urine-chemistry-analyzer-c10651715.html</t>
         </is>
       </c>
-      <c r="R13" s="1" t="inlineStr"/>
-      <c r="S13" s="1" t="inlineStr"/>
-      <c r="T13" s="1" t="inlineStr">
+      <c r="R14" s="1" t="inlineStr">
+        <is>
+          <t>B No C-39, Chandra Puri, Mathura, Uttar Pradesh, 281001, India</t>
+        </is>
+      </c>
+      <c r="S14" s="1" t="inlineStr"/>
+      <c r="T14" s="1" t="inlineStr">
         <is>
           <t>Biosolution Technologies - Offering low price Uriscan Pro Urine Chemistry Analyzer - Color: Different Availabe - Color: Different Availabe in Chandra Puri, Mathura with product details &amp; company information.</t>
         </is>
       </c>
-      <c r="U13" s="1" t="inlineStr"/>
-      <c r="V13" s="1" t="inlineStr"/>
+      <c r="U14" s="1" t="inlineStr"/>
+      <c r="V14" s="1" t="inlineStr"/>
     </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>Human Humastar 600 Automated Clinical Chemistry Analyzer - Dimension (L*w*h): 1000*740*1130 Mm</t>
         </is>
       </c>
-      <c r="B14" s="1" t="inlineStr">
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>INORBVICT HEALTHCARE INDIA PVT. LTD.</t>
         </is>
       </c>
-      <c r="C14" s="1" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>Human Humastar 600 Automated Clinical Chemistry Analyzer</t>
         </is>
       </c>
-      <c r="D14" s="1" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/human-humastar-600-automated-clinical-chemistry-analyzer-c10877025.html</t>
         </is>
       </c>
-      <c r="E14" s="1" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>https://cpimg.tistatic.com/10877025/b/4/Human-Humastar-600-Automated-Clinical-Chemistry-Analyzer.png</t>
         </is>
       </c>
-      <c r="F14" s="1" t="inlineStr"/>
-      <c r="G14" s="1" t="inlineStr">
+      <c r="F15" s="1" t="inlineStr"/>
+      <c r="G15" s="1" t="inlineStr">
         <is>
           <t>Routine clinical chemistry testing in medium to high-throughput laboratories</t>
         </is>
       </c>
-      <c r="H14" s="1" t="inlineStr">
+      <c r="H15" s="1" t="inlineStr">
         <is>
           <t>Portable Biogas Analyzer - Accuracy: 2 %: https://www.tradeindia.com/products/portable-biogas-analyzer-c3391801.html
 Circuit Breaker Operational Analyzer - Automation Grade: Automatic: https://www.tradeindia.com/products/circuit-breaker-operational-analyzer-c11224952.html
@@ -1772,78 +1934,82 @@
 Biochemistry Analyzer Fully Automatic For Laboratory Use: https://www.tradeindia.com/products/biochemistry-analyzer-fully-automatic-for-laboratory-use-c10877154.html</t>
         </is>
       </c>
-      <c r="I14" s="1" t="inlineStr">
+      <c r="I15" s="1" t="inlineStr">
         <is>
           <t>INORBVICT HEALTHCARE INDIA PVT. LTD.</t>
         </is>
       </c>
-      <c r="J14" s="1" t="inlineStr"/>
-      <c r="K14" s="1" t="inlineStr"/>
-      <c r="L14" s="1" t="inlineStr">
+      <c r="J15" s="1" t="inlineStr"/>
+      <c r="K15" s="1" t="inlineStr"/>
+      <c r="L15" s="1" t="inlineStr">
         <is>
           <t>INORBVICT HEALTHCARE INDIA PVT. LTD.</t>
         </is>
       </c>
-      <c r="M14" s="1" t="inlineStr">
+      <c r="M15" s="1" t="inlineStr">
         <is>
           <t>INORBVICT HEALTHCARE INDIA PVT. LTD.</t>
         </is>
       </c>
-      <c r="N14" s="1" t="inlineStr">
+      <c r="N15" s="1" t="inlineStr">
         <is>
           <t>At Inorbvict Healthcare India Pvt. Ltd. , we are passionate about delivering quality healthcare solutions to the world. As a dedicated exporter, we work closely with healthcare providers, hospitals, and institutions across the globe to supply reliable, advanced medical equipment that supports better patient care. We offer a wide range of products including Dental &amp; ENT equipment, OT &amp; ICU setups, Endoscopy systems, X-Ray and Ultrasound machines, NICU and Neurology tools, Radiology and Imaging equipment, Blood bank solutions, Dialysis machines, Dermatology and Ophthalmology equipment, Laboratory instruments, Cardiology devices, Respiratory care systems , and Operating Microscopes . What sets us apart is our commitment to quality, trusted brand associations, and a hands-on approach to every clienta s needs. Whether youa re setting up a new facility or expanding your services, wea re here to make global medical sourcing easier, faster, and more reliable. Business Type Exporter, Manufacturer Employee Count 50 Establishment 2014 Working Days Monday To Saturday GST NO 27AADCI6120M1ZH Payment Mode Others Certification ISO 9001:2015 Related Products Portable Biogas Analyzer - Accuracy: 2 % Price: 280000 INR MOQ - 1 Piece/Pieces Hnl Systems Pvt. Ltd. Mumbai, Maharashtra</t>
         </is>
       </c>
-      <c r="O14" s="1" t="inlineStr"/>
-      <c r="P14" s="1" t="inlineStr"/>
-      <c r="Q14" s="1" t="inlineStr">
+      <c r="O15" s="1" t="inlineStr"/>
+      <c r="P15" s="1" t="inlineStr"/>
+      <c r="Q15" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/inorbvict-healthcare-india-pvt-ltd-8372692/</t>
         </is>
       </c>
-      <c r="R14" s="1" t="inlineStr"/>
-      <c r="S14" s="1" t="inlineStr"/>
-      <c r="T14" s="1" t="inlineStr">
+      <c r="R15" s="1" t="inlineStr">
+        <is>
+          <t>Office No.821 , 8 Floor, Solitaire Business Hub, Balewadi High St, Gaon, Baner, Pune, Maharashtra, 411027, India</t>
+        </is>
+      </c>
+      <c r="S15" s="1" t="inlineStr"/>
+      <c r="T15" s="1" t="inlineStr">
         <is>
           <t>Routine clinical chemistry testing in medium to high-throughput laboratories</t>
         </is>
       </c>
-      <c r="U14" s="1" t="inlineStr">
+      <c r="U15" s="1" t="inlineStr">
         <is>
           <t>Routine clinical chemistry testing in medium to high-throughput laboratories</t>
         </is>
       </c>
-      <c r="V14" s="1" t="inlineStr"/>
+      <c r="V15" s="1" t="inlineStr"/>
     </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>Erba Em200 Fully Automated Biochemistry Analyzer</t>
         </is>
       </c>
-      <c r="B15" s="1" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>DIAGNOSOL HEALTHTECH</t>
         </is>
       </c>
-      <c r="C15" s="1" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>Erba Em200 Fully Automated Biochemistry Analyzer</t>
         </is>
       </c>
-      <c r="D15" s="1" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/erba-em200-fully-automated-biochemistry-analyzer-c11140521.html</t>
         </is>
       </c>
-      <c r="E15" s="1" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>https://cpimg.tistatic.com/11140521/b/4/Erba-Em200-Fully-Automated-Biochemistry-Analyzer..jpg</t>
         </is>
       </c>
-      <c r="F15" s="1" t="inlineStr"/>
-      <c r="G15" s="1" t="inlineStr"/>
-      <c r="H15" s="1" t="inlineStr">
+      <c r="F16" s="1" t="inlineStr"/>
+      <c r="G16" s="1" t="inlineStr"/>
+      <c r="H16" s="1" t="inlineStr">
         <is>
           <t>Erba Em Destiny 180 - Fully Automated Biochemistry Analyzer - Automation Grade: Automatic: https://www.tradeindia.com/products/erba-em-destiny-180-fully-automated-biochemistry-analyzer-c11787573.html
 Erba Biochemistry Analyzer Application: Industrial: https://www.tradeindia.com/products/erba-biochemistry-analyzer-c8544174.html
@@ -1865,78 +2031,82 @@
 Clinical Chemistry Analyzer: https://www.tradeindia.com/products/clinical-chemistry-analyzer-c5395097.html</t>
         </is>
       </c>
-      <c r="I15" s="1" t="inlineStr">
+      <c r="I16" s="1" t="inlineStr">
         <is>
           <t>DIAGNOSOL HEALTHTECH</t>
         </is>
       </c>
-      <c r="J15" s="1" t="inlineStr"/>
-      <c r="K15" s="1" t="inlineStr"/>
-      <c r="L15" s="1" t="inlineStr">
+      <c r="J16" s="1" t="inlineStr"/>
+      <c r="K16" s="1" t="inlineStr"/>
+      <c r="L16" s="1" t="inlineStr">
         <is>
           <t>DIAGNOSOL HEALTHTECH</t>
         </is>
       </c>
-      <c r="M15" s="1" t="inlineStr">
+      <c r="M16" s="1" t="inlineStr">
         <is>
           <t>DIAGNOSOL HEALTHTECH</t>
         </is>
       </c>
-      <c r="N15" s="1" t="inlineStr">
+      <c r="N16" s="1" t="inlineStr">
         <is>
           <t>Our company, Diagnosol Healthtech, is a leading supplier, trader, and exporter in the market, known for our wide range of Hematology Analyzer, Immunoassay Analyzer, Biochemistry Analyzer, Emerald Syringe, Hemoglobin Meter, and more. Established in 2016, we are a vibrant, dedicated, and quality driven organization. Since the beginning, we have become stronger than ever, firmly establishing ourselves in both the domestic and international markets. For diagnostic labs, hospitals, medical clinics, and research centers, we provide a full selection of our products. In how we behave ourselves and conduct business, we are open, honest, and courteous. Ordering lines are open 24 hours a day, and deliveries of critical supplies are made continuously. Because we are committed to the clients that choose to work with us, we are always available to provide superior service. Our success is largely a r Business Type Exporter, Supplier, Trading Company, Wholesaler Employee Count 10 Establishment 2018 Working Days Monday To Sunday GST NO 08AASFD7556L1ZL Payment Mode Online Payments (NEFT/RTGS/IMPS), Cheque/DD, Wallet &amp; UPI Related Products Erba Em Destiny 180 - Fully Automated Biochemistry Analyzer - Automation Grade: Automatic Price: 550000 INR MOQ - 1 Unit/Units Global Biomedicals Inc Jaipur, Rajasthan</t>
         </is>
       </c>
-      <c r="O15" s="1" t="inlineStr"/>
-      <c r="P15" s="1" t="inlineStr"/>
-      <c r="Q15" s="1" t="inlineStr">
+      <c r="O16" s="1" t="inlineStr"/>
+      <c r="P16" s="1" t="inlineStr"/>
+      <c r="Q16" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/diagnosol-healthtech-35405475/</t>
         </is>
       </c>
-      <c r="R15" s="1" t="inlineStr"/>
-      <c r="S15" s="1" t="inlineStr"/>
-      <c r="T15" s="1" t="inlineStr">
+      <c r="R16" s="1" t="inlineStr">
+        <is>
+          <t>T-134, Basemate, Ganesh Nagar, Niwaru Road, Jhotwara, Jaipur, Rajasthan, 302012, India</t>
+        </is>
+      </c>
+      <c r="S16" s="1" t="inlineStr"/>
+      <c r="T16" s="1" t="inlineStr">
         <is>
           <t>Erba Em200 Fully Automated Biochemistry Analyzer</t>
         </is>
       </c>
-      <c r="U15" s="1" t="inlineStr"/>
-      <c r="V15" s="1" t="inlineStr"/>
+      <c r="U16" s="1" t="inlineStr"/>
+      <c r="V16" s="1" t="inlineStr"/>
     </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
         <is>
           <t>Huma Star 100 Biochemistry Analyzer</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>AMBAY ENTERPRISES</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>Huma Star 100 Biochemistry Analyzer</t>
         </is>
       </c>
-      <c r="D16" s="1" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>https://www.tradeindia.com/products/huma-star-100-biochemistry-analyzer-c7839529.html</t>
         </is>
       </c>
-      <c r="E16" s="1" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>https://cpimg.tistatic.com/07839529/b/4/Huma-Star-100-Biochemistry-Analyzer.jpg</t>
         </is>
       </c>
-      <c r="F16" s="1" t="inlineStr"/>
-      <c r="G16" s="1" t="inlineStr">
+      <c r="F17" s="1" t="inlineStr"/>
+      <c r="G17" s="1" t="inlineStr">
         <is>
           <t>Diagnostic Equipment</t>
         </is>
       </c>
-      <c r="H16" s="1" t="inlineStr">
+      <c r="H17" s="1" t="inlineStr">
         <is>
           <t>Semiautomatic HBA1C Abbott Afinion 2 For Laboratory Use: https://www.tradeindia.com/products/auto-biochemistry-analyzer-8968392.html
 Semi-Automated Biochemistry Analyzer - Application: Anlyzer: https://www.tradeindia.com/products/biochemistry-analyzer-c10543245.html
@@ -1970,157 +2140,51 @@
 High Performance Automatic Biochemistry Analyzer For Laboratory: https://www.tradeindia.com/products/high-performance-automatic-biochemistry-analyzer-for-laboratory-8579675.html</t>
         </is>
       </c>
-      <c r="I16" s="1" t="inlineStr">
+      <c r="I17" s="1" t="inlineStr">
         <is>
           <t>AMBAY ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="J16" s="1" t="inlineStr"/>
-      <c r="K16" s="1" t="inlineStr"/>
-      <c r="L16" s="1" t="inlineStr">
-        <is>
-          <t>AMBAY ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="M16" s="1" t="inlineStr">
-        <is>
-          <t>AMBAY ENTERPRISES</t>
-        </is>
-      </c>
-      <c r="N16" s="1" t="inlineStr">
-        <is>
-          <t>We are a Distribution based marketing organisation based at Kolkata, West Bengal dealing in IVD products, delivering all over India &amp; abroad. Business Type Exporter, Supplier, Trading Company Employee Count 12 Establishment 2006 Working Days Monday To Saturday GST NO 19AHMPB8675P1ZD Payment Mode Cash Advance (CA) Certification ISO 9001:2005 Related Products Semiautomatic HBA1C Abbott Afinion 2 For Laboratory Use Price: 190000 INR MOQ - 1 Piece/Pieces Pathimage Instruments Co. Kolkata, West Bengal</t>
-        </is>
-      </c>
-      <c r="O16" s="1" t="inlineStr"/>
-      <c r="P16" s="1" t="inlineStr"/>
-      <c r="Q16" s="1" t="inlineStr">
-        <is>
-          <t>https://www.tradeindia.com/ambay-enterprises-23586489/</t>
-        </is>
-      </c>
-      <c r="R16" s="1" t="inlineStr"/>
-      <c r="S16" s="1" t="inlineStr"/>
-      <c r="T16" s="1" t="inlineStr">
-        <is>
-          <t>Diagnostic Equipment</t>
-        </is>
-      </c>
-      <c r="U16" s="1" t="inlineStr">
-        <is>
-          <t>Diagnostic Equipment</t>
-        </is>
-      </c>
-      <c r="V16" s="1" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr">
-        <is>
-          <t>Bio-Chemistry Analyzer</t>
-        </is>
-      </c>
-      <c r="B17" s="1" t="inlineStr">
-        <is>
-          <t>AJANTA EXPORT INDUSTRIES</t>
-        </is>
-      </c>
-      <c r="C17" s="1" t="inlineStr">
-        <is>
-          <t>Bio-Chemistry Analyzer</t>
-        </is>
-      </c>
-      <c r="D17" s="1" t="inlineStr">
-        <is>
-          <t>https://www.tradeindia.com/products/bio-chemistry-analyzer-c1736368.html</t>
-        </is>
-      </c>
-      <c r="E17" s="1" t="inlineStr">
-        <is>
-          <t>https://cpimg.tistatic.com/01736368/b/4/Bio-Chemistry-Analyzer.jpg</t>
-        </is>
-      </c>
-      <c r="F17" s="1" t="inlineStr">
-        <is>
-          <t>Automatic Sample Mixing, Inbuilt Printer, Data Storage Power Supply AC 220V A+- 10%, 50Hz Accuracy C</t>
-        </is>
-      </c>
-      <c r="G17" s="1" t="inlineStr">
-        <is>
-          <t>For Hospital and Laboratory Use</t>
-        </is>
-      </c>
-      <c r="H17" s="1" t="inlineStr">
-        <is>
-          <t>Medical Microscope - Standard Steel, White Finish | Coarse &amp; Fine Motion Sensitivity 0.002 mm, Mechanical Stage, Abbe Condenser, Dual Eye Pieces: https://www.tradeindia.com/products/medical-microscope-c927191.html
-Newton'S Color Disc: https://www.tradeindia.com/products/newton-s-color-disc-516262.html
-B.O.D. Incubator - Anodized Aluminium &amp; Polished Stainless Steel | Double Wall Design, Removable Perforated Shelves: https://www.tradeindia.com/products/b-o-d-incubator-637751.html
-FLAT BOTTOM FLASK 6000 ML: https://www.tradeindia.com/products/flat-bottom-flask-6000-ml-367631.html
-Optical Bench - High Grade Raw Materials, Durable and Quality Assurance: https://www.tradeindia.com/products/optical-bench-666517.html
-Vacuum Pump - High Grade Materials, Durable &amp; Quality Performance: https://www.tradeindia.com/products/vacuum-pump-666481.html
-Amber Color, Reagent Bottles (Laboratory Glassware Equipment): https://www.tradeindia.com/products/amber-color-reagent-bottles-laboratory-glassware-equipment-c5472389.html
-Laboratory Glassware Equipment: https://www.tradeindia.com/products/laboratory-glassware-equipment-9589715.html
-Laboratory Glassware Equipment: https://www.tradeindia.com/products/laboratory-glassware-equipment-c416087.html
-Laboratory Glassware &amp; Equipment: https://www.tradeindia.com/products/laboratory-glassware-equipment-c605015.html
-Model Earth Quake - Wood Material, 75x100 cms Size | Height 127-254 mm, Weight 1-2 kg, Displays Seismic Waves and Earthquake Effects: https://www.tradeindia.com/products/model-earth-quake-c848319.html
-Stainless Steel Shinnipon Operating Microscope Op-2: https://www.tradeindia.com/products/shinnipon-operating-microscope-op-2-c3670972.html
-Abs Plastic Matronix Digital Auto Lensmeter Slk 5400: https://www.tradeindia.com/products/matronix-digital-auto-lensmeter-slk-5400-c3678055.html
-Stainless Steel Lensometer: https://www.tradeindia.com/products/lensometer-c1440090.html
-Abs Plastic Halogen Headlight: https://www.tradeindia.com/products/halogen-headlight-c1439601.html
-Stainless Steel Slit Lamp: https://www.tradeindia.com/products/slit-lamp-c1440191.html
-Abs Plastic Matronix Lens Edgers: https://www.tradeindia.com/products/matronix-lens-edgers-c3678009.html
-Stainless Steel Matronix Adjustable Trial Frame Imported: https://www.tradeindia.com/products/matronix-adjustable-trial-frame-imported-c3677912.html
-Stainless Steel Matronix Chair Unit Optical Model: https://www.tradeindia.com/products/matronix-chair-unit-optical-model-c3677938.html
-Stainless Steel Welch Alyn Pocketscopetm-Ophthalmoscope: https://www.tradeindia.com/products/welch-alyn-pocketscopetm-ophthalmoscope-c3329139.html
-Touch Screen Bio Chemistry Analyzer - Precision Engineered with Premium Raw Material | Advanced Design, Exceptional Durability, Rigorous Quality Testing: https://www.tradeindia.com/products/touch-screen-bio-chemistry-analyzer-1794313.html
-Bio-Chemistry Analyzer - Premium Quality Materials, Customizable Sizes and Dimensions: https://www.tradeindia.com/products/bio-chemistry-analyzer-1794321.html
-Bio Chemistry Analyser - 85-264V, 10-35Â°C, 20-90% Humidity | Quantitative Clinical Bio-Chemical Analysis, Lamber-Beer Law: https://www.tradeindia.com/products/bio-chemistry-analyser-c4209661.html
-ConXport Bio-Chemistry Analyzer: https://www.tradeindia.com/products/conxport-bio-chemistry-analyzer-c7208608.html
-Aagappe Semi Biio Chemistry Analyzer: https://www.tradeindia.com/products/aagappe-semi-biio-chemistry-analyzer-c5466455.html
-ConXport Touch Screen Bio Chemistry Analyzer - Plastic Stainless Steel, 430x355x340 mm, 7" HD Touch Screen | 100-240V, Photometric Detection, Automatic Sample Loading, Onboard Reagent Cooling, Integrated Incubator, USB LAN RS232 Connectivity: https://www.tradeindia.com/products/conxport-touch-screen-bio-chemistry-analyzer-c7208529.html
-BIO-CHEMISTRY ANALYZER: https://www.tradeindia.com/products/bio-chemistry-analyzer-c2924176.html
-Touch Bio Chemistry Analyzer: https://www.tradeindia.com/products/touch-bio-chemistry-analyzer-c4222428.html
-Erba Semi Bio Chemistry Analyzer: https://www.tradeindia.com/products/erba-semi-bio-chemistry-analyzer-c5466456.html
-Hot Air Oven: https://www.tradeindia.com/products/hot-air-oven-c3853103.html
-Laboratory Conical Flask: https://www.tradeindia.com/products/laboratory-conical-flask-c7045442.html</t>
-        </is>
-      </c>
-      <c r="I17" s="1" t="inlineStr">
-        <is>
-          <t>AJANTA EXPORT INDUSTRIES</t>
         </is>
       </c>
       <c r="J17" s="1" t="inlineStr"/>
       <c r="K17" s="1" t="inlineStr"/>
       <c r="L17" s="1" t="inlineStr">
         <is>
-          <t>AJANTA EXPORT INDUSTRIES</t>
+          <t>AMBAY ENTERPRISES</t>
         </is>
       </c>
       <c r="M17" s="1" t="inlineStr">
         <is>
-          <t>AJANTA EXPORT INDUSTRIES</t>
+          <t>AMBAY ENTERPRISES</t>
         </is>
       </c>
       <c r="N17" s="1" t="inlineStr">
         <is>
-          <t>Established in the year 1957 at Ambala, Haryana (India), we, “Ajanta Export Industries”, are one of the leading manufacturers, exporters &amp; wholesalers of equipment and instruments used in physics, biology and chemistry labs. Besides, we are also meeting the demands of quality laboratory glassware. The complete product range offered by us include biological models, biological charts, dental/ENT equipments, laboratory glassware, laboratory plasticwares, scientific microscopes, physics equipments, physics apparatus, pharmacy instruments, surgical equipments, hospital furnitures, mechanics equipment, soil testing and survey items, generator equipments, muffle furnaces and many more. A Proprietorshi Business Type Exporter, Manufacturer, Distributor, Supplier, Trading Company Employee Count 10 Establishment 1964 Working Days Monday To Sunday GST NO 06DCHPK3570D1ZS Related Products Medical Microscope - Standard Steel, White Finish | Coarse &amp; Fine Motion Sensitivity 0.002 mm, Mechanical Stage, Abbe Condenser, Dual Eye Pieces Price: 2700.0 INR MOQ - 1 Piece/Pieces Standard Steel Ambala Cantt, Haryana</t>
+          <t>We are a Distribution based marketing organisation based at Kolkata, West Bengal dealing in IVD products, delivering all over India &amp; abroad. Business Type Exporter, Supplier, Trading Company Employee Count 12 Establishment 2006 Working Days Monday To Saturday GST NO 19AHMPB8675P1ZD Payment Mode Cash Advance (CA) Certification ISO 9001:2005 Related Products Semiautomatic HBA1C Abbott Afinion 2 For Laboratory Use Price: 190000 INR MOQ - 1 Piece/Pieces Pathimage Instruments Co. Kolkata, West Bengal</t>
         </is>
       </c>
       <c r="O17" s="1" t="inlineStr"/>
       <c r="P17" s="1" t="inlineStr"/>
       <c r="Q17" s="1" t="inlineStr">
         <is>
-          <t>https://www.tradeindia.com/ajanta-export-industries-4895159/</t>
-        </is>
-      </c>
-      <c r="R17" s="1" t="inlineStr"/>
+          <t>https://www.tradeindia.com/ambay-enterprises-23586489/</t>
+        </is>
+      </c>
+      <c r="R17" s="1" t="inlineStr">
+        <is>
+          <t>No. 89, Netaji Subhas Road, 2nd Floor, Room No. 13, Kolkata, West Bengal, 700001, India</t>
+        </is>
+      </c>
       <c r="S17" s="1" t="inlineStr"/>
       <c r="T17" s="1" t="inlineStr">
         <is>
-          <t>For Hospital and Laboratory Use</t>
-        </is>
-      </c>
-      <c r="U17" s="1" t="inlineStr"/>
+          <t>Diagnostic Equipment</t>
+        </is>
+      </c>
+      <c r="U17" s="1" t="inlineStr">
+        <is>
+          <t>Diagnostic Equipment</t>
+        </is>
+      </c>
       <c r="V17" s="1" t="inlineStr"/>
     </row>
     <row r="18">
@@ -2207,7 +2271,11 @@
           <t>https://www.tradeindia.com/labman-scientific-instruments-pvt-ltd-81508453/</t>
         </is>
       </c>
-      <c r="R18" s="1" t="inlineStr"/>
+      <c r="R18" s="1" t="inlineStr">
+        <is>
+          <t>No 2, Abirami Avenue, 12th Street, Kodungaiyur, Kkd Nagar, Chennai, Tamil Nadu, 600118, India</t>
+        </is>
+      </c>
       <c r="S18" s="1" t="inlineStr"/>
       <c r="T18" s="1" t="inlineStr">
         <is>
@@ -2294,7 +2362,11 @@
           <t>https://www.tradeindia.com/mediray-healthcare-1528634/</t>
         </is>
       </c>
-      <c r="R19" s="1" t="inlineStr"/>
+      <c r="R19" s="1" t="inlineStr">
+        <is>
+          <t>Mediray Healthcare, Link Roan Near Car Market, Faridabad, Haryana, 121008, India</t>
+        </is>
+      </c>
       <c r="S19" s="1" t="inlineStr"/>
       <c r="T19" s="1" t="inlineStr">
         <is>
@@ -2383,7 +2455,11 @@
           <t>https://www.tradeindia.com/products/clover-a1c-hba1c-analyzer-c8467399.html</t>
         </is>
       </c>
-      <c r="R20" s="1" t="inlineStr"/>
+      <c r="R20" s="1" t="inlineStr">
+        <is>
+          <t>Corporate Office: - 412, Suncity Trade Tower, Sector 21, Gurugram, Haryana 122016 Gurugram, Haryana, 122016, India</t>
+        </is>
+      </c>
       <c r="S20" s="1" t="inlineStr"/>
       <c r="T20" s="1" t="inlineStr">
         <is>
@@ -2478,7 +2554,11 @@
           <t>https://www.tradeindia.com/labchrom-scientific-llp-7424735/</t>
         </is>
       </c>
-      <c r="R21" s="1" t="inlineStr"/>
+      <c r="R21" s="1" t="inlineStr">
+        <is>
+          <t>Office No. 253, 2nd Floor, Udyog Bhavan, Sonawala Road, Goregaon East, Mumbai, Maharashtra, 400063, India</t>
+        </is>
+      </c>
       <c r="S21" s="1" t="inlineStr"/>
       <c r="T21" s="1" t="inlineStr">
         <is>
@@ -2580,7 +2660,11 @@
           <t>https://www.tradeindia.com/drx-laboratories-india-inc-34596077/</t>
         </is>
       </c>
-      <c r="R22" s="1" t="inlineStr"/>
+      <c r="R22" s="1" t="inlineStr">
+        <is>
+          <t>201, 2nd Floor, M4 - Block, Gupta Plaza, Opp. Kerala Public School, Vikas Puri, New Delhi, Delhi, 110018, India</t>
+        </is>
+      </c>
       <c r="S22" s="1" t="inlineStr"/>
       <c r="T22" s="1" t="inlineStr">
         <is>
@@ -2687,7 +2771,11 @@
           <t>https://www.tradeindia.com/esel-international-10434316/</t>
         </is>
       </c>
-      <c r="R23" s="1" t="inlineStr"/>
+      <c r="R23" s="1" t="inlineStr">
+        <is>
+          <t>62, Azad Nagar, RamPur Chowk, P.O Industrial Area, Ambala Cantt, Haryana, 133001, India</t>
+        </is>
+      </c>
       <c r="S23" s="1" t="inlineStr"/>
       <c r="T23" s="1" t="inlineStr">
         <is>
@@ -2782,7 +2870,11 @@
           <t>https://www.tradeindia.com/biogenix-inc-pvt-ltd-9029995/</t>
         </is>
       </c>
-      <c r="R24" s="1" t="inlineStr"/>
+      <c r="R24" s="1" t="inlineStr">
+        <is>
+          <t>B19/A , S.I.L Ancillary Estate Amausi Industrial Area, Nadarganj, Lucknow, Uttar Pradesh, 226008, India</t>
+        </is>
+      </c>
       <c r="S24" s="1" t="inlineStr"/>
       <c r="T24" s="1" t="inlineStr">
         <is>
@@ -2883,7 +2975,11 @@
           <t>https://www.tradeindia.com/products/bio-chemistry-analyzer-c2951949.html</t>
         </is>
       </c>
-      <c r="R25" s="1" t="inlineStr"/>
+      <c r="R25" s="1" t="inlineStr">
+        <is>
+          <t>Factory: 70, Edutek House, Main Road Vikaspuri, Industrial Area, Ambala Cantt, Haryana, 133006, India</t>
+        </is>
+      </c>
       <c r="S25" s="1" t="inlineStr"/>
       <c r="T25" s="1" t="inlineStr">
         <is>
@@ -2976,7 +3072,11 @@
           <t>https://www.tradeindia.com/marken-healthtech-limited-32168396/</t>
         </is>
       </c>
-      <c r="R26" s="1" t="inlineStr"/>
+      <c r="R26" s="1" t="inlineStr">
+        <is>
+          <t>Street No.17, Shed No.1, Plot No.93/1, Satpur, Nashik, Maharashtra, 422007, India</t>
+        </is>
+      </c>
       <c r="S26" s="1" t="inlineStr"/>
       <c r="T26" s="1" t="inlineStr">
         <is>
@@ -3078,7 +3178,11 @@
           <t>https://www.tradeindia.com/lifeline-distribution-35105571/</t>
         </is>
       </c>
-      <c r="R27" s="1" t="inlineStr"/>
+      <c r="R27" s="1" t="inlineStr">
+        <is>
+          <t>Owais Abad Near - Kargil House, Bemina, Srinagar, Jammu and Kashmir, 190018, India</t>
+        </is>
+      </c>
       <c r="S27" s="1" t="inlineStr"/>
       <c r="T27" s="1" t="inlineStr">
         <is>
@@ -3137,11 +3241,23 @@
 Hospital Phototherapy Machine: https://www.tradeindia.com/products/hospital-phototherapy-machine-5539798.html</t>
         </is>
       </c>
-      <c r="I28" s="1" t="inlineStr"/>
+      <c r="I28" s="1" t="inlineStr">
+        <is>
+          <t>BENAKA HEALTH CARE</t>
+        </is>
+      </c>
       <c r="J28" s="1" t="inlineStr"/>
       <c r="K28" s="1" t="inlineStr"/>
-      <c r="L28" s="1" t="inlineStr"/>
-      <c r="M28" s="1" t="inlineStr"/>
+      <c r="L28" s="1" t="inlineStr">
+        <is>
+          <t>BENAKA HEALTH CARE</t>
+        </is>
+      </c>
+      <c r="M28" s="1" t="inlineStr">
+        <is>
+          <t>BENAKA HEALTH CARE</t>
+        </is>
+      </c>
       <c r="N28" s="1" t="inlineStr">
         <is>
           <t>Know Us Benaka Health Care (A Division Of Benaka Business Consultancy) is a reputed name in the sector of Syringe Pump, Digital X Ray System, Radiation Protection Products, Ultrasound System, Cardiology System, ECG Machine, Critical Care Product, Patient Monitor, etc. Committed to provide innovative, branded and cost-effective products, we have been offering the best solutions to the medical industry. We have developed a business alliance with the major names of the industry to provide clients with the matchless range. With prompt sales, customer service and service efficiency, we have become the icon of trust for the patrons. Incepted in the year of 2009, we Business Type Manufacturer, Service Provider, Supplier, Trading Company Employee Count 25 Establishment 2009 Working Days Monday To Sunday GST NO 29ADHPC5601P1ZC Payment Mode Online Payments (NEFT/RTGS/IMPS), Cheque/DD, Wallet &amp; UPI Related Products Medical Machinery Price: 5000 INR MOQ - 100 Piece/Pieces Naturoinfra Private Limited Indore, Madhya Pradesh</t>
@@ -3154,7 +3270,11 @@
           <t>https://www.tradeindia.com/products/clover-a1c-hba1c-analyzer-c9513981.html</t>
         </is>
       </c>
-      <c r="R28" s="1" t="inlineStr"/>
+      <c r="R28" s="1" t="inlineStr">
+        <is>
+          <t>B No. 36, 6th Cross, 10th Main, 4th Phase, BSK 3rd Stage, Bengaluru, Karnataka, 560085, India</t>
+        </is>
+      </c>
       <c r="S28" s="1" t="inlineStr"/>
       <c r="T28" s="1" t="inlineStr">
         <is>
@@ -3255,7 +3375,11 @@
           <t>https://www.tradeindia.com/products/semi-automatic-analyzer-c11541591.html</t>
         </is>
       </c>
-      <c r="R29" s="1" t="inlineStr"/>
+      <c r="R29" s="1" t="inlineStr">
+        <is>
+          <t>2/283-1, First Floor, Brindhavan Nagar, Bodipalayam, Seerapalayam, Coimbatore, Tamil Nadu, 641006, India</t>
+        </is>
+      </c>
       <c r="S29" s="1" t="inlineStr"/>
       <c r="T29" s="1" t="inlineStr">
         <is>
@@ -3344,7 +3468,11 @@
           <t>https://www.tradeindia.com/products/clinical-chemistry-analyzer-c11977827.html</t>
         </is>
       </c>
-      <c r="R30" s="1" t="inlineStr"/>
+      <c r="R30" s="1" t="inlineStr">
+        <is>
+          <t>262- N Block, Khidwai Nagar, Kanpur, Uttar Pradesh, 271302, India</t>
+        </is>
+      </c>
       <c r="S30" s="1" t="inlineStr"/>
       <c r="T30" s="1" t="inlineStr">
         <is>
@@ -3439,7 +3567,11 @@
           <t>https://www.tradeindia.com/royal-diagnostic-surgical-29441814/</t>
         </is>
       </c>
-      <c r="R31" s="1" t="inlineStr"/>
+      <c r="R31" s="1" t="inlineStr">
+        <is>
+          <t>Shop No. - A - 165, Ground Floor, Rama Park, Uttam Nagar, Near Dwarka More Station Pillar No. -763, New Delhi, Delhi, 110059, India</t>
+        </is>
+      </c>
       <c r="S31" s="1" t="inlineStr"/>
       <c r="T31" s="1" t="inlineStr">
         <is>
@@ -3511,11 +3643,23 @@
 Labcare Export Digital Dissolved Oxygen Meter: https://www.tradeindia.com/products/labcare-export-digital-dissolved-oxygen-meter-c6741226.html</t>
         </is>
       </c>
-      <c r="I32" s="1" t="inlineStr"/>
+      <c r="I32" s="1" t="inlineStr">
+        <is>
+          <t>LABCARE INSTRUMENTS &amp; INTERNATIONAL SERVICES</t>
+        </is>
+      </c>
       <c r="J32" s="1" t="inlineStr"/>
       <c r="K32" s="1" t="inlineStr"/>
-      <c r="L32" s="1" t="inlineStr"/>
-      <c r="M32" s="1" t="inlineStr"/>
+      <c r="L32" s="1" t="inlineStr">
+        <is>
+          <t>LABCARE INSTRUMENTS &amp; INTERNATIONAL SERVICES</t>
+        </is>
+      </c>
+      <c r="M32" s="1" t="inlineStr">
+        <is>
+          <t>LABCARE INSTRUMENTS &amp; INTERNATIONAL SERVICES</t>
+        </is>
+      </c>
       <c r="N32" s="1" t="inlineStr">
         <is>
           <t>LABCARE INSTRUMENTS &amp; INTERNATIONAL SERVICES , Established in 1986 at Ambala Cantt in Haryana, is a leading service provider of Scientific Instruments in India. LABCARE INSTRUMENTS &amp; INTERNATIONAL SERVICES is one of Trade India's verified and trusted names for listed services. With extensive experience in the field of Scientific Instruments, LABCARE INSTRUMENTS &amp; INTERNATIONAL SERVICES has made a reputed name for itself in the market with satisfactory Double Beam UV VIS Spectrophotometer, 2 Jar Digital Programmable Disintegration Apparatus, For Industrial, ABS Bedside locker, etc. Focusing on a customer-centric approach, LABCARE INSTRUMENTS &amp; INTERNATIONAL SERVICES has a pan-India presence and caters to a huge consumer base throughout the country. Get Scientific Instruments from LABCARE INSTRUMENTS &amp; INTERNATIONAL SERVICES at Trade India quality-assured services. Business Type Exporter, Importer, Manufacturer, Service Provider, Distributor, Supplier, Trading Company Employee Count 45 Establishment 1986 Working Days Monday To Sunday GST NO 06DCLPA2906P1ZF Certification ISO 9001 : 2O15 CERTIFIED CO. CE CERTIFIED Related Products Digital Thermometers - Color: Blue Price: 500.0 INR MOQ - 10 Piece/Pieces Micro Teknik Ambala Cantt, Haryana</t>
@@ -3528,7 +3672,11 @@
           <t>https://www.tradeindia.com/products/labcare-export-auto-biochemistry-analyzer-c6741418.html</t>
         </is>
       </c>
-      <c r="R32" s="1" t="inlineStr"/>
+      <c r="R32" s="1" t="inlineStr">
+        <is>
+          <t>Plant No 18, Near Shiv Mandir, Behind B D Flour Mill, Pragati Vihar, Ambala Cantt, Haryana, 133001, India</t>
+        </is>
+      </c>
       <c r="S32" s="1" t="inlineStr"/>
       <c r="T32" s="1" t="inlineStr">
         <is>
@@ -3622,7 +3770,11 @@
           <t>https://www.tradeindia.com/surgical-wholesale-mart-private-limited-39977655/</t>
         </is>
       </c>
-      <c r="R33" s="1" t="inlineStr"/>
+      <c r="R33" s="1" t="inlineStr">
+        <is>
+          <t>Kh 75/02, Ground Floor, Sri Sai Complex, Kapashera Border, New Delhi, Delhi, 110037, India</t>
+        </is>
+      </c>
       <c r="S33" s="1" t="inlineStr"/>
       <c r="T33" s="1" t="inlineStr">
         <is>
@@ -3685,11 +3837,23 @@
 Mini Urine Analyzer For Medical Use: https://www.tradeindia.com/products/mini-urine-analyzer-for-medical-use-139649.html</t>
         </is>
       </c>
-      <c r="I34" s="1" t="inlineStr"/>
+      <c r="I34" s="1" t="inlineStr">
+        <is>
+          <t>Saaskin Corporation Private Limited.</t>
+        </is>
+      </c>
       <c r="J34" s="1" t="inlineStr"/>
       <c r="K34" s="1" t="inlineStr"/>
-      <c r="L34" s="1" t="inlineStr"/>
-      <c r="M34" s="1" t="inlineStr"/>
+      <c r="L34" s="1" t="inlineStr">
+        <is>
+          <t>Saaskin Corporation Private Limited.</t>
+        </is>
+      </c>
+      <c r="M34" s="1" t="inlineStr">
+        <is>
+          <t>Saaskin Corporation Private Limited.</t>
+        </is>
+      </c>
       <c r="N34" s="1" t="inlineStr">
         <is>
           <t>SAASKIN Corporation Private Limited is a Healthcare and Life Sciences Company that provides Manufacturing , Distribution and Consulting to different markets across globe. Business Type Exporter, Manufacturer, Distributor, Supplier, Trading Company, Wholesaler, Dealer Employee Count 10 Establishment 2011 Working Days Monday To Saturday GST NO 33AAZCS6003M1ZU Payment Mode Telegraphic Transfer (T/T) Certification IS0 9001 : 2015 Related Products Mission U120 Urine Analyzer - Manual Operation, White Color | 120 Tests Per Hour, 2000 Results Memory, Accurate Real-Time Results Price: 30000 INR MOQ - 2 Unit/Units Saaskin Corporation Private Limited. Chennai, Tamil Nadu</t>
@@ -3702,7 +3866,11 @@
           <t>https://www.tradeindia.com/products/acon-mission-u500-urine-analyzer-c9992154.html</t>
         </is>
       </c>
-      <c r="R34" s="1" t="inlineStr"/>
+      <c r="R34" s="1" t="inlineStr">
+        <is>
+          <t>275/184, 1st Floor, Office No: 2, Golden Enclave, Periyar E V R Salai, P.H. Road, Kilpauk, Chennai, Tamil Nadu, 600010, India</t>
+        </is>
+      </c>
       <c r="S34" s="1" t="inlineStr"/>
       <c r="T34" s="1" t="inlineStr">
         <is>
@@ -3806,7 +3974,11 @@
           <t>https://www.tradeindia.com/anvi-diagnostics-61709470/</t>
         </is>
       </c>
-      <c r="R35" s="1" t="inlineStr"/>
+      <c r="R35" s="1" t="inlineStr">
+        <is>
+          <t>No.3, Sai Prasad soc, Singh Est, Rd No 2, Basra Film Studio, Kandivali (E), Mumbai, Maharashtra, 400101, India</t>
+        </is>
+      </c>
       <c r="S35" s="1" t="inlineStr"/>
       <c r="T35" s="1" t="inlineStr">
         <is>
@@ -3908,7 +4080,11 @@
           <t>https://www.tradeindia.com/pc-enterprises-149880218/</t>
         </is>
       </c>
-      <c r="R36" s="1" t="inlineStr"/>
+      <c r="R36" s="1" t="inlineStr">
+        <is>
+          <t>Third Floor, WZ-26, Room No. 50, Village Nangli Zalib, B-1 Janak Puri, New Delhi, Delhi, 110058, India</t>
+        </is>
+      </c>
       <c r="S36" s="1" t="inlineStr"/>
       <c r="T36" s="1" t="inlineStr">
         <is>
@@ -4006,7 +4182,11 @@
           <t>https://www.tradeindia.com/products/vector-v-chem-next-programmable-biochemistry-analyzer-c11872770.html</t>
         </is>
       </c>
-      <c r="R37" s="1" t="inlineStr"/>
+      <c r="R37" s="1" t="inlineStr">
+        <is>
+          <t>Plot No. 24 Shivdashpura, Baullia Lahartara, Varanasi, Uttar Pradesh, 221002, India</t>
+        </is>
+      </c>
       <c r="S37" s="1" t="inlineStr"/>
       <c r="T37" s="1" t="inlineStr">
         <is>
@@ -4102,7 +4282,11 @@
           <t>https://www.tradeindia.com/medica-solutions-26010478/</t>
         </is>
       </c>
-      <c r="R38" s="1" t="inlineStr"/>
+      <c r="R38" s="1" t="inlineStr">
+        <is>
+          <t>E-1018, Saraswati Vihar, Delhi, Delhi, 110034, India</t>
+        </is>
+      </c>
       <c r="S38" s="1" t="inlineStr"/>
       <c r="T38" s="1" t="inlineStr">
         <is>
@@ -4201,7 +4385,11 @@
           <t>https://www.tradeindia.com/products/unikon-gh-hba1c-analyzer-c12491593.html</t>
         </is>
       </c>
-      <c r="R39" s="1" t="inlineStr"/>
+      <c r="R39" s="1" t="inlineStr">
+        <is>
+          <t>Gt Road, Mahesh Pur Industrial Estate, Varanasi, Uttar Pradesh, 221106, India</t>
+        </is>
+      </c>
       <c r="S39" s="1" t="inlineStr"/>
       <c r="T39" s="1" t="inlineStr">
         <is>
@@ -4293,7 +4481,11 @@
           <t>https://www.tradeindia.com/majumder-enterprises-27873101/</t>
         </is>
       </c>
-      <c r="R40" s="1" t="inlineStr"/>
+      <c r="R40" s="1" t="inlineStr">
+        <is>
+          <t>156/33, Bt Road, Dunlop, Northarn Park Road, Near Sonali Cinema Hall, Kolkata, West Bengal, 700108, India</t>
+        </is>
+      </c>
       <c r="S40" s="1" t="inlineStr"/>
       <c r="T40" s="1" t="inlineStr">
         <is>
@@ -4393,7 +4585,11 @@
           <t>https://www.tradeindia.com/testcare-instruments-90878291/</t>
         </is>
       </c>
-      <c r="R41" s="1" t="inlineStr"/>
+      <c r="R41" s="1" t="inlineStr">
+        <is>
+          <t>424/1/93/1-1, Totadamane, Antony street, Mylasandra, Bengaluru, Karnataka, 560068, India</t>
+        </is>
+      </c>
       <c r="S41" s="1" t="inlineStr"/>
       <c r="T41" s="1" t="inlineStr">
         <is>
@@ -4495,7 +4691,11 @@
           <t>https://www.tradeindia.com/darshi-biomedical-5228411/</t>
         </is>
       </c>
-      <c r="R42" s="1" t="inlineStr"/>
+      <c r="R42" s="1" t="inlineStr">
+        <is>
+          <t>5, Laxminagar Corner, Diagnostic Vally, Nana Mava Main Road, Rajkot, Gujarat, 360004, India</t>
+        </is>
+      </c>
       <c r="S42" s="1" t="inlineStr"/>
       <c r="T42" s="1" t="inlineStr">
         <is>
@@ -4586,7 +4786,11 @@
           <t>https://www.tradeindia.com/products/bio-chemistry-analyzer-c2393205.html</t>
         </is>
       </c>
-      <c r="R43" s="1" t="inlineStr"/>
+      <c r="R43" s="1" t="inlineStr">
+        <is>
+          <t>B.O : 5430/3, Anaj Mandi, Science Market, Near Nigar Cinema, R.O : 102-B Ram Nagar, Ambala Cantt, Haryana, 133001, India</t>
+        </is>
+      </c>
       <c r="S43" s="1" t="inlineStr"/>
       <c r="T43" s="1" t="inlineStr">
         <is>
@@ -4680,7 +4884,11 @@
           <t>https://www.tradeindia.com/biotex-life-science-5237582/</t>
         </is>
       </c>
-      <c r="R44" s="1" t="inlineStr"/>
+      <c r="R44" s="1" t="inlineStr">
+        <is>
+          <t>Bhukhand No 48, Khasra No 3, Vikas Nagar, Lucknow, Uttar Pradesh, 226022, India</t>
+        </is>
+      </c>
       <c r="S44" s="1" t="inlineStr"/>
       <c r="T44" s="1" t="inlineStr">
         <is>
@@ -4748,11 +4956,23 @@
 KANAD 8MPC PLUS Clinical Chemistry Analyzer: https://www.tradeindia.com/products/kanad-8mpc-plus-clinical-chemistry-analyzer-6521743.html</t>
         </is>
       </c>
-      <c r="I45" s="1" t="inlineStr"/>
+      <c r="I45" s="1" t="inlineStr">
+        <is>
+          <t>River View Bio Chemical</t>
+        </is>
+      </c>
       <c r="J45" s="1" t="inlineStr"/>
       <c r="K45" s="1" t="inlineStr"/>
-      <c r="L45" s="1" t="inlineStr"/>
-      <c r="M45" s="1" t="inlineStr"/>
+      <c r="L45" s="1" t="inlineStr">
+        <is>
+          <t>River View Bio Chemical</t>
+        </is>
+      </c>
+      <c r="M45" s="1" t="inlineStr">
+        <is>
+          <t>River View Bio Chemical</t>
+        </is>
+      </c>
       <c r="N45" s="1" t="inlineStr">
         <is>
           <t>Welcome to River View Bio Chemical, where precision diagnostics meet dependable supply. As a trusted supplier and trader in the field of laboratory and healthcare solutions, we are committed to empowering diagnostic centers, hospitals, and pathology labs with reliable, high-quality products that support accurate patient care.Our comprehensive product range includes Hematology Analyzers, Edge Lyse, Analyzer Quality Control Kit, Rinse Cleanzer and many more, each carefully sourced to meet the diverse needs of modern diagnostic laboratories. From accurate blood cell analysis to optimal cell lysis, quality control, and analyzer maintenance, our range covers the essential requirements of a well-equipped, efficient laboratory setup.At River View Bio Chemical, we understand that in healthcare, precision is not just important it is essential. That is why we prioritize sourcing q Business Type Supplier, Trading Company Employee Count 6 Establishment 2020 Working Days Monday To Sunday GST NO 21FTKPS4474J1Z6 Payment Mode Online Payments (NEFT/RTGS/IMPS), Cheque/DD, Cash Related Products Clinical Chemistry Analyzer MOQ - 1 Unit/Units River View Bio Chemical Cuttack, Odisha</t>
@@ -4765,7 +4985,11 @@
           <t>https://www.tradeindia.com/products/clinical-chemistry-analyzer-c13295107.html</t>
         </is>
       </c>
-      <c r="R45" s="1" t="inlineStr"/>
+      <c r="R45" s="1" t="inlineStr">
+        <is>
+          <t>Ground Floor, Plot No-161/1751, Khata No-527/356, Unit No-38, Arundoya Nagar, Badambadi, Cuttack, Odisha, 753012, India</t>
+        </is>
+      </c>
       <c r="S45" s="1" t="inlineStr"/>
       <c r="T45" s="1" t="inlineStr">
         <is>
@@ -4872,7 +5096,11 @@
           <t>https://www.tradeindia.com/truvic-healthcare-40589588/</t>
         </is>
       </c>
-      <c r="R46" s="1" t="inlineStr"/>
+      <c r="R46" s="1" t="inlineStr">
+        <is>
+          <t>Flat No 301, 2nd Floor, Second Floor, 1624/a, Lav Kush Purma, Old Shivli Road, Kalyanpur, Kanpur, Uttar Pradesh, 208017, India</t>
+        </is>
+      </c>
       <c r="S46" s="1" t="inlineStr"/>
       <c r="T46" s="1" t="inlineStr">
         <is>
@@ -4962,7 +5190,11 @@
           <t>https://www.tradeindia.com/psj-biochem-diagnostic-pvt-ltd-2376460/</t>
         </is>
       </c>
-      <c r="R47" s="1" t="inlineStr"/>
+      <c r="R47" s="1" t="inlineStr">
+        <is>
+          <t>Khasra No.-1109, Village Rithala, Delhi, Delhi, 110085, India</t>
+        </is>
+      </c>
       <c r="S47" s="1" t="inlineStr"/>
       <c r="T47" s="1" t="inlineStr">
         <is>
@@ -5032,11 +5264,23 @@
 Stable Performance Biochemistry Analyzer: https://www.tradeindia.com/products/stable-performance-biochemistry-analyzer-85757.html</t>
         </is>
       </c>
-      <c r="I48" s="1" t="inlineStr"/>
+      <c r="I48" s="1" t="inlineStr">
+        <is>
+          <t>Martand Medical Services</t>
+        </is>
+      </c>
       <c r="J48" s="1" t="inlineStr"/>
       <c r="K48" s="1" t="inlineStr"/>
-      <c r="L48" s="1" t="inlineStr"/>
-      <c r="M48" s="1" t="inlineStr"/>
+      <c r="L48" s="1" t="inlineStr">
+        <is>
+          <t>Martand Medical Services</t>
+        </is>
+      </c>
+      <c r="M48" s="1" t="inlineStr">
+        <is>
+          <t>Martand Medical Services</t>
+        </is>
+      </c>
       <c r="N48" s="1" t="inlineStr">
         <is>
           <t>Martand Medical Services is a renowned supplier of haematology analyser and other biochemistry analyser and laboratory testing equipment. Established in 2015, we have been providing advanced laboratory testing equipment and analyser including Business Type Exporter, Importer, Distributor, Supplier, Trading Company Employee Count 20 Establishment 2015 Working Days Monday To Sunday Related Products Autoquant 400 Supremus Biochemistry Analyzer - Color: Different Available Price: 1060000 INR MOQ - 5 Unit/Units Drx Laboratories India Inc New Delhi, Delhi</t>
@@ -5049,7 +5293,11 @@
           <t>https://www.tradeindia.com/products/clinical-biochemistry-analyzer-c3774440.html</t>
         </is>
       </c>
-      <c r="R48" s="1" t="inlineStr"/>
+      <c r="R48" s="1" t="inlineStr">
+        <is>
+          <t>Plot No-F-21 Dwarkapuri, Vijay Enclave, Palam Dabri Road, New Delhi, Delhi, 110045, India</t>
+        </is>
+      </c>
       <c r="S48" s="1" t="inlineStr"/>
       <c r="T48" s="1" t="inlineStr">
         <is>
@@ -5118,11 +5366,23 @@
 Neo 4000 Chemistry Analyzer: https://www.tradeindia.com/products/neo-4000-chemistry-analyzer-6469074.html</t>
         </is>
       </c>
-      <c r="I49" s="1" t="inlineStr"/>
+      <c r="I49" s="1" t="inlineStr">
+        <is>
+          <t>U. R. DIAGNOSTICS PVT. LTD.</t>
+        </is>
+      </c>
       <c r="J49" s="1" t="inlineStr"/>
       <c r="K49" s="1" t="inlineStr"/>
-      <c r="L49" s="1" t="inlineStr"/>
-      <c r="M49" s="1" t="inlineStr"/>
+      <c r="L49" s="1" t="inlineStr">
+        <is>
+          <t>U. R. DIAGNOSTICS PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="M49" s="1" t="inlineStr">
+        <is>
+          <t>U. R. DIAGNOSTICS PVT. LTD.</t>
+        </is>
+      </c>
       <c r="N49" s="1" t="inlineStr">
         <is>
           <t>Company Preface To cater to the requirements of pharmaceutical and diagnostic industries, we, U.R. Diagnostics Pvt Ltd., were founded in 2007. Since our foundation, we have remained committed in meeting and exceeding our clients expectations with our entire assortment of quality assured products. Acquisition of immense knowledge and rich experience has assisted in achieving a prominent position of one of the noted importers, traders and suppliers in this competitive industry. Banking on valuable contribution of reliable vendors, we are able to showcase a quality range of products such as Clinical Chemistry (Two Reagents ), Clinical Chemistry ( Single Reagents), Serology ( Including Blood Group Business Type Exporter, Supplier, Trading Company Employee Count 50 Establishment 2001 Related Products Mediray- Semi Auto Biochemistry Analyzer - Material: Plastic Price: 52000 INR MOQ - 1 Piece/Pieces Mediray Healthcare Faridabad, Haryana</t>
@@ -5135,7 +5395,11 @@
           <t>https://www.tradeindia.com/products/clinical-chemistry-analyzer-c720406.html</t>
         </is>
       </c>
-      <c r="R49" s="1" t="inlineStr"/>
+      <c r="R49" s="1" t="inlineStr">
+        <is>
+          <t>204, First Floor, Mittal Shopping Complex, Kulbir Singh Marg, NH-5, N.I.T., Faridabad, Haryana, 121001, India</t>
+        </is>
+      </c>
       <c r="S49" s="1" t="inlineStr"/>
       <c r="T49" s="1" t="inlineStr">
         <is>
@@ -5228,7 +5492,11 @@
           <t>https://www.tradeindia.com/udit-agencies-2241277/</t>
         </is>
       </c>
-      <c r="R50" s="1" t="inlineStr"/>
+      <c r="R50" s="1" t="inlineStr">
+        <is>
+          <t>Plot No-21, Alok Press Chouraha, 1st Floor, Tallaiya Road, Bhopal, Madhya Pradesh, 462001, India</t>
+        </is>
+      </c>
       <c r="S50" s="1" t="inlineStr"/>
       <c r="T50" s="1" t="inlineStr">
         <is>
@@ -5338,7 +5606,11 @@
           <t>https://www.tradeindia.com/didac-international-11078877/</t>
         </is>
       </c>
-      <c r="R51" s="1" t="inlineStr"/>
+      <c r="R51" s="1" t="inlineStr">
+        <is>
+          <t>Regd. Office Address : 507, Shahpuri Tower, C- 58, Janakpuri New Delhi, Delhi, 110058, India</t>
+        </is>
+      </c>
       <c r="S51" s="1" t="inlineStr"/>
       <c r="T51" s="1" t="inlineStr">
         <is>
@@ -5397,11 +5669,23 @@
 PH Analyser: https://www.tradeindia.com/products/ph-analyser-c698762.html</t>
         </is>
       </c>
-      <c r="I52" s="1" t="inlineStr"/>
+      <c r="I52" s="1" t="inlineStr">
+        <is>
+          <t>ELICO LIMITED</t>
+        </is>
+      </c>
       <c r="J52" s="1" t="inlineStr"/>
       <c r="K52" s="1" t="inlineStr"/>
-      <c r="L52" s="1" t="inlineStr"/>
-      <c r="M52" s="1" t="inlineStr"/>
+      <c r="L52" s="1" t="inlineStr">
+        <is>
+          <t>ELICO LIMITED</t>
+        </is>
+      </c>
+      <c r="M52" s="1" t="inlineStr">
+        <is>
+          <t>ELICO LIMITED</t>
+        </is>
+      </c>
       <c r="N52" s="1" t="inlineStr">
         <is>
           <t>ELICO LIMITED , Established in 1959 at Hyderabad in Telangana, is a leading Exporter,Manufacturer,Supplier of Measuring Tools &amp; Equipment in India. ELICO LIMITED is one of Trade India's verified and trusted sellers of listed products. With extensive experience in supplying and trading Clinical Chemistry Analyzers, ELICO LIMITED has made a reputed name for itself in the market with high-quality True Double Beam Atomic Absorption Spectrophotometer, Variable Bandwidth UV VIS Spectrophotometers, Bio Spectrophotometers, etc. Focusing on a customer-centric approach, ELICO LIMITED has a pan-India presence and caters to a huge consumer base throughout the country. Buy Measuring Tools &amp; Equipment in bulk from ELICO LIMITED at Trade India quality-assured products. Business Type Exporter, Manufacturer, Supplier Establishment 1959 Working Days Monday To Sunday GST NO 36AAACE5140L1ZP Certification ISO:9001 Related Products Emp 168 Semi Automatic Chemistry Analyzer Dimension(L*W*H): 420(L) X 310(W) X 152(H) Centimeter (Cm) Vishnu Bio Sciences Hyderabad, Telangana</t>
@@ -5414,7 +5698,11 @@
           <t>https://www.tradeindia.com/products/clinical-chemistry-analyzers-c698758.html</t>
         </is>
       </c>
-      <c r="R52" s="1" t="inlineStr"/>
+      <c r="R52" s="1" t="inlineStr">
+        <is>
+          <t>B-90, A.P.E.I, Sanathnagar Industrial Estate, Hyderabad, Telangana, 500018, India</t>
+        </is>
+      </c>
       <c r="S52" s="1" t="inlineStr"/>
       <c r="T52" s="1" t="inlineStr">
         <is>
@@ -5498,7 +5786,11 @@
           <t>https://www.tradeindia.com/pulse-medical-services-9769229/</t>
         </is>
       </c>
-      <c r="R53" s="1" t="inlineStr"/>
+      <c r="R53" s="1" t="inlineStr">
+        <is>
+          <t>Plot no :- 204/B, Yaddamnagar Colony, Tirumalagiri, Secunderabad, Telangana, 500015, India</t>
+        </is>
+      </c>
       <c r="S53" s="1" t="inlineStr"/>
       <c r="T53" s="1" t="inlineStr">
         <is>
@@ -5561,11 +5853,23 @@
 Sinocare Safe-Accu (Bood Glucose Monitoring System) - Use: Pathlab / Hospital / Clinic: https://www.tradeindia.com/products/sinocare-safe-accu-bood-glucose-monitoring-system-c8639911.html</t>
         </is>
       </c>
-      <c r="I54" s="1" t="inlineStr"/>
+      <c r="I54" s="1" t="inlineStr">
+        <is>
+          <t>Ank Cares Pvt Ltd</t>
+        </is>
+      </c>
       <c r="J54" s="1" t="inlineStr"/>
       <c r="K54" s="1" t="inlineStr"/>
-      <c r="L54" s="1" t="inlineStr"/>
-      <c r="M54" s="1" t="inlineStr"/>
+      <c r="L54" s="1" t="inlineStr">
+        <is>
+          <t>Ank Cares Pvt Ltd</t>
+        </is>
+      </c>
+      <c r="M54" s="1" t="inlineStr">
+        <is>
+          <t>Ank Cares Pvt Ltd</t>
+        </is>
+      </c>
       <c r="N54" s="1" t="inlineStr">
         <is>
           <t>Ank Cares Pvt Ltd , Established in 2015 at Ahmedabad in Gujarat, is a leading Exporter,Manufacturer,Supplier,Trading Company of Personal Safety Equipment in India. Ank Cares Pvt Ltd is one of Trade India's verified and trusted sellers of listed products. With extensive experience in supplying and trading CPC Turbochem Prime Fully Automated Clinical Chemistry Analyzer, Ank Cares Pvt Ltd has made a reputed name for itself in the market with high-quality 100 Bp DNA Ladder 500ul, Abon Multi Drug Test Kit 6 Panel, Abon-Alere Multi Line Drug Screen Test (Urine) 10 Para, etc. Focusing on a customer-centric approach, Ank Cares Pvt Ltd has a pan-India presence and caters to a huge consumer base throughout the country. Buy Personal Safety Equipment in bulk from Ank Cares Pvt Ltd at Trade India quality-assured products. Business Type Exporter, Manufacturer, Supplier, Trading Company Employee Count 25 Establishment 2015 Working Days Monday To Sunday GST NO 24AAQCA0109F1Z4 Payment Mode Cash Advance (CA) Related Products Clinical Chemistry Analyzer - Application: Laboratory Use Price: 105000.00 INR MOQ - 1 Piece/Pieces Microlab Instruments Private Limited Ahmedabad, Gujarat</t>
@@ -5578,7 +5882,11 @@
           <t>https://www.tradeindia.com/products/cpc-turbochem-prime-fully-automated-clinical-chemistry-analyzer-c8761098.html</t>
         </is>
       </c>
-      <c r="R54" s="1" t="inlineStr"/>
+      <c r="R54" s="1" t="inlineStr">
+        <is>
+          <t>Sakar - 5, 103, 1st Floor, Ashram Road, Behind Croma, Ahmedabad, Gujarat, 380001, India</t>
+        </is>
+      </c>
       <c r="S54" s="1" t="inlineStr"/>
       <c r="T54" s="1" t="inlineStr">
         <is>
@@ -5635,11 +5943,23 @@
 Erba Chem 5x Clinical Chemistry Analyzer: https://www.tradeindia.com/products/erba-chem-5x-clinical-chemistry-analyzer-c8379215.html</t>
         </is>
       </c>
-      <c r="I55" s="1" t="inlineStr"/>
+      <c r="I55" s="1" t="inlineStr">
+        <is>
+          <t>HEALTH TECH HEALTHCARE</t>
+        </is>
+      </c>
       <c r="J55" s="1" t="inlineStr"/>
       <c r="K55" s="1" t="inlineStr"/>
-      <c r="L55" s="1" t="inlineStr"/>
-      <c r="M55" s="1" t="inlineStr"/>
+      <c r="L55" s="1" t="inlineStr">
+        <is>
+          <t>HEALTH TECH HEALTHCARE</t>
+        </is>
+      </c>
+      <c r="M55" s="1" t="inlineStr">
+        <is>
+          <t>HEALTH TECH HEALTHCARE</t>
+        </is>
+      </c>
       <c r="N55" s="1" t="inlineStr">
         <is>
           <t>HEALTH TECH HEALTHCARE , Established in 2016 at Delhi in Delhi, is a leading Supplier,Trading Company,Wholesaler of Medical Equipment in India. HEALTH TECH HEALTHCARE is one of Trade India's verified and trusted sellers of listed products. With extensive experience in supplying and trading Star 20 Clinical Chemistry Analyzer, HEALTH TECH HEALTHCARE has made a reputed name for itself in the market with high-quality 60 ABX Micros Analyzer, AD 3200 Plus Hematology Analyzers, Aspen Star 20 Clinical Chemistry Analyzer, etc. Focusing on a customer-centric approach, HEALTH TECH HEALTHCARE has a pan-India presence and caters to a huge consumer base throughout the country. Buy Medical Equipment in bulk from HEALTH TECH HEALTHCARE at Trade India quality-assured products. Business Type Supplier, Trading Company, Wholesaler Employee Count 10 Establishment 2016 Working Days Monday To Saturday GST NO 07BKMPA3262M1Z0 Payment Mode Online Payments (NEFT/RTGS/IMPS) Related Products Full Automatic Chemistry Analyzer - Application: Commercial MOQ - 1 Unit/Units Weldon Biotech (india) Pvt. Ltd. Delhi, Delhi</t>
@@ -5652,7 +5972,11 @@
           <t>https://www.tradeindia.com/products/star-20-clinical-chemistry-analyzer-c9495038.html</t>
         </is>
       </c>
-      <c r="R55" s="1" t="inlineStr"/>
+      <c r="R55" s="1" t="inlineStr">
+        <is>
+          <t>Shop No. 26, Aggrawal City Mall, Rani Bagh, Delhi, Delhi, 110034, India</t>
+        </is>
+      </c>
       <c r="S55" s="1" t="inlineStr"/>
       <c r="T55" s="1" t="inlineStr">
         <is>
@@ -5760,7 +6084,11 @@
           <t>https://www.tradeindia.com/krishco-medical-products-pvt-ltd-3014067/</t>
         </is>
       </c>
-      <c r="R56" s="1" t="inlineStr"/>
+      <c r="R56" s="1" t="inlineStr">
+        <is>
+          <t>No .181, 3rd Main, 5th Cross, Srinivasa Nagar, Bsk 1st Stage, Near Vidyapeeta Circle, Bengaluru, Karnataka, 560050, India</t>
+        </is>
+      </c>
       <c r="S56" s="1" t="inlineStr"/>
       <c r="T56" s="1" t="inlineStr">
         <is>
@@ -5827,11 +6155,23 @@
 Neo 4000 Chemistry Analyzer: https://www.tradeindia.com/products/neo-4000-chemistry-analyzer-6469074.html</t>
         </is>
       </c>
-      <c r="I57" s="1" t="inlineStr"/>
+      <c r="I57" s="1" t="inlineStr">
+        <is>
+          <t>BHARGAVA BIO - MEDICS</t>
+        </is>
+      </c>
       <c r="J57" s="1" t="inlineStr"/>
       <c r="K57" s="1" t="inlineStr"/>
-      <c r="L57" s="1" t="inlineStr"/>
-      <c r="M57" s="1" t="inlineStr"/>
+      <c r="L57" s="1" t="inlineStr">
+        <is>
+          <t>BHARGAVA BIO - MEDICS</t>
+        </is>
+      </c>
+      <c r="M57" s="1" t="inlineStr">
+        <is>
+          <t>BHARGAVA BIO - MEDICS</t>
+        </is>
+      </c>
       <c r="N57" s="1" t="inlineStr">
         <is>
           <t>About Us Based in Madhya Pradesh (India), Bhargava Bio-Medics is a reputed Manufacturer, Supplier, Exporter and Service Provider of medical instruments. Our company was set up in the year 2009 with a mission to be the preferred choice to acquire Electrolyte Analyzer, Laboratory Reagents and similar products in the marketplace. Products we offer to our reputed clients are Biochemistry Analyzer, Cleaner Reagent, Diluent Reagents, Electrolyte Analyzer, Hematology Analyzer, Laboratory Reagents, Lyzer Reagents, Pathology Instruments, Probe Cleaner, etc. We manufacture all these products adhering to the global quality parameters to serve the clients with unmatched quality in all goods. In addition to this, our infrastructure supports us efficiently to fabricate medical equipment with dimensional accuracy. Also, all our products are covered by warranty period which marks our market authenticity. We attain complete client satisfaction by surpassing our performance to keep things balanced. In our endeavor to stand apart from the regular manufacturers in the market, we also provide after sales service to focus on different requirements of our customers. Our technical team provides consultation and give information regarding the product usages. Our customer service comes under our top most priorities to achieve our organizational goals. Business Type Exporter, Manufacturer, Service Provider, Supplier Employee Count 15 Establishment 2009 Working Days Monday To Saturday GST NO 23ATQPB3374D1ZY Payment Mode Cash in Advance (CID) Related Products Chemistry Analyzer - Automated, Discrete, Random Access | 330 Tests/Hour, Refrigerated Reagent Compartment, Bi-Directional LIS Interface, 40 Reagent &amp; Sample Positions, 80 Semi-Permanent Cuvettes, Automatic Cleaning &amp; Collision Protection Bhargava Bio - Medics Ujjain, Madhya Pradesh</t>
@@ -5844,7 +6184,11 @@
           <t>https://www.tradeindia.com/products/semi-auto-chemistry-analyzer-c2840515.html</t>
         </is>
       </c>
-      <c r="R57" s="1" t="inlineStr"/>
+      <c r="R57" s="1" t="inlineStr">
+        <is>
+          <t>Plot No. 16, Bhargava Complex, Varah Mihir Marg, Freeganj, Ujjain, Madhya Pradesh, 456010, India</t>
+        </is>
+      </c>
       <c r="S57" s="1" t="inlineStr"/>
       <c r="T57" s="1" t="inlineStr">
         <is>
@@ -5944,7 +6288,11 @@
           <t>https://www.tradeindia.com/tuljai-labpoint-private-limited-27267008/</t>
         </is>
       </c>
-      <c r="R58" s="1" t="inlineStr"/>
+      <c r="R58" s="1" t="inlineStr">
+        <is>
+          <t>Flat No 001, Konark Appartment, Plot No 151/A, Khare Town, Nagpur, Maharashtra, 440010, India</t>
+        </is>
+      </c>
       <c r="S58" s="1" t="inlineStr"/>
       <c r="T58" s="1" t="inlineStr">
         <is>
@@ -6005,11 +6353,23 @@
 Abbott UROMETER 120 URINE CHEMISTRY ANALYZER: https://www.tradeindia.com/products/abbott-urometer-120-urine-chemistry-analyzer-c9991917.html</t>
         </is>
       </c>
-      <c r="I59" s="1" t="inlineStr"/>
+      <c r="I59" s="1" t="inlineStr">
+        <is>
+          <t>Invitro Biotech Ltd</t>
+        </is>
+      </c>
       <c r="J59" s="1" t="inlineStr"/>
       <c r="K59" s="1" t="inlineStr"/>
-      <c r="L59" s="1" t="inlineStr"/>
-      <c r="M59" s="1" t="inlineStr"/>
+      <c r="L59" s="1" t="inlineStr">
+        <is>
+          <t>Invitro Biotech Ltd</t>
+        </is>
+      </c>
+      <c r="M59" s="1" t="inlineStr">
+        <is>
+          <t>Invitro Biotech Ltd</t>
+        </is>
+      </c>
       <c r="N59" s="1" t="inlineStr">
         <is>
           <t>Laboratory Equipment &amp; Reagents - accuracy, precision and reliabilityEstablished in the year 2002, Invitro Biotech Ltd. is a renowned manufacturer, supplier and exporter of a wide array of laboratory products with application in clinical, biotech, research and college laboratories. Laboratories can avail from us microprocessor based Digital Colorimeter, Chemistry Analyzer, Hemoglobin Meter, Single and Multi Channel Micropipettes, various models of regular Lab Centrifuge, Lab Accessories Clinical Chemistry Reagents, and many more. Manufactured as per best industrial practices and norms, our products are known for best quality &amp; standards. Our quality management systems are ISO 9001: 2008 certified and SOPs are laid out for Business Type Exporter, Manufacturer, Supplier Employee Count 20 Establishment 2002 Working Days Monday To Sunday GST NO 36AAACI8264R1ZU Related Products Emp 168 Semi Automatic Chemistry Analyzer Dimension(L*W*H): 420(L) X 310(W) X 152(H) Centimeter (Cm) Vishnu Bio Sciences Hyderabad, Telangana</t>
@@ -6022,7 +6382,11 @@
           <t>https://www.tradeindia.com/products/clinical-chemistry-analyzer-c2000683.html</t>
         </is>
       </c>
-      <c r="R59" s="1" t="inlineStr"/>
+      <c r="R59" s="1" t="inlineStr">
+        <is>
+          <t>Building Number- 177, Prasanth Nagar, Industrial Area, Kukatpally, Hyderabad, Telangana, 500072, India</t>
+        </is>
+      </c>
       <c r="S59" s="1" t="inlineStr"/>
       <c r="T59" s="1" t="inlineStr">
         <is>
@@ -6085,11 +6449,23 @@
 Kanad Semi Auto Clinical Analyser 6FX: https://www.tradeindia.com/products/kanad-semi-auto-clinical-analyser-6fx-c8379206.html</t>
         </is>
       </c>
-      <c r="I60" s="1" t="inlineStr"/>
+      <c r="I60" s="1" t="inlineStr">
+        <is>
+          <t>CLINDIAG INDIA (a division of Monash International)</t>
+        </is>
+      </c>
       <c r="J60" s="1" t="inlineStr"/>
       <c r="K60" s="1" t="inlineStr"/>
-      <c r="L60" s="1" t="inlineStr"/>
-      <c r="M60" s="1" t="inlineStr"/>
+      <c r="L60" s="1" t="inlineStr">
+        <is>
+          <t>CLINDIAG INDIA (a division of Monash International)</t>
+        </is>
+      </c>
+      <c r="M60" s="1" t="inlineStr">
+        <is>
+          <t>CLINDIAG INDIA (a division of Monash International)</t>
+        </is>
+      </c>
       <c r="N60" s="1" t="inlineStr">
         <is>
           <t>Clindiag is a newly founded company by a group of experienced international specialists, located in Belgium, the heart of Europe. Having the many years of experience of our engineers, Clindiag provides a full range of customer orientated, innovative products to the clinical laboratory world market.By producing high quality products combined with an excellent service to our customers, Clindiag is planning to become an important player in the clinical laboratory market over the next few years... 25792_ 25792_HOME2.jpg Clindiag India a divis Business Type Exporter, Service Provider, Distributor, Supplier, Trading Company Establishment 1998 Working Days Monday To Saturday Related Products Fully Automated Biochemistry Analyzer - Color: White Price: 300000 INR MOQ - 1 Unit/Units Medica Solutions Delhi, Delhi</t>
@@ -6102,7 +6478,11 @@
           <t>https://www.tradeindia.com/products/semi-automatic-clinical-analyzer-c478186.html</t>
         </is>
       </c>
-      <c r="R60" s="1" t="inlineStr"/>
+      <c r="R60" s="1" t="inlineStr">
+        <is>
+          <t>B-1177-78, G.D.Colony, Mayur Vihar, Phase-III, Delhi, Delhi, 110096, India</t>
+        </is>
+      </c>
       <c r="S60" s="1" t="inlineStr"/>
       <c r="T60" s="1" t="inlineStr">
         <is>
@@ -6172,11 +6552,23 @@
 Tissue Stabilizer: https://www.tradeindia.com/products/tissue-stabilizer-8317845.html</t>
         </is>
       </c>
-      <c r="I61" s="1" t="inlineStr"/>
+      <c r="I61" s="1" t="inlineStr">
+        <is>
+          <t>PIKA MEDICAL (P) LTD.</t>
+        </is>
+      </c>
       <c r="J61" s="1" t="inlineStr"/>
       <c r="K61" s="1" t="inlineStr"/>
-      <c r="L61" s="1" t="inlineStr"/>
-      <c r="M61" s="1" t="inlineStr"/>
+      <c r="L61" s="1" t="inlineStr">
+        <is>
+          <t>PIKA MEDICAL (P) LTD.</t>
+        </is>
+      </c>
+      <c r="M61" s="1" t="inlineStr">
+        <is>
+          <t>PIKA MEDICAL (P) LTD.</t>
+        </is>
+      </c>
       <c r="N61" s="1" t="inlineStr">
         <is>
           <t>Founded in the year of 1994, we, Pika Medical (P) Limited, have established ourselves as a renowned Supplier and Trader of an unmatched array of medical equipment which includes Karl Storz Endoscopic Equipment, Endoscopic Medical Equipment, Inventis Audiometers, Inventi Tympanometers, Emed Electrocautery Unit, Middle Ear Analyzers and more. These are procured from a trusted base of experienced vendors who manufacture these products using licensed components. Our entire range of hospital equipment has an enormous market demand owing to their steady performance, long operational life, portable design, accurate information, low power consumption etc. We have an in-house fully Business Type Distributor, Supplier, Trading Company Employee Count 19 Establishment 1994 Working Days Monday To Sunday GST NO 29AAACP8185A1ZD Related Products Medical Diagnostic Equipments Geneva Industries Ltd. Bengaluru, Karnataka</t>
@@ -6189,7 +6581,11 @@
           <t>https://www.tradeindia.com/products/clinical-middle-ear-analyzer-c4413153.html</t>
         </is>
       </c>
-      <c r="R61" s="1" t="inlineStr"/>
+      <c r="R61" s="1" t="inlineStr">
+        <is>
+          <t>1212B, Mittal Tower, 6 M.G. Road, Bengaluru, Karnataka, 560001, India</t>
+        </is>
+      </c>
       <c r="S61" s="1" t="inlineStr"/>
       <c r="T61" s="1" t="inlineStr">
         <is>
@@ -6258,11 +6654,23 @@
 Biochemistry Analyzer: https://www.tradeindia.com/products/biochemistry-analyzer-c4729653.html</t>
         </is>
       </c>
-      <c r="I62" s="1" t="inlineStr"/>
+      <c r="I62" s="1" t="inlineStr">
+        <is>
+          <t>RADIANT BIOMED PVT. LTD.</t>
+        </is>
+      </c>
       <c r="J62" s="1" t="inlineStr"/>
       <c r="K62" s="1" t="inlineStr"/>
-      <c r="L62" s="1" t="inlineStr"/>
-      <c r="M62" s="1" t="inlineStr"/>
+      <c r="L62" s="1" t="inlineStr">
+        <is>
+          <t>RADIANT BIOMED PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="M62" s="1" t="inlineStr">
+        <is>
+          <t>RADIANT BIOMED PVT. LTD.</t>
+        </is>
+      </c>
       <c r="N62" s="1" t="inlineStr">
         <is>
           <t>We prefer inquiries from north India only, like Delhi NCR, Rajasthan, UP, Punjab etc. Established in 2011, we, RADIANT BIOMED PVT. LTD, are a renowned importer, supplier and wholesaler/distributor of Laboratory Equipment such as, Hematology Analyzer, (Blood Cell Counter) and Biochemistry Analyzer. We are offering these products to several hospitals, laboratories and health clinics.All our laboratory equipments are of reputed brands and appreciated for their advanced technology. They are reliable and affordable. They provide accurate results to the doctors and help them to diagnose the patient's disease Business Type Importer, Distributor, Supplier Employee Count 8 Establishment 2011 Working Days Monday To Sunday GST NO 07AAGCR7834J1ZY Related Products Autoquant 400 Supremus Biochemistry Analyzer - Color: Different Available Price: 1060000 INR MOQ - 5 Unit/Units Drx Laboratories India Inc New Delhi, Delhi</t>
@@ -6275,7 +6683,11 @@
           <t>https://www.tradeindia.com/products/clinical-biochemistry-analyzer-c3310429.html</t>
         </is>
       </c>
-      <c r="R62" s="1" t="inlineStr"/>
+      <c r="R62" s="1" t="inlineStr">
+        <is>
+          <t>C-159, 1st Floor, Main Road, Naraina Industrial Area Phase - 1, New Delhi, Delhi, 110028, India</t>
+        </is>
+      </c>
       <c r="S62" s="1" t="inlineStr"/>
       <c r="T62" s="1" t="inlineStr">
         <is>
@@ -6346,11 +6758,23 @@
 Biochemistry Analyzer: https://www.tradeindia.com/products/biochemistry-analyzer-c6350610.html</t>
         </is>
       </c>
-      <c r="I63" s="1" t="inlineStr"/>
+      <c r="I63" s="1" t="inlineStr">
+        <is>
+          <t>PRANA'S 4 EVER DIAGNOSTICS</t>
+        </is>
+      </c>
       <c r="J63" s="1" t="inlineStr"/>
       <c r="K63" s="1" t="inlineStr"/>
-      <c r="L63" s="1" t="inlineStr"/>
-      <c r="M63" s="1" t="inlineStr"/>
+      <c r="L63" s="1" t="inlineStr">
+        <is>
+          <t>PRANA'S 4 EVER DIAGNOSTICS</t>
+        </is>
+      </c>
+      <c r="M63" s="1" t="inlineStr">
+        <is>
+          <t>PRANA'S 4 EVER DIAGNOSTICS</t>
+        </is>
+      </c>
       <c r="N63" s="1" t="inlineStr">
         <is>
           <t>We are the right place for the customer who in looking for and authentic firm for buying the top-class and items like Activated Clotting Time Machine, Elisa Readwell Touch, Prietest Easylab Biochemistry Analyzer, Wash Well Strip etc. Our company named Prana's 4 Ever Diagnostics is a one-stop destinations and a leading supplier, wholesaler and trader of wide array of products. Since our foundation in 2014, we have become one of the favourite choice of the customers and have made a vast client base form various ends of the country. We feel beaming to see that our attempts are being successful, as we are getting positive reviews from our customer in majority. We promise that in future too, we will stay loyal in our business deals and satisfy the needs of the customers. Give us a chance to serve, we Business Type Distributor, Supplier, Trading Company Employee Count 5 Establishment 2014 Working Days Monday To Sunday GST NO 27ALTPS3435P1Z3 Related Products Agappe Mispa Viva Infinity Diagnochem Mumbai, Maharashtra</t>
@@ -6363,7 +6787,11 @@
           <t>https://www.tradeindia.com/products/biochemistry-analyzer-c4729653.html</t>
         </is>
       </c>
-      <c r="R63" s="1" t="inlineStr"/>
+      <c r="R63" s="1" t="inlineStr">
+        <is>
+          <t>J-11, Nancy Cottage, Nancy Colony, Near ST Bus Depot, Borivali (E), Mumbai, Maharashtra, 400066, India</t>
+        </is>
+      </c>
       <c r="S63" s="1" t="inlineStr"/>
       <c r="T63" s="1" t="inlineStr">
         <is>
@@ -6432,11 +6860,23 @@
 TDS Conductivity Meter with High Accuracy: https://www.tradeindia.com/products/tds-conductivity-meter-with-high-accuracy-7182450.html</t>
         </is>
       </c>
-      <c r="I64" s="1" t="inlineStr"/>
+      <c r="I64" s="1" t="inlineStr">
+        <is>
+          <t>ACCUSTER TECHNOLOGIES PVT. LTD.</t>
+        </is>
+      </c>
       <c r="J64" s="1" t="inlineStr"/>
       <c r="K64" s="1" t="inlineStr"/>
-      <c r="L64" s="1" t="inlineStr"/>
-      <c r="M64" s="1" t="inlineStr"/>
+      <c r="L64" s="1" t="inlineStr">
+        <is>
+          <t>ACCUSTER TECHNOLOGIES PVT. LTD.</t>
+        </is>
+      </c>
+      <c r="M64" s="1" t="inlineStr">
+        <is>
+          <t>ACCUSTER TECHNOLOGIES PVT. LTD.</t>
+        </is>
+      </c>
       <c r="N64" s="1" t="inlineStr">
         <is>
           <t>ACCUSTER TECHNOLOGIES PVT. LTD. , Established in 2009 at Gurugram in Haryana, is a leading service provider of Laboratory Glassware &amp; Equipment in India. ACCUSTER TECHNOLOGIES PVT. LTD. is one of Trade India's verified and trusted names for listed services. With extensive experience in the field of Laboratory Glassware &amp; Equipment, ACCUSTER TECHNOLOGIES PVT. LTD. has made a reputed name for itself in the market with satisfactory Accurate All, Accurate-8, Autoclave, etc. Focusing on a customer-centric approach, ACCUSTER TECHNOLOGIES PVT. LTD. has a pan-India presence and caters to a huge consumer base throughout the country. Get Laboratory Glassware &amp; Equipment from ACCUSTER TECHNOLOGIES PVT. LTD. at Trade India quality-assured services. Business Type Exporter, Manufacturer, Service Provider, Supplier, Trading Company Employee Count 100 Establishment 2009 Working Days Monday To Sunday GST NO 06AABCU0629H1ZK Related Products Chemistry Analyzers Accuster Technologies Pvt. Ltd. Gurugram, Haryana</t>
@@ -6449,7 +6889,11 @@
           <t>https://www.tradeindia.com/products/chemistry-analyzers-c3905784.html</t>
         </is>
       </c>
-      <c r="R64" s="1" t="inlineStr"/>
+      <c r="R64" s="1" t="inlineStr">
+        <is>
+          <t>Plot No. 758, First Floor Sector 47, Near Bharat Petroleum, Gurugram, Haryana, 122018, India</t>
+        </is>
+      </c>
       <c r="S64" s="1" t="inlineStr"/>
       <c r="T64" s="1" t="inlineStr">
         <is>

</xml_diff>